<commit_message>
Updates scenario specific data and solver options
Refactors scenario price reading to handle separate price sheets for import and manufacturing costs for different technologies. It also enhances solver configuration by adding detailed logging for binary variables and limiting solutions.

- Modifies the price reading logic to accommodate separate excel sheets dedicated to manufacturing and import costs for each technology
- Enables detailed logging for binary variables in the solver.
- Fixes a condition in the decommissioned capacity rule in the scrap extension.
- Adjusts the cost reduction for wind technologies.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6FA9B08-323D-4013-A62E-287D8C61B49C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF064698-A154-4B25-BE65-5FA2D3540356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="67080" yWindow="-1935" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
@@ -860,7 +860,7 @@
         <v>414000</v>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F2">
         <v>1775265.6417320003</v>
@@ -869,22 +869,22 @@
         <v>2337972.5216000001</v>
       </c>
       <c r="H2">
-        <v>9999999</v>
-      </c>
-      <c r="I2" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
       </c>
       <c r="J2">
         <v>1052044.8400000001</v>
       </c>
       <c r="K2">
-        <v>1673707.7000000002</v>
+        <v>1673707.7</v>
       </c>
       <c r="L2">
-        <v>9999999</v>
-      </c>
-      <c r="M2" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
       </c>
       <c r="N2">
         <v>90210</v>
@@ -913,7 +913,7 @@
         <v>414000</v>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F3">
         <v>1722922.372057667</v>
@@ -922,10 +922,10 @@
         <v>2318026.381866667</v>
       </c>
       <c r="H3">
-        <v>9999999</v>
-      </c>
-      <c r="I3" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
       </c>
       <c r="J3">
         <v>1042480.7960000001</v>
@@ -934,10 +934,10 @@
         <v>1660955.6413333334</v>
       </c>
       <c r="L3">
-        <v>9999999</v>
-      </c>
-      <c r="M3" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
       </c>
       <c r="N3">
         <v>88856.85</v>
@@ -966,7 +966,7 @@
         <v>414000</v>
       </c>
       <c r="E4">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F4">
         <v>1670579.1023833335</v>
@@ -975,10 +975,10 @@
         <v>2298080.2421333333</v>
       </c>
       <c r="H4">
-        <v>9999999</v>
-      </c>
-      <c r="I4" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
       </c>
       <c r="J4">
         <v>1032916.7520000001</v>
@@ -987,10 +987,10 @@
         <v>1648203.5826666667</v>
       </c>
       <c r="L4">
-        <v>9999999</v>
-      </c>
-      <c r="M4" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
       </c>
       <c r="N4">
         <v>87523</v>
@@ -1019,7 +1019,7 @@
         <v>414000</v>
       </c>
       <c r="E5">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F5">
         <v>1618235.832709</v>
@@ -1028,10 +1028,10 @@
         <v>2278134.1023999997</v>
       </c>
       <c r="H5">
-        <v>9999999</v>
-      </c>
-      <c r="I5" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
       </c>
       <c r="J5">
         <v>1023352.708</v>
@@ -1040,10 +1040,10 @@
         <v>1635451.524</v>
       </c>
       <c r="L5">
-        <v>9999999</v>
-      </c>
-      <c r="M5" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
       </c>
       <c r="N5">
         <v>86209.15</v>
@@ -1072,7 +1072,7 @@
         <v>414000</v>
       </c>
       <c r="E6">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F6">
         <v>1565892.5630346665</v>
@@ -1081,10 +1081,10 @@
         <v>2258187.9626666661</v>
       </c>
       <c r="H6">
-        <v>9999999</v>
-      </c>
-      <c r="I6" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
       </c>
       <c r="J6">
         <v>1013788.6639999999</v>
@@ -1093,10 +1093,10 @@
         <v>1622699.4653333335</v>
       </c>
       <c r="L6">
-        <v>9999999</v>
-      </c>
-      <c r="M6" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
       </c>
       <c r="N6">
         <v>84915.01</v>
@@ -1125,7 +1125,7 @@
         <v>414000</v>
       </c>
       <c r="E7">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F7">
         <v>1513549.293360333</v>
@@ -1134,10 +1134,10 @@
         <v>2238241.8229333302</v>
       </c>
       <c r="H7">
-        <v>9999999</v>
-      </c>
-      <c r="I7" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
       </c>
       <c r="J7">
         <v>1004224.62</v>
@@ -1146,10 +1146,10 @@
         <v>1609947.4066666667</v>
       </c>
       <c r="L7">
-        <v>9999999</v>
-      </c>
-      <c r="M7" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
       </c>
       <c r="N7">
         <v>83640.289999999994</v>
@@ -1178,7 +1178,7 @@
         <v>414000</v>
       </c>
       <c r="E8">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F8">
         <v>1461206.0236859999</v>
@@ -1187,10 +1187,10 @@
         <v>2218295.6831999999</v>
       </c>
       <c r="H8">
-        <v>9999999</v>
-      </c>
-      <c r="I8" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
       </c>
       <c r="J8">
         <v>994660.57600000012</v>
@@ -1199,10 +1199,10 @@
         <v>1597195.3480000002</v>
       </c>
       <c r="L8">
-        <v>9999999</v>
-      </c>
-      <c r="M8" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
       </c>
       <c r="N8">
         <v>82384.69</v>
@@ -1231,7 +1231,7 @@
         <v>414000</v>
       </c>
       <c r="E9">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F9">
         <v>1444015.15599508</v>
@@ -1240,10 +1240,10 @@
         <v>2205259.4561600001</v>
       </c>
       <c r="H9">
-        <v>9999999</v>
-      </c>
-      <c r="I9" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
       </c>
       <c r="J9">
         <v>992747.76720000012</v>
@@ -1252,10 +1252,10 @@
         <v>1594326.1348000003</v>
       </c>
       <c r="L9">
-        <v>9999999</v>
-      </c>
-      <c r="M9" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
       </c>
       <c r="N9">
         <v>81147.92</v>
@@ -1284,7 +1284,7 @@
         <v>414000</v>
       </c>
       <c r="E10">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F10">
         <v>1426824.2883041599</v>
@@ -1293,10 +1293,10 @@
         <v>2192223.2291199998</v>
       </c>
       <c r="H10">
-        <v>9999999</v>
-      </c>
-      <c r="I10" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
       </c>
       <c r="J10">
         <v>990834.9584</v>
@@ -1305,10 +1305,10 @@
         <v>1591456.9216000002</v>
       </c>
       <c r="L10">
-        <v>9999999</v>
-      </c>
-      <c r="M10" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
       </c>
       <c r="N10">
         <v>79929.7</v>
@@ -1337,7 +1337,7 @@
         <v>414000</v>
       </c>
       <c r="E11">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F11">
         <v>1409633.42061324</v>
@@ -1346,10 +1346,10 @@
         <v>2179187.0020799995</v>
       </c>
       <c r="H11">
-        <v>9999999</v>
-      </c>
-      <c r="I11" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
       </c>
       <c r="J11">
         <v>988922.1496</v>
@@ -1358,10 +1358,10 @@
         <v>1588587.7084000004</v>
       </c>
       <c r="L11">
-        <v>9999999</v>
-      </c>
-      <c r="M11" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
       </c>
       <c r="N11">
         <v>78729.759999999995</v>
@@ -1390,7 +1390,7 @@
         <v>414000</v>
       </c>
       <c r="E12">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F12">
         <v>1392442.5529223196</v>
@@ -1399,10 +1399,10 @@
         <v>2166150.7750399997</v>
       </c>
       <c r="H12">
-        <v>9999999</v>
-      </c>
-      <c r="I12" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
       </c>
       <c r="J12">
         <v>987009.34079999989</v>
@@ -1411,10 +1411,10 @@
         <v>1585718.4952000002</v>
       </c>
       <c r="L12">
-        <v>9999999</v>
-      </c>
-      <c r="M12" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
       </c>
       <c r="N12">
         <v>77547.820000000007</v>
@@ -1443,7 +1443,7 @@
         <v>414000</v>
       </c>
       <c r="E13">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F13">
         <v>1375251.6852313997</v>
@@ -1452,10 +1452,10 @@
         <v>2153114.5479999995</v>
       </c>
       <c r="H13">
-        <v>9999999</v>
-      </c>
-      <c r="I13" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
       </c>
       <c r="J13">
         <v>985096.53199999989</v>
@@ -1464,10 +1464,10 @@
         <v>1582849.2820000004</v>
       </c>
       <c r="L13">
-        <v>9999999</v>
-      </c>
-      <c r="M13" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
       </c>
       <c r="N13">
         <v>76383.600000000006</v>
@@ -1496,7 +1496,7 @@
         <v>414000</v>
       </c>
       <c r="E14">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F14">
         <v>1358060.8175404796</v>
@@ -1505,10 +1505,10 @@
         <v>2140078.3209599997</v>
       </c>
       <c r="H14">
-        <v>9999999</v>
-      </c>
-      <c r="I14" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
       </c>
       <c r="J14">
         <v>983183.72319999977</v>
@@ -1517,10 +1517,10 @@
         <v>1579980.0688000005</v>
       </c>
       <c r="L14">
-        <v>9999999</v>
-      </c>
-      <c r="M14" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M14">
+        <v>1</v>
       </c>
       <c r="N14">
         <v>75236.84</v>
@@ -1549,7 +1549,7 @@
         <v>414000</v>
       </c>
       <c r="E15">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F15">
         <v>1340869.9498495597</v>
@@ -1558,10 +1558,10 @@
         <v>2127042.0939199994</v>
       </c>
       <c r="H15">
-        <v>9999999</v>
-      </c>
-      <c r="I15" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
       </c>
       <c r="J15">
         <v>981270.91439999978</v>
@@ -1570,10 +1570,10 @@
         <v>1577110.8556000004</v>
       </c>
       <c r="L15">
-        <v>9999999</v>
-      </c>
-      <c r="M15" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M15">
+        <v>1</v>
       </c>
       <c r="N15">
         <v>74107.289999999994</v>
@@ -1602,7 +1602,7 @@
         <v>414000</v>
       </c>
       <c r="E16">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F16">
         <v>1323679.0821586396</v>
@@ -1611,10 +1611,10 @@
         <v>2114005.8668799992</v>
       </c>
       <c r="H16">
-        <v>9999999</v>
-      </c>
-      <c r="I16" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
       </c>
       <c r="J16">
         <v>979358.10559999966</v>
@@ -1623,10 +1623,10 @@
         <v>1574241.6424000005</v>
       </c>
       <c r="L16">
-        <v>9999999</v>
-      </c>
-      <c r="M16" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
       </c>
       <c r="N16">
         <v>72994.679999999993</v>
@@ -1655,7 +1655,7 @@
         <v>414000</v>
       </c>
       <c r="E17">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F17">
         <v>1306488.2144677194</v>
@@ -1664,10 +1664,10 @@
         <v>2100969.6398399994</v>
       </c>
       <c r="H17">
-        <v>9999999</v>
-      </c>
-      <c r="I17" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
       </c>
       <c r="J17">
         <v>977445.29679999966</v>
@@ -1676,10 +1676,10 @@
         <v>1571372.4292000004</v>
       </c>
       <c r="L17">
-        <v>9999999</v>
-      </c>
-      <c r="M17" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M17">
+        <v>1</v>
       </c>
       <c r="N17">
         <v>71898.759999999995</v>
@@ -1708,7 +1708,7 @@
         <v>414000</v>
       </c>
       <c r="E18">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F18">
         <v>1288027.7959324</v>
@@ -1717,10 +1717,10 @@
         <v>2087933.4128</v>
       </c>
       <c r="H18">
-        <v>9999999</v>
-      </c>
-      <c r="I18" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
       </c>
       <c r="J18">
         <v>975532.48799999955</v>
@@ -1729,10 +1729,10 @@
         <v>1568503.2160000005</v>
       </c>
       <c r="L18">
-        <v>9999999</v>
-      </c>
-      <c r="M18" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M18">
+        <v>1</v>
       </c>
       <c r="N18">
         <v>70819.28</v>
@@ -1761,7 +1761,7 @@
         <v>414000</v>
       </c>
       <c r="E19">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F19">
         <v>1288154.7510168403</v>
@@ -1770,10 +1770,10 @@
         <v>2076927.41784</v>
       </c>
       <c r="H19">
-        <v>9999999</v>
-      </c>
-      <c r="I19" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I19">
+        <v>1</v>
       </c>
       <c r="J19">
         <v>973619.67919999966</v>
@@ -1782,10 +1782,10 @@
         <v>1565634.0028000006</v>
       </c>
       <c r="L19">
-        <v>9999999</v>
-      </c>
-      <c r="M19" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M19">
+        <v>1</v>
       </c>
       <c r="N19">
         <v>69755.990000000005</v>
@@ -1814,7 +1814,7 @@
         <v>414000</v>
       </c>
       <c r="E20">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F20">
         <v>1288281.7061012802</v>
@@ -1823,10 +1823,10 @@
         <v>2065921.4228800002</v>
       </c>
       <c r="H20">
-        <v>9999999</v>
-      </c>
-      <c r="I20" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
       </c>
       <c r="J20">
         <v>971706.87039999955</v>
@@ -1835,10 +1835,10 @@
         <v>1562764.7896000005</v>
       </c>
       <c r="L20">
-        <v>9999999</v>
-      </c>
-      <c r="M20" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M20">
+        <v>1</v>
       </c>
       <c r="N20">
         <v>68708.649999999994</v>
@@ -1867,7 +1867,7 @@
         <v>414000</v>
       </c>
       <c r="E21">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F21">
         <v>1288408.6611857202</v>
@@ -1876,10 +1876,10 @@
         <v>2054915.4279200002</v>
       </c>
       <c r="H21">
-        <v>9999999</v>
-      </c>
-      <c r="I21" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
       </c>
       <c r="J21">
         <v>969794.06159999955</v>
@@ -1888,10 +1888,10 @@
         <v>1559895.5764000006</v>
       </c>
       <c r="L21">
-        <v>9999999</v>
-      </c>
-      <c r="M21" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M21">
+        <v>1</v>
       </c>
       <c r="N21">
         <v>67677.02</v>
@@ -1920,7 +1920,7 @@
         <v>414000</v>
       </c>
       <c r="E22">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F22">
         <v>1288535.6162701603</v>
@@ -1929,10 +1929,10 @@
         <v>2043909.4329600004</v>
       </c>
       <c r="H22">
-        <v>9999999</v>
-      </c>
-      <c r="I22" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I22">
+        <v>1</v>
       </c>
       <c r="J22">
         <v>967881.25279999943</v>
@@ -1941,10 +1941,10 @@
         <v>1557026.3632000005</v>
       </c>
       <c r="L22">
-        <v>9999999</v>
-      </c>
-      <c r="M22" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M22">
+        <v>1</v>
       </c>
       <c r="N22">
         <v>66660.86</v>
@@ -1973,7 +1973,7 @@
         <v>414000</v>
       </c>
       <c r="E23">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F23">
         <v>1288662.5713546001</v>
@@ -1982,10 +1982,10 @@
         <v>2032903.4380000005</v>
       </c>
       <c r="H23">
-        <v>9999999</v>
-      </c>
-      <c r="I23" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I23">
+        <v>1</v>
       </c>
       <c r="J23">
         <v>965968.44399999944</v>
@@ -1994,10 +1994,10 @@
         <v>1554157.1500000006</v>
       </c>
       <c r="L23">
-        <v>9999999</v>
-      </c>
-      <c r="M23" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M23">
+        <v>1</v>
       </c>
       <c r="N23">
         <v>65659.95</v>
@@ -2026,7 +2026,7 @@
         <v>414000</v>
       </c>
       <c r="E24">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F24">
         <v>1288789.5264390404</v>
@@ -2035,10 +2035,10 @@
         <v>2021897.4430400007</v>
       </c>
       <c r="H24">
-        <v>9999999</v>
-      </c>
-      <c r="I24" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
       </c>
       <c r="J24">
         <v>964055.63519999932</v>
@@ -2047,10 +2047,10 @@
         <v>1551287.9368000007</v>
       </c>
       <c r="L24">
-        <v>9999999</v>
-      </c>
-      <c r="M24" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M24">
+        <v>1</v>
       </c>
       <c r="N24">
         <v>64674.05</v>
@@ -2079,7 +2079,7 @@
         <v>414000</v>
       </c>
       <c r="E25">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F25">
         <v>1288916.4815234803</v>
@@ -2088,10 +2088,10 @@
         <v>2010891.4480800009</v>
       </c>
       <c r="H25">
-        <v>9999999</v>
-      </c>
-      <c r="I25" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I25">
+        <v>1</v>
       </c>
       <c r="J25">
         <v>962142.82639999932</v>
@@ -2100,10 +2100,10 @@
         <v>1548418.7236000006</v>
       </c>
       <c r="L25">
-        <v>9999999</v>
-      </c>
-      <c r="M25" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M25">
+        <v>1</v>
       </c>
       <c r="N25">
         <v>63702.94</v>
@@ -2132,7 +2132,7 @@
         <v>414000</v>
       </c>
       <c r="E26">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F26">
         <v>1289043.4366079206</v>
@@ -2141,10 +2141,10 @@
         <v>1999885.4531200009</v>
       </c>
       <c r="H26">
-        <v>9999999</v>
-      </c>
-      <c r="I26" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I26">
+        <v>1</v>
       </c>
       <c r="J26">
         <v>960230.01759999921</v>
@@ -2153,10 +2153,10 @@
         <v>1545549.5104000007</v>
       </c>
       <c r="L26">
-        <v>9999999</v>
-      </c>
-      <c r="M26" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M26">
+        <v>1</v>
       </c>
       <c r="N26">
         <v>62746.400000000001</v>
@@ -2185,7 +2185,7 @@
         <v>414000</v>
       </c>
       <c r="E27">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F27">
         <v>1289170.3916923604</v>
@@ -2194,10 +2194,10 @@
         <v>1988879.4581600011</v>
       </c>
       <c r="H27">
-        <v>9999999</v>
-      </c>
-      <c r="I27" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I27">
+        <v>1</v>
       </c>
       <c r="J27">
         <v>958317.20879999921</v>
@@ -2206,10 +2206,10 @@
         <v>1542680.2972000006</v>
       </c>
       <c r="L27">
-        <v>9999999</v>
-      </c>
-      <c r="M27" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M27">
+        <v>1</v>
       </c>
       <c r="N27">
         <v>61804.2</v>
@@ -2238,7 +2238,7 @@
         <v>414000</v>
       </c>
       <c r="E28">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F28">
         <v>1289297.3467768</v>
@@ -2247,10 +2247,10 @@
         <v>1977873.4631999999</v>
       </c>
       <c r="H28">
-        <v>9999999</v>
-      </c>
-      <c r="I28" s="5">
-        <v>11000</v>
+        <v>2380000</v>
+      </c>
+      <c r="I28">
+        <v>1</v>
       </c>
       <c r="J28">
         <v>956404.40000000026</v>
@@ -2259,10 +2259,10 @@
         <v>1539811.0840000003</v>
       </c>
       <c r="L28">
-        <v>9999999</v>
-      </c>
-      <c r="M28" s="5">
-        <v>11000</v>
+        <v>1700000</v>
+      </c>
+      <c r="M28">
+        <v>1</v>
       </c>
       <c r="N28">
         <v>60876.14</v>
@@ -9050,7 +9050,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E3" s="5">
         <v>0.25</v>
@@ -9059,25 +9059,25 @@
         <v>0</v>
       </c>
       <c r="G3" s="6">
-        <v>6000</v>
+        <v>7000</v>
       </c>
       <c r="H3" s="5">
         <v>0</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="5">
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="J3" s="5">
-        <v>8.5999999999999993E-2</v>
+      <c r="J3" s="6">
+        <v>0.2</v>
       </c>
       <c r="K3" s="5">
         <v>0.8</v>
       </c>
       <c r="L3" s="5">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="M3">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="N3" s="5">
         <v>5</v>
@@ -9094,8 +9094,8 @@
       <c r="R3" s="6">
         <v>0.85</v>
       </c>
-      <c r="S3" s="5">
-        <v>8.5999999999999993E-2</v>
+      <c r="S3" s="6">
+        <v>0.2</v>
       </c>
       <c r="T3" s="5">
         <v>25000</v>
@@ -9130,7 +9130,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E4" s="5">
         <v>0.25</v>
@@ -9138,23 +9138,23 @@
       <c r="F4" s="5">
         <v>0</v>
       </c>
-      <c r="G4" s="7">
-        <v>24000</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4" s="6">
+      <c r="G4" s="6">
+        <v>23000</v>
+      </c>
+      <c r="H4" s="5">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5">
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="J4" s="5">
-        <v>8.5999999999999993E-2</v>
+      <c r="J4" s="6">
+        <v>0.2</v>
       </c>
       <c r="K4" s="5">
         <v>0.8</v>
       </c>
       <c r="L4" s="5">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="M4" s="5">
         <v>20</v>
@@ -9171,11 +9171,11 @@
       <c r="Q4" s="6">
         <v>10000</v>
       </c>
-      <c r="R4" s="5">
-        <v>0.7</v>
-      </c>
-      <c r="S4" s="5">
-        <v>8.5999999999999993E-2</v>
+      <c r="R4" s="6">
+        <v>0.85</v>
+      </c>
+      <c r="S4" s="6">
+        <v>0.2</v>
       </c>
       <c r="T4" s="5">
         <v>25000</v>
@@ -9234,7 +9234,7 @@
         <v>0.8</v>
       </c>
       <c r="L5" s="5">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="M5">
         <v>30</v>
@@ -10323,7 +10323,7 @@
         <v>2024</v>
       </c>
       <c r="B2">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C2">
         <v>26250</v>
@@ -10340,7 +10340,7 @@
         <v>2025</v>
       </c>
       <c r="B3">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C3">
         <v>26250</v>
@@ -10357,7 +10357,7 @@
         <v>2026</v>
       </c>
       <c r="B4">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C4">
         <v>26250</v>
@@ -10374,7 +10374,7 @@
         <v>2027</v>
       </c>
       <c r="B5">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C5">
         <v>26250</v>
@@ -10391,7 +10391,7 @@
         <v>2028</v>
       </c>
       <c r="B6">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C6">
         <v>26250</v>
@@ -10408,7 +10408,7 @@
         <v>2029</v>
       </c>
       <c r="B7">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C7">
         <v>26250</v>
@@ -10425,7 +10425,7 @@
         <v>2030</v>
       </c>
       <c r="B8">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C8">
         <v>26250</v>
@@ -10442,7 +10442,7 @@
         <v>2031</v>
       </c>
       <c r="B9">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C9">
         <v>26250</v>
@@ -10459,7 +10459,7 @@
         <v>2032</v>
       </c>
       <c r="B10">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C10">
         <v>26250</v>
@@ -10476,7 +10476,7 @@
         <v>2033</v>
       </c>
       <c r="B11">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C11">
         <v>26250</v>
@@ -10493,7 +10493,7 @@
         <v>2034</v>
       </c>
       <c r="B12">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C12">
         <v>26250</v>
@@ -10510,7 +10510,7 @@
         <v>2035</v>
       </c>
       <c r="B13">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C13">
         <v>26250</v>
@@ -10527,7 +10527,7 @@
         <v>2036</v>
       </c>
       <c r="B14">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C14">
         <v>26250</v>
@@ -10544,7 +10544,7 @@
         <v>2037</v>
       </c>
       <c r="B15">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C15">
         <v>26250</v>
@@ -10561,7 +10561,7 @@
         <v>2038</v>
       </c>
       <c r="B16">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C16">
         <v>26250</v>
@@ -10578,7 +10578,7 @@
         <v>2039</v>
       </c>
       <c r="B17">
-        <v>74200</v>
+        <v>70000</v>
       </c>
       <c r="C17">
         <v>26250</v>

</xml_diff>

<commit_message>
Refactors scenario definitions and plotting
Updates the scenario definitions in `run_model.py` to include new scenarios.
Removes the plotting script and adjusts the cost calculations for solar capacity.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{150F7FBD-CA77-4252-8E4F-5DD69389CF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B845115B-BB82-49DB-B75B-FF27A4EBAF4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="67080" yWindow="-1935" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -395,7 +395,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -441,6 +441,12 @@
       <color rgb="FF648C1A"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -2445,6 +2451,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -9161,7 +9168,7 @@
         <v>0.38879999999999998</v>
       </c>
       <c r="K2" s="5">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="L2" s="5">
         <v>0.2</v>
@@ -9244,7 +9251,7 @@
         <v>0.2</v>
       </c>
       <c r="K3" s="5">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="L3" s="5">
         <v>0.2</v>
@@ -9327,7 +9334,7 @@
         <v>0.2</v>
       </c>
       <c r="K4" s="5">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="L4" s="5">
         <v>0.2</v>
@@ -9410,7 +9417,7 @@
         <v>0.3</v>
       </c>
       <c r="K5" s="5">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="L5" s="5">
         <v>0.2</v>

</xml_diff>

<commit_message>
Added first basics for block_pricing, works so far, testes read in, does it correct
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gerald\Desktop\urbsextension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76775CF2-2FE5-492A-BD98-4162FA4A53CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C09D9B4-4F64-4E34-98C5-550EE28DFFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="-5565" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="28680" yWindow="-7545" windowWidth="16440" windowHeight="28440" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="dcr" sheetId="6" r:id="rId6"/>
     <sheet name="stocklvl" sheetId="7" r:id="rId7"/>
     <sheet name="installable_capacity" sheetId="3" r:id="rId8"/>
+    <sheet name="lng_block" sheetId="13" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="124">
   <si>
     <t>Value</t>
   </si>
@@ -385,6 +386,36 @@
   </si>
   <si>
     <t>308 477,99</t>
+  </si>
+  <si>
+    <t>block</t>
+  </si>
+  <si>
+    <t>limit</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>Algeria</t>
+  </si>
+  <si>
+    <t>Nigeria</t>
+  </si>
+  <si>
+    <t>Other Europe</t>
+  </si>
+  <si>
+    <t>Other Africa</t>
+  </si>
+  <si>
+    <t>Trinidad &amp; Tobago</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>Other Americas</t>
   </si>
 </sst>
 </file>
@@ -449,7 +480,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -483,6 +514,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -544,7 +581,7 @@
     </xf>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -565,6 +602,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{1C1ADB5D-62B2-4A88-A962-14B0B3D457AA}"/>
@@ -909,9 +947,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31FF74EF-7037-4139-88AF-F295C305C1F7}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -919,7 +957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -927,7 +965,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -935,7 +973,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -951,25 +989,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6185AF38-42FD-4CFF-B287-2FCFFF6C6EF3}">
   <dimension ref="A1:Q28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.6640625" customWidth="1"/>
-    <col min="3" max="3" width="26.6640625" customWidth="1"/>
-    <col min="4" max="4" width="37.33203125" customWidth="1"/>
-    <col min="5" max="5" width="29.88671875" customWidth="1"/>
-    <col min="6" max="6" width="39.88671875" customWidth="1"/>
-    <col min="7" max="7" width="21.44140625" customWidth="1"/>
-    <col min="9" max="9" width="22.5546875" customWidth="1"/>
-    <col min="10" max="10" width="24.109375" customWidth="1"/>
-    <col min="11" max="11" width="27.6640625" customWidth="1"/>
-    <col min="12" max="12" width="22.88671875" customWidth="1"/>
-    <col min="13" max="13" width="20.109375" customWidth="1"/>
-    <col min="15" max="15" width="32.77734375" customWidth="1"/>
-    <col min="16" max="16" width="35.21875" customWidth="1"/>
-    <col min="17" max="17" width="31.44140625" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="26.7109375" customWidth="1"/>
+    <col min="4" max="4" width="37.28515625" customWidth="1"/>
+    <col min="5" max="5" width="29.85546875" customWidth="1"/>
+    <col min="6" max="6" width="39.85546875" customWidth="1"/>
+    <col min="7" max="7" width="21.42578125" customWidth="1"/>
+    <col min="9" max="9" width="22.5703125" customWidth="1"/>
+    <col min="10" max="10" width="24.140625" customWidth="1"/>
+    <col min="11" max="11" width="27.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.85546875" customWidth="1"/>
+    <col min="13" max="13" width="20.140625" customWidth="1"/>
+    <col min="15" max="15" width="32.7109375" customWidth="1"/>
+    <col min="16" max="16" width="35.28515625" customWidth="1"/>
+    <col min="17" max="17" width="31.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1022,7 +1060,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -1075,7 +1113,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -1128,7 +1166,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -1181,7 +1219,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -1234,7 +1272,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -1287,7 +1325,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -1340,7 +1378,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -1393,7 +1431,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -1446,7 +1484,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -1499,7 +1537,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -1552,7 +1590,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -1605,7 +1643,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -1658,7 +1696,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -1711,7 +1749,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -1764,7 +1802,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -1817,7 +1855,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -1870,7 +1908,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -1923,7 +1961,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -1976,7 +2014,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -2029,7 +2067,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -2082,7 +2120,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -2135,7 +2173,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -2188,7 +2226,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -2241,7 +2279,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -2294,7 +2332,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -2347,7 +2385,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -2400,7 +2438,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -2462,64 +2500,64 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC0D039F-A3AA-471E-A6A2-F25F8348E84D}">
   <dimension ref="A1:A17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
     </row>
   </sheetData>
@@ -2530,12 +2568,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6341E4C-4AB4-44A4-8119-B6BB3BEB6E84}">
   <dimension ref="A1:F325"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -2555,7 +2593,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2575,7 +2613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2595,7 +2633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2615,7 +2653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2635,7 +2673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2655,7 +2693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2675,7 +2713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2695,7 +2733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2715,7 +2753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2735,7 +2773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2755,7 +2793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2775,7 +2813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2795,7 +2833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1</v>
       </c>
@@ -2815,7 +2853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
@@ -2835,7 +2873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>3</v>
       </c>
@@ -2855,7 +2893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>4</v>
       </c>
@@ -2875,7 +2913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>5</v>
       </c>
@@ -2895,7 +2933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>6</v>
       </c>
@@ -2915,7 +2953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>7</v>
       </c>
@@ -2935,7 +2973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>8</v>
       </c>
@@ -2955,7 +2993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>9</v>
       </c>
@@ -2975,7 +3013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>10</v>
       </c>
@@ -2995,7 +3033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>11</v>
       </c>
@@ -3015,7 +3053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>12</v>
       </c>
@@ -3035,7 +3073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1</v>
       </c>
@@ -3055,7 +3093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2</v>
       </c>
@@ -3075,7 +3113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>3</v>
       </c>
@@ -3095,7 +3133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>4</v>
       </c>
@@ -3115,7 +3153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>5</v>
       </c>
@@ -3135,7 +3173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>6</v>
       </c>
@@ -3155,7 +3193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>7</v>
       </c>
@@ -3175,7 +3213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>8</v>
       </c>
@@ -3195,7 +3233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>9</v>
       </c>
@@ -3215,7 +3253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>10</v>
       </c>
@@ -3235,7 +3273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>11</v>
       </c>
@@ -3255,7 +3293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>12</v>
       </c>
@@ -3275,7 +3313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>1</v>
       </c>
@@ -3295,7 +3333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2</v>
       </c>
@@ -3315,7 +3353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>3</v>
       </c>
@@ -3335,7 +3373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>4</v>
       </c>
@@ -3355,7 +3393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>5</v>
       </c>
@@ -3375,7 +3413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>6</v>
       </c>
@@ -3395,7 +3433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>7</v>
       </c>
@@ -3415,7 +3453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>8</v>
       </c>
@@ -3435,7 +3473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>9</v>
       </c>
@@ -3455,7 +3493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>10</v>
       </c>
@@ -3475,7 +3513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>11</v>
       </c>
@@ -3495,7 +3533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>12</v>
       </c>
@@ -3515,7 +3553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>1</v>
       </c>
@@ -3535,7 +3573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2</v>
       </c>
@@ -3555,7 +3593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>3</v>
       </c>
@@ -3575,7 +3613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>4</v>
       </c>
@@ -3595,7 +3633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>5</v>
       </c>
@@ -3615,7 +3653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>6</v>
       </c>
@@ -3635,7 +3673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>7</v>
       </c>
@@ -3655,7 +3693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>8</v>
       </c>
@@ -3675,7 +3713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>9</v>
       </c>
@@ -3695,7 +3733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>10</v>
       </c>
@@ -3715,7 +3753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>11</v>
       </c>
@@ -3735,7 +3773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>12</v>
       </c>
@@ -3755,7 +3793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>1</v>
       </c>
@@ -3775,7 +3813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>2</v>
       </c>
@@ -3795,7 +3833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>3</v>
       </c>
@@ -3815,7 +3853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>4</v>
       </c>
@@ -3835,7 +3873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>5</v>
       </c>
@@ -3855,7 +3893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>6</v>
       </c>
@@ -3875,7 +3913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>7</v>
       </c>
@@ -3895,7 +3933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>8</v>
       </c>
@@ -3915,7 +3953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>9</v>
       </c>
@@ -3935,7 +3973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>10</v>
       </c>
@@ -3955,7 +3993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>11</v>
       </c>
@@ -3975,7 +4013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>12</v>
       </c>
@@ -3995,7 +4033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>1</v>
       </c>
@@ -4015,7 +4053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>2</v>
       </c>
@@ -4035,7 +4073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>3</v>
       </c>
@@ -4055,7 +4093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>4</v>
       </c>
@@ -4075,7 +4113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>5</v>
       </c>
@@ -4095,7 +4133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>6</v>
       </c>
@@ -4115,7 +4153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>7</v>
       </c>
@@ -4135,7 +4173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>8</v>
       </c>
@@ -4155,7 +4193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>9</v>
       </c>
@@ -4175,7 +4213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>10</v>
       </c>
@@ -4195,7 +4233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>11</v>
       </c>
@@ -4215,7 +4253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>12</v>
       </c>
@@ -4235,7 +4273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>1</v>
       </c>
@@ -4255,7 +4293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>2</v>
       </c>
@@ -4275,7 +4313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>3</v>
       </c>
@@ -4295,7 +4333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>4</v>
       </c>
@@ -4315,7 +4353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>5</v>
       </c>
@@ -4335,7 +4373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>6</v>
       </c>
@@ -4355,7 +4393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>7</v>
       </c>
@@ -4375,7 +4413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>8</v>
       </c>
@@ -4395,7 +4433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>9</v>
       </c>
@@ -4415,7 +4453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>10</v>
       </c>
@@ -4435,7 +4473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>11</v>
       </c>
@@ -4455,7 +4493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>12</v>
       </c>
@@ -4475,7 +4513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>1</v>
       </c>
@@ -4495,7 +4533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>2</v>
       </c>
@@ -4515,7 +4553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>3</v>
       </c>
@@ -4535,7 +4573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>4</v>
       </c>
@@ -4555,7 +4593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>5</v>
       </c>
@@ -4575,7 +4613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>6</v>
       </c>
@@ -4595,7 +4633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>7</v>
       </c>
@@ -4615,7 +4653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>8</v>
       </c>
@@ -4635,7 +4673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>9</v>
       </c>
@@ -4655,7 +4693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>10</v>
       </c>
@@ -4675,7 +4713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>11</v>
       </c>
@@ -4695,7 +4733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>12</v>
       </c>
@@ -4715,7 +4753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>1</v>
       </c>
@@ -4735,7 +4773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>2</v>
       </c>
@@ -4755,7 +4793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>3</v>
       </c>
@@ -4775,7 +4813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>4</v>
       </c>
@@ -4795,7 +4833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>5</v>
       </c>
@@ -4815,7 +4853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>6</v>
       </c>
@@ -4835,7 +4873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>7</v>
       </c>
@@ -4855,7 +4893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>8</v>
       </c>
@@ -4875,7 +4913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>9</v>
       </c>
@@ -4895,7 +4933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>10</v>
       </c>
@@ -4915,7 +4953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>11</v>
       </c>
@@ -4935,7 +4973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>12</v>
       </c>
@@ -4955,7 +4993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>1</v>
       </c>
@@ -4975,7 +5013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>2</v>
       </c>
@@ -4995,7 +5033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>3</v>
       </c>
@@ -5015,7 +5053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>4</v>
       </c>
@@ -5035,7 +5073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>5</v>
       </c>
@@ -5055,7 +5093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>6</v>
       </c>
@@ -5075,7 +5113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>7</v>
       </c>
@@ -5095,7 +5133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>8</v>
       </c>
@@ -5115,7 +5153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>9</v>
       </c>
@@ -5135,7 +5173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>10</v>
       </c>
@@ -5155,7 +5193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>11</v>
       </c>
@@ -5175,7 +5213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>12</v>
       </c>
@@ -5195,7 +5233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>1</v>
       </c>
@@ -5215,7 +5253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>2</v>
       </c>
@@ -5235,7 +5273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>3</v>
       </c>
@@ -5255,7 +5293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>4</v>
       </c>
@@ -5275,7 +5313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>5</v>
       </c>
@@ -5295,7 +5333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>6</v>
       </c>
@@ -5315,7 +5353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>7</v>
       </c>
@@ -5335,7 +5373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>8</v>
       </c>
@@ -5355,7 +5393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>9</v>
       </c>
@@ -5375,7 +5413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>10</v>
       </c>
@@ -5395,7 +5433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>11</v>
       </c>
@@ -5415,7 +5453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>12</v>
       </c>
@@ -5435,7 +5473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>1</v>
       </c>
@@ -5455,7 +5493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>2</v>
       </c>
@@ -5475,7 +5513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>3</v>
       </c>
@@ -5495,7 +5533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>4</v>
       </c>
@@ -5515,7 +5553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>5</v>
       </c>
@@ -5535,7 +5573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>6</v>
       </c>
@@ -5555,7 +5593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>7</v>
       </c>
@@ -5575,7 +5613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>8</v>
       </c>
@@ -5595,7 +5633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>9</v>
       </c>
@@ -5615,7 +5653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>10</v>
       </c>
@@ -5635,7 +5673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>11</v>
       </c>
@@ -5655,7 +5693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>12</v>
       </c>
@@ -5675,7 +5713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>1</v>
       </c>
@@ -5695,7 +5733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>2</v>
       </c>
@@ -5715,7 +5753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>3</v>
       </c>
@@ -5735,7 +5773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>4</v>
       </c>
@@ -5755,7 +5793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>5</v>
       </c>
@@ -5775,7 +5813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>6</v>
       </c>
@@ -5795,7 +5833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>7</v>
       </c>
@@ -5815,7 +5853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>8</v>
       </c>
@@ -5835,7 +5873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>9</v>
       </c>
@@ -5855,7 +5893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>10</v>
       </c>
@@ -5875,7 +5913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>11</v>
       </c>
@@ -5895,7 +5933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>12</v>
       </c>
@@ -5915,7 +5953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>1</v>
       </c>
@@ -5935,7 +5973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>2</v>
       </c>
@@ -5955,7 +5993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>3</v>
       </c>
@@ -5975,7 +6013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>4</v>
       </c>
@@ -5995,7 +6033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>5</v>
       </c>
@@ -6015,7 +6053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>6</v>
       </c>
@@ -6035,7 +6073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>7</v>
       </c>
@@ -6055,7 +6093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>8</v>
       </c>
@@ -6075,7 +6113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>9</v>
       </c>
@@ -6095,7 +6133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>10</v>
       </c>
@@ -6115,7 +6153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>11</v>
       </c>
@@ -6135,7 +6173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>12</v>
       </c>
@@ -6155,7 +6193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>1</v>
       </c>
@@ -6175,7 +6213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>2</v>
       </c>
@@ -6195,7 +6233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>3</v>
       </c>
@@ -6215,7 +6253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>4</v>
       </c>
@@ -6235,7 +6273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>5</v>
       </c>
@@ -6255,7 +6293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>6</v>
       </c>
@@ -6275,7 +6313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>7</v>
       </c>
@@ -6295,7 +6333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>8</v>
       </c>
@@ -6315,7 +6353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>9</v>
       </c>
@@ -6335,7 +6373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>10</v>
       </c>
@@ -6355,7 +6393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>11</v>
       </c>
@@ -6375,7 +6413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>12</v>
       </c>
@@ -6395,7 +6433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>1</v>
       </c>
@@ -6415,7 +6453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>2</v>
       </c>
@@ -6435,7 +6473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>3</v>
       </c>
@@ -6455,7 +6493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>4</v>
       </c>
@@ -6475,7 +6513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>5</v>
       </c>
@@ -6495,7 +6533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>6</v>
       </c>
@@ -6515,7 +6553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>7</v>
       </c>
@@ -6535,7 +6573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>8</v>
       </c>
@@ -6555,7 +6593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>9</v>
       </c>
@@ -6575,7 +6613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>10</v>
       </c>
@@ -6595,7 +6633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>11</v>
       </c>
@@ -6615,7 +6653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>12</v>
       </c>
@@ -6635,7 +6673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>1</v>
       </c>
@@ -6655,7 +6693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>2</v>
       </c>
@@ -6675,7 +6713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>3</v>
       </c>
@@ -6695,7 +6733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>4</v>
       </c>
@@ -6715,7 +6753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>5</v>
       </c>
@@ -6735,7 +6773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>6</v>
       </c>
@@ -6755,7 +6793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>7</v>
       </c>
@@ -6775,7 +6813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>8</v>
       </c>
@@ -6795,7 +6833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>9</v>
       </c>
@@ -6815,7 +6853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>10</v>
       </c>
@@ -6835,7 +6873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>11</v>
       </c>
@@ -6855,7 +6893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>12</v>
       </c>
@@ -6875,7 +6913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>1</v>
       </c>
@@ -6895,7 +6933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>2</v>
       </c>
@@ -6915,7 +6953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>3</v>
       </c>
@@ -6935,7 +6973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>4</v>
       </c>
@@ -6955,7 +6993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>5</v>
       </c>
@@ -6975,7 +7013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>6</v>
       </c>
@@ -6995,7 +7033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>7</v>
       </c>
@@ -7015,7 +7053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>8</v>
       </c>
@@ -7035,7 +7073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>9</v>
       </c>
@@ -7055,7 +7093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>10</v>
       </c>
@@ -7075,7 +7113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>11</v>
       </c>
@@ -7095,7 +7133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>12</v>
       </c>
@@ -7115,7 +7153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>1</v>
       </c>
@@ -7135,7 +7173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>2</v>
       </c>
@@ -7155,7 +7193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>3</v>
       </c>
@@ -7175,7 +7213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>4</v>
       </c>
@@ -7195,7 +7233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>5</v>
       </c>
@@ -7215,7 +7253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>6</v>
       </c>
@@ -7235,7 +7273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>7</v>
       </c>
@@ -7255,7 +7293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>8</v>
       </c>
@@ -7275,7 +7313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>9</v>
       </c>
@@ -7295,7 +7333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>10</v>
       </c>
@@ -7315,7 +7353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>11</v>
       </c>
@@ -7335,7 +7373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>12</v>
       </c>
@@ -7355,7 +7393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>1</v>
       </c>
@@ -7375,7 +7413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>2</v>
       </c>
@@ -7395,7 +7433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>3</v>
       </c>
@@ -7415,7 +7453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>4</v>
       </c>
@@ -7435,7 +7473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>5</v>
       </c>
@@ -7455,7 +7493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>6</v>
       </c>
@@ -7475,7 +7513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>7</v>
       </c>
@@ -7495,7 +7533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>8</v>
       </c>
@@ -7515,7 +7553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>9</v>
       </c>
@@ -7535,7 +7573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>10</v>
       </c>
@@ -7555,7 +7593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>11</v>
       </c>
@@ -7575,7 +7613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>12</v>
       </c>
@@ -7595,7 +7633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A254">
         <v>1</v>
       </c>
@@ -7615,7 +7653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A255">
         <v>2</v>
       </c>
@@ -7635,7 +7673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A256">
         <v>3</v>
       </c>
@@ -7655,7 +7693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>4</v>
       </c>
@@ -7675,7 +7713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>5</v>
       </c>
@@ -7695,7 +7733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A259">
         <v>6</v>
       </c>
@@ -7715,7 +7753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A260">
         <v>7</v>
       </c>
@@ -7735,7 +7773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A261">
         <v>8</v>
       </c>
@@ -7755,7 +7793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A262">
         <v>9</v>
       </c>
@@ -7775,7 +7813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A263">
         <v>10</v>
       </c>
@@ -7795,7 +7833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A264">
         <v>11</v>
       </c>
@@ -7815,7 +7853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A265">
         <v>12</v>
       </c>
@@ -7835,7 +7873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A266">
         <v>1</v>
       </c>
@@ -7855,7 +7893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A267">
         <v>2</v>
       </c>
@@ -7875,7 +7913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A268">
         <v>3</v>
       </c>
@@ -7895,7 +7933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A269">
         <v>4</v>
       </c>
@@ -7915,7 +7953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A270">
         <v>5</v>
       </c>
@@ -7935,7 +7973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A271">
         <v>6</v>
       </c>
@@ -7955,7 +7993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A272">
         <v>7</v>
       </c>
@@ -7975,7 +8013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A273">
         <v>8</v>
       </c>
@@ -7995,7 +8033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>9</v>
       </c>
@@ -8015,7 +8053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A275">
         <v>10</v>
       </c>
@@ -8035,7 +8073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A276">
         <v>11</v>
       </c>
@@ -8055,7 +8093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A277">
         <v>12</v>
       </c>
@@ -8075,7 +8113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A278">
         <v>1</v>
       </c>
@@ -8095,7 +8133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A279">
         <v>2</v>
       </c>
@@ -8115,7 +8153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A280">
         <v>3</v>
       </c>
@@ -8135,7 +8173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A281">
         <v>4</v>
       </c>
@@ -8155,7 +8193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A282">
         <v>5</v>
       </c>
@@ -8175,7 +8213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A283">
         <v>6</v>
       </c>
@@ -8195,7 +8233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A284">
         <v>7</v>
       </c>
@@ -8215,7 +8253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A285">
         <v>8</v>
       </c>
@@ -8235,7 +8273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A286">
         <v>9</v>
       </c>
@@ -8255,7 +8293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A287">
         <v>10</v>
       </c>
@@ -8275,7 +8313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A288">
         <v>11</v>
       </c>
@@ -8295,7 +8333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A289">
         <v>12</v>
       </c>
@@ -8315,7 +8353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A290">
         <v>1</v>
       </c>
@@ -8335,7 +8373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A291">
         <v>2</v>
       </c>
@@ -8355,7 +8393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>3</v>
       </c>
@@ -8375,7 +8413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>4</v>
       </c>
@@ -8395,7 +8433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>5</v>
       </c>
@@ -8415,7 +8453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A295">
         <v>6</v>
       </c>
@@ -8435,7 +8473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>7</v>
       </c>
@@ -8455,7 +8493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>8</v>
       </c>
@@ -8475,7 +8513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>9</v>
       </c>
@@ -8495,7 +8533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A299">
         <v>10</v>
       </c>
@@ -8515,7 +8553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>11</v>
       </c>
@@ -8535,7 +8573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>12</v>
       </c>
@@ -8555,7 +8593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A302">
         <v>1</v>
       </c>
@@ -8575,7 +8613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A303">
         <v>2</v>
       </c>
@@ -8595,7 +8633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A304">
         <v>3</v>
       </c>
@@ -8615,7 +8653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A305">
         <v>4</v>
       </c>
@@ -8635,7 +8673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A306">
         <v>5</v>
       </c>
@@ -8655,7 +8693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A307">
         <v>6</v>
       </c>
@@ -8675,7 +8713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A308">
         <v>7</v>
       </c>
@@ -8695,7 +8733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A309">
         <v>8</v>
       </c>
@@ -8715,7 +8753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A310">
         <v>9</v>
       </c>
@@ -8735,7 +8773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A311">
         <v>10</v>
       </c>
@@ -8755,7 +8793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A312">
         <v>11</v>
       </c>
@@ -8775,7 +8813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A313">
         <v>12</v>
       </c>
@@ -8795,7 +8833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A314">
         <v>1</v>
       </c>
@@ -8815,7 +8853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A315">
         <v>2</v>
       </c>
@@ -8835,7 +8873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A316">
         <v>3</v>
       </c>
@@ -8855,7 +8893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A317">
         <v>4</v>
       </c>
@@ -8875,7 +8913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="318" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A318">
         <v>5</v>
       </c>
@@ -8895,7 +8933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="319" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A319">
         <v>6</v>
       </c>
@@ -8915,7 +8953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A320">
         <v>7</v>
       </c>
@@ -8935,7 +8973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A321">
         <v>8</v>
       </c>
@@ -8955,7 +8993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A322">
         <v>9</v>
       </c>
@@ -8975,7 +9013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A323">
         <v>10</v>
       </c>
@@ -8995,7 +9033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A324">
         <v>11</v>
       </c>
@@ -9015,7 +9053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="325" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A325">
         <v>12</v>
       </c>
@@ -9043,20 +9081,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71493739-45C2-4A8D-9266-24BB3FC8F4DB}">
   <dimension ref="A1:AA18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" customWidth="1"/>
-    <col min="7" max="7" width="18.33203125" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="18.28515625" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="19.33203125" customWidth="1"/>
-    <col min="10" max="10" width="21.88671875" customWidth="1"/>
-    <col min="14" max="14" width="20.109375" customWidth="1"/>
-    <col min="20" max="20" width="20.5546875" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" customWidth="1"/>
+    <col min="10" max="10" width="21.85546875" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" customWidth="1"/>
+    <col min="20" max="20" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>18</v>
       </c>
@@ -9139,7 +9177,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
@@ -9222,7 +9260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>31</v>
       </c>
@@ -9305,7 +9343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>41</v>
       </c>
@@ -9388,7 +9426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>56</v>
       </c>
@@ -9471,43 +9509,43 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
     </row>
   </sheetData>
@@ -9519,9 +9557,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69FD329D-454B-4A8C-B502-49D79ABB4242}">
   <dimension ref="A1:E28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -9538,7 +9576,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -9555,7 +9593,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -9572,7 +9610,7 @@
         <v>2.2200000000000001E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -9589,7 +9627,7 @@
         <v>2.4400000000000002E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -9606,7 +9644,7 @@
         <v>2.6599999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -9623,7 +9661,7 @@
         <v>2.8799999999999999E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -9640,7 +9678,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -9657,7 +9695,7 @@
         <v>3.32E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -9674,7 +9712,7 @@
         <v>3.5400000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -9691,7 +9729,7 @@
         <v>3.7600000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -9708,7 +9746,7 @@
         <v>3.9800000000000002E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -9725,7 +9763,7 @@
         <v>3.9800000000000002E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -9742,7 +9780,7 @@
         <v>4.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -9759,7 +9797,7 @@
         <v>4.4200000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -9776,7 +9814,7 @@
         <v>4.6399999999999997E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -9793,7 +9831,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -9810,7 +9848,7 @@
         <v>5.0799999999999998E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -9827,7 +9865,7 @@
         <v>5.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -9844,7 +9882,7 @@
         <v>5.5199999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -9861,7 +9899,7 @@
         <v>5.74E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -9878,7 +9916,7 @@
         <v>5.96E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -9895,7 +9933,7 @@
         <v>6.1800000000000001E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -9912,7 +9950,7 @@
         <v>6.4000000000000001E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -9929,7 +9967,7 @@
         <v>6.6199999999999995E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -9946,7 +9984,7 @@
         <v>6.8400000000000002E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -9963,7 +10001,7 @@
         <v>7.0599999999999996E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -9980,7 +10018,7 @@
         <v>7.2800000000000004E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -10005,9 +10043,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1143316B-9FC2-4B52-982D-1F4DD6859A8E}">
   <dimension ref="A1:E28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -10024,7 +10062,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -10041,7 +10079,7 @@
         <v>26229.707720000002</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -10058,7 +10096,7 @@
         <v>26589.174669999997</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -10075,7 +10113,7 @@
         <v>60431.69513</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -10092,7 +10130,7 @@
         <v>95314.195130000007</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -10109,7 +10147,7 @@
         <v>130196.6951</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -10126,7 +10164,7 @@
         <v>165780.465</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -10143,7 +10181,7 @@
         <v>179750.54879999999</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -10160,7 +10198,7 @@
         <v>195610.7611</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -10177,7 +10215,7 @@
         <v>196499.72339999999</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -10194,7 +10232,7 @@
         <v>198853.9976</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -10211,7 +10249,7 @@
         <v>202089.00579999998</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -10228,7 +10266,7 @@
         <v>164077.8836</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -10245,7 +10283,7 @@
         <v>126654.49769999999</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -10262,7 +10300,7 @@
         <v>90701.344779999999</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -10279,7 +10317,7 @@
         <v>57298.538379999998</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -10296,7 +10334,7 @@
         <v>40938.322699999997</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -10313,7 +10351,7 @@
         <v>30788.296410000003</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -10330,7 +10368,7 @@
         <v>28368.054080000002</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -10347,7 +10385,7 @@
         <v>31250.81408</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -10364,7 +10402,7 @@
         <v>34011.350160000002</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -10381,7 +10419,7 @@
         <v>35066.675019999995</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -10398,7 +10436,7 @@
         <v>33453.543590000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -10415,7 +10453,7 @@
         <v>25310.301890000002</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -10432,7 +10470,7 @@
         <v>11877.08452</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -10449,7 +10487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -10466,7 +10504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -10491,9 +10529,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3790A601-26C3-4DCA-97B6-9342C547A4A0}">
   <dimension ref="A1:E28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -10510,7 +10548,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -10527,7 +10565,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -10545,7 +10583,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -10563,7 +10601,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -10581,7 +10619,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -10599,7 +10637,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -10617,7 +10655,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -10635,7 +10673,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -10654,7 +10692,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -10673,7 +10711,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -10692,7 +10730,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -10711,7 +10749,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -10730,7 +10768,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -10747,7 +10785,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -10764,7 +10802,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -10781,7 +10819,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -10798,7 +10836,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -10815,7 +10853,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -10832,7 +10870,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -10849,7 +10887,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -10866,7 +10904,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -10883,7 +10921,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -10900,7 +10938,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -10917,7 +10955,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -10934,7 +10972,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -10951,7 +10989,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -10968,7 +11006,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -10983,6 +11021,139 @@
       </c>
       <c r="E28">
         <v>999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="25.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>138105619</v>
+      </c>
+      <c r="C2">
+        <v>15.87</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>471381508</v>
+      </c>
+      <c r="C3">
+        <v>28.56</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>27736037</v>
+      </c>
+      <c r="C4">
+        <v>29.18</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>61588793</v>
+      </c>
+      <c r="C5">
+        <v>30.15</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>144907263</v>
+      </c>
+      <c r="C6">
+        <v>33.33</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>471381508</v>
+      </c>
+      <c r="C7">
+        <v>39.69</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>98828156</v>
+      </c>
+      <c r="C8">
+        <v>43.14</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>999999999999</v>
+      </c>
+      <c r="C9">
+        <v>79.319999999999993</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Successfully implemented LNG Block Pricing.
Approach: every year there is a certain amount available per supplier for a certain price
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gerald\Desktop\urbsextension\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C09D9B4-4F64-4E34-98C5-550EE28DFFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F918984-D2CD-4EB7-B7E0-942DB386408D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-7545" windowWidth="16440" windowHeight="28440" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="67080" yWindow="-5565" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -947,9 +947,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31FF74EF-7037-4139-88AF-F295C305C1F7}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -957,7 +957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -965,7 +965,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -973,7 +973,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -989,25 +989,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6185AF38-42FD-4CFF-B287-2FCFFF6C6EF3}">
   <dimension ref="A1:Q28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
-    <col min="3" max="3" width="26.7109375" customWidth="1"/>
-    <col min="4" max="4" width="37.28515625" customWidth="1"/>
-    <col min="5" max="5" width="29.85546875" customWidth="1"/>
-    <col min="6" max="6" width="39.85546875" customWidth="1"/>
-    <col min="7" max="7" width="21.42578125" customWidth="1"/>
-    <col min="9" max="9" width="22.5703125" customWidth="1"/>
-    <col min="10" max="10" width="24.140625" customWidth="1"/>
-    <col min="11" max="11" width="27.7109375" customWidth="1"/>
-    <col min="12" max="12" width="22.85546875" customWidth="1"/>
-    <col min="13" max="13" width="20.140625" customWidth="1"/>
-    <col min="15" max="15" width="32.7109375" customWidth="1"/>
-    <col min="16" max="16" width="35.28515625" customWidth="1"/>
-    <col min="17" max="17" width="31.42578125" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" customWidth="1"/>
+    <col min="3" max="3" width="26.6640625" customWidth="1"/>
+    <col min="4" max="4" width="37.33203125" customWidth="1"/>
+    <col min="5" max="5" width="29.88671875" customWidth="1"/>
+    <col min="6" max="6" width="39.88671875" customWidth="1"/>
+    <col min="7" max="7" width="21.44140625" customWidth="1"/>
+    <col min="9" max="9" width="22.5546875" customWidth="1"/>
+    <col min="10" max="10" width="24.109375" customWidth="1"/>
+    <col min="11" max="11" width="27.6640625" customWidth="1"/>
+    <col min="12" max="12" width="22.88671875" customWidth="1"/>
+    <col min="13" max="13" width="20.109375" customWidth="1"/>
+    <col min="15" max="15" width="32.6640625" customWidth="1"/>
+    <col min="16" max="16" width="35.33203125" customWidth="1"/>
+    <col min="17" max="17" width="31.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1060,7 +1060,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -1113,7 +1113,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -1219,7 +1219,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -1272,7 +1272,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -1325,7 +1325,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -1431,7 +1431,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -1537,7 +1537,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -1590,7 +1590,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -1802,7 +1802,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -1855,7 +1855,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -1908,7 +1908,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -2173,7 +2173,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -2332,7 +2332,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -2385,7 +2385,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -2438,7 +2438,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -2500,64 +2500,64 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC0D039F-A3AA-471E-A6A2-F25F8348E84D}">
   <dimension ref="A1:A17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
     </row>
   </sheetData>
@@ -2568,12 +2568,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6341E4C-4AB4-44A4-8119-B6BB3BEB6E84}">
   <dimension ref="A1:F325"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -2593,7 +2593,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2633,7 +2633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2653,7 +2653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2673,7 +2673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2693,7 +2693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2713,7 +2713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2773,7 +2773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2793,7 +2793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2813,7 +2813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1</v>
       </c>
@@ -2853,7 +2853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2</v>
       </c>
@@ -2873,7 +2873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>3</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>4</v>
       </c>
@@ -2913,7 +2913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>5</v>
       </c>
@@ -2933,7 +2933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>6</v>
       </c>
@@ -2953,7 +2953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>7</v>
       </c>
@@ -2973,7 +2973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>8</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>9</v>
       </c>
@@ -3013,7 +3013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>10</v>
       </c>
@@ -3033,7 +3033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>11</v>
       </c>
@@ -3053,7 +3053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>12</v>
       </c>
@@ -3073,7 +3073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>1</v>
       </c>
@@ -3093,7 +3093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2</v>
       </c>
@@ -3113,7 +3113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>3</v>
       </c>
@@ -3133,7 +3133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>4</v>
       </c>
@@ -3153,7 +3153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>5</v>
       </c>
@@ -3173,7 +3173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>6</v>
       </c>
@@ -3193,7 +3193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>7</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>8</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>9</v>
       </c>
@@ -3253,7 +3253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>10</v>
       </c>
@@ -3273,7 +3273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>11</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>12</v>
       </c>
@@ -3313,7 +3313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>1</v>
       </c>
@@ -3333,7 +3333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>2</v>
       </c>
@@ -3353,7 +3353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>3</v>
       </c>
@@ -3373,7 +3373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>4</v>
       </c>
@@ -3393,7 +3393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>5</v>
       </c>
@@ -3413,7 +3413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>6</v>
       </c>
@@ -3433,7 +3433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>7</v>
       </c>
@@ -3453,7 +3453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>8</v>
       </c>
@@ -3473,7 +3473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>9</v>
       </c>
@@ -3493,7 +3493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>10</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>11</v>
       </c>
@@ -3533,7 +3533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>12</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>1</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>2</v>
       </c>
@@ -3593,7 +3593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>3</v>
       </c>
@@ -3613,7 +3613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>4</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>5</v>
       </c>
@@ -3653,7 +3653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>6</v>
       </c>
@@ -3673,7 +3673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>7</v>
       </c>
@@ -3693,7 +3693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>8</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>9</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>10</v>
       </c>
@@ -3753,7 +3753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>11</v>
       </c>
@@ -3773,7 +3773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>12</v>
       </c>
@@ -3793,7 +3793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>1</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>2</v>
       </c>
@@ -3833,7 +3833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>3</v>
       </c>
@@ -3853,7 +3853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>4</v>
       </c>
@@ -3873,7 +3873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>5</v>
       </c>
@@ -3893,7 +3893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>6</v>
       </c>
@@ -3913,7 +3913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>7</v>
       </c>
@@ -3933,7 +3933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>8</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>9</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>10</v>
       </c>
@@ -3993,7 +3993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>11</v>
       </c>
@@ -4013,7 +4013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>12</v>
       </c>
@@ -4033,7 +4033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>1</v>
       </c>
@@ -4053,7 +4053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>2</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>3</v>
       </c>
@@ -4093,7 +4093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>4</v>
       </c>
@@ -4113,7 +4113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>5</v>
       </c>
@@ -4133,7 +4133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>6</v>
       </c>
@@ -4153,7 +4153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>7</v>
       </c>
@@ -4173,7 +4173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>8</v>
       </c>
@@ -4193,7 +4193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>9</v>
       </c>
@@ -4213,7 +4213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>10</v>
       </c>
@@ -4233,7 +4233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>11</v>
       </c>
@@ -4253,7 +4253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>12</v>
       </c>
@@ -4273,7 +4273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>1</v>
       </c>
@@ -4293,7 +4293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>2</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>3</v>
       </c>
@@ -4333,7 +4333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>4</v>
       </c>
@@ -4353,7 +4353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>5</v>
       </c>
@@ -4373,7 +4373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>6</v>
       </c>
@@ -4393,7 +4393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>7</v>
       </c>
@@ -4413,7 +4413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>8</v>
       </c>
@@ -4433,7 +4433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>9</v>
       </c>
@@ -4453,7 +4453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>10</v>
       </c>
@@ -4473,7 +4473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>11</v>
       </c>
@@ -4493,7 +4493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>12</v>
       </c>
@@ -4513,7 +4513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>1</v>
       </c>
@@ -4533,7 +4533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>2</v>
       </c>
@@ -4553,7 +4553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>3</v>
       </c>
@@ -4573,7 +4573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>4</v>
       </c>
@@ -4593,7 +4593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>5</v>
       </c>
@@ -4613,7 +4613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>6</v>
       </c>
@@ -4633,7 +4633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>7</v>
       </c>
@@ -4653,7 +4653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>8</v>
       </c>
@@ -4673,7 +4673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>9</v>
       </c>
@@ -4693,7 +4693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>10</v>
       </c>
@@ -4713,7 +4713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>11</v>
       </c>
@@ -4733,7 +4733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>12</v>
       </c>
@@ -4753,7 +4753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>1</v>
       </c>
@@ -4773,7 +4773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>2</v>
       </c>
@@ -4793,7 +4793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>3</v>
       </c>
@@ -4813,7 +4813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>4</v>
       </c>
@@ -4833,7 +4833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>5</v>
       </c>
@@ -4853,7 +4853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>6</v>
       </c>
@@ -4873,7 +4873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>7</v>
       </c>
@@ -4893,7 +4893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>8</v>
       </c>
@@ -4913,7 +4913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>9</v>
       </c>
@@ -4933,7 +4933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>10</v>
       </c>
@@ -4953,7 +4953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>11</v>
       </c>
@@ -4973,7 +4973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>12</v>
       </c>
@@ -4993,7 +4993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>1</v>
       </c>
@@ -5013,7 +5013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>2</v>
       </c>
@@ -5033,7 +5033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>3</v>
       </c>
@@ -5053,7 +5053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>4</v>
       </c>
@@ -5073,7 +5073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>5</v>
       </c>
@@ -5093,7 +5093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>6</v>
       </c>
@@ -5113,7 +5113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>7</v>
       </c>
@@ -5133,7 +5133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>8</v>
       </c>
@@ -5153,7 +5153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>9</v>
       </c>
@@ -5173,7 +5173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>10</v>
       </c>
@@ -5193,7 +5193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>11</v>
       </c>
@@ -5213,7 +5213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>12</v>
       </c>
@@ -5233,7 +5233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>1</v>
       </c>
@@ -5253,7 +5253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>2</v>
       </c>
@@ -5273,7 +5273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>3</v>
       </c>
@@ -5293,7 +5293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>4</v>
       </c>
@@ -5313,7 +5313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>5</v>
       </c>
@@ -5333,7 +5333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>6</v>
       </c>
@@ -5353,7 +5353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>7</v>
       </c>
@@ -5373,7 +5373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>8</v>
       </c>
@@ -5393,7 +5393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>9</v>
       </c>
@@ -5413,7 +5413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>10</v>
       </c>
@@ -5433,7 +5433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>11</v>
       </c>
@@ -5453,7 +5453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>12</v>
       </c>
@@ -5473,7 +5473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>1</v>
       </c>
@@ -5493,7 +5493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>2</v>
       </c>
@@ -5513,7 +5513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>3</v>
       </c>
@@ -5533,7 +5533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>4</v>
       </c>
@@ -5553,7 +5553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>5</v>
       </c>
@@ -5573,7 +5573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>6</v>
       </c>
@@ -5593,7 +5593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>7</v>
       </c>
@@ -5613,7 +5613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>8</v>
       </c>
@@ -5633,7 +5633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>9</v>
       </c>
@@ -5653,7 +5653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>10</v>
       </c>
@@ -5673,7 +5673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>11</v>
       </c>
@@ -5693,7 +5693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>12</v>
       </c>
@@ -5713,7 +5713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>1</v>
       </c>
@@ -5733,7 +5733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>2</v>
       </c>
@@ -5753,7 +5753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>3</v>
       </c>
@@ -5773,7 +5773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>4</v>
       </c>
@@ -5793,7 +5793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>5</v>
       </c>
@@ -5813,7 +5813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>6</v>
       </c>
@@ -5833,7 +5833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>7</v>
       </c>
@@ -5853,7 +5853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>8</v>
       </c>
@@ -5873,7 +5873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>9</v>
       </c>
@@ -5893,7 +5893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>10</v>
       </c>
@@ -5913,7 +5913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>11</v>
       </c>
@@ -5933,7 +5933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>12</v>
       </c>
@@ -5953,7 +5953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>1</v>
       </c>
@@ -5973,7 +5973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>2</v>
       </c>
@@ -5993,7 +5993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>3</v>
       </c>
@@ -6013,7 +6013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>4</v>
       </c>
@@ -6033,7 +6033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>5</v>
       </c>
@@ -6053,7 +6053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>6</v>
       </c>
@@ -6073,7 +6073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>7</v>
       </c>
@@ -6093,7 +6093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>8</v>
       </c>
@@ -6113,7 +6113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>9</v>
       </c>
@@ -6133,7 +6133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>10</v>
       </c>
@@ -6153,7 +6153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>11</v>
       </c>
@@ -6173,7 +6173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>12</v>
       </c>
@@ -6193,7 +6193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>1</v>
       </c>
@@ -6213,7 +6213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>2</v>
       </c>
@@ -6233,7 +6233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>3</v>
       </c>
@@ -6253,7 +6253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>4</v>
       </c>
@@ -6273,7 +6273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>5</v>
       </c>
@@ -6293,7 +6293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>6</v>
       </c>
@@ -6313,7 +6313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>7</v>
       </c>
@@ -6333,7 +6333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>8</v>
       </c>
@@ -6353,7 +6353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>9</v>
       </c>
@@ -6373,7 +6373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>10</v>
       </c>
@@ -6393,7 +6393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>11</v>
       </c>
@@ -6413,7 +6413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>12</v>
       </c>
@@ -6433,7 +6433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>1</v>
       </c>
@@ -6453,7 +6453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>2</v>
       </c>
@@ -6473,7 +6473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>3</v>
       </c>
@@ -6493,7 +6493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>4</v>
       </c>
@@ -6513,7 +6513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>5</v>
       </c>
@@ -6533,7 +6533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>6</v>
       </c>
@@ -6553,7 +6553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>7</v>
       </c>
@@ -6573,7 +6573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>8</v>
       </c>
@@ -6593,7 +6593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>9</v>
       </c>
@@ -6613,7 +6613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>10</v>
       </c>
@@ -6633,7 +6633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>11</v>
       </c>
@@ -6653,7 +6653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>12</v>
       </c>
@@ -6673,7 +6673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>1</v>
       </c>
@@ -6693,7 +6693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>2</v>
       </c>
@@ -6713,7 +6713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>3</v>
       </c>
@@ -6733,7 +6733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>4</v>
       </c>
@@ -6753,7 +6753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>5</v>
       </c>
@@ -6773,7 +6773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>6</v>
       </c>
@@ -6793,7 +6793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>7</v>
       </c>
@@ -6813,7 +6813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>8</v>
       </c>
@@ -6833,7 +6833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>9</v>
       </c>
@@ -6853,7 +6853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>10</v>
       </c>
@@ -6873,7 +6873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>11</v>
       </c>
@@ -6893,7 +6893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>12</v>
       </c>
@@ -6913,7 +6913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>1</v>
       </c>
@@ -6933,7 +6933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>2</v>
       </c>
@@ -6953,7 +6953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>3</v>
       </c>
@@ -6973,7 +6973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>4</v>
       </c>
@@ -6993,7 +6993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>5</v>
       </c>
@@ -7013,7 +7013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>6</v>
       </c>
@@ -7033,7 +7033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>7</v>
       </c>
@@ -7053,7 +7053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>8</v>
       </c>
@@ -7073,7 +7073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>9</v>
       </c>
@@ -7093,7 +7093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>10</v>
       </c>
@@ -7113,7 +7113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>11</v>
       </c>
@@ -7133,7 +7133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>12</v>
       </c>
@@ -7153,7 +7153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>1</v>
       </c>
@@ -7173,7 +7173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>2</v>
       </c>
@@ -7193,7 +7193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>3</v>
       </c>
@@ -7213,7 +7213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>4</v>
       </c>
@@ -7233,7 +7233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>5</v>
       </c>
@@ -7253,7 +7253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>6</v>
       </c>
@@ -7273,7 +7273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>7</v>
       </c>
@@ -7293,7 +7293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>8</v>
       </c>
@@ -7313,7 +7313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>9</v>
       </c>
@@ -7333,7 +7333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>10</v>
       </c>
@@ -7353,7 +7353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>11</v>
       </c>
@@ -7373,7 +7373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>12</v>
       </c>
@@ -7393,7 +7393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>1</v>
       </c>
@@ -7413,7 +7413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>2</v>
       </c>
@@ -7433,7 +7433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>3</v>
       </c>
@@ -7453,7 +7453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>4</v>
       </c>
@@ -7473,7 +7473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>5</v>
       </c>
@@ -7493,7 +7493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>6</v>
       </c>
@@ -7513,7 +7513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>7</v>
       </c>
@@ -7533,7 +7533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>8</v>
       </c>
@@ -7553,7 +7553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>9</v>
       </c>
@@ -7573,7 +7573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>10</v>
       </c>
@@ -7593,7 +7593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>11</v>
       </c>
@@ -7613,7 +7613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>12</v>
       </c>
@@ -7633,7 +7633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>1</v>
       </c>
@@ -7653,7 +7653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>2</v>
       </c>
@@ -7673,7 +7673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>3</v>
       </c>
@@ -7693,7 +7693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>4</v>
       </c>
@@ -7713,7 +7713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>5</v>
       </c>
@@ -7733,7 +7733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>6</v>
       </c>
@@ -7753,7 +7753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>7</v>
       </c>
@@ -7773,7 +7773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>8</v>
       </c>
@@ -7793,7 +7793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>9</v>
       </c>
@@ -7813,7 +7813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>10</v>
       </c>
@@ -7833,7 +7833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>11</v>
       </c>
@@ -7853,7 +7853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>12</v>
       </c>
@@ -7873,7 +7873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>1</v>
       </c>
@@ -7893,7 +7893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>2</v>
       </c>
@@ -7913,7 +7913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>3</v>
       </c>
@@ -7933,7 +7933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>4</v>
       </c>
@@ -7953,7 +7953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>5</v>
       </c>
@@ -7973,7 +7973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>6</v>
       </c>
@@ -7993,7 +7993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>7</v>
       </c>
@@ -8013,7 +8013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>8</v>
       </c>
@@ -8033,7 +8033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>9</v>
       </c>
@@ -8053,7 +8053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>10</v>
       </c>
@@ -8073,7 +8073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>11</v>
       </c>
@@ -8093,7 +8093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>12</v>
       </c>
@@ -8113,7 +8113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>1</v>
       </c>
@@ -8133,7 +8133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>2</v>
       </c>
@@ -8153,7 +8153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>3</v>
       </c>
@@ -8173,7 +8173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>4</v>
       </c>
@@ -8193,7 +8193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>5</v>
       </c>
@@ -8213,7 +8213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>6</v>
       </c>
@@ -8233,7 +8233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>7</v>
       </c>
@@ -8253,7 +8253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>8</v>
       </c>
@@ -8273,7 +8273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>9</v>
       </c>
@@ -8293,7 +8293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>10</v>
       </c>
@@ -8313,7 +8313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>11</v>
       </c>
@@ -8333,7 +8333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>12</v>
       </c>
@@ -8353,7 +8353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>1</v>
       </c>
@@ -8373,7 +8373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>2</v>
       </c>
@@ -8393,7 +8393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>3</v>
       </c>
@@ -8413,7 +8413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>4</v>
       </c>
@@ -8433,7 +8433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>5</v>
       </c>
@@ -8453,7 +8453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>6</v>
       </c>
@@ -8473,7 +8473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>7</v>
       </c>
@@ -8493,7 +8493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>8</v>
       </c>
@@ -8513,7 +8513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>9</v>
       </c>
@@ -8533,7 +8533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>10</v>
       </c>
@@ -8553,7 +8553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>11</v>
       </c>
@@ -8573,7 +8573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>12</v>
       </c>
@@ -8593,7 +8593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>1</v>
       </c>
@@ -8613,7 +8613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>2</v>
       </c>
@@ -8633,7 +8633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>3</v>
       </c>
@@ -8653,7 +8653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>4</v>
       </c>
@@ -8673,7 +8673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>5</v>
       </c>
@@ -8693,7 +8693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>6</v>
       </c>
@@ -8713,7 +8713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>7</v>
       </c>
@@ -8733,7 +8733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>8</v>
       </c>
@@ -8753,7 +8753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A310">
         <v>9</v>
       </c>
@@ -8773,7 +8773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A311">
         <v>10</v>
       </c>
@@ -8793,7 +8793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A312">
         <v>11</v>
       </c>
@@ -8813,7 +8813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>12</v>
       </c>
@@ -8833,7 +8833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A314">
         <v>1</v>
       </c>
@@ -8853,7 +8853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>2</v>
       </c>
@@ -8873,7 +8873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>3</v>
       </c>
@@ -8893,7 +8893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>4</v>
       </c>
@@ -8913,7 +8913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="318" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>5</v>
       </c>
@@ -8933,7 +8933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A319">
         <v>6</v>
       </c>
@@ -8953,7 +8953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A320">
         <v>7</v>
       </c>
@@ -8973,7 +8973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>8</v>
       </c>
@@ -8993,7 +8993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A322">
         <v>9</v>
       </c>
@@ -9013,7 +9013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A323">
         <v>10</v>
       </c>
@@ -9033,7 +9033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A324">
         <v>11</v>
       </c>
@@ -9053,7 +9053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="325" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A325">
         <v>12</v>
       </c>
@@ -9081,20 +9081,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71493739-45C2-4A8D-9266-24BB3FC8F4DB}">
   <dimension ref="A1:AA18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" customWidth="1"/>
-    <col min="7" max="7" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="19.28515625" customWidth="1"/>
-    <col min="10" max="10" width="21.85546875" customWidth="1"/>
-    <col min="14" max="14" width="20.140625" customWidth="1"/>
-    <col min="20" max="20" width="20.5703125" customWidth="1"/>
+    <col min="9" max="9" width="19.33203125" customWidth="1"/>
+    <col min="10" max="10" width="21.88671875" customWidth="1"/>
+    <col min="14" max="14" width="20.109375" customWidth="1"/>
+    <col min="20" max="20" width="20.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>18</v>
       </c>
@@ -9177,7 +9177,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
@@ -9260,7 +9260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>31</v>
       </c>
@@ -9343,7 +9343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>41</v>
       </c>
@@ -9426,7 +9426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>56</v>
       </c>
@@ -9509,43 +9509,43 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
     </row>
   </sheetData>
@@ -9557,9 +9557,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69FD329D-454B-4A8C-B502-49D79ABB4242}">
   <dimension ref="A1:E28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -9576,7 +9576,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -9593,7 +9593,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -9610,7 +9610,7 @@
         <v>2.2200000000000001E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -9627,7 +9627,7 @@
         <v>2.4400000000000002E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -9644,7 +9644,7 @@
         <v>2.6599999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -9661,7 +9661,7 @@
         <v>2.8799999999999999E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -9678,7 +9678,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -9695,7 +9695,7 @@
         <v>3.32E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -9712,7 +9712,7 @@
         <v>3.5400000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -9729,7 +9729,7 @@
         <v>3.7600000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -9746,7 +9746,7 @@
         <v>3.9800000000000002E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -9763,7 +9763,7 @@
         <v>3.9800000000000002E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -9780,7 +9780,7 @@
         <v>4.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -9797,7 +9797,7 @@
         <v>4.4200000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -9814,7 +9814,7 @@
         <v>4.6399999999999997E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -9831,7 +9831,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -9848,7 +9848,7 @@
         <v>5.0799999999999998E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -9865,7 +9865,7 @@
         <v>5.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -9882,7 +9882,7 @@
         <v>5.5199999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -9899,7 +9899,7 @@
         <v>5.74E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -9916,7 +9916,7 @@
         <v>5.96E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -9933,7 +9933,7 @@
         <v>6.1800000000000001E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -9950,7 +9950,7 @@
         <v>6.4000000000000001E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -9967,7 +9967,7 @@
         <v>6.6199999999999995E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -9984,7 +9984,7 @@
         <v>6.8400000000000002E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -10001,7 +10001,7 @@
         <v>7.0599999999999996E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -10018,7 +10018,7 @@
         <v>7.2800000000000004E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -10043,9 +10043,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1143316B-9FC2-4B52-982D-1F4DD6859A8E}">
   <dimension ref="A1:E28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -10062,7 +10062,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -10079,7 +10079,7 @@
         <v>26229.707720000002</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -10096,7 +10096,7 @@
         <v>26589.174669999997</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -10113,7 +10113,7 @@
         <v>60431.69513</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -10130,7 +10130,7 @@
         <v>95314.195130000007</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -10147,7 +10147,7 @@
         <v>130196.6951</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -10164,7 +10164,7 @@
         <v>165780.465</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -10181,7 +10181,7 @@
         <v>179750.54879999999</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -10198,7 +10198,7 @@
         <v>195610.7611</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -10215,7 +10215,7 @@
         <v>196499.72339999999</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -10232,7 +10232,7 @@
         <v>198853.9976</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -10249,7 +10249,7 @@
         <v>202089.00579999998</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -10266,7 +10266,7 @@
         <v>164077.8836</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -10283,7 +10283,7 @@
         <v>126654.49769999999</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -10300,7 +10300,7 @@
         <v>90701.344779999999</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -10317,7 +10317,7 @@
         <v>57298.538379999998</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -10334,7 +10334,7 @@
         <v>40938.322699999997</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -10351,7 +10351,7 @@
         <v>30788.296410000003</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -10368,7 +10368,7 @@
         <v>28368.054080000002</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -10385,7 +10385,7 @@
         <v>31250.81408</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -10402,7 +10402,7 @@
         <v>34011.350160000002</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -10419,7 +10419,7 @@
         <v>35066.675019999995</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -10436,7 +10436,7 @@
         <v>33453.543590000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -10453,7 +10453,7 @@
         <v>25310.301890000002</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -10470,7 +10470,7 @@
         <v>11877.08452</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -10487,7 +10487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -10504,7 +10504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -10529,9 +10529,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3790A601-26C3-4DCA-97B6-9342C547A4A0}">
   <dimension ref="A1:E28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -10548,7 +10548,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -10565,7 +10565,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -10583,7 +10583,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -10601,7 +10601,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -10619,7 +10619,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -10637,7 +10637,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -10655,7 +10655,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -10673,7 +10673,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -10692,7 +10692,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -10711,7 +10711,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -10730,7 +10730,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -10749,7 +10749,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -10768,7 +10768,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -10785,7 +10785,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -10802,7 +10802,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -10819,7 +10819,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -10836,7 +10836,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -10853,7 +10853,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -10870,7 +10870,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -10887,7 +10887,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -10904,7 +10904,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -10921,7 +10921,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -10938,7 +10938,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -10955,7 +10955,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -10972,7 +10972,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -10989,7 +10989,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -11006,7 +11006,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -11031,12 +11031,12 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="25.5703125" customWidth="1"/>
+    <col min="5" max="5" width="25.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>114</v>
       </c>
@@ -11047,7 +11047,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -11055,13 +11055,13 @@
         <v>138105619</v>
       </c>
       <c r="C2">
-        <v>15.87</v>
+        <v>1000</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -11069,13 +11069,13 @@
         <v>471381508</v>
       </c>
       <c r="C3">
-        <v>28.56</v>
+        <v>1000</v>
       </c>
       <c r="E3" s="10" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -11083,13 +11083,13 @@
         <v>27736037</v>
       </c>
       <c r="C4">
-        <v>29.18</v>
+        <v>1000</v>
       </c>
       <c r="E4" s="10" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -11097,13 +11097,13 @@
         <v>61588793</v>
       </c>
       <c r="C5">
-        <v>30.15</v>
+        <v>1000</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -11111,13 +11111,13 @@
         <v>144907263</v>
       </c>
       <c r="C6">
-        <v>33.33</v>
+        <v>1000</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -11125,13 +11125,13 @@
         <v>471381508</v>
       </c>
       <c r="C7">
-        <v>39.69</v>
+        <v>1000</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -11139,13 +11139,13 @@
         <v>98828156</v>
       </c>
       <c r="C8">
-        <v>43.14</v>
+        <v>1000</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -11153,7 +11153,7 @@
         <v>999999999999</v>
       </c>
       <c r="C9">
-        <v>79.319999999999993</v>
+        <v>1000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Pricing mechanism does not work properly
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1294A14-454B-4C12-A610-4EBC208C09E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{242CF2B7-D5E0-4759-9FC3-53FB16E4A55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="67080" yWindow="-5565" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -11058,7 +11058,7 @@
   <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -11202,7 +11202,7 @@
       <c r="B9">
         <v>2321122320</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9">
         <v>23.61</v>
       </c>
       <c r="D9">
@@ -11219,7 +11219,7 @@
       <c r="B10">
         <v>633033360</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10">
         <v>25.71</v>
       </c>
       <c r="D10">
@@ -11236,7 +11236,7 @@
       <c r="B11">
         <v>453673908.00000006</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11">
         <v>27.37</v>
       </c>
       <c r="D11">
@@ -11253,7 +11253,7 @@
       <c r="B12">
         <v>397755961.20000005</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12">
         <v>27.66</v>
       </c>
       <c r="D12">
@@ -11270,7 +11270,7 @@
       <c r="B13">
         <v>1477077840.0000002</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13">
         <v>34.409999999999997</v>
       </c>
       <c r="D13">
@@ -11287,7 +11287,7 @@
       <c r="B14">
         <v>220506620.40000001</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14">
         <v>34.409999999999997</v>
       </c>
       <c r="D14">

</xml_diff>

<commit_message>
just some lng stuff
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B802C3-58CC-41DB-9A14-CDBF4AD62AEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4527232-E70C-4408-BA96-E521B1020982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="7" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <sheet name="lng_block" sheetId="13" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">lng_block!$C$1:$C$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">lng_block!$C$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="71">
   <si>
     <t>Value</t>
   </si>
@@ -229,168 +229,6 @@
     <t>total_facility_cap_initial</t>
   </si>
   <si>
-    <t>280 439,83</t>
-  </si>
-  <si>
-    <t>274 754,91</t>
-  </si>
-  <si>
-    <t>269 179,44</t>
-  </si>
-  <si>
-    <t>263 711,78</t>
-  </si>
-  <si>
-    <t>258 350,32</t>
-  </si>
-  <si>
-    <t>253 093,46</t>
-  </si>
-  <si>
-    <t>247 939,65</t>
-  </si>
-  <si>
-    <t>242 887,37</t>
-  </si>
-  <si>
-    <t>237 935,10</t>
-  </si>
-  <si>
-    <t>233 081,40</t>
-  </si>
-  <si>
-    <t>228 324,82</t>
-  </si>
-  <si>
-    <t>223 663,91</t>
-  </si>
-  <si>
-    <t>219 097,32</t>
-  </si>
-  <si>
-    <t>214 623,65</t>
-  </si>
-  <si>
-    <t>210 241,60</t>
-  </si>
-  <si>
-    <t>205 949,84</t>
-  </si>
-  <si>
-    <t>201 747,12</t>
-  </si>
-  <si>
-    <t>197 632,19</t>
-  </si>
-  <si>
-    <t>193 603,83</t>
-  </si>
-  <si>
-    <t>189 660,87</t>
-  </si>
-  <si>
-    <t>185 802,14</t>
-  </si>
-  <si>
-    <t>182 026,51</t>
-  </si>
-  <si>
-    <t>178 332,87</t>
-  </si>
-  <si>
-    <t>174 720,11</t>
-  </si>
-  <si>
-    <t>171 187,17</t>
-  </si>
-  <si>
-    <t>167 732,98</t>
-  </si>
-  <si>
-    <t>164 356,52</t>
-  </si>
-  <si>
-    <t>527 469,86</t>
-  </si>
-  <si>
-    <t>516 785,56</t>
-  </si>
-  <si>
-    <t>506 302,50</t>
-  </si>
-  <si>
-    <t>496 017,89</t>
-  </si>
-  <si>
-    <t>485 929,01</t>
-  </si>
-  <si>
-    <t>476 033,18</t>
-  </si>
-  <si>
-    <t>466 327,80</t>
-  </si>
-  <si>
-    <t>456 810,30</t>
-  </si>
-  <si>
-    <t>447 478,16</t>
-  </si>
-  <si>
-    <t>438 328,91</t>
-  </si>
-  <si>
-    <t>429 360,14</t>
-  </si>
-  <si>
-    <t>420 569,49</t>
-  </si>
-  <si>
-    <t>411 954,65</t>
-  </si>
-  <si>
-    <t>403 513,36</t>
-  </si>
-  <si>
-    <t>395 243,39</t>
-  </si>
-  <si>
-    <t>387 142,59</t>
-  </si>
-  <si>
-    <t>379 208,83</t>
-  </si>
-  <si>
-    <t>371 440,05</t>
-  </si>
-  <si>
-    <t>363 834,24</t>
-  </si>
-  <si>
-    <t>356 389,41</t>
-  </si>
-  <si>
-    <t>349 103,66</t>
-  </si>
-  <si>
-    <t>341 975,10</t>
-  </si>
-  <si>
-    <t>334 991,90</t>
-  </si>
-  <si>
-    <t>328 152,29</t>
-  </si>
-  <si>
-    <t>321 454,54</t>
-  </si>
-  <si>
-    <t>314 897,00</t>
-  </si>
-  <si>
-    <t>308 477,99</t>
-  </si>
-  <si>
     <t>block</t>
   </si>
   <si>
@@ -400,49 +238,7 @@
     <t>price</t>
   </si>
   <si>
-    <t>Algeria</t>
-  </si>
-  <si>
-    <t>Other Europe</t>
-  </si>
-  <si>
-    <t>Other Africa</t>
-  </si>
-  <si>
-    <t>Trinidad &amp; Tobago</t>
-  </si>
-  <si>
-    <t>USA</t>
-  </si>
-  <si>
-    <t>Other Americas</t>
-  </si>
-  <si>
     <t>emissions</t>
-  </si>
-  <si>
-    <t>dummy block</t>
-  </si>
-  <si>
-    <t>Qatar</t>
-  </si>
-  <si>
-    <t>Australia</t>
-  </si>
-  <si>
-    <t>Malaysia</t>
-  </si>
-  <si>
-    <t>Indonesia</t>
-  </si>
-  <si>
-    <t>Oman</t>
-  </si>
-  <si>
-    <t>Other Asia Pacific</t>
-  </si>
-  <si>
-    <t>Other ME</t>
   </si>
   <si>
     <t>oandm_EU27_solarPV</t>
@@ -456,6 +252,15 @@
   <si>
     <t>oandm_EU27_Batteries</t>
   </si>
+  <si>
+    <t>Net Zero Demand</t>
+  </si>
+  <si>
+    <t>New Momentum Demand</t>
+  </si>
+  <si>
+    <t>What the heck Demand</t>
+  </si>
 </sst>
 </file>
 
@@ -465,7 +270,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -518,12 +323,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -564,12 +363,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEBF1DE"/>
-        <bgColor rgb="FF000000"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -601,6 +400,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -626,7 +434,7 @@
     </xf>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -647,9 +455,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{1C1ADB5D-62B2-4A88-A962-14B0B3D457AA}"/>
@@ -1071,7 +879,7 @@
         <v>37</v>
       </c>
       <c r="F1" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="G1" t="s">
         <v>28</v>
@@ -1086,7 +894,7 @@
         <v>38</v>
       </c>
       <c r="K1" t="s">
-        <v>133</v>
+        <v>65</v>
       </c>
       <c r="L1" t="s">
         <v>43</v>
@@ -1101,7 +909,7 @@
         <v>46</v>
       </c>
       <c r="P1" t="s">
-        <v>134</v>
+        <v>66</v>
       </c>
       <c r="Q1" t="s">
         <v>52</v>
@@ -1116,7 +924,7 @@
         <v>55</v>
       </c>
       <c r="U1" t="s">
-        <v>135</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
@@ -1168,11 +976,11 @@
       <c r="P2">
         <v>17386.633918245541</v>
       </c>
-      <c r="Q2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>87</v>
+      <c r="Q2">
+        <v>280439.83</v>
+      </c>
+      <c r="R2">
+        <v>527469.86</v>
       </c>
       <c r="S2" s="8">
         <v>489061.86</v>
@@ -1233,11 +1041,11 @@
       <c r="P3">
         <v>17386.633918245541</v>
       </c>
-      <c r="Q3" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>88</v>
+      <c r="Q3">
+        <v>274754.90999999997</v>
+      </c>
+      <c r="R3">
+        <v>516785.56</v>
       </c>
       <c r="S3" s="8">
         <v>489061.86</v>
@@ -1298,11 +1106,11 @@
       <c r="P4">
         <v>17386.633918245541</v>
       </c>
-      <c r="Q4" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="R4" s="2" t="s">
-        <v>89</v>
+      <c r="Q4">
+        <v>269179.44</v>
+      </c>
+      <c r="R4">
+        <v>506302.5</v>
       </c>
       <c r="S4" s="8">
         <v>489061.86</v>
@@ -1363,11 +1171,11 @@
       <c r="P5">
         <v>17386.633918245541</v>
       </c>
-      <c r="Q5" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>90</v>
+      <c r="Q5">
+        <v>263711.78000000003</v>
+      </c>
+      <c r="R5">
+        <v>496017.89</v>
       </c>
       <c r="S5" s="8">
         <v>489061.86</v>
@@ -1428,11 +1236,11 @@
       <c r="P6">
         <v>17386.633918245541</v>
       </c>
-      <c r="Q6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="R6" s="2" t="s">
-        <v>91</v>
+      <c r="Q6">
+        <v>258350.32</v>
+      </c>
+      <c r="R6">
+        <v>485929.01</v>
       </c>
       <c r="S6" s="8">
         <v>489061.86</v>
@@ -1493,11 +1301,11 @@
       <c r="P7">
         <v>17386.633918245541</v>
       </c>
-      <c r="Q7" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>92</v>
+      <c r="Q7">
+        <v>253093.46</v>
+      </c>
+      <c r="R7">
+        <v>476033.18</v>
       </c>
       <c r="S7" s="8">
         <v>489061.86</v>
@@ -1558,11 +1366,11 @@
       <c r="P8">
         <v>16662.667964091612</v>
       </c>
-      <c r="Q8" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="R8" s="2" t="s">
-        <v>93</v>
+      <c r="Q8">
+        <v>247939.65</v>
+      </c>
+      <c r="R8">
+        <v>466327.8</v>
       </c>
       <c r="S8" s="8">
         <v>489061.86</v>
@@ -1623,11 +1431,11 @@
       <c r="P9">
         <v>16662.667964091612</v>
       </c>
-      <c r="Q9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="R9" s="2" t="s">
-        <v>94</v>
+      <c r="Q9">
+        <v>242887.37</v>
+      </c>
+      <c r="R9">
+        <v>456810.3</v>
       </c>
       <c r="S9" s="8">
         <v>489061.86</v>
@@ -1688,11 +1496,11 @@
       <c r="P10">
         <v>16662.667964091612</v>
       </c>
-      <c r="Q10" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="R10" s="2" t="s">
-        <v>95</v>
+      <c r="Q10">
+        <v>237935.1</v>
+      </c>
+      <c r="R10">
+        <v>447478.16</v>
       </c>
       <c r="S10" s="8">
         <v>489061.86</v>
@@ -1753,11 +1561,11 @@
       <c r="P11">
         <v>16662.667964091612</v>
       </c>
-      <c r="Q11" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="R11" s="2" t="s">
-        <v>96</v>
+      <c r="Q11">
+        <v>233081.4</v>
+      </c>
+      <c r="R11">
+        <v>438328.91</v>
       </c>
       <c r="S11" s="8">
         <v>489061.86</v>
@@ -1818,11 +1626,11 @@
       <c r="P12">
         <v>16662.667964091612</v>
       </c>
-      <c r="Q12" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="R12" s="2" t="s">
-        <v>97</v>
+      <c r="Q12">
+        <v>228324.82</v>
+      </c>
+      <c r="R12">
+        <v>429360.14</v>
       </c>
       <c r="S12" s="8">
         <v>489061.86</v>
@@ -1883,11 +1691,11 @@
       <c r="P13">
         <v>16662.667964091612</v>
       </c>
-      <c r="Q13" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="R13" s="2" t="s">
-        <v>98</v>
+      <c r="Q13">
+        <v>223663.91</v>
+      </c>
+      <c r="R13">
+        <v>420569.49</v>
       </c>
       <c r="S13" s="8">
         <v>489061.86</v>
@@ -1948,11 +1756,11 @@
       <c r="P14">
         <v>16662.667964091612</v>
       </c>
-      <c r="Q14" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="R14" s="2" t="s">
-        <v>99</v>
+      <c r="Q14">
+        <v>219097.32</v>
+      </c>
+      <c r="R14">
+        <v>411954.65</v>
       </c>
       <c r="S14" s="8">
         <v>489061.86</v>
@@ -2013,11 +1821,11 @@
       <c r="P15">
         <v>16662.667964091612</v>
       </c>
-      <c r="Q15" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="R15" s="2" t="s">
-        <v>100</v>
+      <c r="Q15">
+        <v>214623.65</v>
+      </c>
+      <c r="R15">
+        <v>403513.36</v>
       </c>
       <c r="S15" s="8">
         <v>489061.86</v>
@@ -2078,11 +1886,11 @@
       <c r="P16">
         <v>16662.667964091612</v>
       </c>
-      <c r="Q16" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="R16" s="2" t="s">
-        <v>101</v>
+      <c r="Q16">
+        <v>210241.6</v>
+      </c>
+      <c r="R16">
+        <v>395243.39</v>
       </c>
       <c r="S16" s="8">
         <v>489061.86</v>
@@ -2143,11 +1951,11 @@
       <c r="P17">
         <v>16662.667964091612</v>
       </c>
-      <c r="Q17" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="R17" s="2" t="s">
-        <v>102</v>
+      <c r="Q17">
+        <v>205949.84</v>
+      </c>
+      <c r="R17">
+        <v>387142.59</v>
       </c>
       <c r="S17" s="8">
         <v>489061.86</v>
@@ -2208,11 +2016,11 @@
       <c r="P18">
         <v>15965.364846295015</v>
       </c>
-      <c r="Q18" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="R18" s="2" t="s">
-        <v>103</v>
+      <c r="Q18">
+        <v>201747.12</v>
+      </c>
+      <c r="R18">
+        <v>379208.83</v>
       </c>
       <c r="S18" s="8">
         <v>489061.86</v>
@@ -2273,11 +2081,11 @@
       <c r="P19">
         <v>15965.364846295015</v>
       </c>
-      <c r="Q19" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="R19" s="2" t="s">
-        <v>104</v>
+      <c r="Q19">
+        <v>197632.19</v>
+      </c>
+      <c r="R19">
+        <v>371440.05</v>
       </c>
       <c r="S19" s="8">
         <v>489061.86</v>
@@ -2338,11 +2146,11 @@
       <c r="P20">
         <v>15965.364846295015</v>
       </c>
-      <c r="Q20" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="R20" s="2" t="s">
-        <v>105</v>
+      <c r="Q20">
+        <v>193603.83</v>
+      </c>
+      <c r="R20">
+        <v>363834.24</v>
       </c>
       <c r="S20" s="8">
         <v>489061.86</v>
@@ -2403,11 +2211,11 @@
       <c r="P21">
         <v>15965.364846295015</v>
       </c>
-      <c r="Q21" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="R21" s="2" t="s">
-        <v>106</v>
+      <c r="Q21">
+        <v>189660.87</v>
+      </c>
+      <c r="R21">
+        <v>356389.41</v>
       </c>
       <c r="S21" s="8">
         <v>489061.86</v>
@@ -2468,11 +2276,11 @@
       <c r="P22">
         <v>15965.364846295015</v>
       </c>
-      <c r="Q22" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="R22" s="2" t="s">
-        <v>107</v>
+      <c r="Q22">
+        <v>185802.14</v>
+      </c>
+      <c r="R22">
+        <v>349103.66</v>
       </c>
       <c r="S22" s="8">
         <v>489061.86</v>
@@ -2533,11 +2341,11 @@
       <c r="P23">
         <v>15965.364846295015</v>
       </c>
-      <c r="Q23" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="R23" s="2" t="s">
-        <v>108</v>
+      <c r="Q23">
+        <v>182026.51</v>
+      </c>
+      <c r="R23">
+        <v>341975.1</v>
       </c>
       <c r="S23" s="8">
         <v>489061.86</v>
@@ -2598,11 +2406,11 @@
       <c r="P24">
         <v>15965.364846295015</v>
       </c>
-      <c r="Q24" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="R24" s="2" t="s">
-        <v>109</v>
+      <c r="Q24">
+        <v>178332.87</v>
+      </c>
+      <c r="R24">
+        <v>334991.90000000002</v>
       </c>
       <c r="S24" s="8">
         <v>489061.86</v>
@@ -2663,11 +2471,11 @@
       <c r="P25">
         <v>15965.364846295015</v>
       </c>
-      <c r="Q25" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="R25" s="2" t="s">
-        <v>110</v>
+      <c r="Q25">
+        <v>174720.11</v>
+      </c>
+      <c r="R25">
+        <v>328152.28999999998</v>
       </c>
       <c r="S25" s="8">
         <v>489061.86</v>
@@ -2728,11 +2536,11 @@
       <c r="P26">
         <v>15965.364846295015</v>
       </c>
-      <c r="Q26" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="R26" s="2" t="s">
-        <v>111</v>
+      <c r="Q26">
+        <v>171187.17</v>
+      </c>
+      <c r="R26">
+        <v>321454.53999999998</v>
       </c>
       <c r="S26" s="8">
         <v>489061.86</v>
@@ -2793,11 +2601,11 @@
       <c r="P27">
         <v>15965.364846295015</v>
       </c>
-      <c r="Q27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="R27" s="2" t="s">
-        <v>112</v>
+      <c r="Q27">
+        <v>167732.98000000001</v>
+      </c>
+      <c r="R27">
+        <v>314897</v>
       </c>
       <c r="S27" s="8">
         <v>489061.86</v>
@@ -2858,11 +2666,11 @@
       <c r="P28">
         <v>15602.06928231802</v>
       </c>
-      <c r="Q28" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="R28" s="2" t="s">
-        <v>113</v>
+      <c r="Q28">
+        <v>164356.51999999999</v>
+      </c>
+      <c r="R28">
+        <v>308477.99</v>
       </c>
       <c r="S28" s="8">
         <v>489061.86</v>
@@ -10953,7 +10761,6 @@
         <v>2025</v>
       </c>
       <c r="B3">
-        <f>SUM(B2*1.04)</f>
         <v>68120</v>
       </c>
       <c r="C3">
@@ -10971,7 +10778,6 @@
         <v>2026</v>
       </c>
       <c r="B4">
-        <f t="shared" ref="B4:B8" si="0">SUM(B3*1.04)</f>
         <v>70844.800000000003</v>
       </c>
       <c r="C4">
@@ -10989,7 +10795,6 @@
         <v>2027</v>
       </c>
       <c r="B5">
-        <f t="shared" si="0"/>
         <v>73678.592000000004</v>
       </c>
       <c r="C5">
@@ -11007,7 +10812,6 @@
         <v>2028</v>
       </c>
       <c r="B6">
-        <f t="shared" si="0"/>
         <v>76625.735680000013</v>
       </c>
       <c r="C6">
@@ -11025,8 +10829,7 @@
         <v>2029</v>
       </c>
       <c r="B7">
-        <f t="shared" si="0"/>
-        <v>79690.765107200015</v>
+        <v>79690.765107200001</v>
       </c>
       <c r="C7">
         <v>6410</v>
@@ -11043,7 +10846,6 @@
         <v>2030</v>
       </c>
       <c r="B8">
-        <f t="shared" si="0"/>
         <v>82878.395711488018</v>
       </c>
       <c r="C8">
@@ -11152,7 +10954,7 @@
         <v>20887.355507945696</v>
       </c>
       <c r="D14">
-        <v>29532.863049035175</v>
+        <v>31009.506201486936</v>
       </c>
       <c r="E14">
         <v>999999</v>
@@ -11169,7 +10971,7 @@
         <v>22976.091058740265</v>
       </c>
       <c r="D15">
-        <v>29532.863049035175</v>
+        <v>32559.981511561284</v>
       </c>
       <c r="E15">
         <v>999999</v>
@@ -11186,7 +10988,7 @@
         <v>25273.700164614293</v>
       </c>
       <c r="D16">
-        <v>29532.863049035175</v>
+        <v>34187.980587139347</v>
       </c>
       <c r="E16">
         <v>999999</v>
@@ -11203,7 +11005,7 @@
         <v>27801.070181075727</v>
       </c>
       <c r="D17">
-        <v>29532.863049035175</v>
+        <v>35897.379616496313</v>
       </c>
       <c r="E17">
         <v>999999</v>
@@ -11220,7 +11022,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D18">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E18">
         <v>999999</v>
@@ -11237,7 +11039,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D19">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E19">
         <v>999999</v>
@@ -11254,7 +11056,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D20">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E20">
         <v>999999</v>
@@ -11271,7 +11073,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D21">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E21">
         <v>999999</v>
@@ -11288,7 +11090,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D22">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E22">
         <v>999999</v>
@@ -11305,7 +11107,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D23">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E23">
         <v>999999</v>
@@ -11322,7 +11124,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D24">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E24">
         <v>999999</v>
@@ -11339,7 +11141,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D25">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E25">
         <v>999999</v>
@@ -11356,7 +11158,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D26">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E26">
         <v>999999</v>
@@ -11373,7 +11175,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D27">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E27">
         <v>999999</v>
@@ -11390,7 +11192,7 @@
         <v>30581.177199183301</v>
       </c>
       <c r="D28">
-        <v>30581.177199183301</v>
+        <v>37692.24859732113</v>
       </c>
       <c r="E28">
         <v>999999</v>
@@ -11403,263 +11205,76 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" customWidth="1"/>
     <col min="5" max="5" width="25.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>114</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
-        <v>115</v>
+        <v>61</v>
       </c>
       <c r="C1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D1" t="s">
-        <v>123</v>
+        <v>62</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>211011120.00000003</v>
+      <c r="B2" s="8">
+        <v>286654747.94721401</v>
       </c>
       <c r="C2" s="8">
-        <v>9.61</v>
-      </c>
-      <c r="D2">
+        <v>29.19</v>
+      </c>
+      <c r="D2" s="12">
         <v>6.9372000000000003E-2</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>117</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>2126230105.0000002</v>
+      <c r="B3" s="8">
+        <v>1109104864.5590901</v>
       </c>
       <c r="C3" s="8">
-        <v>13.66</v>
-      </c>
-      <c r="D3">
+        <v>42.69</v>
+      </c>
+      <c r="D3" s="12">
         <v>4.9157999999999993E-2</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>81239281.200000003</v>
+      <c r="B4" s="8">
+        <v>293070999999.70697</v>
       </c>
       <c r="C4" s="8">
-        <v>15.66</v>
-      </c>
-      <c r="D4">
+        <v>94.17</v>
+      </c>
+      <c r="D4" s="12">
         <v>4.4639999999999999E-2</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>167331818.16000003</v>
-      </c>
-      <c r="C5" s="8">
-        <v>17.489999999999998</v>
-      </c>
-      <c r="D5">
-        <v>4.4639999999999999E-2</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>90734781.600000009</v>
-      </c>
-      <c r="C6" s="8">
-        <v>18.18</v>
-      </c>
-      <c r="D6">
-        <v>4.6440000000000002E-2</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>1055055600.0000001</v>
-      </c>
-      <c r="C7" s="8">
-        <v>18.87</v>
-      </c>
-      <c r="D7">
-        <v>4.4639999999999999E-2</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>179359452.00000003</v>
-      </c>
-      <c r="C8" s="8">
-        <v>20.09</v>
-      </c>
-      <c r="D8">
-        <v>4.0806000000000002E-2</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>2321122320</v>
-      </c>
-      <c r="C9" s="8">
-        <v>23.61</v>
-      </c>
-      <c r="D9">
-        <v>0.19746</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>633033360</v>
-      </c>
-      <c r="C10" s="8">
-        <v>25.71</v>
-      </c>
-      <c r="D10">
-        <v>5.1839999999999997E-2</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>453673908.00000006</v>
-      </c>
-      <c r="C11" s="8">
-        <v>27.37</v>
-      </c>
-      <c r="D11">
-        <v>5.7239999999999999E-2</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>397755961.20000005</v>
-      </c>
-      <c r="C12" s="8">
-        <v>27.66</v>
-      </c>
-      <c r="D12">
-        <v>5.7239999999999999E-2</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>1477077840.0000002</v>
-      </c>
-      <c r="C13" s="8">
-        <v>34.409999999999997</v>
-      </c>
-      <c r="D13">
-        <v>3.9239999999999997E-2</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>220506620.40000001</v>
-      </c>
-      <c r="C14" s="8">
-        <v>34.409999999999997</v>
-      </c>
-      <c r="D14">
-        <v>5.7239999999999999E-2</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>99999999999</v>
-      </c>
-      <c r="C15" s="8">
-        <v>1000</v>
-      </c>
-      <c r="D15">
-        <v>0.19746</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>124</v>
+      <c r="E4" s="11" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Did some more changes to installable Capacity
Maybe Elec Demand is too high
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4527232-E70C-4408-BA96-E521B1020982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25E8F9F3-0BF6-4B0F-8696-ACA83E9A43F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="7" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -11231,7 +11231,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="8">
-        <v>286654747.94721401</v>
+        <v>270613611.10000002</v>
       </c>
       <c r="C2" s="8">
         <v>29.19</v>
@@ -11248,7 +11248,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="8">
-        <v>1109104864.5590901</v>
+        <v>1047284444.4400001</v>
       </c>
       <c r="C3" s="8">
         <v>42.69</v>
@@ -11265,10 +11265,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="8">
-        <v>293070999999.70697</v>
+        <v>2930833333.3299999</v>
       </c>
       <c r="C4" s="8">
-        <v>94.17</v>
+        <v>150</v>
       </c>
       <c r="D4" s="12">
         <v>4.4639999999999999E-2</v>

</xml_diff>

<commit_message>
Changed the formulation of maximum Increase and limited eu prim and eusec by available build out
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB3966CB-6233-4861-A1AB-524FA1662BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EE77B3D-C3B4-4E0C-AFC1-23B6CEAF6A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="-5565" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -9413,10 +9413,10 @@
         <v>0</v>
       </c>
       <c r="I2" s="6">
-        <v>0.24030000000000001</v>
+        <v>9.8000000000000004E-2</v>
       </c>
       <c r="J2" s="6">
-        <v>0.38879999999999998</v>
+        <v>0.2</v>
       </c>
       <c r="K2" s="5">
         <v>0.8</v>
@@ -9495,7 +9495,7 @@
       <c r="H3" s="5">
         <v>0</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="6">
         <v>8.5999999999999993E-2</v>
       </c>
       <c r="J3" s="6">
@@ -9578,7 +9578,7 @@
       <c r="H4" s="5">
         <v>0</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="6">
         <v>8.5999999999999993E-2</v>
       </c>
       <c r="J4" s="6">
@@ -9662,7 +9662,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="6">
-        <v>0.27439999999999998</v>
+        <v>0.3</v>
       </c>
       <c r="J5" s="6">
         <v>0.3</v>

</xml_diff>

<commit_message>
Adds comprehensive plotting and analysis suite
Adds a comprehensive suite of plotting and analysis functions for scenario results. This includes functions for:

- Loading and processing data from Excel files.
- Plotting generation mixes, renewable breakdowns, and scrap comparisons.
- Performing LNG demand analysis with range plots and boxplots.
- Analyzing system costs with boxplots.
- Generating scatter plots of cumulative capacities with optional clustering.
- Visualizing capacity clusters and flows using bar charts and Sankey diagrams.

These tools provide a more detailed and insightful analysis of different energy scenarios.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89486067-0CA3-4462-89DC-4E65E91C57C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67065" yWindow="-5580" windowWidth="38670" windowHeight="21150" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="67230" yWindow="-4800" windowWidth="13830" windowHeight="7035" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -9419,7 +9419,7 @@
         <v>0.2</v>
       </c>
       <c r="K2" s="5">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L2" s="5">
         <v>0.8</v>
@@ -9502,7 +9502,7 @@
         <v>0.2</v>
       </c>
       <c r="K3" s="5">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L3" s="5">
         <v>0.8</v>
@@ -9585,7 +9585,7 @@
         <v>0.2</v>
       </c>
       <c r="K4" s="5">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L4" s="5">
         <v>0.8</v>
@@ -9668,7 +9668,7 @@
         <v>0.3</v>
       </c>
       <c r="K5" s="5">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L5" s="5">
         <v>0.8</v>
@@ -12638,26 +12638,6 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -12665,6 +12645,26 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Model runs through with new package. there is a calculation error somewhere, way less caps then prior runs suggested installed
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-extension/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F8DECA5-D051-4C44-8AE6-0B1E7095FB46}"/>
+  <xr:revisionPtr revIDLastSave="229" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AD15F06-E503-4891-AF71-B5AEAB14D995}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="735" yWindow="735" windowWidth="28800" windowHeight="15345" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" firstSheet="6" activeTab="11" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -22,6 +22,11 @@
     <sheet name="stocklvl" sheetId="7" r:id="rId7"/>
     <sheet name="installable_capacity" sheetId="3" r:id="rId8"/>
     <sheet name="gas_block" sheetId="13" r:id="rId9"/>
+    <sheet name="Tech_Stage_Specs" sheetId="14" r:id="rId10"/>
+    <sheet name="Materieal_Intensity" sheetId="15" r:id="rId11"/>
+    <sheet name="Material_Market" sheetId="17" r:id="rId12"/>
+    <sheet name="Component_Map" sheetId="18" r:id="rId13"/>
+    <sheet name="Cost_Data" sheetId="16" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">gas_block!$B$1:$B$109</definedName>
@@ -47,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="157">
   <si>
     <t>Value</t>
   </si>
@@ -263,6 +268,261 @@
   </si>
   <si>
     <t>WTF_LNG</t>
+  </si>
+  <si>
+    <t>build_time_lag</t>
+  </si>
+  <si>
+    <t>energy_needs</t>
+  </si>
+  <si>
+    <t>is_final_stage</t>
+  </si>
+  <si>
+    <t>solarPV</t>
+  </si>
+  <si>
+    <t>windon</t>
+  </si>
+  <si>
+    <t>windoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">note </t>
+  </si>
+  <si>
+    <t>finished</t>
+  </si>
+  <si>
+    <t>host</t>
+  </si>
+  <si>
+    <t>unique</t>
+  </si>
+  <si>
+    <t>Technology</t>
+  </si>
+  <si>
+    <t>Stage</t>
+  </si>
+  <si>
+    <t>Material</t>
+  </si>
+  <si>
+    <t>Ingot</t>
+  </si>
+  <si>
+    <t>Silicon</t>
+  </si>
+  <si>
+    <t>3.0</t>
+  </si>
+  <si>
+    <t>0.95</t>
+  </si>
+  <si>
+    <t>Cell</t>
+  </si>
+  <si>
+    <t>Silver</t>
+  </si>
+  <si>
+    <t>0.05</t>
+  </si>
+  <si>
+    <t>0.98</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Glass</t>
+  </si>
+  <si>
+    <t>40.0</t>
+  </si>
+  <si>
+    <t>38.0</t>
+  </si>
+  <si>
+    <t>0.90</t>
+  </si>
+  <si>
+    <t>Aluminum</t>
+  </si>
+  <si>
+    <t>5.0</t>
+  </si>
+  <si>
+    <t>0.85</t>
+  </si>
+  <si>
+    <t>Blade</t>
+  </si>
+  <si>
+    <t>Composite</t>
+  </si>
+  <si>
+    <t>12.0</t>
+  </si>
+  <si>
+    <t>0.50</t>
+  </si>
+  <si>
+    <t>Tower</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
+    <t>150.0</t>
+  </si>
+  <si>
+    <t>Nacelle</t>
+  </si>
+  <si>
+    <t>Copper</t>
+  </si>
+  <si>
+    <t>2.0</t>
+  </si>
+  <si>
+    <t>RareEarth</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>0.80</t>
+  </si>
+  <si>
+    <t>Batteries</t>
+  </si>
+  <si>
+    <t>Lithium</t>
+  </si>
+  <si>
+    <t>0.8</t>
+  </si>
+  <si>
+    <t>Cobalt</t>
+  </si>
+  <si>
+    <t>0.2</t>
+  </si>
+  <si>
+    <t>wndon</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Wafer</t>
+  </si>
+  <si>
+    <t>80.0</t>
+  </si>
+  <si>
+    <t>20.0</t>
+  </si>
+  <si>
+    <t>4.0</t>
+  </si>
+  <si>
+    <t>120.0</t>
+  </si>
+  <si>
+    <t>70.0</t>
+  </si>
+  <si>
+    <t>60.0</t>
+  </si>
+  <si>
+    <t>25.0</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>90.0</t>
+  </si>
+  <si>
+    <t>Assembly</t>
+  </si>
+  <si>
+    <t>10.0</t>
+  </si>
+  <si>
+    <t>15.0</t>
+  </si>
+  <si>
+    <t>Foundation</t>
+  </si>
+  <si>
+    <t>200.0</t>
+  </si>
+  <si>
+    <t>250.0</t>
+  </si>
+  <si>
+    <t>30.0</t>
+  </si>
+  <si>
+    <t>Pack</t>
+  </si>
+  <si>
+    <t>0.9</t>
+  </si>
+  <si>
+    <t>0.10</t>
+  </si>
+  <si>
+    <t>Cons_Tech</t>
+  </si>
+  <si>
+    <t>Cons_Stage</t>
+  </si>
+  <si>
+    <t>Input_Tech</t>
+  </si>
+  <si>
+    <t>Input_Stage</t>
+  </si>
+  <si>
+    <t>Ratio</t>
+  </si>
+  <si>
+    <t>rec_efficiency</t>
+  </si>
+  <si>
+    <t>intensity</t>
+  </si>
+  <si>
+    <t>scrap_content</t>
+  </si>
+  <si>
+    <t>mining_cost</t>
+  </si>
+  <si>
+    <t>import_cost</t>
+  </si>
+  <si>
+    <t>mining_limit</t>
+  </si>
+  <si>
+    <t>capex_base</t>
+  </si>
+  <si>
+    <t>opex_var_base</t>
+  </si>
+  <si>
+    <t>import_cost_part</t>
+  </si>
+  <si>
+    <t>init_cap</t>
   </si>
 </sst>
 </file>
@@ -491,6 +751,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -850,6 +1114,1292 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8C0D52F-0ADA-4AC5-8A50-4699398C8904}">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" t="s">
+        <v>156</v>
+      </c>
+      <c r="G1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>150</v>
+      </c>
+      <c r="F2">
+        <v>100</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>100</v>
+      </c>
+      <c r="F3">
+        <v>100</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>100</v>
+      </c>
+      <c r="F4">
+        <v>100</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>100</v>
+      </c>
+      <c r="F5">
+        <v>100</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>100</v>
+      </c>
+      <c r="F6">
+        <v>100</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>100</v>
+      </c>
+      <c r="F7">
+        <v>100</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" t="s">
+        <v>108</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>100</v>
+      </c>
+      <c r="F8">
+        <v>100</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>100</v>
+      </c>
+      <c r="F9">
+        <v>100</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" t="s">
+        <v>135</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>100</v>
+      </c>
+      <c r="F10">
+        <v>100</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>100</v>
+      </c>
+      <c r="F11">
+        <v>100</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>80</v>
+      </c>
+      <c r="F12">
+        <v>100</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>114</v>
+      </c>
+      <c r="C13" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>20</v>
+      </c>
+      <c r="F13">
+        <v>100</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FA1A697-84AA-4F97-BE70-81695B57512E}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E3" t="s">
+        <v>91</v>
+      </c>
+      <c r="F3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" t="s">
+        <v>103</v>
+      </c>
+      <c r="E6" t="s">
+        <v>103</v>
+      </c>
+      <c r="F6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" t="s">
+        <v>107</v>
+      </c>
+      <c r="F7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" t="s">
+        <v>109</v>
+      </c>
+      <c r="D8" t="s">
+        <v>110</v>
+      </c>
+      <c r="E8" t="s">
+        <v>110</v>
+      </c>
+      <c r="F8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" t="s">
+        <v>112</v>
+      </c>
+      <c r="E9" t="s">
+        <v>112</v>
+      </c>
+      <c r="F9" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>114</v>
+      </c>
+      <c r="B10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D10" t="s">
+        <v>116</v>
+      </c>
+      <c r="E10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>114</v>
+      </c>
+      <c r="B11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D11" t="s">
+        <v>118</v>
+      </c>
+      <c r="E11" t="s">
+        <v>118</v>
+      </c>
+      <c r="F11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03BB5A9E-0DE2-4C9D-A6F4-EBF765E41A9E}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2024</v>
+      </c>
+      <c r="B2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2">
+        <v>1000000</v>
+      </c>
+      <c r="D2">
+        <v>1800</v>
+      </c>
+      <c r="E2">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2024</v>
+      </c>
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3">
+        <v>5000</v>
+      </c>
+      <c r="D3">
+        <v>650000</v>
+      </c>
+      <c r="E3">
+        <v>700000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2024</v>
+      </c>
+      <c r="B4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4">
+        <v>5000000</v>
+      </c>
+      <c r="D4">
+        <v>100</v>
+      </c>
+      <c r="E4">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C5">
+        <v>2000000</v>
+      </c>
+      <c r="D5">
+        <v>2000</v>
+      </c>
+      <c r="E5">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2024</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>500000</v>
+      </c>
+      <c r="D6">
+        <v>3000</v>
+      </c>
+      <c r="E6">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2024</v>
+      </c>
+      <c r="B7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7">
+        <v>10000000</v>
+      </c>
+      <c r="D7">
+        <v>600</v>
+      </c>
+      <c r="E7">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C8">
+        <v>800000</v>
+      </c>
+      <c r="D8">
+        <v>8000</v>
+      </c>
+      <c r="E8">
+        <v>9500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2024</v>
+      </c>
+      <c r="B9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9">
+        <v>20000</v>
+      </c>
+      <c r="D9">
+        <v>40000</v>
+      </c>
+      <c r="E9">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2024</v>
+      </c>
+      <c r="B10" t="s">
+        <v>115</v>
+      </c>
+      <c r="C10">
+        <v>150000</v>
+      </c>
+      <c r="D10">
+        <v>15000</v>
+      </c>
+      <c r="E10">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2024</v>
+      </c>
+      <c r="B11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11">
+        <v>50000</v>
+      </c>
+      <c r="D11">
+        <v>30000</v>
+      </c>
+      <c r="E11">
+        <v>35000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{996B2112-D2EE-4E9F-B294-4222E881A3C9}">
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" t="s">
+        <v>132</v>
+      </c>
+      <c r="C6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" t="s">
+        <v>132</v>
+      </c>
+      <c r="C9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C10" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C11" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" t="s">
+        <v>108</v>
+      </c>
+      <c r="E11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" t="s">
+        <v>135</v>
+      </c>
+      <c r="E12" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CE844EE-882F-4833-8B87-00A8BB665263}">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F1" t="s">
+        <v>154</v>
+      </c>
+      <c r="G1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2024</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E2" t="s">
+        <v>126</v>
+      </c>
+      <c r="F2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2024</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E3" t="s">
+        <v>127</v>
+      </c>
+      <c r="F3" t="s">
+        <v>141</v>
+      </c>
+      <c r="G3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2024</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2024</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E5" t="s">
+        <v>129</v>
+      </c>
+      <c r="F5" t="s">
+        <v>116</v>
+      </c>
+      <c r="G5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2024</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E6" t="s">
+        <v>131</v>
+      </c>
+      <c r="F6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2024</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E7" t="s">
+        <v>123</v>
+      </c>
+      <c r="F7" t="s">
+        <v>141</v>
+      </c>
+      <c r="G7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F8" t="s">
+        <v>125</v>
+      </c>
+      <c r="G8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2024</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" t="s">
+        <v>132</v>
+      </c>
+      <c r="E9" t="s">
+        <v>133</v>
+      </c>
+      <c r="F9" t="s">
+        <v>130</v>
+      </c>
+      <c r="G9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2024</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" t="s">
+        <v>135</v>
+      </c>
+      <c r="E10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F10" t="s">
+        <v>99</v>
+      </c>
+      <c r="G10" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2024</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G11" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2024</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>114</v>
+      </c>
+      <c r="D12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" t="s">
+        <v>123</v>
+      </c>
+      <c r="F12" t="s">
+        <v>87</v>
+      </c>
+      <c r="G12" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2024</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" t="s">
+        <v>139</v>
+      </c>
+      <c r="E13" t="s">
+        <v>138</v>
+      </c>
+      <c r="F13" t="s">
+        <v>130</v>
+      </c>
+      <c r="G13" t="s">
+        <v>141</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6185AF38-42FD-4CFF-B287-2FCFFF6C6EF3}">
   <dimension ref="A1:U28"/>

</xml_diff>

<commit_message>
Refactors material constraints and data loading
Streamlines the data loading process for material constraints by switching from a monolithic Excel reader to targeted sheet processing, improving modularity and maintainability.

Fixes an issue with legacy capacity lookup, ensuring correct values are used. Adds optional retirement logic for legacy factories.

Introduces a stockpile holding cost to reflect storage expenses and updates variable indexing to enhance model accuracy.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-extension/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="229" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AD15F06-E503-4891-AF71-B5AEAB14D995}"/>
+  <xr:revisionPtr revIDLastSave="270" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A20A2E7-1617-4C82-9341-AEA66E3C0C5A}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" firstSheet="6" activeTab="11" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="14" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -23,10 +23,11 @@
     <sheet name="installable_capacity" sheetId="3" r:id="rId8"/>
     <sheet name="gas_block" sheetId="13" r:id="rId9"/>
     <sheet name="Tech_Stage_Specs" sheetId="14" r:id="rId10"/>
-    <sheet name="Materieal_Intensity" sheetId="15" r:id="rId11"/>
+    <sheet name="Material_Intensity" sheetId="15" r:id="rId11"/>
     <sheet name="Material_Market" sheetId="17" r:id="rId12"/>
     <sheet name="Component_Map" sheetId="18" r:id="rId13"/>
     <sheet name="Cost_Data" sheetId="16" r:id="rId14"/>
+    <sheet name="Import_Cost_Stage" sheetId="19" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">gas_block!$B$1:$B$109</definedName>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="167">
   <si>
     <t>Value</t>
   </si>
@@ -411,9 +412,6 @@
     <t>0.2</t>
   </si>
   <si>
-    <t>wndon</t>
-  </si>
-  <si>
     <t>Year</t>
   </si>
   <si>
@@ -474,9 +472,6 @@
     <t>Pack</t>
   </si>
   <si>
-    <t>0.9</t>
-  </si>
-  <si>
     <t>0.10</t>
   </si>
   <si>
@@ -523,6 +518,42 @@
   </si>
   <si>
     <t>init_cap</t>
+  </si>
+  <si>
+    <t>solarPV_Ingot</t>
+  </si>
+  <si>
+    <t>solarPV_Wafer</t>
+  </si>
+  <si>
+    <t>solarPV_Cell</t>
+  </si>
+  <si>
+    <t>windon_Blade</t>
+  </si>
+  <si>
+    <t>windon_Tower</t>
+  </si>
+  <si>
+    <t>windon_Nacelle</t>
+  </si>
+  <si>
+    <t>windon_Assembly</t>
+  </si>
+  <si>
+    <t>windoff_Foundation</t>
+  </si>
+  <si>
+    <t>windoff_Assembly</t>
+  </si>
+  <si>
+    <t>bateries_Cell</t>
+  </si>
+  <si>
+    <t>batteries_Pack</t>
+  </si>
+  <si>
+    <t>solarPV_Module</t>
   </si>
 </sst>
 </file>
@@ -1121,7 +1152,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B1" t="s">
         <v>82</v>
@@ -1136,7 +1167,7 @@
         <v>73</v>
       </c>
       <c r="F1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="G1" t="s">
         <v>74</v>
@@ -1176,7 +1207,7 @@
         <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1326,7 +1357,7 @@
         <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1352,7 +1383,7 @@
         <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1378,7 +1409,7 @@
         <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1427,7 +1458,7 @@
         <v>114</v>
       </c>
       <c r="C13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1464,13 +1495,13 @@
         <v>84</v>
       </c>
       <c r="D1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1615,7 +1646,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>119</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
         <v>108</v>
@@ -1686,19 +1717,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B1" t="s">
         <v>84</v>
       </c>
       <c r="C1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1883,19 +1914,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1" t="s">
         <v>142</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>143</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>144</v>
-      </c>
-      <c r="D1" t="s">
-        <v>145</v>
-      </c>
-      <c r="E1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1903,7 +1934,7 @@
         <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C2" t="s">
         <v>75</v>
@@ -1912,7 +1943,7 @@
         <v>85</v>
       </c>
       <c r="E2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1926,10 +1957,10 @@
         <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1946,7 +1977,7 @@
         <v>89</v>
       </c>
       <c r="E4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1954,7 +1985,7 @@
         <v>114</v>
       </c>
       <c r="B5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C5" t="s">
         <v>114</v>
@@ -1963,7 +1994,7 @@
         <v>89</v>
       </c>
       <c r="E5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1971,7 +2002,7 @@
         <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C6" t="s">
         <v>76</v>
@@ -1980,7 +2011,7 @@
         <v>101</v>
       </c>
       <c r="E6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1988,7 +2019,7 @@
         <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C7" t="s">
         <v>76</v>
@@ -1997,7 +2028,7 @@
         <v>105</v>
       </c>
       <c r="E7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2005,7 +2036,7 @@
         <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C8" t="s">
         <v>76</v>
@@ -2014,7 +2045,7 @@
         <v>108</v>
       </c>
       <c r="E8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2022,7 +2053,7 @@
         <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C9" t="s">
         <v>76</v>
@@ -2031,7 +2062,7 @@
         <v>101</v>
       </c>
       <c r="E9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2039,7 +2070,7 @@
         <v>77</v>
       </c>
       <c r="B10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C10" t="s">
         <v>76</v>
@@ -2048,7 +2079,7 @@
         <v>105</v>
       </c>
       <c r="E10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2056,7 +2087,7 @@
         <v>77</v>
       </c>
       <c r="B11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C11" t="s">
         <v>76</v>
@@ -2065,7 +2096,7 @@
         <v>108</v>
       </c>
       <c r="E11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2073,16 +2104,16 @@
         <v>77</v>
       </c>
       <c r="B12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C12" t="s">
         <v>77</v>
       </c>
       <c r="D12" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -2097,10 +2128,10 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" t="s">
         <v>120</v>
-      </c>
-      <c r="B1" t="s">
-        <v>121</v>
       </c>
       <c r="C1" t="s">
         <v>82</v>
@@ -2109,13 +2140,13 @@
         <v>83</v>
       </c>
       <c r="E1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G1" t="s">
         <v>153</v>
-      </c>
-      <c r="F1" t="s">
-        <v>154</v>
-      </c>
-      <c r="G1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -2132,10 +2163,10 @@
         <v>85</v>
       </c>
       <c r="E2" t="s">
-        <v>126</v>
-      </c>
-      <c r="F2" t="s">
         <v>125</v>
+      </c>
+      <c r="F2">
+        <v>1000000</v>
       </c>
       <c r="G2" t="s">
         <v>99</v>
@@ -2152,16 +2183,16 @@
         <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E3" t="s">
-        <v>127</v>
-      </c>
-      <c r="F3" t="s">
-        <v>141</v>
+        <v>126</v>
+      </c>
+      <c r="F3">
+        <v>1000000</v>
       </c>
       <c r="G3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -2178,13 +2209,13 @@
         <v>89</v>
       </c>
       <c r="E4" t="s">
-        <v>128</v>
-      </c>
-      <c r="F4" t="s">
-        <v>110</v>
+        <v>127</v>
+      </c>
+      <c r="F4">
+        <v>1000000</v>
       </c>
       <c r="G4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -2201,13 +2232,13 @@
         <v>93</v>
       </c>
       <c r="E5" t="s">
+        <v>128</v>
+      </c>
+      <c r="F5">
+        <v>1000000</v>
+      </c>
+      <c r="G5" t="s">
         <v>129</v>
-      </c>
-      <c r="F5" t="s">
-        <v>116</v>
-      </c>
-      <c r="G5" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -2224,10 +2255,10 @@
         <v>101</v>
       </c>
       <c r="E6" t="s">
-        <v>131</v>
-      </c>
-      <c r="F6" t="s">
-        <v>140</v>
+        <v>130</v>
+      </c>
+      <c r="F6">
+        <v>1000000</v>
       </c>
       <c r="G6" t="s">
         <v>87</v>
@@ -2247,10 +2278,10 @@
         <v>105</v>
       </c>
       <c r="E7" t="s">
-        <v>123</v>
-      </c>
-      <c r="F7" t="s">
-        <v>141</v>
+        <v>122</v>
+      </c>
+      <c r="F7">
+        <v>1000000</v>
       </c>
       <c r="G7" t="s">
         <v>110</v>
@@ -2272,8 +2303,8 @@
       <c r="E8" t="s">
         <v>107</v>
       </c>
-      <c r="F8" t="s">
-        <v>125</v>
+      <c r="F8">
+        <v>1000000</v>
       </c>
       <c r="G8" t="s">
         <v>99</v>
@@ -2290,16 +2321,16 @@
         <v>76</v>
       </c>
       <c r="D9" t="s">
+        <v>131</v>
+      </c>
+      <c r="E9" t="s">
         <v>132</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9">
+        <v>1000000</v>
+      </c>
+      <c r="G9" t="s">
         <v>133</v>
-      </c>
-      <c r="F9" t="s">
-        <v>130</v>
-      </c>
-      <c r="G9" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -2313,16 +2344,16 @@
         <v>77</v>
       </c>
       <c r="D10" t="s">
+        <v>134</v>
+      </c>
+      <c r="E10" t="s">
         <v>135</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10">
+        <v>1000000</v>
+      </c>
+      <c r="G10" t="s">
         <v>136</v>
-      </c>
-      <c r="F10" t="s">
-        <v>99</v>
-      </c>
-      <c r="G10" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -2336,16 +2367,16 @@
         <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E11" t="s">
-        <v>124</v>
-      </c>
-      <c r="F11" t="s">
-        <v>110</v>
+        <v>123</v>
+      </c>
+      <c r="F11">
+        <v>1000000</v>
       </c>
       <c r="G11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -2362,13 +2393,13 @@
         <v>89</v>
       </c>
       <c r="E12" t="s">
-        <v>123</v>
-      </c>
-      <c r="F12" t="s">
-        <v>87</v>
+        <v>122</v>
+      </c>
+      <c r="F12">
+        <v>1000000</v>
       </c>
       <c r="G12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -2382,21 +2413,1180 @@
         <v>114</v>
       </c>
       <c r="D13" t="s">
+        <v>138</v>
+      </c>
+      <c r="E13" t="s">
+        <v>137</v>
+      </c>
+      <c r="F13">
+        <v>1000000</v>
+      </c>
+      <c r="G13" t="s">
         <v>139</v>
-      </c>
-      <c r="E13" t="s">
-        <v>138</v>
-      </c>
-      <c r="F13" t="s">
-        <v>130</v>
-      </c>
-      <c r="G13" t="s">
-        <v>141</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B74DFEF-01D9-4B2D-A936-BF616F091054}">
+  <dimension ref="A1:M28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F1" t="s">
+        <v>158</v>
+      </c>
+      <c r="G1" t="s">
+        <v>159</v>
+      </c>
+      <c r="H1" t="s">
+        <v>160</v>
+      </c>
+      <c r="I1" t="s">
+        <v>161</v>
+      </c>
+      <c r="J1" t="s">
+        <v>162</v>
+      </c>
+      <c r="K1" t="s">
+        <v>163</v>
+      </c>
+      <c r="L1" t="s">
+        <v>164</v>
+      </c>
+      <c r="M1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2024</v>
+      </c>
+      <c r="B2">
+        <v>9999999</v>
+      </c>
+      <c r="C2">
+        <v>9999999</v>
+      </c>
+      <c r="D2">
+        <v>9999999</v>
+      </c>
+      <c r="E2">
+        <v>250240</v>
+      </c>
+      <c r="F2">
+        <v>9999999</v>
+      </c>
+      <c r="G2">
+        <v>9999999</v>
+      </c>
+      <c r="H2">
+        <v>9999999</v>
+      </c>
+      <c r="I2" s="8">
+        <v>1052044.8400000001</v>
+      </c>
+      <c r="J2">
+        <v>9999999</v>
+      </c>
+      <c r="K2" s="8">
+        <v>1775265.6417320003</v>
+      </c>
+      <c r="L2">
+        <v>9999999</v>
+      </c>
+      <c r="M2">
+        <v>280439.83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2025</v>
+      </c>
+      <c r="B3">
+        <v>9999999</v>
+      </c>
+      <c r="C3">
+        <v>9999999</v>
+      </c>
+      <c r="D3">
+        <v>9999999</v>
+      </c>
+      <c r="E3">
+        <v>246486.39999999999</v>
+      </c>
+      <c r="F3">
+        <v>9999999</v>
+      </c>
+      <c r="G3">
+        <v>9999999</v>
+      </c>
+      <c r="H3">
+        <v>9999999</v>
+      </c>
+      <c r="I3" s="8">
+        <v>1042480.7960000001</v>
+      </c>
+      <c r="J3">
+        <v>9999999</v>
+      </c>
+      <c r="K3" s="8">
+        <v>1722922.372057667</v>
+      </c>
+      <c r="L3">
+        <v>9999999</v>
+      </c>
+      <c r="M3">
+        <v>274754.90999999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2026</v>
+      </c>
+      <c r="B4">
+        <v>9999999</v>
+      </c>
+      <c r="C4">
+        <v>9999999</v>
+      </c>
+      <c r="D4">
+        <v>9999999</v>
+      </c>
+      <c r="E4">
+        <v>242789.10399999999</v>
+      </c>
+      <c r="F4">
+        <v>9999999</v>
+      </c>
+      <c r="G4">
+        <v>9999999</v>
+      </c>
+      <c r="H4">
+        <v>9999999</v>
+      </c>
+      <c r="I4" s="8">
+        <v>1032916.7520000001</v>
+      </c>
+      <c r="J4">
+        <v>9999999</v>
+      </c>
+      <c r="K4" s="8">
+        <v>1670579.1023833335</v>
+      </c>
+      <c r="L4">
+        <v>9999999</v>
+      </c>
+      <c r="M4">
+        <v>269179.44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2027</v>
+      </c>
+      <c r="B5">
+        <v>9999999</v>
+      </c>
+      <c r="C5">
+        <v>9999999</v>
+      </c>
+      <c r="D5">
+        <v>9999999</v>
+      </c>
+      <c r="E5">
+        <v>239147.26740000001</v>
+      </c>
+      <c r="F5">
+        <v>9999999</v>
+      </c>
+      <c r="G5">
+        <v>9999999</v>
+      </c>
+      <c r="H5">
+        <v>9999999</v>
+      </c>
+      <c r="I5" s="8">
+        <v>1023352.708</v>
+      </c>
+      <c r="J5">
+        <v>9999999</v>
+      </c>
+      <c r="K5" s="8">
+        <v>1618235.832709</v>
+      </c>
+      <c r="L5">
+        <v>9999999</v>
+      </c>
+      <c r="M5">
+        <v>263711.78000000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2028</v>
+      </c>
+      <c r="B6">
+        <v>9999999</v>
+      </c>
+      <c r="C6">
+        <v>9999999</v>
+      </c>
+      <c r="D6">
+        <v>9999999</v>
+      </c>
+      <c r="E6">
+        <v>235560.05840000001</v>
+      </c>
+      <c r="F6">
+        <v>9999999</v>
+      </c>
+      <c r="G6">
+        <v>9999999</v>
+      </c>
+      <c r="H6">
+        <v>9999999</v>
+      </c>
+      <c r="I6" s="8">
+        <v>1013788.6639999999</v>
+      </c>
+      <c r="J6">
+        <v>9999999</v>
+      </c>
+      <c r="K6" s="8">
+        <v>1565892.5630346665</v>
+      </c>
+      <c r="L6">
+        <v>9999999</v>
+      </c>
+      <c r="M6">
+        <v>258350.32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2029</v>
+      </c>
+      <c r="B7">
+        <v>9999999</v>
+      </c>
+      <c r="C7">
+        <v>9999999</v>
+      </c>
+      <c r="D7">
+        <v>9999999</v>
+      </c>
+      <c r="E7">
+        <v>232026.65760000001</v>
+      </c>
+      <c r="F7">
+        <v>9999999</v>
+      </c>
+      <c r="G7">
+        <v>9999999</v>
+      </c>
+      <c r="H7">
+        <v>9999999</v>
+      </c>
+      <c r="I7" s="8">
+        <v>1004224.62</v>
+      </c>
+      <c r="J7">
+        <v>9999999</v>
+      </c>
+      <c r="K7" s="8">
+        <v>1513549.293360333</v>
+      </c>
+      <c r="L7">
+        <v>9999999</v>
+      </c>
+      <c r="M7">
+        <v>253093.46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2030</v>
+      </c>
+      <c r="B8">
+        <v>9999999</v>
+      </c>
+      <c r="C8">
+        <v>9999999</v>
+      </c>
+      <c r="D8">
+        <v>9999999</v>
+      </c>
+      <c r="E8">
+        <v>228546.25769999999</v>
+      </c>
+      <c r="F8">
+        <v>9999999</v>
+      </c>
+      <c r="G8">
+        <v>9999999</v>
+      </c>
+      <c r="H8">
+        <v>9999999</v>
+      </c>
+      <c r="I8" s="8">
+        <v>994660.57600000012</v>
+      </c>
+      <c r="J8">
+        <v>9999999</v>
+      </c>
+      <c r="K8" s="8">
+        <v>1461206.0236859999</v>
+      </c>
+      <c r="L8">
+        <v>9999999</v>
+      </c>
+      <c r="M8">
+        <v>247939.65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2031</v>
+      </c>
+      <c r="B9">
+        <v>9999999</v>
+      </c>
+      <c r="C9">
+        <v>9999999</v>
+      </c>
+      <c r="D9">
+        <v>9999999</v>
+      </c>
+      <c r="E9">
+        <v>225118.0638</v>
+      </c>
+      <c r="F9">
+        <v>9999999</v>
+      </c>
+      <c r="G9">
+        <v>9999999</v>
+      </c>
+      <c r="H9">
+        <v>9999999</v>
+      </c>
+      <c r="I9" s="8">
+        <v>992747.76720000012</v>
+      </c>
+      <c r="J9">
+        <v>9999999</v>
+      </c>
+      <c r="K9" s="8">
+        <v>1444015.15599508</v>
+      </c>
+      <c r="L9">
+        <v>9999999</v>
+      </c>
+      <c r="M9">
+        <v>242887.37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2032</v>
+      </c>
+      <c r="B10">
+        <v>9999999</v>
+      </c>
+      <c r="C10">
+        <v>9999999</v>
+      </c>
+      <c r="D10">
+        <v>9999999</v>
+      </c>
+      <c r="E10">
+        <v>221741.2929</v>
+      </c>
+      <c r="F10">
+        <v>9999999</v>
+      </c>
+      <c r="G10">
+        <v>9999999</v>
+      </c>
+      <c r="H10">
+        <v>9999999</v>
+      </c>
+      <c r="I10" s="8">
+        <v>990834.9584</v>
+      </c>
+      <c r="J10">
+        <v>9999999</v>
+      </c>
+      <c r="K10" s="8">
+        <v>1426824.2883041599</v>
+      </c>
+      <c r="L10">
+        <v>9999999</v>
+      </c>
+      <c r="M10">
+        <v>237935.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2033</v>
+      </c>
+      <c r="B11">
+        <v>9999999</v>
+      </c>
+      <c r="C11">
+        <v>9999999</v>
+      </c>
+      <c r="D11">
+        <v>9999999</v>
+      </c>
+      <c r="E11">
+        <v>218415.1735</v>
+      </c>
+      <c r="F11">
+        <v>9999999</v>
+      </c>
+      <c r="G11">
+        <v>9999999</v>
+      </c>
+      <c r="H11">
+        <v>9999999</v>
+      </c>
+      <c r="I11" s="8">
+        <v>988922.1496</v>
+      </c>
+      <c r="J11">
+        <v>9999999</v>
+      </c>
+      <c r="K11" s="8">
+        <v>1409633.42061324</v>
+      </c>
+      <c r="L11">
+        <v>9999999</v>
+      </c>
+      <c r="M11">
+        <v>233081.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2034</v>
+      </c>
+      <c r="B12">
+        <v>9999999</v>
+      </c>
+      <c r="C12">
+        <v>9999999</v>
+      </c>
+      <c r="D12">
+        <v>9999999</v>
+      </c>
+      <c r="E12">
+        <v>215138.94589999999</v>
+      </c>
+      <c r="F12">
+        <v>9999999</v>
+      </c>
+      <c r="G12">
+        <v>9999999</v>
+      </c>
+      <c r="H12">
+        <v>9999999</v>
+      </c>
+      <c r="I12" s="8">
+        <v>987009.34079999989</v>
+      </c>
+      <c r="J12">
+        <v>9999999</v>
+      </c>
+      <c r="K12" s="8">
+        <v>1392442.5529223196</v>
+      </c>
+      <c r="L12">
+        <v>9999999</v>
+      </c>
+      <c r="M12">
+        <v>228324.82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2035</v>
+      </c>
+      <c r="B13">
+        <v>9999999</v>
+      </c>
+      <c r="C13">
+        <v>9999999</v>
+      </c>
+      <c r="D13">
+        <v>9999999</v>
+      </c>
+      <c r="E13">
+        <v>211911.86170000001</v>
+      </c>
+      <c r="F13">
+        <v>9999999</v>
+      </c>
+      <c r="G13">
+        <v>9999999</v>
+      </c>
+      <c r="H13">
+        <v>9999999</v>
+      </c>
+      <c r="I13" s="8">
+        <v>985096.53199999989</v>
+      </c>
+      <c r="J13">
+        <v>9999999</v>
+      </c>
+      <c r="K13" s="8">
+        <v>1375251.6852313997</v>
+      </c>
+      <c r="L13">
+        <v>9999999</v>
+      </c>
+      <c r="M13">
+        <v>223663.91</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2036</v>
+      </c>
+      <c r="B14">
+        <v>9999999</v>
+      </c>
+      <c r="C14">
+        <v>9999999</v>
+      </c>
+      <c r="D14">
+        <v>9999999</v>
+      </c>
+      <c r="E14">
+        <v>208733.1838</v>
+      </c>
+      <c r="F14">
+        <v>9999999</v>
+      </c>
+      <c r="G14">
+        <v>9999999</v>
+      </c>
+      <c r="H14">
+        <v>9999999</v>
+      </c>
+      <c r="I14" s="8">
+        <v>983183.72319999977</v>
+      </c>
+      <c r="J14">
+        <v>9999999</v>
+      </c>
+      <c r="K14" s="8">
+        <v>1358060.8175404796</v>
+      </c>
+      <c r="L14">
+        <v>9999999</v>
+      </c>
+      <c r="M14">
+        <v>219097.32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2037</v>
+      </c>
+      <c r="B15">
+        <v>9999999</v>
+      </c>
+      <c r="C15">
+        <v>9999999</v>
+      </c>
+      <c r="D15">
+        <v>9999999</v>
+      </c>
+      <c r="E15">
+        <v>205602.18599999999</v>
+      </c>
+      <c r="F15">
+        <v>9999999</v>
+      </c>
+      <c r="G15">
+        <v>9999999</v>
+      </c>
+      <c r="H15">
+        <v>9999999</v>
+      </c>
+      <c r="I15" s="8">
+        <v>981270.91439999978</v>
+      </c>
+      <c r="J15">
+        <v>9999999</v>
+      </c>
+      <c r="K15" s="8">
+        <v>1340869.9498495597</v>
+      </c>
+      <c r="L15">
+        <v>9999999</v>
+      </c>
+      <c r="M15">
+        <v>214623.65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2038</v>
+      </c>
+      <c r="B16">
+        <v>9999999</v>
+      </c>
+      <c r="C16">
+        <v>9999999</v>
+      </c>
+      <c r="D16">
+        <v>9999999</v>
+      </c>
+      <c r="E16">
+        <v>202518.1532</v>
+      </c>
+      <c r="F16">
+        <v>9999999</v>
+      </c>
+      <c r="G16">
+        <v>9999999</v>
+      </c>
+      <c r="H16">
+        <v>9999999</v>
+      </c>
+      <c r="I16" s="8">
+        <v>979358.10559999966</v>
+      </c>
+      <c r="J16">
+        <v>9999999</v>
+      </c>
+      <c r="K16" s="8">
+        <v>1323679.0821586396</v>
+      </c>
+      <c r="L16">
+        <v>9999999</v>
+      </c>
+      <c r="M16">
+        <v>210241.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>2039</v>
+      </c>
+      <c r="B17">
+        <v>9999999</v>
+      </c>
+      <c r="C17">
+        <v>9999999</v>
+      </c>
+      <c r="D17">
+        <v>9999999</v>
+      </c>
+      <c r="E17">
+        <v>199480.38089999999</v>
+      </c>
+      <c r="F17">
+        <v>9999999</v>
+      </c>
+      <c r="G17">
+        <v>9999999</v>
+      </c>
+      <c r="H17">
+        <v>9999999</v>
+      </c>
+      <c r="I17" s="8">
+        <v>977445.29679999966</v>
+      </c>
+      <c r="J17">
+        <v>9999999</v>
+      </c>
+      <c r="K17" s="8">
+        <v>1306488.2144677194</v>
+      </c>
+      <c r="L17">
+        <v>9999999</v>
+      </c>
+      <c r="M17">
+        <v>205949.84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>2040</v>
+      </c>
+      <c r="B18">
+        <v>9999999</v>
+      </c>
+      <c r="C18">
+        <v>9999999</v>
+      </c>
+      <c r="D18">
+        <v>9999999</v>
+      </c>
+      <c r="E18">
+        <v>196488.1752</v>
+      </c>
+      <c r="F18">
+        <v>9999999</v>
+      </c>
+      <c r="G18">
+        <v>9999999</v>
+      </c>
+      <c r="H18">
+        <v>9999999</v>
+      </c>
+      <c r="I18" s="8">
+        <v>975532.48799999955</v>
+      </c>
+      <c r="J18">
+        <v>9999999</v>
+      </c>
+      <c r="K18" s="8">
+        <v>1288027.7959324</v>
+      </c>
+      <c r="L18">
+        <v>9999999</v>
+      </c>
+      <c r="M18">
+        <v>201747.12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2041</v>
+      </c>
+      <c r="B19">
+        <v>9999999</v>
+      </c>
+      <c r="C19">
+        <v>9999999</v>
+      </c>
+      <c r="D19">
+        <v>9999999</v>
+      </c>
+      <c r="E19">
+        <v>193540.85260000001</v>
+      </c>
+      <c r="F19">
+        <v>9999999</v>
+      </c>
+      <c r="G19">
+        <v>9999999</v>
+      </c>
+      <c r="H19">
+        <v>9999999</v>
+      </c>
+      <c r="I19" s="8">
+        <v>973619.67919999966</v>
+      </c>
+      <c r="J19">
+        <v>9999999</v>
+      </c>
+      <c r="K19" s="8">
+        <v>1288154.7510168403</v>
+      </c>
+      <c r="L19">
+        <v>9999999</v>
+      </c>
+      <c r="M19">
+        <v>197632.19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>2042</v>
+      </c>
+      <c r="B20">
+        <v>9999999</v>
+      </c>
+      <c r="C20">
+        <v>9999999</v>
+      </c>
+      <c r="D20">
+        <v>9999999</v>
+      </c>
+      <c r="E20">
+        <v>190637.73980000001</v>
+      </c>
+      <c r="F20">
+        <v>9999999</v>
+      </c>
+      <c r="G20">
+        <v>9999999</v>
+      </c>
+      <c r="H20">
+        <v>9999999</v>
+      </c>
+      <c r="I20" s="8">
+        <v>971706.87039999955</v>
+      </c>
+      <c r="J20">
+        <v>9999999</v>
+      </c>
+      <c r="K20" s="8">
+        <v>1288281.7061012802</v>
+      </c>
+      <c r="L20">
+        <v>9999999</v>
+      </c>
+      <c r="M20">
+        <v>193603.83</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>2043</v>
+      </c>
+      <c r="B21">
+        <v>9999999</v>
+      </c>
+      <c r="C21">
+        <v>9999999</v>
+      </c>
+      <c r="D21">
+        <v>9999999</v>
+      </c>
+      <c r="E21">
+        <v>187778.17370000001</v>
+      </c>
+      <c r="F21">
+        <v>9999999</v>
+      </c>
+      <c r="G21">
+        <v>9999999</v>
+      </c>
+      <c r="H21">
+        <v>9999999</v>
+      </c>
+      <c r="I21" s="8">
+        <v>969794.06159999955</v>
+      </c>
+      <c r="J21">
+        <v>9999999</v>
+      </c>
+      <c r="K21" s="8">
+        <v>1288408.6611857202</v>
+      </c>
+      <c r="L21">
+        <v>9999999</v>
+      </c>
+      <c r="M21">
+        <v>189660.87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>2044</v>
+      </c>
+      <c r="B22">
+        <v>9999999</v>
+      </c>
+      <c r="C22">
+        <v>9999999</v>
+      </c>
+      <c r="D22">
+        <v>9999999</v>
+      </c>
+      <c r="E22">
+        <v>184961.50109999999</v>
+      </c>
+      <c r="F22">
+        <v>9999999</v>
+      </c>
+      <c r="G22">
+        <v>9999999</v>
+      </c>
+      <c r="H22">
+        <v>9999999</v>
+      </c>
+      <c r="I22" s="8">
+        <v>967881.25279999943</v>
+      </c>
+      <c r="J22">
+        <v>9999999</v>
+      </c>
+      <c r="K22" s="8">
+        <v>1288535.6162701603</v>
+      </c>
+      <c r="L22">
+        <v>9999999</v>
+      </c>
+      <c r="M22">
+        <v>185802.14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>2045</v>
+      </c>
+      <c r="B23">
+        <v>9999999</v>
+      </c>
+      <c r="C23">
+        <v>9999999</v>
+      </c>
+      <c r="D23">
+        <v>9999999</v>
+      </c>
+      <c r="E23">
+        <v>182187.07860000001</v>
+      </c>
+      <c r="F23">
+        <v>9999999</v>
+      </c>
+      <c r="G23">
+        <v>9999999</v>
+      </c>
+      <c r="H23">
+        <v>9999999</v>
+      </c>
+      <c r="I23" s="8">
+        <v>965968.44399999944</v>
+      </c>
+      <c r="J23">
+        <v>9999999</v>
+      </c>
+      <c r="K23" s="8">
+        <v>1288662.5713546001</v>
+      </c>
+      <c r="L23">
+        <v>9999999</v>
+      </c>
+      <c r="M23">
+        <v>182026.51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>2046</v>
+      </c>
+      <c r="B24">
+        <v>9999999</v>
+      </c>
+      <c r="C24">
+        <v>9999999</v>
+      </c>
+      <c r="D24">
+        <v>9999999</v>
+      </c>
+      <c r="E24">
+        <v>179454.27239999999</v>
+      </c>
+      <c r="F24">
+        <v>9999999</v>
+      </c>
+      <c r="G24">
+        <v>9999999</v>
+      </c>
+      <c r="H24">
+        <v>9999999</v>
+      </c>
+      <c r="I24" s="8">
+        <v>964055.63519999932</v>
+      </c>
+      <c r="J24">
+        <v>9999999</v>
+      </c>
+      <c r="K24" s="8">
+        <v>1288789.5264390404</v>
+      </c>
+      <c r="L24">
+        <v>9999999</v>
+      </c>
+      <c r="M24">
+        <v>178332.87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2047</v>
+      </c>
+      <c r="B25">
+        <v>9999999</v>
+      </c>
+      <c r="C25">
+        <v>9999999</v>
+      </c>
+      <c r="D25">
+        <v>9999999</v>
+      </c>
+      <c r="E25">
+        <v>176762.4583</v>
+      </c>
+      <c r="F25">
+        <v>9999999</v>
+      </c>
+      <c r="G25">
+        <v>9999999</v>
+      </c>
+      <c r="H25">
+        <v>9999999</v>
+      </c>
+      <c r="I25" s="8">
+        <v>962142.82639999932</v>
+      </c>
+      <c r="J25">
+        <v>9999999</v>
+      </c>
+      <c r="K25" s="8">
+        <v>1288916.4815234803</v>
+      </c>
+      <c r="L25">
+        <v>9999999</v>
+      </c>
+      <c r="M25">
+        <v>174720.11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>2048</v>
+      </c>
+      <c r="B26">
+        <v>9999999</v>
+      </c>
+      <c r="C26">
+        <v>9999999</v>
+      </c>
+      <c r="D26">
+        <v>9999999</v>
+      </c>
+      <c r="E26">
+        <v>174111.0214</v>
+      </c>
+      <c r="F26">
+        <v>9999999</v>
+      </c>
+      <c r="G26">
+        <v>9999999</v>
+      </c>
+      <c r="H26">
+        <v>9999999</v>
+      </c>
+      <c r="I26" s="8">
+        <v>960230.01759999921</v>
+      </c>
+      <c r="J26">
+        <v>9999999</v>
+      </c>
+      <c r="K26" s="8">
+        <v>1289043.4366079206</v>
+      </c>
+      <c r="L26">
+        <v>9999999</v>
+      </c>
+      <c r="M26">
+        <v>171187.17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>2049</v>
+      </c>
+      <c r="B27">
+        <v>9999999</v>
+      </c>
+      <c r="C27">
+        <v>9999999</v>
+      </c>
+      <c r="D27">
+        <v>9999999</v>
+      </c>
+      <c r="E27">
+        <v>171499.3561</v>
+      </c>
+      <c r="F27">
+        <v>9999999</v>
+      </c>
+      <c r="G27">
+        <v>9999999</v>
+      </c>
+      <c r="H27">
+        <v>9999999</v>
+      </c>
+      <c r="I27" s="8">
+        <v>958317.20879999921</v>
+      </c>
+      <c r="J27">
+        <v>9999999</v>
+      </c>
+      <c r="K27" s="8">
+        <v>1289170.3916923604</v>
+      </c>
+      <c r="L27">
+        <v>9999999</v>
+      </c>
+      <c r="M27">
+        <v>167732.98000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>2050</v>
+      </c>
+      <c r="B28">
+        <v>9999999</v>
+      </c>
+      <c r="C28">
+        <v>9999999</v>
+      </c>
+      <c r="D28">
+        <v>9999999</v>
+      </c>
+      <c r="E28">
+        <v>168926.8658</v>
+      </c>
+      <c r="F28">
+        <v>9999999</v>
+      </c>
+      <c r="G28">
+        <v>9999999</v>
+      </c>
+      <c r="H28">
+        <v>9999999</v>
+      </c>
+      <c r="I28" s="8">
+        <v>956404.40000000026</v>
+      </c>
+      <c r="J28">
+        <v>9999999</v>
+      </c>
+      <c r="K28" s="8">
+        <v>1289297.3467768</v>
+      </c>
+      <c r="L28">
+        <v>9999999</v>
+      </c>
+      <c r="M28">
+        <v>164356.51999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Updates the urbsextension Excel file.
Updates the urbsextension Excel file to reflect current data.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-extension/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="270" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A20A2E7-1617-4C82-9341-AEA66E3C0C5A}"/>
+  <xr:revisionPtr revIDLastSave="301" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11A5AAD5-D1C8-4FB3-A394-84735324E4CB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="14" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" firstSheet="8" activeTab="9" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="152">
   <si>
     <t>Value</t>
   </si>
@@ -310,9 +310,6 @@
     <t>Material</t>
   </si>
   <si>
-    <t>Ingot</t>
-  </si>
-  <si>
     <t>Silicon</t>
   </si>
   <si>
@@ -421,58 +418,16 @@
     <t>Wafer</t>
   </si>
   <si>
-    <t>80.0</t>
-  </si>
-  <si>
-    <t>20.0</t>
-  </si>
-  <si>
-    <t>4.0</t>
-  </si>
-  <si>
-    <t>120.0</t>
-  </si>
-  <si>
-    <t>70.0</t>
-  </si>
-  <si>
-    <t>60.0</t>
-  </si>
-  <si>
-    <t>25.0</t>
-  </si>
-  <si>
     <t>1.0</t>
-  </si>
-  <si>
-    <t>90.0</t>
   </si>
   <si>
     <t>Assembly</t>
   </si>
   <si>
-    <t>10.0</t>
-  </si>
-  <si>
-    <t>15.0</t>
-  </si>
-  <si>
     <t>Foundation</t>
   </si>
   <si>
-    <t>200.0</t>
-  </si>
-  <si>
-    <t>250.0</t>
-  </si>
-  <si>
-    <t>30.0</t>
-  </si>
-  <si>
     <t>Pack</t>
-  </si>
-  <si>
-    <t>0.10</t>
   </si>
   <si>
     <t>Cons_Tech</t>
@@ -514,13 +469,7 @@
     <t>opex_var_base</t>
   </si>
   <si>
-    <t>import_cost_part</t>
-  </si>
-  <si>
     <t>init_cap</t>
-  </si>
-  <si>
-    <t>solarPV_Ingot</t>
   </si>
   <si>
     <t>solarPV_Wafer</t>
@@ -554,6 +503,12 @@
   </si>
   <si>
     <t>solarPV_Module</t>
+  </si>
+  <si>
+    <t>Polysilicon</t>
+  </si>
+  <si>
+    <t>solarPV_Polysilicon</t>
   </si>
 </sst>
 </file>
@@ -1152,7 +1107,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B1" t="s">
         <v>82</v>
@@ -1167,7 +1122,7 @@
         <v>73</v>
       </c>
       <c r="F1" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="G1" t="s">
         <v>74</v>
@@ -1184,7 +1139,7 @@
         <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>150</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1193,7 +1148,7 @@
         <v>150</v>
       </c>
       <c r="F2">
-        <v>100</v>
+        <v>24000</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1207,7 +1162,7 @@
         <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1216,7 +1171,7 @@
         <v>100</v>
       </c>
       <c r="F3">
-        <v>100</v>
+        <v>2000</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1230,7 +1185,7 @@
         <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1239,7 +1194,7 @@
         <v>100</v>
       </c>
       <c r="F4">
-        <v>100</v>
+        <v>7000</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -1253,7 +1208,7 @@
         <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1262,7 +1217,7 @@
         <v>100</v>
       </c>
       <c r="F5">
-        <v>100</v>
+        <v>22000</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -1279,7 +1234,7 @@
         <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1305,7 +1260,7 @@
         <v>76</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1331,7 +1286,7 @@
         <v>76</v>
       </c>
       <c r="C8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1357,7 +1312,7 @@
         <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1383,7 +1338,7 @@
         <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1409,7 +1364,7 @@
         <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1432,10 +1387,10 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1455,10 +1410,10 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C13" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1495,13 +1450,13 @@
         <v>84</v>
       </c>
       <c r="D1" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="E1" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="F1" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1509,19 +1464,19 @@
         <v>75</v>
       </c>
       <c r="B2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C2" t="s">
         <v>85</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" t="s">
         <v>86</v>
       </c>
-      <c r="D2" t="s">
-        <v>91</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>87</v>
-      </c>
-      <c r="F2" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1529,19 +1484,19 @@
         <v>75</v>
       </c>
       <c r="B3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" t="s">
         <v>89</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>90</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F3" t="s">
         <v>91</v>
-      </c>
-      <c r="E3" t="s">
-        <v>91</v>
-      </c>
-      <c r="F3" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1549,19 +1504,19 @@
         <v>75</v>
       </c>
       <c r="B4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C4" t="s">
         <v>93</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>94</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>95</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>96</v>
-      </c>
-      <c r="F4" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1569,19 +1524,19 @@
         <v>75</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" t="s">
         <v>98</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>98</v>
+      </c>
+      <c r="F5" t="s">
         <v>99</v>
-      </c>
-      <c r="E5" t="s">
-        <v>99</v>
-      </c>
-      <c r="F5" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1589,19 +1544,19 @@
         <v>76</v>
       </c>
       <c r="B6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" t="s">
         <v>101</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>102</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>102</v>
+      </c>
+      <c r="F6" t="s">
         <v>103</v>
-      </c>
-      <c r="E6" t="s">
-        <v>103</v>
-      </c>
-      <c r="F6" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1609,19 +1564,19 @@
         <v>76</v>
       </c>
       <c r="B7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C7" t="s">
         <v>105</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>106</v>
       </c>
-      <c r="D7" t="s">
-        <v>107</v>
-      </c>
       <c r="E7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1629,19 +1584,19 @@
         <v>76</v>
       </c>
       <c r="B8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" t="s">
         <v>108</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>109</v>
       </c>
-      <c r="D8" t="s">
-        <v>110</v>
-      </c>
       <c r="E8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1649,59 +1604,59 @@
         <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D9" t="s">
         <v>111</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
+        <v>111</v>
+      </c>
+      <c r="F9" t="s">
         <v>112</v>
-      </c>
-      <c r="E9" t="s">
-        <v>112</v>
-      </c>
-      <c r="F9" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" t="s">
         <v>114</v>
       </c>
-      <c r="B10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>115</v>
       </c>
-      <c r="D10" t="s">
-        <v>116</v>
-      </c>
       <c r="E10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C11" t="s">
+        <v>116</v>
+      </c>
+      <c r="D11" t="s">
         <v>117</v>
       </c>
-      <c r="D11" t="s">
-        <v>118</v>
-      </c>
       <c r="E11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1717,19 +1672,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1" t="s">
         <v>84</v>
       </c>
       <c r="C1" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="D1" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="E1" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1737,7 +1692,7 @@
         <v>2024</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C2">
         <v>1000000</v>
@@ -1754,7 +1709,7 @@
         <v>2024</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C3">
         <v>5000</v>
@@ -1771,7 +1726,7 @@
         <v>2024</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C4">
         <v>5000000</v>
@@ -1788,7 +1743,7 @@
         <v>2024</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C5">
         <v>2000000</v>
@@ -1805,7 +1760,7 @@
         <v>2024</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C6">
         <v>500000</v>
@@ -1822,7 +1777,7 @@
         <v>2024</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C7">
         <v>10000000</v>
@@ -1839,7 +1794,7 @@
         <v>2024</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C8">
         <v>800000</v>
@@ -1856,7 +1811,7 @@
         <v>2024</v>
       </c>
       <c r="B9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C9">
         <v>20000</v>
@@ -1873,7 +1828,7 @@
         <v>2024</v>
       </c>
       <c r="B10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C10">
         <v>150000</v>
@@ -1890,7 +1845,7 @@
         <v>2024</v>
       </c>
       <c r="B11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C11">
         <v>50000</v>
@@ -1914,19 +1869,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="B1" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="C1" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
       <c r="D1" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="E1" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1934,16 +1889,16 @@
         <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C2" t="s">
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>150</v>
       </c>
       <c r="E2" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1951,16 +1906,16 @@
         <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C3" t="s">
         <v>75</v>
       </c>
       <c r="D3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E3" t="s">
         <v>121</v>
-      </c>
-      <c r="E3" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1968,33 +1923,33 @@
         <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
         <v>75</v>
       </c>
       <c r="D4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E4" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E5" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2002,16 +1957,16 @@
         <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C6" t="s">
         <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2019,16 +1974,16 @@
         <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C7" t="s">
         <v>76</v>
       </c>
       <c r="D7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E7" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2036,16 +1991,16 @@
         <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C8" t="s">
         <v>76</v>
       </c>
       <c r="D8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E8" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2053,16 +2008,16 @@
         <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C9" t="s">
         <v>76</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E9" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2070,16 +2025,16 @@
         <v>77</v>
       </c>
       <c r="B10" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C10" t="s">
         <v>76</v>
       </c>
       <c r="D10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E10" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2087,16 +2042,16 @@
         <v>77</v>
       </c>
       <c r="B11" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C11" t="s">
         <v>76</v>
       </c>
       <c r="D11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E11" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2104,16 +2059,16 @@
         <v>77</v>
       </c>
       <c r="B12" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C12" t="s">
         <v>77</v>
       </c>
       <c r="D12" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="E12" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2123,15 +2078,15 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CE844EE-882F-4833-8B87-00A8BB665263}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" t="s">
         <v>119</v>
-      </c>
-      <c r="B1" t="s">
-        <v>120</v>
       </c>
       <c r="C1" t="s">
         <v>82</v>
@@ -2140,16 +2095,13 @@
         <v>83</v>
       </c>
       <c r="E1" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="F1" t="s">
-        <v>152</v>
-      </c>
-      <c r="G1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -2160,19 +2112,16 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E2" t="s">
-        <v>125</v>
+        <v>150</v>
+      </c>
+      <c r="E2">
+        <v>1000</v>
       </c>
       <c r="F2">
         <v>1000000</v>
       </c>
-      <c r="G2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2024</v>
       </c>
@@ -2183,19 +2132,16 @@
         <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E3" t="s">
-        <v>126</v>
+        <v>120</v>
+      </c>
+      <c r="E3">
+        <v>1000</v>
       </c>
       <c r="F3">
         <v>1000000</v>
       </c>
-      <c r="G3" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2024</v>
       </c>
@@ -2206,19 +2152,16 @@
         <v>75</v>
       </c>
       <c r="D4" t="s">
-        <v>89</v>
-      </c>
-      <c r="E4" t="s">
-        <v>127</v>
+        <v>88</v>
+      </c>
+      <c r="E4">
+        <v>1000</v>
       </c>
       <c r="F4">
         <v>1000000</v>
       </c>
-      <c r="G4" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2024</v>
       </c>
@@ -2229,19 +2172,16 @@
         <v>75</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
-      </c>
-      <c r="E5" t="s">
-        <v>128</v>
+        <v>92</v>
+      </c>
+      <c r="E5">
+        <v>1000</v>
       </c>
       <c r="F5">
         <v>1000000</v>
       </c>
-      <c r="G5" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2024</v>
       </c>
@@ -2252,19 +2192,16 @@
         <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>101</v>
-      </c>
-      <c r="E6" t="s">
-        <v>130</v>
+        <v>100</v>
+      </c>
+      <c r="E6">
+        <v>1000</v>
       </c>
       <c r="F6">
         <v>1000000</v>
       </c>
-      <c r="G6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2024</v>
       </c>
@@ -2275,19 +2212,16 @@
         <v>76</v>
       </c>
       <c r="D7" t="s">
-        <v>105</v>
-      </c>
-      <c r="E7" t="s">
-        <v>122</v>
+        <v>104</v>
+      </c>
+      <c r="E7">
+        <v>1000</v>
       </c>
       <c r="F7">
         <v>1000000</v>
       </c>
-      <c r="G7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -2298,19 +2232,16 @@
         <v>76</v>
       </c>
       <c r="D8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E8" t="s">
         <v>107</v>
+      </c>
+      <c r="E8">
+        <v>1000</v>
       </c>
       <c r="F8">
         <v>1000000</v>
       </c>
-      <c r="G8" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2024</v>
       </c>
@@ -2321,19 +2252,16 @@
         <v>76</v>
       </c>
       <c r="D9" t="s">
-        <v>131</v>
-      </c>
-      <c r="E9" t="s">
-        <v>132</v>
+        <v>122</v>
+      </c>
+      <c r="E9">
+        <v>1000</v>
       </c>
       <c r="F9">
         <v>1000000</v>
       </c>
-      <c r="G9" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2024</v>
       </c>
@@ -2344,19 +2272,16 @@
         <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>134</v>
-      </c>
-      <c r="E10" t="s">
-        <v>135</v>
+        <v>123</v>
+      </c>
+      <c r="E10">
+        <v>1000</v>
       </c>
       <c r="F10">
         <v>1000000</v>
       </c>
-      <c r="G10" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2024</v>
       </c>
@@ -2367,19 +2292,16 @@
         <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>131</v>
-      </c>
-      <c r="E11" t="s">
-        <v>123</v>
+        <v>122</v>
+      </c>
+      <c r="E11">
+        <v>1000</v>
       </c>
       <c r="F11">
         <v>1000000</v>
       </c>
-      <c r="G11" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2024</v>
       </c>
@@ -2387,22 +2309,19 @@
         <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D12" t="s">
-        <v>89</v>
-      </c>
-      <c r="E12" t="s">
-        <v>122</v>
+        <v>88</v>
+      </c>
+      <c r="E12">
+        <v>1000</v>
       </c>
       <c r="F12">
         <v>1000000</v>
       </c>
-      <c r="G12" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2024</v>
       </c>
@@ -2410,19 +2329,16 @@
         <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D13" t="s">
-        <v>138</v>
-      </c>
-      <c r="E13" t="s">
-        <v>137</v>
+        <v>124</v>
+      </c>
+      <c r="E13">
+        <v>1000</v>
       </c>
       <c r="F13">
         <v>1000000</v>
-      </c>
-      <c r="G13" t="s">
-        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2441,40 +2357,40 @@
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C1" t="s">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="D1" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="E1" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
       <c r="F1" t="s">
-        <v>158</v>
+        <v>141</v>
       </c>
       <c r="G1" t="s">
-        <v>159</v>
+        <v>142</v>
       </c>
       <c r="H1" t="s">
-        <v>160</v>
+        <v>143</v>
       </c>
       <c r="I1" t="s">
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="J1" t="s">
-        <v>162</v>
+        <v>145</v>
       </c>
       <c r="K1" t="s">
-        <v>163</v>
+        <v>146</v>
       </c>
       <c r="L1" t="s">
-        <v>164</v>
+        <v>147</v>
       </c>
       <c r="M1" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2482,7 +2398,7 @@
         <v>2024</v>
       </c>
       <c r="B2">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C2">
         <v>9999999</v>

</xml_diff>

<commit_message>
Refactors processing capacity and import costs
Improves processing capacity constraints by introducing a buildout rule, a growth limit rule, and adjusting the output limit rule.

This change enhances the model's ability to represent realistic factory buildout scenarios. It also fixes issues with import costs, ensuring that the solver receives accurate data and avoids defaulting to unrealistic values.

The implementation also introduces new validation checks to ensure import costs are correctly loaded and used by the solver. A new set is added to define valid tech-stage combinations.

Addresses inconsistencies in legacy capacity handling and applies corrections to cost calculations to provide a more robust and reliable model.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-extension/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="301" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11A5AAD5-D1C8-4FB3-A394-84735324E4CB}"/>
+  <xr:revisionPtr revIDLastSave="313" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{109EDEA0-1EB9-4F59-9537-2F6A9E6EB3A3}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" firstSheet="8" activeTab="9" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="14" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="151">
   <si>
     <t>Value</t>
   </si>
@@ -427,9 +427,6 @@
     <t>Foundation</t>
   </si>
   <si>
-    <t>Pack</t>
-  </si>
-  <si>
     <t>Cons_Tech</t>
   </si>
   <si>
@@ -496,12 +493,6 @@
     <t>windoff_Assembly</t>
   </si>
   <si>
-    <t>bateries_Cell</t>
-  </si>
-  <si>
-    <t>batteries_Pack</t>
-  </si>
-  <si>
     <t>solarPV_Module</t>
   </si>
   <si>
@@ -509,6 +500,12 @@
   </si>
   <si>
     <t>solarPV_Polysilicon</t>
+  </si>
+  <si>
+    <t>Batteries_Assembly</t>
+  </si>
+  <si>
+    <t>Batteries_Cell</t>
   </si>
 </sst>
 </file>
@@ -1122,7 +1119,7 @@
         <v>73</v>
       </c>
       <c r="F1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G1" t="s">
         <v>74</v>
@@ -1139,7 +1136,7 @@
         <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1413,7 +1410,7 @@
         <v>113</v>
       </c>
       <c r="C13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1450,13 +1447,13 @@
         <v>84</v>
       </c>
       <c r="D1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" t="s">
-        <v>132</v>
-      </c>
       <c r="F1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1464,7 +1461,7 @@
         <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C2" t="s">
         <v>85</v>
@@ -1678,13 +1675,13 @@
         <v>84</v>
       </c>
       <c r="C1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E1" t="s">
         <v>133</v>
-      </c>
-      <c r="E1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1869,19 +1866,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" t="s">
         <v>125</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>126</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>128</v>
-      </c>
-      <c r="E1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1895,7 +1892,7 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E2" t="s">
         <v>121</v>
@@ -1940,7 +1937,7 @@
         <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C5" t="s">
         <v>113</v>
@@ -2095,10 +2092,10 @@
         <v>83</v>
       </c>
       <c r="E1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F1" t="s">
         <v>136</v>
-      </c>
-      <c r="F1" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -2112,7 +2109,7 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E2">
         <v>1000</v>
@@ -2332,7 +2329,7 @@
         <v>113</v>
       </c>
       <c r="D13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E13">
         <v>1000</v>
@@ -2357,40 +2354,40 @@
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D1" t="s">
         <v>139</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F1" t="s">
         <v>140</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
+        <v>141</v>
+      </c>
+      <c r="H1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I1" t="s">
+        <v>143</v>
+      </c>
+      <c r="J1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K1" t="s">
+        <v>145</v>
+      </c>
+      <c r="L1" t="s">
+        <v>150</v>
+      </c>
+      <c r="M1" t="s">
         <v>149</v>
-      </c>
-      <c r="F1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G1" t="s">
-        <v>142</v>
-      </c>
-      <c r="H1" t="s">
-        <v>143</v>
-      </c>
-      <c r="I1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J1" t="s">
-        <v>145</v>
-      </c>
-      <c r="K1" t="s">
-        <v>146</v>
-      </c>
-      <c r="L1" t="s">
-        <v>147</v>
-      </c>
-      <c r="M1" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2425,7 +2422,7 @@
         <v>9999999</v>
       </c>
       <c r="K2" s="8">
-        <v>1775265.6417320003</v>
+        <v>1775265.64</v>
       </c>
       <c r="L2">
         <v>9999999</v>
@@ -2460,13 +2457,13 @@
         <v>9999999</v>
       </c>
       <c r="I3" s="8">
-        <v>1042480.7960000001</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J3">
         <v>9999999</v>
       </c>
       <c r="K3" s="8">
-        <v>1722922.372057667</v>
+        <v>1775265.64</v>
       </c>
       <c r="L3">
         <v>9999999</v>
@@ -2501,13 +2498,13 @@
         <v>9999999</v>
       </c>
       <c r="I4" s="8">
-        <v>1032916.7520000001</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J4">
         <v>9999999</v>
       </c>
       <c r="K4" s="8">
-        <v>1670579.1023833335</v>
+        <v>1775265.64</v>
       </c>
       <c r="L4">
         <v>9999999</v>
@@ -2542,13 +2539,13 @@
         <v>9999999</v>
       </c>
       <c r="I5" s="8">
-        <v>1023352.708</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J5">
         <v>9999999</v>
       </c>
       <c r="K5" s="8">
-        <v>1618235.832709</v>
+        <v>1775265.64</v>
       </c>
       <c r="L5">
         <v>9999999</v>
@@ -2583,13 +2580,13 @@
         <v>9999999</v>
       </c>
       <c r="I6" s="8">
-        <v>1013788.6639999999</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J6">
         <v>9999999</v>
       </c>
       <c r="K6" s="8">
-        <v>1565892.5630346665</v>
+        <v>1775265.64</v>
       </c>
       <c r="L6">
         <v>9999999</v>
@@ -2624,13 +2621,13 @@
         <v>9999999</v>
       </c>
       <c r="I7" s="8">
-        <v>1004224.62</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J7">
         <v>9999999</v>
       </c>
       <c r="K7" s="8">
-        <v>1513549.293360333</v>
+        <v>1775265.64</v>
       </c>
       <c r="L7">
         <v>9999999</v>
@@ -2665,13 +2662,13 @@
         <v>9999999</v>
       </c>
       <c r="I8" s="8">
-        <v>994660.57600000012</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J8">
         <v>9999999</v>
       </c>
       <c r="K8" s="8">
-        <v>1461206.0236859999</v>
+        <v>1775265.64</v>
       </c>
       <c r="L8">
         <v>9999999</v>
@@ -2706,13 +2703,13 @@
         <v>9999999</v>
       </c>
       <c r="I9" s="8">
-        <v>992747.76720000012</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J9">
         <v>9999999</v>
       </c>
       <c r="K9" s="8">
-        <v>1444015.15599508</v>
+        <v>1775265.64</v>
       </c>
       <c r="L9">
         <v>9999999</v>
@@ -2747,13 +2744,13 @@
         <v>9999999</v>
       </c>
       <c r="I10" s="8">
-        <v>990834.9584</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J10">
         <v>9999999</v>
       </c>
       <c r="K10" s="8">
-        <v>1426824.2883041599</v>
+        <v>1775265.64</v>
       </c>
       <c r="L10">
         <v>9999999</v>
@@ -2788,13 +2785,13 @@
         <v>9999999</v>
       </c>
       <c r="I11" s="8">
-        <v>988922.1496</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J11">
         <v>9999999</v>
       </c>
       <c r="K11" s="8">
-        <v>1409633.42061324</v>
+        <v>1775265.64</v>
       </c>
       <c r="L11">
         <v>9999999</v>
@@ -2829,13 +2826,13 @@
         <v>9999999</v>
       </c>
       <c r="I12" s="8">
-        <v>987009.34079999989</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J12">
         <v>9999999</v>
       </c>
       <c r="K12" s="8">
-        <v>1392442.5529223196</v>
+        <v>1775265.64</v>
       </c>
       <c r="L12">
         <v>9999999</v>
@@ -2870,13 +2867,13 @@
         <v>9999999</v>
       </c>
       <c r="I13" s="8">
-        <v>985096.53199999989</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J13">
         <v>9999999</v>
       </c>
       <c r="K13" s="8">
-        <v>1375251.6852313997</v>
+        <v>1775265.64</v>
       </c>
       <c r="L13">
         <v>9999999</v>
@@ -2911,13 +2908,13 @@
         <v>9999999</v>
       </c>
       <c r="I14" s="8">
-        <v>983183.72319999977</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J14">
         <v>9999999</v>
       </c>
       <c r="K14" s="8">
-        <v>1358060.8175404796</v>
+        <v>1775265.64</v>
       </c>
       <c r="L14">
         <v>9999999</v>
@@ -2952,13 +2949,13 @@
         <v>9999999</v>
       </c>
       <c r="I15" s="8">
-        <v>981270.91439999978</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J15">
         <v>9999999</v>
       </c>
       <c r="K15" s="8">
-        <v>1340869.9498495597</v>
+        <v>1775265.64</v>
       </c>
       <c r="L15">
         <v>9999999</v>
@@ -2993,13 +2990,13 @@
         <v>9999999</v>
       </c>
       <c r="I16" s="8">
-        <v>979358.10559999966</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J16">
         <v>9999999</v>
       </c>
       <c r="K16" s="8">
-        <v>1323679.0821586396</v>
+        <v>1775265.64</v>
       </c>
       <c r="L16">
         <v>9999999</v>
@@ -3034,13 +3031,13 @@
         <v>9999999</v>
       </c>
       <c r="I17" s="8">
-        <v>977445.29679999966</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J17">
         <v>9999999</v>
       </c>
       <c r="K17" s="8">
-        <v>1306488.2144677194</v>
+        <v>1775265.64</v>
       </c>
       <c r="L17">
         <v>9999999</v>
@@ -3075,13 +3072,13 @@
         <v>9999999</v>
       </c>
       <c r="I18" s="8">
-        <v>975532.48799999955</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J18">
         <v>9999999</v>
       </c>
       <c r="K18" s="8">
-        <v>1288027.7959324</v>
+        <v>1775265.64</v>
       </c>
       <c r="L18">
         <v>9999999</v>
@@ -3116,13 +3113,13 @@
         <v>9999999</v>
       </c>
       <c r="I19" s="8">
-        <v>973619.67919999966</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J19">
         <v>9999999</v>
       </c>
       <c r="K19" s="8">
-        <v>1288154.7510168403</v>
+        <v>1775265.64</v>
       </c>
       <c r="L19">
         <v>9999999</v>
@@ -3157,13 +3154,13 @@
         <v>9999999</v>
       </c>
       <c r="I20" s="8">
-        <v>971706.87039999955</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J20">
         <v>9999999</v>
       </c>
       <c r="K20" s="8">
-        <v>1288281.7061012802</v>
+        <v>1775265.64</v>
       </c>
       <c r="L20">
         <v>9999999</v>
@@ -3198,13 +3195,13 @@
         <v>9999999</v>
       </c>
       <c r="I21" s="8">
-        <v>969794.06159999955</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J21">
         <v>9999999</v>
       </c>
       <c r="K21" s="8">
-        <v>1288408.6611857202</v>
+        <v>1775265.64</v>
       </c>
       <c r="L21">
         <v>9999999</v>
@@ -3239,13 +3236,13 @@
         <v>9999999</v>
       </c>
       <c r="I22" s="8">
-        <v>967881.25279999943</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J22">
         <v>9999999</v>
       </c>
       <c r="K22" s="8">
-        <v>1288535.6162701603</v>
+        <v>1775265.64</v>
       </c>
       <c r="L22">
         <v>9999999</v>
@@ -3280,13 +3277,13 @@
         <v>9999999</v>
       </c>
       <c r="I23" s="8">
-        <v>965968.44399999944</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J23">
         <v>9999999</v>
       </c>
       <c r="K23" s="8">
-        <v>1288662.5713546001</v>
+        <v>1775265.64</v>
       </c>
       <c r="L23">
         <v>9999999</v>
@@ -3321,13 +3318,13 @@
         <v>9999999</v>
       </c>
       <c r="I24" s="8">
-        <v>964055.63519999932</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J24">
         <v>9999999</v>
       </c>
       <c r="K24" s="8">
-        <v>1288789.5264390404</v>
+        <v>1775265.64</v>
       </c>
       <c r="L24">
         <v>9999999</v>
@@ -3362,13 +3359,13 @@
         <v>9999999</v>
       </c>
       <c r="I25" s="8">
-        <v>962142.82639999932</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J25">
         <v>9999999</v>
       </c>
       <c r="K25" s="8">
-        <v>1288916.4815234803</v>
+        <v>1775265.64</v>
       </c>
       <c r="L25">
         <v>9999999</v>
@@ -3403,13 +3400,13 @@
         <v>9999999</v>
       </c>
       <c r="I26" s="8">
-        <v>960230.01759999921</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J26">
         <v>9999999</v>
       </c>
       <c r="K26" s="8">
-        <v>1289043.4366079206</v>
+        <v>1775265.64</v>
       </c>
       <c r="L26">
         <v>9999999</v>
@@ -3444,13 +3441,13 @@
         <v>9999999</v>
       </c>
       <c r="I27" s="8">
-        <v>958317.20879999921</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J27">
         <v>9999999</v>
       </c>
       <c r="K27" s="8">
-        <v>1289170.3916923604</v>
+        <v>1775265.64</v>
       </c>
       <c r="L27">
         <v>9999999</v>
@@ -3485,13 +3482,13 @@
         <v>9999999</v>
       </c>
       <c r="I28" s="8">
-        <v>956404.40000000026</v>
+        <v>1052044.8400000001</v>
       </c>
       <c r="J28">
         <v>9999999</v>
       </c>
       <c r="K28" s="8">
-        <v>1289297.3467768</v>
+        <v>1775265.64</v>
       </c>
       <c r="L28">
         <v>9999999</v>
@@ -15272,26 +15269,6 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -15299,6 +15276,26 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implements scenario constraints and refactors scrap
Applies scenario constraints related to NZIA and CRMA targets for domestic production, extraction and recycling.

Refactors scrap constraints, removing the obsolete recycling constraint and adjusts solver tolerances for feasibility and optimality.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-extension/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="314" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48D5A401-35C7-4493-814E-E5354DD6F0B1}"/>
+  <xr:revisionPtr revIDLastSave="388" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39C07CE4-8C5D-4311-B8B6-913E977DEB40}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="14" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="9" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="151">
   <si>
     <t>Value</t>
   </si>
@@ -424,9 +424,6 @@
     <t>Assembly</t>
   </si>
   <si>
-    <t>Foundation</t>
-  </si>
-  <si>
     <t>Cons_Tech</t>
   </si>
   <si>
@@ -507,6 +504,9 @@
   <si>
     <t>Batteries_Cell</t>
   </si>
+  <si>
+    <t>finished, happens on-site so no limitation, will be limited by installable capacity</t>
+  </si>
 </sst>
 </file>
 
@@ -570,7 +570,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -604,6 +604,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -680,7 +686,7 @@
     </xf>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -710,6 +716,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{1C1ADB5D-62B2-4A88-A962-14B0B3D457AA}"/>
@@ -1099,7 +1106,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8C0D52F-0ADA-4AC5-8A50-4699398C8904}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1119,7 +1126,7 @@
         <v>73</v>
       </c>
       <c r="F1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G1" t="s">
         <v>74</v>
@@ -1136,7 +1143,7 @@
         <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1144,7 +1151,7 @@
       <c r="E2">
         <v>150</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="7">
         <v>24000</v>
       </c>
       <c r="G2">
@@ -1167,7 +1174,7 @@
       <c r="E3">
         <v>100</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="7">
         <v>2000</v>
       </c>
       <c r="G3">
@@ -1190,7 +1197,7 @@
       <c r="E4">
         <v>100</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="7">
         <v>7000</v>
       </c>
       <c r="G4">
@@ -1213,7 +1220,7 @@
       <c r="E5">
         <v>100</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="7">
         <v>22000</v>
       </c>
       <c r="G5">
@@ -1239,8 +1246,8 @@
       <c r="E6">
         <v>100</v>
       </c>
-      <c r="F6">
-        <v>100</v>
+      <c r="F6" s="7">
+        <v>27000</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -1265,8 +1272,8 @@
       <c r="E7">
         <v>100</v>
       </c>
-      <c r="F7">
-        <v>100</v>
+      <c r="F7" s="7">
+        <v>27000</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -1291,8 +1298,8 @@
       <c r="E8">
         <v>100</v>
       </c>
-      <c r="F8">
-        <v>100</v>
+      <c r="F8" s="7">
+        <v>27000</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -1317,14 +1324,14 @@
       <c r="E9">
         <v>100</v>
       </c>
-      <c r="F9">
-        <v>100</v>
+      <c r="F9" s="7">
+        <v>999999</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>79</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1335,7 +1342,7 @@
         <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1361,22 +1368,19 @@
         <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
       <c r="E11">
-        <v>100</v>
-      </c>
-      <c r="F11">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="F11" s="7">
+        <v>1</v>
       </c>
       <c r="G11">
-        <v>1</v>
-      </c>
-      <c r="H11" t="s">
-        <v>79</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1384,19 +1388,16 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
-      </c>
-      <c r="D12">
+        <v>107</v>
+      </c>
+      <c r="E12">
         <v>1</v>
       </c>
-      <c r="E12">
-        <v>80</v>
-      </c>
-      <c r="F12">
-        <v>100</v>
+      <c r="F12" s="7">
+        <v>1</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1407,7 +1408,7 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="C13" t="s">
         <v>122</v>
@@ -1416,13 +1417,62 @@
         <v>1</v>
       </c>
       <c r="E13">
-        <v>20</v>
-      </c>
-      <c r="F13">
         <v>100</v>
+      </c>
+      <c r="F13" s="7">
+        <v>999999</v>
       </c>
       <c r="G13">
         <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" t="s">
+        <v>113</v>
+      </c>
+      <c r="C14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>80</v>
+      </c>
+      <c r="F14">
+        <v>100</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>20</v>
+      </c>
+      <c r="F15">
+        <v>100</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1433,7 +1483,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FA1A697-84AA-4F97-BE70-81695B57512E}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -1447,13 +1497,13 @@
         <v>84</v>
       </c>
       <c r="D1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" t="s">
-        <v>131</v>
-      </c>
       <c r="F1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1461,7 +1511,7 @@
         <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C2" t="s">
         <v>85</v>
@@ -1618,41 +1668,121 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="C10" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="D10" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="E10" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="F10" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" t="s">
+        <v>106</v>
+      </c>
+      <c r="F11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" t="s">
+        <v>109</v>
+      </c>
+      <c r="E12" t="s">
+        <v>109</v>
+      </c>
+      <c r="F12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" t="s">
+        <v>111</v>
+      </c>
+      <c r="E13" t="s">
+        <v>111</v>
+      </c>
+      <c r="F13" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>113</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B14" t="s">
         <v>88</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C14" t="s">
+        <v>114</v>
+      </c>
+      <c r="D14" t="s">
+        <v>115</v>
+      </c>
+      <c r="E14" t="s">
+        <v>115</v>
+      </c>
+      <c r="F14" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>113</v>
+      </c>
+      <c r="B15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C15" t="s">
         <v>116</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D15" t="s">
         <v>117</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E15" t="s">
         <v>117</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F15" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1675,13 +1805,13 @@
         <v>84</v>
       </c>
       <c r="C1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E1" t="s">
         <v>132</v>
-      </c>
-      <c r="E1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1861,24 +1991,24 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{996B2112-D2EE-4E9F-B294-4222E881A3C9}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" t="s">
         <v>124</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>125</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>126</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>127</v>
-      </c>
-      <c r="E1" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1892,7 +2022,7 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E2" t="s">
         <v>121</v>
@@ -2008,7 +2138,7 @@
         <v>122</v>
       </c>
       <c r="C9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D9" t="s">
         <v>100</v>
@@ -2025,7 +2155,7 @@
         <v>122</v>
       </c>
       <c r="C10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D10" t="s">
         <v>104</v>
@@ -2042,29 +2172,12 @@
         <v>122</v>
       </c>
       <c r="C11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D11" t="s">
         <v>107</v>
       </c>
       <c r="E11" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>77</v>
-      </c>
-      <c r="B12" t="s">
-        <v>122</v>
-      </c>
-      <c r="C12" t="s">
-        <v>77</v>
-      </c>
-      <c r="D12" t="s">
-        <v>123</v>
-      </c>
-      <c r="E12" t="s">
         <v>121</v>
       </c>
     </row>
@@ -2075,7 +2188,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CE844EE-882F-4833-8B87-00A8BB665263}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2092,10 +2205,10 @@
         <v>83</v>
       </c>
       <c r="E1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F1" t="s">
         <v>135</v>
-      </c>
-      <c r="F1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -2109,13 +2222,13 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E2">
-        <v>1000</v>
-      </c>
-      <c r="F2">
-        <v>1000000</v>
+        <v>146</v>
+      </c>
+      <c r="E2" s="13">
+        <v>55200</v>
+      </c>
+      <c r="F2" s="13">
+        <v>3220.0000000000005</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2131,11 +2244,11 @@
       <c r="D3" t="s">
         <v>120</v>
       </c>
-      <c r="E3">
-        <v>1000</v>
-      </c>
-      <c r="F3">
-        <v>1000000</v>
+      <c r="E3" s="13">
+        <v>92000</v>
+      </c>
+      <c r="F3" s="13">
+        <v>4600</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2151,11 +2264,11 @@
       <c r="D4" t="s">
         <v>88</v>
       </c>
-      <c r="E4">
-        <v>1000</v>
-      </c>
-      <c r="F4">
-        <v>1000000</v>
+      <c r="E4" s="13">
+        <v>165600</v>
+      </c>
+      <c r="F4" s="13">
+        <v>8280</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -2171,11 +2284,11 @@
       <c r="D5" t="s">
         <v>92</v>
       </c>
-      <c r="E5">
-        <v>1000</v>
-      </c>
-      <c r="F5">
-        <v>1000000</v>
+      <c r="E5" s="13">
+        <v>46000</v>
+      </c>
+      <c r="F5" s="13">
+        <v>2300</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -2191,11 +2304,11 @@
       <c r="D6" t="s">
         <v>100</v>
       </c>
-      <c r="E6">
-        <v>1000</v>
-      </c>
-      <c r="F6">
-        <v>1000000</v>
+      <c r="E6" s="13">
+        <v>73600</v>
+      </c>
+      <c r="F6" s="13">
+        <v>3680.0000000000009</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -2211,11 +2324,11 @@
       <c r="D7" t="s">
         <v>104</v>
       </c>
-      <c r="E7">
-        <v>1000</v>
-      </c>
-      <c r="F7">
-        <v>1000000</v>
+      <c r="E7" s="13">
+        <v>82800</v>
+      </c>
+      <c r="F7" s="13">
+        <v>4140</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -2231,11 +2344,11 @@
       <c r="D8" t="s">
         <v>107</v>
       </c>
-      <c r="E8">
-        <v>1000</v>
-      </c>
-      <c r="F8">
-        <v>1000000</v>
+      <c r="E8" s="13">
+        <v>276000</v>
+      </c>
+      <c r="F8" s="13">
+        <v>13800</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2251,11 +2364,11 @@
       <c r="D9" t="s">
         <v>122</v>
       </c>
-      <c r="E9">
-        <v>1000</v>
-      </c>
-      <c r="F9">
-        <v>1000000</v>
+      <c r="E9" s="13">
+        <v>1</v>
+      </c>
+      <c r="F9" s="13">
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2269,13 +2382,13 @@
         <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>123</v>
-      </c>
-      <c r="E10">
-        <v>1000</v>
-      </c>
-      <c r="F10">
-        <v>1000000</v>
+        <v>100</v>
+      </c>
+      <c r="E10" s="13">
+        <v>165600</v>
+      </c>
+      <c r="F10" s="13">
+        <v>8280</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2289,13 +2402,13 @@
         <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>122</v>
-      </c>
-      <c r="E11">
-        <v>1000</v>
-      </c>
-      <c r="F11">
-        <v>1000000</v>
+        <v>104</v>
+      </c>
+      <c r="E11" s="13">
+        <v>202400</v>
+      </c>
+      <c r="F11" s="13">
+        <v>10120</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -2306,16 +2419,16 @@
         <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="D12" t="s">
-        <v>88</v>
-      </c>
-      <c r="E12">
-        <v>1000</v>
-      </c>
-      <c r="F12">
-        <v>1000000</v>
+        <v>107</v>
+      </c>
+      <c r="E12" s="13">
+        <v>202400</v>
+      </c>
+      <c r="F12" s="13">
+        <v>10120</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -2326,16 +2439,56 @@
         <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
         <v>122</v>
       </c>
-      <c r="E13">
-        <v>1000</v>
-      </c>
-      <c r="F13">
-        <v>1000000</v>
+      <c r="E13" s="13">
+        <v>1</v>
+      </c>
+      <c r="F13" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2024</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" t="s">
+        <v>113</v>
+      </c>
+      <c r="D14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E14" s="13">
+        <v>92000</v>
+      </c>
+      <c r="F14" s="13">
+        <v>4600</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2024</v>
+      </c>
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" t="s">
+        <v>113</v>
+      </c>
+      <c r="D15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" s="13">
+        <v>1</v>
+      </c>
+      <c r="F15" s="13">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2354,40 +2507,40 @@
         <v>15</v>
       </c>
       <c r="B1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F1" t="s">
+        <v>139</v>
+      </c>
+      <c r="G1" t="s">
+        <v>140</v>
+      </c>
+      <c r="H1" t="s">
+        <v>141</v>
+      </c>
+      <c r="I1" t="s">
+        <v>142</v>
+      </c>
+      <c r="J1" t="s">
+        <v>143</v>
+      </c>
+      <c r="K1" t="s">
+        <v>144</v>
+      </c>
+      <c r="L1" t="s">
+        <v>149</v>
+      </c>
+      <c r="M1" t="s">
         <v>148</v>
-      </c>
-      <c r="C1" t="s">
-        <v>138</v>
-      </c>
-      <c r="D1" t="s">
-        <v>139</v>
-      </c>
-      <c r="E1" t="s">
-        <v>146</v>
-      </c>
-      <c r="F1" t="s">
-        <v>140</v>
-      </c>
-      <c r="G1" t="s">
-        <v>141</v>
-      </c>
-      <c r="H1" t="s">
-        <v>142</v>
-      </c>
-      <c r="I1" t="s">
-        <v>143</v>
-      </c>
-      <c r="J1" t="s">
-        <v>144</v>
-      </c>
-      <c r="K1" t="s">
-        <v>145</v>
-      </c>
-      <c r="L1" t="s">
-        <v>150</v>
-      </c>
-      <c r="M1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -15269,26 +15422,6 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -15296,6 +15429,26 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implemented variable and fixed opex
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-extension/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="388" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39C07CE4-8C5D-4311-B8B6-913E977DEB40}"/>
+  <xr:revisionPtr revIDLastSave="403" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEF8DBB7-6D38-454A-A4D6-ADC9D831B385}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="9" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" firstSheet="6" activeTab="13" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="154">
   <si>
     <t>Value</t>
   </si>
@@ -484,9 +484,6 @@
     <t>windon_Assembly</t>
   </si>
   <si>
-    <t>windoff_Foundation</t>
-  </si>
-  <si>
     <t>windoff_Assembly</t>
   </si>
   <si>
@@ -506,6 +503,18 @@
   </si>
   <si>
     <t>finished, happens on-site so no limitation, will be limited by installable capacity</t>
+  </si>
+  <si>
+    <t>windoff_Blade</t>
+  </si>
+  <si>
+    <t>windoff_Tower</t>
+  </si>
+  <si>
+    <t>windoff_Nacelle</t>
+  </si>
+  <si>
+    <t>opex_fixed</t>
   </si>
 </sst>
 </file>
@@ -713,10 +722,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{1C1ADB5D-62B2-4A88-A962-14B0B3D457AA}"/>
@@ -1143,7 +1152,7 @@
         <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1331,7 +1340,7 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1472,7 +1481,7 @@
         <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -1511,7 +1520,7 @@
         <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C2" t="s">
         <v>85</v>
@@ -2022,7 +2031,7 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E2" t="s">
         <v>121</v>
@@ -2188,10 +2197,10 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CE844EE-882F-4833-8B87-00A8BB665263}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>118</v>
       </c>
@@ -2210,8 +2219,11 @@
       <c r="F1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -2222,16 +2234,19 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>146</v>
-      </c>
-      <c r="E2" s="13">
+        <v>145</v>
+      </c>
+      <c r="E2" s="12">
         <v>55200</v>
       </c>
-      <c r="F2" s="13">
+      <c r="F2" s="12">
+        <v>1449.0000000000002</v>
+      </c>
+      <c r="G2" s="12">
         <v>3220.0000000000005</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2024</v>
       </c>
@@ -2244,14 +2259,17 @@
       <c r="D3" t="s">
         <v>120</v>
       </c>
-      <c r="E3" s="13">
+      <c r="E3" s="12">
         <v>92000</v>
       </c>
-      <c r="F3" s="13">
+      <c r="F3" s="12">
+        <v>3312</v>
+      </c>
+      <c r="G3" s="12">
         <v>4600</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2024</v>
       </c>
@@ -2264,14 +2282,17 @@
       <c r="D4" t="s">
         <v>88</v>
       </c>
-      <c r="E4" s="13">
+      <c r="E4" s="12">
         <v>165600</v>
       </c>
-      <c r="F4" s="13">
+      <c r="F4" s="12">
+        <v>14904</v>
+      </c>
+      <c r="G4" s="12">
         <v>8280</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2024</v>
       </c>
@@ -2284,14 +2305,17 @@
       <c r="D5" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="12">
         <v>46000</v>
       </c>
-      <c r="F5" s="13">
+      <c r="F5" s="12">
+        <v>12420</v>
+      </c>
+      <c r="G5" s="12">
         <v>2300</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2024</v>
       </c>
@@ -2304,14 +2328,17 @@
       <c r="D6" t="s">
         <v>100</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="12">
         <v>73600</v>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="12">
+        <v>20976.000000000007</v>
+      </c>
+      <c r="G6" s="12">
         <v>3680.0000000000009</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2024</v>
       </c>
@@ -2324,14 +2351,17 @@
       <c r="D7" t="s">
         <v>104</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="12">
         <v>82800</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="12">
+        <v>7866</v>
+      </c>
+      <c r="G7" s="12">
         <v>4140</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -2344,14 +2374,17 @@
       <c r="D8" t="s">
         <v>107</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="12">
         <v>276000</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="12">
+        <v>26220</v>
+      </c>
+      <c r="G8" s="12">
         <v>13800</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2024</v>
       </c>
@@ -2364,14 +2397,17 @@
       <c r="D9" t="s">
         <v>122</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="12">
         <v>1</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F9" s="12">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2024</v>
       </c>
@@ -2384,14 +2420,17 @@
       <c r="D10" t="s">
         <v>100</v>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="12">
         <v>165600</v>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="12">
+        <v>47196</v>
+      </c>
+      <c r="G10" s="12">
         <v>8280</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2024</v>
       </c>
@@ -2404,14 +2443,17 @@
       <c r="D11" t="s">
         <v>104</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="12">
         <v>202400</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="12">
+        <v>19228</v>
+      </c>
+      <c r="G11" s="12">
         <v>10120</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2024</v>
       </c>
@@ -2424,14 +2466,17 @@
       <c r="D12" t="s">
         <v>107</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="12">
         <v>202400</v>
       </c>
-      <c r="F12" s="13">
+      <c r="F12" s="12">
+        <v>19228</v>
+      </c>
+      <c r="G12" s="12">
         <v>10120</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2024</v>
       </c>
@@ -2444,14 +2489,17 @@
       <c r="D13" t="s">
         <v>122</v>
       </c>
-      <c r="E13" s="13">
+      <c r="E13" s="12">
         <v>1</v>
       </c>
-      <c r="F13" s="13">
+      <c r="F13" s="12">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2024</v>
       </c>
@@ -2464,14 +2512,17 @@
       <c r="D14" t="s">
         <v>88</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="12">
         <v>92000</v>
       </c>
-      <c r="F14" s="13">
+      <c r="F14" s="12">
+        <v>13524</v>
+      </c>
+      <c r="G14" s="12">
         <v>4600</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2024</v>
       </c>
@@ -2484,10 +2535,13 @@
       <c r="D15" t="s">
         <v>122</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="12">
         <v>1</v>
       </c>
-      <c r="F15" s="13">
+      <c r="F15" s="12">
+        <v>1</v>
+      </c>
+      <c r="G15" s="12">
         <v>1</v>
       </c>
     </row>
@@ -2499,15 +2553,15 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B74DFEF-01D9-4B2D-A936-BF616F091054}">
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C1" t="s">
         <v>137</v>
@@ -2516,7 +2570,7 @@
         <v>138</v>
       </c>
       <c r="E1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F1" t="s">
         <v>139</v>
@@ -2531,19 +2585,25 @@
         <v>142</v>
       </c>
       <c r="J1" t="s">
+        <v>150</v>
+      </c>
+      <c r="K1" t="s">
+        <v>151</v>
+      </c>
+      <c r="L1" t="s">
+        <v>152</v>
+      </c>
+      <c r="M1" t="s">
         <v>143</v>
       </c>
-      <c r="K1" t="s">
-        <v>144</v>
-      </c>
-      <c r="L1" t="s">
-        <v>149</v>
-      </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -2574,17 +2634,23 @@
       <c r="J2">
         <v>9999999</v>
       </c>
-      <c r="K2" s="8">
+      <c r="K2">
+        <v>9999999</v>
+      </c>
+      <c r="L2">
+        <v>9999999</v>
+      </c>
+      <c r="M2" s="8">
         <v>1775265.64</v>
       </c>
-      <c r="L2">
-        <v>9999999</v>
-      </c>
-      <c r="M2">
+      <c r="N2">
+        <v>9999999</v>
+      </c>
+      <c r="O2">
         <v>280439.83</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -2615,17 +2681,23 @@
       <c r="J3">
         <v>9999999</v>
       </c>
-      <c r="K3" s="8">
+      <c r="K3">
+        <v>9999999</v>
+      </c>
+      <c r="L3">
+        <v>9999999</v>
+      </c>
+      <c r="M3" s="8">
         <v>1722922.37</v>
       </c>
-      <c r="L3">
-        <v>9999999</v>
-      </c>
-      <c r="M3">
+      <c r="N3">
+        <v>9999999</v>
+      </c>
+      <c r="O3">
         <v>274754.90999999997</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -2656,17 +2728,23 @@
       <c r="J4">
         <v>9999999</v>
       </c>
-      <c r="K4" s="8">
+      <c r="K4">
+        <v>9999999</v>
+      </c>
+      <c r="L4">
+        <v>9999999</v>
+      </c>
+      <c r="M4" s="8">
         <v>1670579.1</v>
       </c>
-      <c r="L4">
-        <v>9999999</v>
-      </c>
-      <c r="M4">
+      <c r="N4">
+        <v>9999999</v>
+      </c>
+      <c r="O4">
         <v>269179.44</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -2697,17 +2775,23 @@
       <c r="J5">
         <v>9999999</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5">
+        <v>9999999</v>
+      </c>
+      <c r="L5">
+        <v>9999999</v>
+      </c>
+      <c r="M5" s="8">
         <v>1618235.83</v>
       </c>
-      <c r="L5">
-        <v>9999999</v>
-      </c>
-      <c r="M5">
+      <c r="N5">
+        <v>9999999</v>
+      </c>
+      <c r="O5">
         <v>263711.78000000003</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -2738,17 +2822,23 @@
       <c r="J6">
         <v>9999999</v>
       </c>
-      <c r="K6" s="8">
+      <c r="K6">
+        <v>9999999</v>
+      </c>
+      <c r="L6">
+        <v>9999999</v>
+      </c>
+      <c r="M6" s="8">
         <v>1565892.56</v>
       </c>
-      <c r="L6">
-        <v>9999999</v>
-      </c>
-      <c r="M6">
+      <c r="N6">
+        <v>9999999</v>
+      </c>
+      <c r="O6">
         <v>258350.32</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -2779,17 +2869,23 @@
       <c r="J7">
         <v>9999999</v>
       </c>
-      <c r="K7" s="8">
+      <c r="K7">
+        <v>9999999</v>
+      </c>
+      <c r="L7">
+        <v>9999999</v>
+      </c>
+      <c r="M7" s="8">
         <v>1513549.29</v>
       </c>
-      <c r="L7">
-        <v>9999999</v>
-      </c>
-      <c r="M7">
+      <c r="N7">
+        <v>9999999</v>
+      </c>
+      <c r="O7">
         <v>253093.46</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -2820,17 +2916,23 @@
       <c r="J8">
         <v>9999999</v>
       </c>
-      <c r="K8" s="8">
+      <c r="K8">
+        <v>9999999</v>
+      </c>
+      <c r="L8">
+        <v>9999999</v>
+      </c>
+      <c r="M8" s="8">
         <v>1461206.02</v>
       </c>
-      <c r="L8">
-        <v>9999999</v>
-      </c>
-      <c r="M8">
+      <c r="N8">
+        <v>9999999</v>
+      </c>
+      <c r="O8">
         <v>247939.65</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -2861,17 +2963,23 @@
       <c r="J9">
         <v>9999999</v>
       </c>
-      <c r="K9" s="8">
+      <c r="K9">
+        <v>9999999</v>
+      </c>
+      <c r="L9">
+        <v>9999999</v>
+      </c>
+      <c r="M9" s="8">
         <v>1444015.16</v>
       </c>
-      <c r="L9">
-        <v>9999999</v>
-      </c>
-      <c r="M9">
+      <c r="N9">
+        <v>9999999</v>
+      </c>
+      <c r="O9">
         <v>242887.37</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -2902,17 +3010,23 @@
       <c r="J10">
         <v>9999999</v>
       </c>
-      <c r="K10" s="8">
+      <c r="K10">
+        <v>9999999</v>
+      </c>
+      <c r="L10">
+        <v>9999999</v>
+      </c>
+      <c r="M10" s="8">
         <v>1426824.29</v>
       </c>
-      <c r="L10">
-        <v>9999999</v>
-      </c>
-      <c r="M10">
+      <c r="N10">
+        <v>9999999</v>
+      </c>
+      <c r="O10">
         <v>237935.1</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -2943,17 +3057,23 @@
       <c r="J11">
         <v>9999999</v>
       </c>
-      <c r="K11" s="8">
+      <c r="K11">
+        <v>9999999</v>
+      </c>
+      <c r="L11">
+        <v>9999999</v>
+      </c>
+      <c r="M11" s="8">
         <v>1409633.42</v>
       </c>
-      <c r="L11">
-        <v>9999999</v>
-      </c>
-      <c r="M11">
+      <c r="N11">
+        <v>9999999</v>
+      </c>
+      <c r="O11">
         <v>233081.4</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -2984,17 +3104,23 @@
       <c r="J12">
         <v>9999999</v>
       </c>
-      <c r="K12" s="8">
+      <c r="K12">
+        <v>9999999</v>
+      </c>
+      <c r="L12">
+        <v>9999999</v>
+      </c>
+      <c r="M12" s="8">
         <v>1392442.55</v>
       </c>
-      <c r="L12">
-        <v>9999999</v>
-      </c>
-      <c r="M12">
+      <c r="N12">
+        <v>9999999</v>
+      </c>
+      <c r="O12">
         <v>228324.82</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -3025,17 +3151,23 @@
       <c r="J13">
         <v>9999999</v>
       </c>
-      <c r="K13" s="8">
+      <c r="K13">
+        <v>9999999</v>
+      </c>
+      <c r="L13">
+        <v>9999999</v>
+      </c>
+      <c r="M13" s="8">
         <v>1375251.69</v>
       </c>
-      <c r="L13">
-        <v>9999999</v>
-      </c>
-      <c r="M13">
+      <c r="N13">
+        <v>9999999</v>
+      </c>
+      <c r="O13">
         <v>223663.91</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -3066,17 +3198,23 @@
       <c r="J14">
         <v>9999999</v>
       </c>
-      <c r="K14" s="8">
+      <c r="K14">
+        <v>9999999</v>
+      </c>
+      <c r="L14">
+        <v>9999999</v>
+      </c>
+      <c r="M14" s="8">
         <v>1358060.82</v>
       </c>
-      <c r="L14">
-        <v>9999999</v>
-      </c>
-      <c r="M14">
+      <c r="N14">
+        <v>9999999</v>
+      </c>
+      <c r="O14">
         <v>219097.32</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -3107,17 +3245,23 @@
       <c r="J15">
         <v>9999999</v>
       </c>
-      <c r="K15" s="8">
+      <c r="K15">
+        <v>9999999</v>
+      </c>
+      <c r="L15">
+        <v>9999999</v>
+      </c>
+      <c r="M15" s="8">
         <v>1340869.95</v>
       </c>
-      <c r="L15">
-        <v>9999999</v>
-      </c>
-      <c r="M15">
+      <c r="N15">
+        <v>9999999</v>
+      </c>
+      <c r="O15">
         <v>214623.65</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -3148,17 +3292,23 @@
       <c r="J16">
         <v>9999999</v>
       </c>
-      <c r="K16" s="8">
+      <c r="K16">
+        <v>9999999</v>
+      </c>
+      <c r="L16">
+        <v>9999999</v>
+      </c>
+      <c r="M16" s="8">
         <v>1323679.08</v>
       </c>
-      <c r="L16">
-        <v>9999999</v>
-      </c>
-      <c r="M16">
+      <c r="N16">
+        <v>9999999</v>
+      </c>
+      <c r="O16">
         <v>210241.6</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -3189,17 +3339,23 @@
       <c r="J17">
         <v>9999999</v>
       </c>
-      <c r="K17" s="8">
+      <c r="K17">
+        <v>9999999</v>
+      </c>
+      <c r="L17">
+        <v>9999999</v>
+      </c>
+      <c r="M17" s="8">
         <v>1306488.21</v>
       </c>
-      <c r="L17">
-        <v>9999999</v>
-      </c>
-      <c r="M17">
+      <c r="N17">
+        <v>9999999</v>
+      </c>
+      <c r="O17">
         <v>205949.84</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -3230,17 +3386,23 @@
       <c r="J18">
         <v>9999999</v>
       </c>
-      <c r="K18" s="8">
+      <c r="K18">
+        <v>9999999</v>
+      </c>
+      <c r="L18">
+        <v>9999999</v>
+      </c>
+      <c r="M18" s="8">
         <v>1288027.8</v>
       </c>
-      <c r="L18">
-        <v>9999999</v>
-      </c>
-      <c r="M18">
+      <c r="N18">
+        <v>9999999</v>
+      </c>
+      <c r="O18">
         <v>201747.12</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -3271,17 +3433,23 @@
       <c r="J19">
         <v>9999999</v>
       </c>
-      <c r="K19" s="8">
+      <c r="K19">
+        <v>9999999</v>
+      </c>
+      <c r="L19">
+        <v>9999999</v>
+      </c>
+      <c r="M19" s="8">
         <v>1288154.75</v>
       </c>
-      <c r="L19">
-        <v>9999999</v>
-      </c>
-      <c r="M19">
+      <c r="N19">
+        <v>9999999</v>
+      </c>
+      <c r="O19">
         <v>197632.19</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -3312,17 +3480,23 @@
       <c r="J20">
         <v>9999999</v>
       </c>
-      <c r="K20" s="8">
+      <c r="K20">
+        <v>9999999</v>
+      </c>
+      <c r="L20">
+        <v>9999999</v>
+      </c>
+      <c r="M20" s="8">
         <v>1288281.71</v>
       </c>
-      <c r="L20">
-        <v>9999999</v>
-      </c>
-      <c r="M20">
+      <c r="N20">
+        <v>9999999</v>
+      </c>
+      <c r="O20">
         <v>193603.83</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -3353,17 +3527,23 @@
       <c r="J21">
         <v>9999999</v>
       </c>
-      <c r="K21" s="8">
+      <c r="K21">
+        <v>9999999</v>
+      </c>
+      <c r="L21">
+        <v>9999999</v>
+      </c>
+      <c r="M21" s="8">
         <v>1288408.6599999999</v>
       </c>
-      <c r="L21">
-        <v>9999999</v>
-      </c>
-      <c r="M21">
+      <c r="N21">
+        <v>9999999</v>
+      </c>
+      <c r="O21">
         <v>189660.87</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -3394,17 +3574,23 @@
       <c r="J22">
         <v>9999999</v>
       </c>
-      <c r="K22" s="8">
+      <c r="K22">
+        <v>9999999</v>
+      </c>
+      <c r="L22">
+        <v>9999999</v>
+      </c>
+      <c r="M22" s="8">
         <v>1288535.6200000001</v>
       </c>
-      <c r="L22">
-        <v>9999999</v>
-      </c>
-      <c r="M22">
+      <c r="N22">
+        <v>9999999</v>
+      </c>
+      <c r="O22">
         <v>185802.14</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -3435,17 +3621,23 @@
       <c r="J23">
         <v>9999999</v>
       </c>
-      <c r="K23" s="8">
+      <c r="K23">
+        <v>9999999</v>
+      </c>
+      <c r="L23">
+        <v>9999999</v>
+      </c>
+      <c r="M23" s="8">
         <v>1288662.57</v>
       </c>
-      <c r="L23">
-        <v>9999999</v>
-      </c>
-      <c r="M23">
+      <c r="N23">
+        <v>9999999</v>
+      </c>
+      <c r="O23">
         <v>182026.51</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -3476,17 +3668,23 @@
       <c r="J24">
         <v>9999999</v>
       </c>
-      <c r="K24" s="8">
+      <c r="K24">
+        <v>9999999</v>
+      </c>
+      <c r="L24">
+        <v>9999999</v>
+      </c>
+      <c r="M24" s="8">
         <v>1288789.53</v>
       </c>
-      <c r="L24">
-        <v>9999999</v>
-      </c>
-      <c r="M24">
+      <c r="N24">
+        <v>9999999</v>
+      </c>
+      <c r="O24">
         <v>178332.87</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -3517,17 +3715,23 @@
       <c r="J25">
         <v>9999999</v>
       </c>
-      <c r="K25" s="8">
+      <c r="K25">
+        <v>9999999</v>
+      </c>
+      <c r="L25">
+        <v>9999999</v>
+      </c>
+      <c r="M25" s="8">
         <v>1288916.48</v>
       </c>
-      <c r="L25">
-        <v>9999999</v>
-      </c>
-      <c r="M25">
+      <c r="N25">
+        <v>9999999</v>
+      </c>
+      <c r="O25">
         <v>174720.11</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -3558,17 +3762,23 @@
       <c r="J26">
         <v>9999999</v>
       </c>
-      <c r="K26" s="8">
+      <c r="K26">
+        <v>9999999</v>
+      </c>
+      <c r="L26">
+        <v>9999999</v>
+      </c>
+      <c r="M26" s="8">
         <v>1289043.44</v>
       </c>
-      <c r="L26">
-        <v>9999999</v>
-      </c>
-      <c r="M26">
+      <c r="N26">
+        <v>9999999</v>
+      </c>
+      <c r="O26">
         <v>171187.17</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -3599,17 +3809,23 @@
       <c r="J27">
         <v>9999999</v>
       </c>
-      <c r="K27" s="8">
+      <c r="K27">
+        <v>9999999</v>
+      </c>
+      <c r="L27">
+        <v>9999999</v>
+      </c>
+      <c r="M27" s="8">
         <v>1289170.3899999999</v>
       </c>
-      <c r="L27">
-        <v>9999999</v>
-      </c>
-      <c r="M27">
+      <c r="N27">
+        <v>9999999</v>
+      </c>
+      <c r="O27">
         <v>167732.98000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -3640,13 +3856,19 @@
       <c r="J28">
         <v>9999999</v>
       </c>
-      <c r="K28" s="8">
+      <c r="K28">
+        <v>9999999</v>
+      </c>
+      <c r="L28">
+        <v>9999999</v>
+      </c>
+      <c r="M28" s="8">
         <v>1289297.3500000001</v>
       </c>
-      <c r="L28">
-        <v>9999999</v>
-      </c>
-      <c r="M28">
+      <c r="N28">
+        <v>9999999</v>
+      </c>
+      <c r="O28">
         <v>164356.51999999999</v>
       </c>
     </row>
@@ -14043,7 +14265,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="12">
+      <c r="A2" s="13">
         <v>2024</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -14057,7 +14279,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="12"/>
+      <c r="A3" s="13"/>
       <c r="B3" s="11" t="s">
         <v>70</v>
       </c>
@@ -14070,7 +14292,7 @@
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="12"/>
+      <c r="A4" s="13"/>
       <c r="B4" s="11" t="s">
         <v>71</v>
       </c>
@@ -14082,7 +14304,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="12"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="11" t="s">
         <v>68</v>
       </c>
@@ -14094,7 +14316,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
+      <c r="A6" s="13">
         <v>2025</v>
       </c>
       <c r="B6" s="11" t="s">
@@ -14108,7 +14330,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="12"/>
+      <c r="A7" s="13"/>
       <c r="B7" s="11" t="s">
         <v>70</v>
       </c>
@@ -14120,7 +14342,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="12"/>
+      <c r="A8" s="13"/>
       <c r="B8" s="11" t="s">
         <v>71</v>
       </c>
@@ -14132,7 +14354,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="11" t="s">
         <v>68</v>
       </c>
@@ -14145,7 +14367,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
+      <c r="A10" s="13">
         <v>2026</v>
       </c>
       <c r="B10" s="11" t="s">
@@ -14159,7 +14381,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
+      <c r="A11" s="13"/>
       <c r="B11" s="11" t="s">
         <v>70</v>
       </c>
@@ -14171,7 +14393,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
+      <c r="A12" s="13"/>
       <c r="B12" s="11" t="s">
         <v>71</v>
       </c>
@@ -14183,7 +14405,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
+      <c r="A13" s="13"/>
       <c r="B13" s="11" t="s">
         <v>68</v>
       </c>
@@ -14196,7 +14418,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
+      <c r="A14" s="13">
         <v>2027</v>
       </c>
       <c r="B14" s="11" t="s">
@@ -14210,7 +14432,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
+      <c r="A15" s="13"/>
       <c r="B15" s="11" t="s">
         <v>70</v>
       </c>
@@ -14222,7 +14444,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="12"/>
+      <c r="A16" s="13"/>
       <c r="B16" s="11" t="s">
         <v>71</v>
       </c>
@@ -14234,7 +14456,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="12"/>
+      <c r="A17" s="13"/>
       <c r="B17" s="11" t="s">
         <v>68</v>
       </c>
@@ -14247,7 +14469,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="12">
+      <c r="A18" s="13">
         <v>2028</v>
       </c>
       <c r="B18" s="11" t="s">
@@ -14261,7 +14483,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="12"/>
+      <c r="A19" s="13"/>
       <c r="B19" s="11" t="s">
         <v>70</v>
       </c>
@@ -14273,7 +14495,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="12"/>
+      <c r="A20" s="13"/>
       <c r="B20" s="11" t="s">
         <v>71</v>
       </c>
@@ -14285,7 +14507,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="12"/>
+      <c r="A21" s="13"/>
       <c r="B21" s="11" t="s">
         <v>68</v>
       </c>
@@ -14298,7 +14520,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="12">
+      <c r="A22" s="13">
         <v>2029</v>
       </c>
       <c r="B22" s="11" t="s">
@@ -14312,7 +14534,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="12"/>
+      <c r="A23" s="13"/>
       <c r="B23" s="11" t="s">
         <v>70</v>
       </c>
@@ -14324,7 +14546,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="12"/>
+      <c r="A24" s="13"/>
       <c r="B24" s="11" t="s">
         <v>71</v>
       </c>
@@ -14336,7 +14558,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="12"/>
+      <c r="A25" s="13"/>
       <c r="B25" s="11" t="s">
         <v>68</v>
       </c>
@@ -14349,7 +14571,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="12">
+      <c r="A26" s="13">
         <v>2030</v>
       </c>
       <c r="B26" s="11" t="s">
@@ -14363,7 +14585,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="12"/>
+      <c r="A27" s="13"/>
       <c r="B27" s="11" t="s">
         <v>70</v>
       </c>
@@ -14375,7 +14597,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="12"/>
+      <c r="A28" s="13"/>
       <c r="B28" s="11" t="s">
         <v>71</v>
       </c>
@@ -14387,7 +14609,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="12"/>
+      <c r="A29" s="13"/>
       <c r="B29" s="11" t="s">
         <v>68</v>
       </c>
@@ -14400,7 +14622,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="12">
+      <c r="A30" s="13">
         <v>2031</v>
       </c>
       <c r="B30" s="11" t="s">
@@ -14414,7 +14636,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="12"/>
+      <c r="A31" s="13"/>
       <c r="B31" s="11" t="s">
         <v>70</v>
       </c>
@@ -14426,7 +14648,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="12"/>
+      <c r="A32" s="13"/>
       <c r="B32" s="11" t="s">
         <v>71</v>
       </c>
@@ -14438,7 +14660,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="12"/>
+      <c r="A33" s="13"/>
       <c r="B33" s="11" t="s">
         <v>68</v>
       </c>
@@ -14451,7 +14673,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="12">
+      <c r="A34" s="13">
         <v>2032</v>
       </c>
       <c r="B34" s="11" t="s">
@@ -14465,7 +14687,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="12"/>
+      <c r="A35" s="13"/>
       <c r="B35" s="11" t="s">
         <v>70</v>
       </c>
@@ -14477,7 +14699,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="12"/>
+      <c r="A36" s="13"/>
       <c r="B36" s="11" t="s">
         <v>71</v>
       </c>
@@ -14489,7 +14711,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="12"/>
+      <c r="A37" s="13"/>
       <c r="B37" s="11" t="s">
         <v>68</v>
       </c>
@@ -14502,7 +14724,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="12">
+      <c r="A38" s="13">
         <v>2033</v>
       </c>
       <c r="B38" s="11" t="s">
@@ -14516,7 +14738,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="12"/>
+      <c r="A39" s="13"/>
       <c r="B39" s="11" t="s">
         <v>70</v>
       </c>
@@ -14528,7 +14750,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="12"/>
+      <c r="A40" s="13"/>
       <c r="B40" s="11" t="s">
         <v>71</v>
       </c>
@@ -14540,7 +14762,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="12"/>
+      <c r="A41" s="13"/>
       <c r="B41" s="11" t="s">
         <v>68</v>
       </c>
@@ -14553,7 +14775,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="12">
+      <c r="A42" s="13">
         <v>2034</v>
       </c>
       <c r="B42" s="11" t="s">
@@ -14567,7 +14789,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="12"/>
+      <c r="A43" s="13"/>
       <c r="B43" s="11" t="s">
         <v>70</v>
       </c>
@@ -14579,7 +14801,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="12"/>
+      <c r="A44" s="13"/>
       <c r="B44" s="11" t="s">
         <v>71</v>
       </c>
@@ -14591,7 +14813,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="12"/>
+      <c r="A45" s="13"/>
       <c r="B45" s="11" t="s">
         <v>68</v>
       </c>
@@ -14604,7 +14826,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="12">
+      <c r="A46" s="13">
         <v>2035</v>
       </c>
       <c r="B46" s="11" t="s">
@@ -14618,7 +14840,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="12"/>
+      <c r="A47" s="13"/>
       <c r="B47" s="11" t="s">
         <v>70</v>
       </c>
@@ -14630,7 +14852,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="12"/>
+      <c r="A48" s="13"/>
       <c r="B48" s="11" t="s">
         <v>71</v>
       </c>
@@ -14642,7 +14864,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="12"/>
+      <c r="A49" s="13"/>
       <c r="B49" s="11" t="s">
         <v>68</v>
       </c>
@@ -14655,7 +14877,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="12">
+      <c r="A50" s="13">
         <v>2036</v>
       </c>
       <c r="B50" s="11" t="s">
@@ -14669,7 +14891,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="12"/>
+      <c r="A51" s="13"/>
       <c r="B51" s="11" t="s">
         <v>70</v>
       </c>
@@ -14681,7 +14903,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="12"/>
+      <c r="A52" s="13"/>
       <c r="B52" s="11" t="s">
         <v>71</v>
       </c>
@@ -14693,7 +14915,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="12"/>
+      <c r="A53" s="13"/>
       <c r="B53" s="11" t="s">
         <v>68</v>
       </c>
@@ -14706,7 +14928,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="12">
+      <c r="A54" s="13">
         <v>2037</v>
       </c>
       <c r="B54" s="11" t="s">
@@ -14720,7 +14942,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="12"/>
+      <c r="A55" s="13"/>
       <c r="B55" s="11" t="s">
         <v>70</v>
       </c>
@@ -14732,7 +14954,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="12"/>
+      <c r="A56" s="13"/>
       <c r="B56" s="11" t="s">
         <v>71</v>
       </c>
@@ -14744,7 +14966,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="12"/>
+      <c r="A57" s="13"/>
       <c r="B57" s="11" t="s">
         <v>68</v>
       </c>
@@ -14757,7 +14979,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="12">
+      <c r="A58" s="13">
         <v>2038</v>
       </c>
       <c r="B58" s="11" t="s">
@@ -14771,7 +14993,7 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="12"/>
+      <c r="A59" s="13"/>
       <c r="B59" s="11" t="s">
         <v>70</v>
       </c>
@@ -14783,7 +15005,7 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="12"/>
+      <c r="A60" s="13"/>
       <c r="B60" s="11" t="s">
         <v>71</v>
       </c>
@@ -14795,7 +15017,7 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="12"/>
+      <c r="A61" s="13"/>
       <c r="B61" s="11" t="s">
         <v>68</v>
       </c>
@@ -14808,7 +15030,7 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="12">
+      <c r="A62" s="13">
         <v>2039</v>
       </c>
       <c r="B62" s="11" t="s">
@@ -14822,7 +15044,7 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="12"/>
+      <c r="A63" s="13"/>
       <c r="B63" s="11" t="s">
         <v>70</v>
       </c>
@@ -14834,7 +15056,7 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="12"/>
+      <c r="A64" s="13"/>
       <c r="B64" s="11" t="s">
         <v>71</v>
       </c>
@@ -14846,7 +15068,7 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="12"/>
+      <c r="A65" s="13"/>
       <c r="B65" s="11" t="s">
         <v>68</v>
       </c>
@@ -14859,7 +15081,7 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="12">
+      <c r="A66" s="13">
         <v>2040</v>
       </c>
       <c r="B66" s="11" t="s">
@@ -14873,7 +15095,7 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="12"/>
+      <c r="A67" s="13"/>
       <c r="B67" s="11" t="s">
         <v>70</v>
       </c>
@@ -14885,7 +15107,7 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="12"/>
+      <c r="A68" s="13"/>
       <c r="B68" s="11" t="s">
         <v>71</v>
       </c>
@@ -14897,7 +15119,7 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="12"/>
+      <c r="A69" s="13"/>
       <c r="B69" s="11" t="s">
         <v>68</v>
       </c>
@@ -14910,7 +15132,7 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="12">
+      <c r="A70" s="13">
         <v>2041</v>
       </c>
       <c r="B70" s="11" t="s">
@@ -14924,7 +15146,7 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="12"/>
+      <c r="A71" s="13"/>
       <c r="B71" s="11" t="s">
         <v>70</v>
       </c>
@@ -14936,7 +15158,7 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="12"/>
+      <c r="A72" s="13"/>
       <c r="B72" s="11" t="s">
         <v>71</v>
       </c>
@@ -14948,7 +15170,7 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="12"/>
+      <c r="A73" s="13"/>
       <c r="B73" s="11" t="s">
         <v>68</v>
       </c>
@@ -14961,7 +15183,7 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="12">
+      <c r="A74" s="13">
         <v>2042</v>
       </c>
       <c r="B74" s="11" t="s">
@@ -14975,7 +15197,7 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="12"/>
+      <c r="A75" s="13"/>
       <c r="B75" s="11" t="s">
         <v>70</v>
       </c>
@@ -14987,7 +15209,7 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="12"/>
+      <c r="A76" s="13"/>
       <c r="B76" s="11" t="s">
         <v>71</v>
       </c>
@@ -14999,7 +15221,7 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="12"/>
+      <c r="A77" s="13"/>
       <c r="B77" s="11" t="s">
         <v>68</v>
       </c>
@@ -15012,7 +15234,7 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="12">
+      <c r="A78" s="13">
         <v>2043</v>
       </c>
       <c r="B78" s="11" t="s">
@@ -15026,7 +15248,7 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="12"/>
+      <c r="A79" s="13"/>
       <c r="B79" s="11" t="s">
         <v>70</v>
       </c>
@@ -15038,7 +15260,7 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="12"/>
+      <c r="A80" s="13"/>
       <c r="B80" s="11" t="s">
         <v>71</v>
       </c>
@@ -15050,7 +15272,7 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="12"/>
+      <c r="A81" s="13"/>
       <c r="B81" s="11" t="s">
         <v>68</v>
       </c>
@@ -15063,7 +15285,7 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="12">
+      <c r="A82" s="13">
         <v>2044</v>
       </c>
       <c r="B82" s="11" t="s">
@@ -15077,7 +15299,7 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="12"/>
+      <c r="A83" s="13"/>
       <c r="B83" s="11" t="s">
         <v>70</v>
       </c>
@@ -15089,7 +15311,7 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="12"/>
+      <c r="A84" s="13"/>
       <c r="B84" s="11" t="s">
         <v>71</v>
       </c>
@@ -15101,7 +15323,7 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="12"/>
+      <c r="A85" s="13"/>
       <c r="B85" s="11" t="s">
         <v>68</v>
       </c>
@@ -15114,7 +15336,7 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="12">
+      <c r="A86" s="13">
         <v>2045</v>
       </c>
       <c r="B86" s="11" t="s">
@@ -15128,7 +15350,7 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="12"/>
+      <c r="A87" s="13"/>
       <c r="B87" s="11" t="s">
         <v>70</v>
       </c>
@@ -15140,7 +15362,7 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="12"/>
+      <c r="A88" s="13"/>
       <c r="B88" s="11" t="s">
         <v>71</v>
       </c>
@@ -15152,7 +15374,7 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="12"/>
+      <c r="A89" s="13"/>
       <c r="B89" s="11" t="s">
         <v>68</v>
       </c>
@@ -15165,7 +15387,7 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="12">
+      <c r="A90" s="13">
         <v>2046</v>
       </c>
       <c r="B90" s="11" t="s">
@@ -15179,7 +15401,7 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="12"/>
+      <c r="A91" s="13"/>
       <c r="B91" s="11" t="s">
         <v>70</v>
       </c>
@@ -15191,7 +15413,7 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="12"/>
+      <c r="A92" s="13"/>
       <c r="B92" s="11" t="s">
         <v>71</v>
       </c>
@@ -15203,7 +15425,7 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="12"/>
+      <c r="A93" s="13"/>
       <c r="B93" s="11" t="s">
         <v>68</v>
       </c>
@@ -15216,7 +15438,7 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="12">
+      <c r="A94" s="13">
         <v>2047</v>
       </c>
       <c r="B94" s="11" t="s">
@@ -15230,7 +15452,7 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="12"/>
+      <c r="A95" s="13"/>
       <c r="B95" s="11" t="s">
         <v>70</v>
       </c>
@@ -15242,7 +15464,7 @@
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="12"/>
+      <c r="A96" s="13"/>
       <c r="B96" s="11" t="s">
         <v>71</v>
       </c>
@@ -15254,7 +15476,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="12"/>
+      <c r="A97" s="13"/>
       <c r="B97" s="11" t="s">
         <v>68</v>
       </c>
@@ -15267,7 +15489,7 @@
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="12">
+      <c r="A98" s="13">
         <v>2048</v>
       </c>
       <c r="B98" s="11" t="s">
@@ -15281,7 +15503,7 @@
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" s="12"/>
+      <c r="A99" s="13"/>
       <c r="B99" s="11" t="s">
         <v>70</v>
       </c>
@@ -15293,7 +15515,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="12"/>
+      <c r="A100" s="13"/>
       <c r="B100" s="11" t="s">
         <v>71</v>
       </c>
@@ -15305,7 +15527,7 @@
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" s="12"/>
+      <c r="A101" s="13"/>
       <c r="B101" s="11" t="s">
         <v>68</v>
       </c>
@@ -15318,7 +15540,7 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" s="12">
+      <c r="A102" s="13">
         <v>2049</v>
       </c>
       <c r="B102" s="11" t="s">
@@ -15332,7 +15554,7 @@
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A103" s="12"/>
+      <c r="A103" s="13"/>
       <c r="B103" s="11" t="s">
         <v>70</v>
       </c>
@@ -15344,7 +15566,7 @@
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="12"/>
+      <c r="A104" s="13"/>
       <c r="B104" s="11" t="s">
         <v>71</v>
       </c>
@@ -15356,7 +15578,7 @@
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="12"/>
+      <c r="A105" s="13"/>
       <c r="B105" s="11" t="s">
         <v>68</v>
       </c>
@@ -15369,7 +15591,7 @@
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" s="12">
+      <c r="A106" s="13">
         <v>2050</v>
       </c>
       <c r="B106" s="11" t="s">
@@ -15383,7 +15605,7 @@
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" s="12"/>
+      <c r="A107" s="13"/>
       <c r="B107" s="11" t="s">
         <v>70</v>
       </c>
@@ -15395,7 +15617,7 @@
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" s="12"/>
+      <c r="A108" s="13"/>
       <c r="B108" s="11" t="s">
         <v>71</v>
       </c>
@@ -15407,7 +15629,7 @@
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" s="12"/>
+      <c r="A109" s="13"/>
       <c r="B109" s="11" t="s">
         <v>68</v>
       </c>

</xml_diff>

<commit_message>
Refactors material recycling and energy demand
Updates the material recycling constraint to accurately calculate recycled material based on scrap content and recycling efficiency.

Corrects the energy demand calculation by using tech and stage parameters, removing the location parameter to match the data indices.

Renames `material_content` to `scrap_content` for clarity and consistency in scrap processing logic.

Sets a default value of 100 for `energy_needs`.

Removes scenario constraints.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-extension/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="403" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEF8DBB7-6D38-454A-A4D6-ADC9D831B385}"/>
+  <xr:revisionPtr revIDLastSave="483" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A619CE2A-1920-42BB-88FA-2AAB6AD008B4}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" firstSheet="6" activeTab="13" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="7" activeTab="9" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="153">
   <si>
     <t>Value</t>
   </si>
@@ -310,25 +310,10 @@
     <t>Material</t>
   </si>
   <si>
-    <t>Silicon</t>
-  </si>
-  <si>
-    <t>3.0</t>
-  </si>
-  <si>
     <t>0.95</t>
   </si>
   <si>
     <t>Cell</t>
-  </si>
-  <si>
-    <t>Silver</t>
-  </si>
-  <si>
-    <t>0.05</t>
-  </si>
-  <si>
-    <t>0.98</t>
   </si>
   <si>
     <t>Module</t>
@@ -337,34 +322,7 @@
     <t>Glass</t>
   </si>
   <si>
-    <t>40.0</t>
-  </si>
-  <si>
-    <t>38.0</t>
-  </si>
-  <si>
-    <t>0.90</t>
-  </si>
-  <si>
-    <t>Aluminum</t>
-  </si>
-  <si>
-    <t>5.0</t>
-  </si>
-  <si>
-    <t>0.85</t>
-  </si>
-  <si>
     <t>Blade</t>
-  </si>
-  <si>
-    <t>Composite</t>
-  </si>
-  <si>
-    <t>12.0</t>
-  </si>
-  <si>
-    <t>0.50</t>
   </si>
   <si>
     <t>Tower</t>
@@ -373,25 +331,7 @@
     <t>Steel</t>
   </si>
   <si>
-    <t>150.0</t>
-  </si>
-  <si>
     <t>Nacelle</t>
-  </si>
-  <si>
-    <t>Copper</t>
-  </si>
-  <si>
-    <t>2.0</t>
-  </si>
-  <si>
-    <t>RareEarth</t>
-  </si>
-  <si>
-    <t>0.1</t>
-  </si>
-  <si>
-    <t>0.80</t>
   </si>
   <si>
     <t>Batteries</t>
@@ -515,6 +455,63 @@
   </si>
   <si>
     <t>opex_fixed</t>
+  </si>
+  <si>
+    <t>Al</t>
+  </si>
+  <si>
+    <t>Polymers</t>
+  </si>
+  <si>
+    <t>Cu</t>
+  </si>
+  <si>
+    <t>Ag</t>
+  </si>
+  <si>
+    <t>Si</t>
+  </si>
+  <si>
+    <t>CFRP</t>
+  </si>
+  <si>
+    <t>GFRP</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Zn</t>
+  </si>
+  <si>
+    <t>Dy</t>
+  </si>
+  <si>
+    <t>Nd</t>
+  </si>
+  <si>
+    <t>Pr</t>
+  </si>
+  <si>
+    <t>Cast iron</t>
+  </si>
+  <si>
+    <t>Mn</t>
+  </si>
+  <si>
+    <t>Mo</t>
+  </si>
+  <si>
+    <t>Ni</t>
+  </si>
+  <si>
+    <t>Cr</t>
+  </si>
+  <si>
+    <t>0.92</t>
+  </si>
+  <si>
+    <t>0.98</t>
   </si>
 </sst>
 </file>
@@ -695,7 +692,7 @@
     </xf>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -723,6 +720,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1120,7 +1120,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="B1" t="s">
         <v>82</v>
@@ -1135,7 +1135,7 @@
         <v>73</v>
       </c>
       <c r="F1" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
       <c r="G1" t="s">
         <v>74</v>
@@ -1152,12 +1152,12 @@
         <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="12">
         <v>150</v>
       </c>
       <c r="F2" s="7">
@@ -1175,13 +1175,13 @@
         <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
-      <c r="E3">
-        <v>100</v>
+      <c r="E3" s="12">
+        <v>125</v>
       </c>
       <c r="F3" s="7">
         <v>2000</v>
@@ -1198,13 +1198,13 @@
         <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4">
-        <v>100</v>
+      <c r="E4" s="12">
+        <v>76</v>
       </c>
       <c r="F4" s="7">
         <v>7000</v>
@@ -1221,13 +1221,13 @@
         <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5">
-        <v>100</v>
+      <c r="E5" s="12">
+        <v>75</v>
       </c>
       <c r="F5" s="7">
         <v>22000</v>
@@ -1247,15 +1247,15 @@
         <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
-      <c r="E6">
-        <v>100</v>
-      </c>
-      <c r="F6" s="7">
+      <c r="E6" s="12">
+        <v>60</v>
+      </c>
+      <c r="F6">
         <v>27000</v>
       </c>
       <c r="G6">
@@ -1273,15 +1273,15 @@
         <v>76</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
-      <c r="E7">
-        <v>100</v>
-      </c>
-      <c r="F7" s="7">
+      <c r="E7" s="12">
+        <v>55</v>
+      </c>
+      <c r="F7">
         <v>27000</v>
       </c>
       <c r="G7">
@@ -1299,15 +1299,15 @@
         <v>76</v>
       </c>
       <c r="C8" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
-      <c r="E8">
-        <v>100</v>
-      </c>
-      <c r="F8" s="7">
+      <c r="E8" s="12">
+        <v>35</v>
+      </c>
+      <c r="F8">
         <v>27000</v>
       </c>
       <c r="G8">
@@ -1325,22 +1325,22 @@
         <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
-      <c r="E9">
-        <v>100</v>
-      </c>
-      <c r="F9" s="7">
+      <c r="E9" s="12">
+        <v>0</v>
+      </c>
+      <c r="F9" s="12">
         <v>999999</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>149</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1351,13 +1351,13 @@
         <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
-      <c r="E10">
-        <v>100</v>
+      <c r="E10" s="12">
+        <v>60</v>
       </c>
       <c r="F10">
         <v>100</v>
@@ -1377,15 +1377,15 @@
         <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="F11" s="7">
+      <c r="E11" s="12">
+        <v>55</v>
+      </c>
+      <c r="F11">
         <v>1</v>
       </c>
       <c r="G11">
@@ -1400,12 +1400,12 @@
         <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>107</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="F12" s="7">
+        <v>92</v>
+      </c>
+      <c r="E12" s="12">
+        <v>35</v>
+      </c>
+      <c r="F12">
         <v>1</v>
       </c>
       <c r="G12">
@@ -1420,15 +1420,15 @@
         <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13">
-        <v>100</v>
-      </c>
-      <c r="F13" s="7">
+      <c r="E13" s="12">
+        <v>0</v>
+      </c>
+      <c r="F13" s="12">
         <v>999999</v>
       </c>
       <c r="G13">
@@ -1440,16 +1440,16 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D14">
         <v>1</v>
       </c>
-      <c r="E14">
-        <v>80</v>
+      <c r="E14" s="12">
+        <v>40</v>
       </c>
       <c r="F14">
         <v>100</v>
@@ -1463,25 +1463,25 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="C15" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15">
-        <v>20</v>
-      </c>
-      <c r="F15">
-        <v>100</v>
+      <c r="E15" s="12">
+        <v>0</v>
+      </c>
+      <c r="F15" s="12">
+        <v>999999</v>
       </c>
       <c r="G15">
         <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>149</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -1492,7 +1492,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FA1A697-84AA-4F97-BE70-81695B57512E}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -1506,296 +1506,817 @@
         <v>84</v>
       </c>
       <c r="D1" t="s">
-        <v>129</v>
+        <v>109</v>
       </c>
       <c r="E1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="F1" t="s">
-        <v>128</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="D2" s="12">
+        <v>7.5</v>
+      </c>
+      <c r="E2" s="12">
+        <v>7.5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D3" s="12">
+        <v>46.4</v>
+      </c>
+      <c r="E3" s="12">
+        <v>46.4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D4" s="12">
+        <v>8.6000000000000014</v>
+      </c>
+      <c r="E4" s="12">
+        <v>8.6000000000000014</v>
+      </c>
+      <c r="F4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D5" s="12">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="E5" s="12">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="F5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="D6" s="12">
+        <v>1.9012500000000002E-2</v>
+      </c>
+      <c r="E6" s="12">
+        <v>1.9012500000000002E-2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7" s="12">
+        <v>3.803015625</v>
+      </c>
+      <c r="E7" s="12">
+        <v>3.803015625</v>
+      </c>
+      <c r="F7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="D8" s="12">
+        <v>0.94859999999999989</v>
+      </c>
+      <c r="E8" s="12">
+        <v>0.94859999999999989</v>
+      </c>
+      <c r="F8" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="D9" s="12">
+        <v>6.9563999999999995</v>
+      </c>
+      <c r="E9" s="12">
+        <v>6.9563999999999995</v>
+      </c>
+      <c r="F9" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D10" s="12">
+        <v>1.17E-3</v>
+      </c>
+      <c r="E10" s="12">
+        <v>1.17E-3</v>
+      </c>
+      <c r="F10" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" s="12">
+        <v>8.1</v>
+      </c>
+      <c r="E11" s="12">
+        <v>8.1</v>
+      </c>
+      <c r="F11" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="D12" s="12">
+        <v>114.72499999999999</v>
+      </c>
+      <c r="E12" s="12">
+        <v>114.72499999999999</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="D13" s="12">
+        <v>5.5</v>
+      </c>
+      <c r="E13" s="12">
+        <v>5.5</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="D14" s="12">
+        <v>5.47E-3</v>
+      </c>
+      <c r="E14" s="12">
+        <v>5.47E-3</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="D15" s="12">
+        <v>4.7689999999999996E-2</v>
+      </c>
+      <c r="E15" s="12">
+        <v>4.7689999999999996E-2</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C16" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D16" s="12">
+        <v>7.2699999999999996E-3</v>
+      </c>
+      <c r="E16" s="12">
+        <v>7.2699999999999996E-3</v>
+      </c>
+      <c r="F16" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="D17" s="12">
+        <v>2.7909999999999999</v>
+      </c>
+      <c r="E17" s="12">
+        <v>2.7909999999999999</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D18" s="12">
+        <v>2.2925</v>
+      </c>
+      <c r="E18" s="12">
+        <v>2.2925</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="D19" s="12">
+        <v>18.945</v>
+      </c>
+      <c r="E19" s="12">
+        <v>18.945</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="D20" s="12">
+        <v>0.78549999999999998</v>
+      </c>
+      <c r="E20" s="12">
+        <v>0.78549999999999998</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D21" s="12">
+        <v>0.1045</v>
+      </c>
+      <c r="E21" s="12">
+        <v>0.1045</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="D22" s="12">
+        <v>0.39200000000000002</v>
+      </c>
+      <c r="E22" s="12">
+        <v>0.39200000000000002</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="D23" s="12">
+        <v>0.50024999999999997</v>
+      </c>
+      <c r="E23" s="12">
+        <v>0.50024999999999997</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="D24" s="12">
+        <v>0.97139999999999993</v>
+      </c>
+      <c r="E24" s="12">
+        <v>0.97139999999999993</v>
+      </c>
+      <c r="F24" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="D25" s="12">
+        <v>7.1236000000000006</v>
+      </c>
+      <c r="E25" s="12">
+        <v>7.1236000000000006</v>
+      </c>
+      <c r="F25" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D26" s="12">
+        <v>3.4500000000000004E-3</v>
+      </c>
+      <c r="E26" s="12">
+        <v>3.4500000000000004E-3</v>
+      </c>
+      <c r="F26" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D27" s="12">
+        <v>11.6</v>
+      </c>
+      <c r="E27" s="12">
+        <v>11.6</v>
+      </c>
+      <c r="F27" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B28" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="E2" t="s">
+      <c r="C28" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="D28" s="12">
+        <v>116.77</v>
+      </c>
+      <c r="E28" s="12">
+        <v>116.77</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="D29" s="12">
+        <v>5.5</v>
+      </c>
+      <c r="E29" s="12">
+        <v>5.5</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="D30" s="12">
+        <v>1.1259999999999999E-2</v>
+      </c>
+      <c r="E30" s="12">
+        <v>1.1259999999999999E-2</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="D31" s="12">
+        <v>0.11219</v>
+      </c>
+      <c r="E31" s="12">
+        <v>0.11219</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="D32" s="12">
+        <v>2.0460000000000002E-2</v>
+      </c>
+      <c r="E32" s="12">
+        <v>2.0460000000000002E-2</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="D33" s="12">
+        <v>4.04</v>
+      </c>
+      <c r="E33" s="12">
+        <v>4.04</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D34" s="12">
+        <v>3.2574999999999998</v>
+      </c>
+      <c r="E34" s="12">
+        <v>3.2574999999999998</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="D35" s="12">
+        <v>19.89</v>
+      </c>
+      <c r="E35" s="12">
+        <v>19.89</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="D36" s="12">
+        <v>0.79039999999999999</v>
+      </c>
+      <c r="E36" s="12">
+        <v>0.79039999999999999</v>
+      </c>
+      <c r="F36" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D37" s="12">
+        <v>0.10940000000000001</v>
+      </c>
+      <c r="E37" s="12">
+        <v>0.10940000000000001</v>
+      </c>
+      <c r="F37" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="D38" s="12">
+        <v>0.32230000000000003</v>
+      </c>
+      <c r="E38" s="12">
+        <v>0.32230000000000003</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="D39" s="12">
+        <v>0.5272</v>
+      </c>
+      <c r="E39" s="12">
+        <v>0.5272</v>
+      </c>
+      <c r="F39" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>93</v>
+      </c>
+      <c r="B40" t="s">
         <v>86</v>
       </c>
-      <c r="F2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C3" t="s">
-        <v>89</v>
-      </c>
-      <c r="D3" t="s">
-        <v>90</v>
-      </c>
-      <c r="E3" t="s">
-        <v>90</v>
-      </c>
-      <c r="F3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="C40" t="s">
+        <v>94</v>
+      </c>
+      <c r="D40" t="s">
+        <v>95</v>
+      </c>
+      <c r="E40" t="s">
+        <v>95</v>
+      </c>
+      <c r="F40" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>93</v>
       </c>
-      <c r="D4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E4" t="s">
-        <v>95</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="B41" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D41" t="s">
         <v>97</v>
       </c>
-      <c r="D5" t="s">
-        <v>98</v>
-      </c>
-      <c r="E5" t="s">
-        <v>98</v>
-      </c>
-      <c r="F5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C6" t="s">
-        <v>101</v>
-      </c>
-      <c r="D6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E6" t="s">
-        <v>102</v>
-      </c>
-      <c r="F6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>76</v>
-      </c>
-      <c r="B7" t="s">
-        <v>104</v>
-      </c>
-      <c r="C7" t="s">
-        <v>105</v>
-      </c>
-      <c r="D7" t="s">
-        <v>106</v>
-      </c>
-      <c r="E7" t="s">
-        <v>106</v>
-      </c>
-      <c r="F7" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B8" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" t="s">
-        <v>108</v>
-      </c>
-      <c r="D8" t="s">
-        <v>109</v>
-      </c>
-      <c r="E8" t="s">
-        <v>109</v>
-      </c>
-      <c r="F8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B9" t="s">
-        <v>107</v>
-      </c>
-      <c r="C9" t="s">
-        <v>110</v>
-      </c>
-      <c r="D9" t="s">
-        <v>111</v>
-      </c>
-      <c r="E9" t="s">
-        <v>111</v>
-      </c>
-      <c r="F9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>77</v>
-      </c>
-      <c r="B10" t="s">
-        <v>100</v>
-      </c>
-      <c r="C10" t="s">
-        <v>101</v>
-      </c>
-      <c r="D10" t="s">
-        <v>102</v>
-      </c>
-      <c r="E10" t="s">
-        <v>102</v>
-      </c>
-      <c r="F10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>77</v>
-      </c>
-      <c r="B11" t="s">
-        <v>104</v>
-      </c>
-      <c r="C11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D11" t="s">
-        <v>106</v>
-      </c>
-      <c r="E11" t="s">
-        <v>106</v>
-      </c>
-      <c r="F11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>77</v>
-      </c>
-      <c r="B12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D12" t="s">
-        <v>109</v>
-      </c>
-      <c r="E12" t="s">
-        <v>109</v>
-      </c>
-      <c r="F12" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>77</v>
-      </c>
-      <c r="B13" t="s">
-        <v>107</v>
-      </c>
-      <c r="C13" t="s">
-        <v>110</v>
-      </c>
-      <c r="D13" t="s">
-        <v>111</v>
-      </c>
-      <c r="E13" t="s">
-        <v>111</v>
-      </c>
-      <c r="F13" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" t="s">
-        <v>88</v>
-      </c>
-      <c r="C14" t="s">
-        <v>114</v>
-      </c>
-      <c r="D14" t="s">
-        <v>115</v>
-      </c>
-      <c r="E14" t="s">
-        <v>115</v>
-      </c>
-      <c r="F14" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>113</v>
-      </c>
-      <c r="B15" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" t="s">
-        <v>116</v>
-      </c>
-      <c r="D15" t="s">
-        <v>117</v>
-      </c>
-      <c r="E15" t="s">
-        <v>117</v>
-      </c>
-      <c r="F15" t="s">
-        <v>96</v>
+      <c r="E41" t="s">
+        <v>97</v>
+      </c>
+      <c r="F41" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -1803,24 +2324,24 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03BB5A9E-0DE2-4C9D-A6F4-EBF765E41A9E}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="B1" t="s">
         <v>84</v>
       </c>
       <c r="C1" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="D1" t="s">
-        <v>131</v>
+        <v>111</v>
       </c>
       <c r="E1" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1828,7 +2349,7 @@
         <v>2024</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>134</v>
       </c>
       <c r="C2">
         <v>1000000</v>
@@ -1845,7 +2366,7 @@
         <v>2024</v>
       </c>
       <c r="B3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C3">
         <v>5000</v>
@@ -1862,7 +2383,7 @@
         <v>2024</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>135</v>
       </c>
       <c r="C4">
         <v>5000000</v>
@@ -1879,7 +2400,7 @@
         <v>2024</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
+        <v>136</v>
       </c>
       <c r="C5">
         <v>2000000</v>
@@ -1896,7 +2417,7 @@
         <v>2024</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="C6">
         <v>500000</v>
@@ -1913,7 +2434,7 @@
         <v>2024</v>
       </c>
       <c r="B7" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
       <c r="C7">
         <v>10000000</v>
@@ -1930,7 +2451,7 @@
         <v>2024</v>
       </c>
       <c r="B8" t="s">
-        <v>108</v>
+        <v>139</v>
       </c>
       <c r="C8">
         <v>800000</v>
@@ -1947,7 +2468,7 @@
         <v>2024</v>
       </c>
       <c r="B9" t="s">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="C9">
         <v>20000</v>
@@ -1964,7 +2485,7 @@
         <v>2024</v>
       </c>
       <c r="B10" t="s">
-        <v>114</v>
+        <v>141</v>
       </c>
       <c r="C10">
         <v>150000</v>
@@ -1981,15 +2502,253 @@
         <v>2024</v>
       </c>
       <c r="B11" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="C11">
-        <v>50000</v>
+        <v>150000</v>
       </c>
       <c r="D11">
         <v>30000</v>
       </c>
       <c r="E11">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2024</v>
+      </c>
+      <c r="B12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12">
+        <v>150000</v>
+      </c>
+      <c r="D12">
+        <v>30000</v>
+      </c>
+      <c r="E12">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2024</v>
+      </c>
+      <c r="B13" t="s">
+        <v>142</v>
+      </c>
+      <c r="C13">
+        <v>150000</v>
+      </c>
+      <c r="D13">
+        <v>30000</v>
+      </c>
+      <c r="E13">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2024</v>
+      </c>
+      <c r="B14" t="s">
+        <v>143</v>
+      </c>
+      <c r="C14">
+        <v>150000</v>
+      </c>
+      <c r="D14">
+        <v>30000</v>
+      </c>
+      <c r="E14">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2024</v>
+      </c>
+      <c r="B15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C15">
+        <v>150000</v>
+      </c>
+      <c r="D15">
+        <v>30000</v>
+      </c>
+      <c r="E15">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2024</v>
+      </c>
+      <c r="B16" t="s">
+        <v>145</v>
+      </c>
+      <c r="C16">
+        <v>150000</v>
+      </c>
+      <c r="D16">
+        <v>30000</v>
+      </c>
+      <c r="E16">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>2024</v>
+      </c>
+      <c r="B17" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17">
+        <v>150000</v>
+      </c>
+      <c r="D17">
+        <v>30000</v>
+      </c>
+      <c r="E17">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>2024</v>
+      </c>
+      <c r="B18" t="s">
+        <v>136</v>
+      </c>
+      <c r="C18">
+        <v>150000</v>
+      </c>
+      <c r="D18">
+        <v>30000</v>
+      </c>
+      <c r="E18">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2024</v>
+      </c>
+      <c r="B19" t="s">
+        <v>146</v>
+      </c>
+      <c r="C19">
+        <v>150000</v>
+      </c>
+      <c r="D19">
+        <v>30000</v>
+      </c>
+      <c r="E19">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>2024</v>
+      </c>
+      <c r="B20" t="s">
+        <v>147</v>
+      </c>
+      <c r="C20">
+        <v>150000</v>
+      </c>
+      <c r="D20">
+        <v>30000</v>
+      </c>
+      <c r="E20">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>2024</v>
+      </c>
+      <c r="B21" t="s">
+        <v>148</v>
+      </c>
+      <c r="C21">
+        <v>150000</v>
+      </c>
+      <c r="D21">
+        <v>30000</v>
+      </c>
+      <c r="E21">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>2024</v>
+      </c>
+      <c r="B22" t="s">
+        <v>149</v>
+      </c>
+      <c r="C22">
+        <v>150000</v>
+      </c>
+      <c r="D22">
+        <v>30000</v>
+      </c>
+      <c r="E22">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>2024</v>
+      </c>
+      <c r="B23" t="s">
+        <v>150</v>
+      </c>
+      <c r="C23">
+        <v>150000</v>
+      </c>
+      <c r="D23">
+        <v>30000</v>
+      </c>
+      <c r="E23">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>2024</v>
+      </c>
+      <c r="B24" t="s">
+        <v>94</v>
+      </c>
+      <c r="C24">
+        <v>150000</v>
+      </c>
+      <c r="D24">
+        <v>30000</v>
+      </c>
+      <c r="E24">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2024</v>
+      </c>
+      <c r="B25" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25">
+        <v>150000</v>
+      </c>
+      <c r="D25">
+        <v>30000</v>
+      </c>
+      <c r="E25">
         <v>35000</v>
       </c>
     </row>
@@ -2005,19 +2764,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
       <c r="B1" t="s">
-        <v>124</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="D1" t="s">
-        <v>126</v>
+        <v>106</v>
       </c>
       <c r="E1" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -2025,16 +2784,16 @@
         <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="C2" t="s">
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="E2" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -2042,16 +2801,16 @@
         <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C3" t="s">
         <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="E3" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2059,33 +2818,33 @@
         <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C4" t="s">
         <v>75</v>
       </c>
       <c r="D4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E4" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="D5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E5" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2093,16 +2852,16 @@
         <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="C6" t="s">
         <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E6" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2110,16 +2869,16 @@
         <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
         <v>76</v>
       </c>
       <c r="D7" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="E7" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2127,16 +2886,16 @@
         <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="C8" t="s">
         <v>76</v>
       </c>
       <c r="D8" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="E8" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2144,16 +2903,16 @@
         <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="C9" t="s">
         <v>77</v>
       </c>
       <c r="D9" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E9" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2161,16 +2920,16 @@
         <v>77</v>
       </c>
       <c r="B10" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="C10" t="s">
         <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="E10" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2178,16 +2937,16 @@
         <v>77</v>
       </c>
       <c r="B11" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="C11" t="s">
         <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="E11" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -2202,10 +2961,10 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="B1" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="C1" t="s">
         <v>82</v>
@@ -2214,13 +2973,13 @@
         <v>83</v>
       </c>
       <c r="E1" t="s">
-        <v>134</v>
+        <v>114</v>
       </c>
       <c r="F1" t="s">
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="G1" t="s">
-        <v>153</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -2234,7 +2993,7 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="E2" s="12">
         <v>55200</v>
@@ -2257,7 +3016,7 @@
         <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="E3" s="12">
         <v>92000</v>
@@ -2280,7 +3039,7 @@
         <v>75</v>
       </c>
       <c r="D4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E4" s="12">
         <v>165600</v>
@@ -2303,7 +3062,7 @@
         <v>75</v>
       </c>
       <c r="D5" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E5" s="12">
         <v>46000</v>
@@ -2326,7 +3085,7 @@
         <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E6" s="12">
         <v>73600</v>
@@ -2349,7 +3108,7 @@
         <v>76</v>
       </c>
       <c r="D7" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="E7" s="12">
         <v>82800</v>
@@ -2372,7 +3131,7 @@
         <v>76</v>
       </c>
       <c r="D8" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="E8" s="12">
         <v>276000</v>
@@ -2395,7 +3154,7 @@
         <v>76</v>
       </c>
       <c r="D9" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
@@ -2418,7 +3177,7 @@
         <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E10" s="12">
         <v>165600</v>
@@ -2441,7 +3200,7 @@
         <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="E11" s="12">
         <v>202400</v>
@@ -2464,7 +3223,7 @@
         <v>77</v>
       </c>
       <c r="D12" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="E12" s="12">
         <v>202400</v>
@@ -2487,7 +3246,7 @@
         <v>77</v>
       </c>
       <c r="D13" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="E13" s="12">
         <v>1</v>
@@ -2507,10 +3266,10 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="D14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E14" s="12">
         <v>92000</v>
@@ -2530,10 +3289,10 @@
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="D15" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="E15" s="12">
         <v>1</v>
@@ -2561,46 +3320,46 @@
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>146</v>
+        <v>126</v>
       </c>
       <c r="C1" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="D1" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="E1" t="s">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="F1" t="s">
-        <v>139</v>
+        <v>119</v>
       </c>
       <c r="G1" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="H1" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="I1" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="J1" t="s">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="K1" t="s">
-        <v>151</v>
+        <v>131</v>
       </c>
       <c r="L1" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
       <c r="M1" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="N1" t="s">
-        <v>148</v>
+        <v>128</v>
       </c>
       <c r="O1" t="s">
-        <v>147</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -14265,7 +15024,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="13">
+      <c r="A2" s="14">
         <v>2024</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -14279,7 +15038,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="13"/>
+      <c r="A3" s="14"/>
       <c r="B3" s="11" t="s">
         <v>70</v>
       </c>
@@ -14292,7 +15051,7 @@
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
+      <c r="A4" s="14"/>
       <c r="B4" s="11" t="s">
         <v>71</v>
       </c>
@@ -14304,7 +15063,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="13"/>
+      <c r="A5" s="14"/>
       <c r="B5" s="11" t="s">
         <v>68</v>
       </c>
@@ -14316,7 +15075,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="13">
+      <c r="A6" s="14">
         <v>2025</v>
       </c>
       <c r="B6" s="11" t="s">
@@ -14330,7 +15089,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="13"/>
+      <c r="A7" s="14"/>
       <c r="B7" s="11" t="s">
         <v>70</v>
       </c>
@@ -14342,7 +15101,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="13"/>
+      <c r="A8" s="14"/>
       <c r="B8" s="11" t="s">
         <v>71</v>
       </c>
@@ -14354,7 +15113,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="13"/>
+      <c r="A9" s="14"/>
       <c r="B9" s="11" t="s">
         <v>68</v>
       </c>
@@ -14367,7 +15126,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="13">
+      <c r="A10" s="14">
         <v>2026</v>
       </c>
       <c r="B10" s="11" t="s">
@@ -14381,7 +15140,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="13"/>
+      <c r="A11" s="14"/>
       <c r="B11" s="11" t="s">
         <v>70</v>
       </c>
@@ -14393,7 +15152,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="13"/>
+      <c r="A12" s="14"/>
       <c r="B12" s="11" t="s">
         <v>71</v>
       </c>
@@ -14405,7 +15164,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="13"/>
+      <c r="A13" s="14"/>
       <c r="B13" s="11" t="s">
         <v>68</v>
       </c>
@@ -14418,7 +15177,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="13">
+      <c r="A14" s="14">
         <v>2027</v>
       </c>
       <c r="B14" s="11" t="s">
@@ -14432,7 +15191,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="13"/>
+      <c r="A15" s="14"/>
       <c r="B15" s="11" t="s">
         <v>70</v>
       </c>
@@ -14444,7 +15203,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="13"/>
+      <c r="A16" s="14"/>
       <c r="B16" s="11" t="s">
         <v>71</v>
       </c>
@@ -14456,7 +15215,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="13"/>
+      <c r="A17" s="14"/>
       <c r="B17" s="11" t="s">
         <v>68</v>
       </c>
@@ -14469,7 +15228,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="13">
+      <c r="A18" s="14">
         <v>2028</v>
       </c>
       <c r="B18" s="11" t="s">
@@ -14483,7 +15242,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="13"/>
+      <c r="A19" s="14"/>
       <c r="B19" s="11" t="s">
         <v>70</v>
       </c>
@@ -14495,7 +15254,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="13"/>
+      <c r="A20" s="14"/>
       <c r="B20" s="11" t="s">
         <v>71</v>
       </c>
@@ -14507,7 +15266,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="13"/>
+      <c r="A21" s="14"/>
       <c r="B21" s="11" t="s">
         <v>68</v>
       </c>
@@ -14520,7 +15279,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="13">
+      <c r="A22" s="14">
         <v>2029</v>
       </c>
       <c r="B22" s="11" t="s">
@@ -14534,7 +15293,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="13"/>
+      <c r="A23" s="14"/>
       <c r="B23" s="11" t="s">
         <v>70</v>
       </c>
@@ -14546,7 +15305,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="13"/>
+      <c r="A24" s="14"/>
       <c r="B24" s="11" t="s">
         <v>71</v>
       </c>
@@ -14558,7 +15317,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="13"/>
+      <c r="A25" s="14"/>
       <c r="B25" s="11" t="s">
         <v>68</v>
       </c>
@@ -14571,7 +15330,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="13">
+      <c r="A26" s="14">
         <v>2030</v>
       </c>
       <c r="B26" s="11" t="s">
@@ -14585,7 +15344,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="13"/>
+      <c r="A27" s="14"/>
       <c r="B27" s="11" t="s">
         <v>70</v>
       </c>
@@ -14597,7 +15356,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="13"/>
+      <c r="A28" s="14"/>
       <c r="B28" s="11" t="s">
         <v>71</v>
       </c>
@@ -14609,7 +15368,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="13"/>
+      <c r="A29" s="14"/>
       <c r="B29" s="11" t="s">
         <v>68</v>
       </c>
@@ -14622,7 +15381,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="13">
+      <c r="A30" s="14">
         <v>2031</v>
       </c>
       <c r="B30" s="11" t="s">
@@ -14636,7 +15395,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="13"/>
+      <c r="A31" s="14"/>
       <c r="B31" s="11" t="s">
         <v>70</v>
       </c>
@@ -14648,7 +15407,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="13"/>
+      <c r="A32" s="14"/>
       <c r="B32" s="11" t="s">
         <v>71</v>
       </c>
@@ -14660,7 +15419,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="13"/>
+      <c r="A33" s="14"/>
       <c r="B33" s="11" t="s">
         <v>68</v>
       </c>
@@ -14673,7 +15432,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="13">
+      <c r="A34" s="14">
         <v>2032</v>
       </c>
       <c r="B34" s="11" t="s">
@@ -14687,7 +15446,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="13"/>
+      <c r="A35" s="14"/>
       <c r="B35" s="11" t="s">
         <v>70</v>
       </c>
@@ -14699,7 +15458,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="13"/>
+      <c r="A36" s="14"/>
       <c r="B36" s="11" t="s">
         <v>71</v>
       </c>
@@ -14711,7 +15470,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="13"/>
+      <c r="A37" s="14"/>
       <c r="B37" s="11" t="s">
         <v>68</v>
       </c>
@@ -14724,7 +15483,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="13">
+      <c r="A38" s="14">
         <v>2033</v>
       </c>
       <c r="B38" s="11" t="s">
@@ -14738,7 +15497,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="13"/>
+      <c r="A39" s="14"/>
       <c r="B39" s="11" t="s">
         <v>70</v>
       </c>
@@ -14750,7 +15509,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="13"/>
+      <c r="A40" s="14"/>
       <c r="B40" s="11" t="s">
         <v>71</v>
       </c>
@@ -14762,7 +15521,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="13"/>
+      <c r="A41" s="14"/>
       <c r="B41" s="11" t="s">
         <v>68</v>
       </c>
@@ -14775,7 +15534,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="13">
+      <c r="A42" s="14">
         <v>2034</v>
       </c>
       <c r="B42" s="11" t="s">
@@ -14789,7 +15548,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="13"/>
+      <c r="A43" s="14"/>
       <c r="B43" s="11" t="s">
         <v>70</v>
       </c>
@@ -14801,7 +15560,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="13"/>
+      <c r="A44" s="14"/>
       <c r="B44" s="11" t="s">
         <v>71</v>
       </c>
@@ -14813,7 +15572,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="13"/>
+      <c r="A45" s="14"/>
       <c r="B45" s="11" t="s">
         <v>68</v>
       </c>
@@ -14826,7 +15585,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="13">
+      <c r="A46" s="14">
         <v>2035</v>
       </c>
       <c r="B46" s="11" t="s">
@@ -14840,7 +15599,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="13"/>
+      <c r="A47" s="14"/>
       <c r="B47" s="11" t="s">
         <v>70</v>
       </c>
@@ -14852,7 +15611,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="13"/>
+      <c r="A48" s="14"/>
       <c r="B48" s="11" t="s">
         <v>71</v>
       </c>
@@ -14864,7 +15623,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="13"/>
+      <c r="A49" s="14"/>
       <c r="B49" s="11" t="s">
         <v>68</v>
       </c>
@@ -14877,7 +15636,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="13">
+      <c r="A50" s="14">
         <v>2036</v>
       </c>
       <c r="B50" s="11" t="s">
@@ -14891,7 +15650,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="13"/>
+      <c r="A51" s="14"/>
       <c r="B51" s="11" t="s">
         <v>70</v>
       </c>
@@ -14903,7 +15662,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="13"/>
+      <c r="A52" s="14"/>
       <c r="B52" s="11" t="s">
         <v>71</v>
       </c>
@@ -14915,7 +15674,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="13"/>
+      <c r="A53" s="14"/>
       <c r="B53" s="11" t="s">
         <v>68</v>
       </c>
@@ -14928,7 +15687,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="13">
+      <c r="A54" s="14">
         <v>2037</v>
       </c>
       <c r="B54" s="11" t="s">
@@ -14942,7 +15701,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="13"/>
+      <c r="A55" s="14"/>
       <c r="B55" s="11" t="s">
         <v>70</v>
       </c>
@@ -14954,7 +15713,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="13"/>
+      <c r="A56" s="14"/>
       <c r="B56" s="11" t="s">
         <v>71</v>
       </c>
@@ -14966,7 +15725,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="13"/>
+      <c r="A57" s="14"/>
       <c r="B57" s="11" t="s">
         <v>68</v>
       </c>
@@ -14979,7 +15738,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="13">
+      <c r="A58" s="14">
         <v>2038</v>
       </c>
       <c r="B58" s="11" t="s">
@@ -14993,7 +15752,7 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="13"/>
+      <c r="A59" s="14"/>
       <c r="B59" s="11" t="s">
         <v>70</v>
       </c>
@@ -15005,7 +15764,7 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="13"/>
+      <c r="A60" s="14"/>
       <c r="B60" s="11" t="s">
         <v>71</v>
       </c>
@@ -15017,7 +15776,7 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="13"/>
+      <c r="A61" s="14"/>
       <c r="B61" s="11" t="s">
         <v>68</v>
       </c>
@@ -15030,7 +15789,7 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="13">
+      <c r="A62" s="14">
         <v>2039</v>
       </c>
       <c r="B62" s="11" t="s">
@@ -15044,7 +15803,7 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="13"/>
+      <c r="A63" s="14"/>
       <c r="B63" s="11" t="s">
         <v>70</v>
       </c>
@@ -15056,7 +15815,7 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="13"/>
+      <c r="A64" s="14"/>
       <c r="B64" s="11" t="s">
         <v>71</v>
       </c>
@@ -15068,7 +15827,7 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="13"/>
+      <c r="A65" s="14"/>
       <c r="B65" s="11" t="s">
         <v>68</v>
       </c>
@@ -15081,7 +15840,7 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="13">
+      <c r="A66" s="14">
         <v>2040</v>
       </c>
       <c r="B66" s="11" t="s">
@@ -15095,7 +15854,7 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="13"/>
+      <c r="A67" s="14"/>
       <c r="B67" s="11" t="s">
         <v>70</v>
       </c>
@@ -15107,7 +15866,7 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="13"/>
+      <c r="A68" s="14"/>
       <c r="B68" s="11" t="s">
         <v>71</v>
       </c>
@@ -15119,7 +15878,7 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="13"/>
+      <c r="A69" s="14"/>
       <c r="B69" s="11" t="s">
         <v>68</v>
       </c>
@@ -15132,7 +15891,7 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="13">
+      <c r="A70" s="14">
         <v>2041</v>
       </c>
       <c r="B70" s="11" t="s">
@@ -15146,7 +15905,7 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="13"/>
+      <c r="A71" s="14"/>
       <c r="B71" s="11" t="s">
         <v>70</v>
       </c>
@@ -15158,7 +15917,7 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="13"/>
+      <c r="A72" s="14"/>
       <c r="B72" s="11" t="s">
         <v>71</v>
       </c>
@@ -15170,7 +15929,7 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="13"/>
+      <c r="A73" s="14"/>
       <c r="B73" s="11" t="s">
         <v>68</v>
       </c>
@@ -15183,7 +15942,7 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="13">
+      <c r="A74" s="14">
         <v>2042</v>
       </c>
       <c r="B74" s="11" t="s">
@@ -15197,7 +15956,7 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="13"/>
+      <c r="A75" s="14"/>
       <c r="B75" s="11" t="s">
         <v>70</v>
       </c>
@@ -15209,7 +15968,7 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="13"/>
+      <c r="A76" s="14"/>
       <c r="B76" s="11" t="s">
         <v>71</v>
       </c>
@@ -15221,7 +15980,7 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="13"/>
+      <c r="A77" s="14"/>
       <c r="B77" s="11" t="s">
         <v>68</v>
       </c>
@@ -15234,7 +15993,7 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="13">
+      <c r="A78" s="14">
         <v>2043</v>
       </c>
       <c r="B78" s="11" t="s">
@@ -15248,7 +16007,7 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="13"/>
+      <c r="A79" s="14"/>
       <c r="B79" s="11" t="s">
         <v>70</v>
       </c>
@@ -15260,7 +16019,7 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="13"/>
+      <c r="A80" s="14"/>
       <c r="B80" s="11" t="s">
         <v>71</v>
       </c>
@@ -15272,7 +16031,7 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="13"/>
+      <c r="A81" s="14"/>
       <c r="B81" s="11" t="s">
         <v>68</v>
       </c>
@@ -15285,7 +16044,7 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="13">
+      <c r="A82" s="14">
         <v>2044</v>
       </c>
       <c r="B82" s="11" t="s">
@@ -15299,7 +16058,7 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="13"/>
+      <c r="A83" s="14"/>
       <c r="B83" s="11" t="s">
         <v>70</v>
       </c>
@@ -15311,7 +16070,7 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="13"/>
+      <c r="A84" s="14"/>
       <c r="B84" s="11" t="s">
         <v>71</v>
       </c>
@@ -15323,7 +16082,7 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="13"/>
+      <c r="A85" s="14"/>
       <c r="B85" s="11" t="s">
         <v>68</v>
       </c>
@@ -15336,7 +16095,7 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="13">
+      <c r="A86" s="14">
         <v>2045</v>
       </c>
       <c r="B86" s="11" t="s">
@@ -15350,7 +16109,7 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="13"/>
+      <c r="A87" s="14"/>
       <c r="B87" s="11" t="s">
         <v>70</v>
       </c>
@@ -15362,7 +16121,7 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="13"/>
+      <c r="A88" s="14"/>
       <c r="B88" s="11" t="s">
         <v>71</v>
       </c>
@@ -15374,7 +16133,7 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="13"/>
+      <c r="A89" s="14"/>
       <c r="B89" s="11" t="s">
         <v>68</v>
       </c>
@@ -15387,7 +16146,7 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="13">
+      <c r="A90" s="14">
         <v>2046</v>
       </c>
       <c r="B90" s="11" t="s">
@@ -15401,7 +16160,7 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="13"/>
+      <c r="A91" s="14"/>
       <c r="B91" s="11" t="s">
         <v>70</v>
       </c>
@@ -15413,7 +16172,7 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="13"/>
+      <c r="A92" s="14"/>
       <c r="B92" s="11" t="s">
         <v>71</v>
       </c>
@@ -15425,7 +16184,7 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="13"/>
+      <c r="A93" s="14"/>
       <c r="B93" s="11" t="s">
         <v>68</v>
       </c>
@@ -15438,7 +16197,7 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="13">
+      <c r="A94" s="14">
         <v>2047</v>
       </c>
       <c r="B94" s="11" t="s">
@@ -15452,7 +16211,7 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="13"/>
+      <c r="A95" s="14"/>
       <c r="B95" s="11" t="s">
         <v>70</v>
       </c>
@@ -15464,7 +16223,7 @@
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="13"/>
+      <c r="A96" s="14"/>
       <c r="B96" s="11" t="s">
         <v>71</v>
       </c>
@@ -15476,7 +16235,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="13"/>
+      <c r="A97" s="14"/>
       <c r="B97" s="11" t="s">
         <v>68</v>
       </c>
@@ -15489,7 +16248,7 @@
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="13">
+      <c r="A98" s="14">
         <v>2048</v>
       </c>
       <c r="B98" s="11" t="s">
@@ -15503,7 +16262,7 @@
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" s="13"/>
+      <c r="A99" s="14"/>
       <c r="B99" s="11" t="s">
         <v>70</v>
       </c>
@@ -15515,7 +16274,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="13"/>
+      <c r="A100" s="14"/>
       <c r="B100" s="11" t="s">
         <v>71</v>
       </c>
@@ -15527,7 +16286,7 @@
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" s="13"/>
+      <c r="A101" s="14"/>
       <c r="B101" s="11" t="s">
         <v>68</v>
       </c>
@@ -15540,7 +16299,7 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" s="13">
+      <c r="A102" s="14">
         <v>2049</v>
       </c>
       <c r="B102" s="11" t="s">
@@ -15554,7 +16313,7 @@
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A103" s="13"/>
+      <c r="A103" s="14"/>
       <c r="B103" s="11" t="s">
         <v>70</v>
       </c>
@@ -15566,7 +16325,7 @@
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="13"/>
+      <c r="A104" s="14"/>
       <c r="B104" s="11" t="s">
         <v>71</v>
       </c>
@@ -15578,7 +16337,7 @@
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="13"/>
+      <c r="A105" s="14"/>
       <c r="B105" s="11" t="s">
         <v>68</v>
       </c>
@@ -15591,7 +16350,7 @@
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" s="13">
+      <c r="A106" s="14">
         <v>2050</v>
       </c>
       <c r="B106" s="11" t="s">
@@ -15605,7 +16364,7 @@
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" s="13"/>
+      <c r="A107" s="14"/>
       <c r="B107" s="11" t="s">
         <v>70</v>
       </c>
@@ -15617,7 +16376,7 @@
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" s="13"/>
+      <c r="A108" s="14"/>
       <c r="B108" s="11" t="s">
         <v>71</v>
       </c>
@@ -15629,7 +16388,7 @@
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" s="13"/>
+      <c r="A109" s="14"/>
       <c r="B109" s="11" t="s">
         <v>68</v>
       </c>

</xml_diff>

<commit_message>
Refactors material processing and scrap handling
Updates the constraints and variables related to material processing and scrap handling capacities.

Check Polysilicon! High Manufacturing bu t dissapears somewhere.

This involves:
- Replacing factory-based capacity with processing-based capacity for better modularity.
- Introduces new constraints for scrap handling capacity to manage scrap recycling more effectively.
- Adds growth limits to processing and scrap handling capacities, enabling a more realistic simulation of capacity expansion.
- Simplifies stock management by using 2024 as the base year.
- Modifies objective function calculation with new capacity constraints.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-extension/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="605" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60C394FD-8E8C-4C4C-A2B5-938D74E72AFF}"/>
+  <xr:revisionPtr revIDLastSave="613" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77662A64-A8E0-4D4A-B470-EAA904996A10}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="12" activeTab="14" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="9" activeTab="18" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -1506,6 +1506,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FA1A697-84AA-4F97-BE70-81695B57512E}">
   <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="12" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -12517,13 +12520,13 @@
         <v>38640</v>
       </c>
       <c r="C2">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D2">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E2">
-        <v>250240</v>
+        <v>165600</v>
       </c>
       <c r="F2">
         <v>9999999</v>
@@ -12561,16 +12564,16 @@
         <v>2025</v>
       </c>
       <c r="B3">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C3">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D3">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E3">
-        <v>246486.39999999999</v>
+        <v>165600</v>
       </c>
       <c r="F3">
         <v>9999999</v>
@@ -12608,16 +12611,16 @@
         <v>2026</v>
       </c>
       <c r="B4">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C4">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D4">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E4">
-        <v>242789.10399999999</v>
+        <v>165600</v>
       </c>
       <c r="F4">
         <v>9999999</v>
@@ -12655,16 +12658,16 @@
         <v>2027</v>
       </c>
       <c r="B5">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C5">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D5">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E5">
-        <v>239147.26740000001</v>
+        <v>165600</v>
       </c>
       <c r="F5">
         <v>9999999</v>
@@ -12702,16 +12705,16 @@
         <v>2028</v>
       </c>
       <c r="B6">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C6">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D6">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E6">
-        <v>235560.05840000001</v>
+        <v>165600</v>
       </c>
       <c r="F6">
         <v>9999999</v>
@@ -12749,16 +12752,16 @@
         <v>2029</v>
       </c>
       <c r="B7">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C7">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D7">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E7">
-        <v>232026.65760000001</v>
+        <v>165600</v>
       </c>
       <c r="F7">
         <v>9999999</v>
@@ -12796,16 +12799,16 @@
         <v>2030</v>
       </c>
       <c r="B8">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C8">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D8">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E8">
-        <v>228546.25769999999</v>
+        <v>165600</v>
       </c>
       <c r="F8">
         <v>9999999</v>
@@ -12843,16 +12846,16 @@
         <v>2031</v>
       </c>
       <c r="B9">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C9">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D9">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E9">
-        <v>225118.0638</v>
+        <v>165600</v>
       </c>
       <c r="F9">
         <v>9999999</v>
@@ -12890,16 +12893,16 @@
         <v>2032</v>
       </c>
       <c r="B10">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C10">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D10">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E10">
-        <v>221741.2929</v>
+        <v>165600</v>
       </c>
       <c r="F10">
         <v>9999999</v>
@@ -12937,16 +12940,16 @@
         <v>2033</v>
       </c>
       <c r="B11">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C11">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D11">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E11">
-        <v>218415.1735</v>
+        <v>165600</v>
       </c>
       <c r="F11">
         <v>9999999</v>
@@ -12984,16 +12987,16 @@
         <v>2034</v>
       </c>
       <c r="B12">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C12">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D12">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E12">
-        <v>215138.94589999999</v>
+        <v>165600</v>
       </c>
       <c r="F12">
         <v>9999999</v>
@@ -13031,16 +13034,16 @@
         <v>2035</v>
       </c>
       <c r="B13">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C13">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D13">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E13">
-        <v>211911.86170000001</v>
+        <v>165600</v>
       </c>
       <c r="F13">
         <v>9999999</v>
@@ -13078,16 +13081,16 @@
         <v>2036</v>
       </c>
       <c r="B14">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C14">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D14">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E14">
-        <v>208733.1838</v>
+        <v>165600</v>
       </c>
       <c r="F14">
         <v>9999999</v>
@@ -13125,16 +13128,16 @@
         <v>2037</v>
       </c>
       <c r="B15">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C15">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D15">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E15">
-        <v>205602.18599999999</v>
+        <v>165600</v>
       </c>
       <c r="F15">
         <v>9999999</v>
@@ -13172,16 +13175,16 @@
         <v>2038</v>
       </c>
       <c r="B16">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C16">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D16">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E16">
-        <v>202518.1532</v>
+        <v>165600</v>
       </c>
       <c r="F16">
         <v>9999999</v>
@@ -13219,16 +13222,16 @@
         <v>2039</v>
       </c>
       <c r="B17">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C17">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D17">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E17">
-        <v>199480.38089999999</v>
+        <v>165600</v>
       </c>
       <c r="F17">
         <v>9999999</v>
@@ -13266,16 +13269,16 @@
         <v>2040</v>
       </c>
       <c r="B18">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C18">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D18">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E18">
-        <v>196488.1752</v>
+        <v>165600</v>
       </c>
       <c r="F18">
         <v>9999999</v>
@@ -13313,16 +13316,16 @@
         <v>2041</v>
       </c>
       <c r="B19">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C19">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D19">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E19">
-        <v>193540.85260000001</v>
+        <v>165600</v>
       </c>
       <c r="F19">
         <v>9999999</v>
@@ -13360,16 +13363,16 @@
         <v>2042</v>
       </c>
       <c r="B20">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C20">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D20">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E20">
-        <v>190637.73980000001</v>
+        <v>165600</v>
       </c>
       <c r="F20">
         <v>9999999</v>
@@ -13407,16 +13410,16 @@
         <v>2043</v>
       </c>
       <c r="B21">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C21">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D21">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E21">
-        <v>187778.17370000001</v>
+        <v>165600</v>
       </c>
       <c r="F21">
         <v>9999999</v>
@@ -13454,16 +13457,16 @@
         <v>2044</v>
       </c>
       <c r="B22">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C22">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D22">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E22">
-        <v>184961.50109999999</v>
+        <v>165600</v>
       </c>
       <c r="F22">
         <v>9999999</v>
@@ -13501,16 +13504,16 @@
         <v>2045</v>
       </c>
       <c r="B23">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C23">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D23">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E23">
-        <v>182187.07860000001</v>
+        <v>165600</v>
       </c>
       <c r="F23">
         <v>9999999</v>
@@ -13548,16 +13551,16 @@
         <v>2046</v>
       </c>
       <c r="B24">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C24">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D24">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E24">
-        <v>179454.27239999999</v>
+        <v>165600</v>
       </c>
       <c r="F24">
         <v>9999999</v>
@@ -13595,16 +13598,16 @@
         <v>2047</v>
       </c>
       <c r="B25">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C25">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D25">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E25">
-        <v>176762.4583</v>
+        <v>165600</v>
       </c>
       <c r="F25">
         <v>9999999</v>
@@ -13642,16 +13645,16 @@
         <v>2048</v>
       </c>
       <c r="B26">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C26">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D26">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E26">
-        <v>174111.0214</v>
+        <v>165600</v>
       </c>
       <c r="F26">
         <v>9999999</v>
@@ -13689,16 +13692,16 @@
         <v>2049</v>
       </c>
       <c r="B27">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C27">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D27">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E27">
-        <v>171499.3561</v>
+        <v>165600</v>
       </c>
       <c r="F27">
         <v>9999999</v>
@@ -13736,16 +13739,16 @@
         <v>2050</v>
       </c>
       <c r="B28">
-        <v>9999999</v>
+        <v>38640</v>
       </c>
       <c r="C28">
-        <v>9999999</v>
+        <v>55200</v>
       </c>
       <c r="D28">
-        <v>9999999</v>
+        <v>82800</v>
       </c>
       <c r="E28">
-        <v>168926.8658</v>
+        <v>165600</v>
       </c>
       <c r="F28">
         <v>9999999</v>
@@ -25550,6 +25553,26 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -25557,26 +25580,6 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implements soft NZIA target with penalty
Implements a soft target for the NZIA constraint, allowing for shortfalls in domestic production.

Adds a penalty cost to the opex calculation based on the magnitude of the shortfall, incentivizing the model to meet the domestic production target where possible.

Initializes `stock_imported_init` with solarPV stock data.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-extension/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="613" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77662A64-A8E0-4D4A-B470-EAA904996A10}"/>
+  <xr:revisionPtr revIDLastSave="627" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CCA5427-6049-44BF-9AE3-CCDE81E7DAB2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="9" activeTab="18" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="38280" yWindow="-1710" windowWidth="38640" windowHeight="21120" firstSheet="5" activeTab="13" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -4329,67 +4329,67 @@
         <v>2024</v>
       </c>
       <c r="B2">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C2">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D2">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E2">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F2">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N2">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O2">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U2">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V2">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
@@ -4397,67 +4397,67 @@
         <v>2025</v>
       </c>
       <c r="B3">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C3">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D3">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E3">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F3">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N3">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O3">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U3">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V3">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
@@ -4465,67 +4465,67 @@
         <v>2026</v>
       </c>
       <c r="B4">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C4">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D4">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E4">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F4">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H4">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N4">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O4">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U4">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V4">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
@@ -4533,67 +4533,67 @@
         <v>2027</v>
       </c>
       <c r="B5">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C5">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D5">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E5">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F5">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N5">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O5">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U5">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V5">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
@@ -4601,67 +4601,67 @@
         <v>2028</v>
       </c>
       <c r="B6">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C6">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D6">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E6">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F6">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N6">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O6">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U6">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V6">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
@@ -4669,67 +4669,67 @@
         <v>2029</v>
       </c>
       <c r="B7">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C7">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D7">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E7">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F7">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G7">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H7">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N7">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O7">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U7">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V7">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
@@ -4737,67 +4737,67 @@
         <v>2030</v>
       </c>
       <c r="B8">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C8">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D8">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E8">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F8">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G8">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H8">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N8">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O8">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U8">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V8">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
@@ -4805,67 +4805,67 @@
         <v>2031</v>
       </c>
       <c r="B9">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C9">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D9">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E9">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F9">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H9">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N9">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O9">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U9">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V9">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.25">
@@ -4873,67 +4873,67 @@
         <v>2032</v>
       </c>
       <c r="B10">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C10">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D10">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E10">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F10">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G10">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H10">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N10">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O10">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U10">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V10">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
@@ -4941,67 +4941,67 @@
         <v>2033</v>
       </c>
       <c r="B11">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C11">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D11">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E11">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F11">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G11">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N11">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O11">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U11">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V11">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.25">
@@ -5009,67 +5009,67 @@
         <v>2034</v>
       </c>
       <c r="B12">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C12">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D12">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E12">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F12">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N12">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O12">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U12">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V12">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.25">
@@ -5077,67 +5077,67 @@
         <v>2035</v>
       </c>
       <c r="B13">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C13">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D13">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E13">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F13">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H13">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N13">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O13">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U13">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V13">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.25">
@@ -5145,67 +5145,67 @@
         <v>2036</v>
       </c>
       <c r="B14">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C14">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D14">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E14">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F14">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G14">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H14">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N14">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O14">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U14">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V14">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
@@ -5213,67 +5213,67 @@
         <v>2037</v>
       </c>
       <c r="B15">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C15">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D15">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E15">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F15">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G15">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N15">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O15">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U15">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V15">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
@@ -5281,67 +5281,67 @@
         <v>2038</v>
       </c>
       <c r="B16">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C16">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D16">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E16">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F16">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H16">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N16">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O16">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U16">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V16">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
@@ -5349,67 +5349,67 @@
         <v>2039</v>
       </c>
       <c r="B17">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C17">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D17">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E17">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F17">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G17">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N17">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O17">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U17">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V17">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.25">
@@ -5417,67 +5417,67 @@
         <v>2040</v>
       </c>
       <c r="B18">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C18">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D18">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E18">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F18">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G18">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H18">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N18">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O18">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U18">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V18">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.25">
@@ -5485,67 +5485,67 @@
         <v>2041</v>
       </c>
       <c r="B19">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C19">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D19">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E19">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F19">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G19">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H19">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N19">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O19">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U19">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V19">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.25">
@@ -5553,67 +5553,67 @@
         <v>2042</v>
       </c>
       <c r="B20">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C20">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D20">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E20">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F20">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G20">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H20">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N20">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O20">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U20">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V20">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.25">
@@ -5621,67 +5621,67 @@
         <v>2043</v>
       </c>
       <c r="B21">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C21">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D21">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E21">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F21">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G21">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H21">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N21">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O21">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U21">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V21">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.25">
@@ -5689,67 +5689,67 @@
         <v>2044</v>
       </c>
       <c r="B22">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C22">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D22">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E22">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F22">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H22">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N22">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O22">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U22">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V22">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.25">
@@ -5757,67 +5757,67 @@
         <v>2045</v>
       </c>
       <c r="B23">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C23">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D23">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E23">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F23">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G23">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H23">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N23">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O23">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U23">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V23">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
@@ -5825,67 +5825,67 @@
         <v>2046</v>
       </c>
       <c r="B24">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C24">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D24">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E24">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F24">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H24">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N24">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O24">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U24">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V24">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.25">
@@ -5893,67 +5893,67 @@
         <v>2047</v>
       </c>
       <c r="B25">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C25">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D25">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E25">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F25">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G25">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H25">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N25">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O25">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U25">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V25">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.25">
@@ -5961,67 +5961,67 @@
         <v>2048</v>
       </c>
       <c r="B26">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C26">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D26">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E26">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F26">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G26">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H26">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N26">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O26">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U26">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V26">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.25">
@@ -6029,67 +6029,67 @@
         <v>2049</v>
       </c>
       <c r="B27">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C27">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D27">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E27">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F27">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G27">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H27">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N27">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O27">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U27">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V27">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.25">
@@ -6097,67 +6097,67 @@
         <v>2050</v>
       </c>
       <c r="B28">
-        <v>650000</v>
+        <v>83.72</v>
       </c>
       <c r="C28">
-        <v>100</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D28">
-        <v>3000</v>
+        <v>2540000</v>
       </c>
       <c r="E28">
-        <v>600</v>
+        <v>2484</v>
       </c>
       <c r="F28">
-        <v>8000</v>
+        <v>1</v>
       </c>
       <c r="G28">
-        <v>40000</v>
+        <v>1</v>
       </c>
       <c r="H28">
-        <v>15000</v>
+        <v>1</v>
       </c>
       <c r="I28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="J28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="K28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="L28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="M28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="N28">
-        <v>30000</v>
+        <v>1800</v>
       </c>
       <c r="O28">
-        <v>30000</v>
+        <v>6800</v>
       </c>
       <c r="P28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="Q28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="R28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="S28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="T28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="U28">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="V28">
-        <v>30000</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -6243,67 +6243,67 @@
         <v>2024</v>
       </c>
       <c r="B2">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C2">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D2">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E2">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F2">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N2">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O2">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U2">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V2">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
@@ -6311,67 +6311,67 @@
         <v>2025</v>
       </c>
       <c r="B3">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C3">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D3">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E3">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F3">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N3">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O3">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U3">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V3">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
@@ -6379,67 +6379,67 @@
         <v>2026</v>
       </c>
       <c r="B4">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C4">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D4">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E4">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F4">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H4">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N4">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O4">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U4">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V4">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
@@ -6447,67 +6447,67 @@
         <v>2027</v>
       </c>
       <c r="B5">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C5">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D5">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E5">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F5">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N5">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O5">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U5">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V5">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
@@ -6515,67 +6515,67 @@
         <v>2028</v>
       </c>
       <c r="B6">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C6">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D6">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E6">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F6">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N6">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O6">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U6">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V6">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
@@ -6583,67 +6583,67 @@
         <v>2029</v>
       </c>
       <c r="B7">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C7">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D7">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E7">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F7">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G7">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H7">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N7">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O7">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U7">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V7">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
@@ -6651,67 +6651,67 @@
         <v>2030</v>
       </c>
       <c r="B8">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C8">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D8">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E8">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F8">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G8">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H8">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N8">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O8">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U8">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V8">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
@@ -6719,67 +6719,67 @@
         <v>2031</v>
       </c>
       <c r="B9">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C9">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D9">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E9">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F9">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H9">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N9">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O9">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U9">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V9">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.25">
@@ -6787,67 +6787,67 @@
         <v>2032</v>
       </c>
       <c r="B10">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C10">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D10">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E10">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F10">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G10">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H10">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N10">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O10">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U10">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V10">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
@@ -6855,67 +6855,67 @@
         <v>2033</v>
       </c>
       <c r="B11">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C11">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D11">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E11">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F11">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G11">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N11">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O11">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U11">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V11">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.25">
@@ -6923,67 +6923,67 @@
         <v>2034</v>
       </c>
       <c r="B12">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C12">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D12">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E12">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F12">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N12">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O12">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U12">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V12">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.25">
@@ -6991,67 +6991,67 @@
         <v>2035</v>
       </c>
       <c r="B13">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C13">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D13">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E13">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F13">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H13">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N13">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O13">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U13">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V13">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.25">
@@ -7059,67 +7059,67 @@
         <v>2036</v>
       </c>
       <c r="B14">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C14">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D14">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E14">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F14">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G14">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H14">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N14">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O14">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U14">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V14">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
@@ -7127,67 +7127,67 @@
         <v>2037</v>
       </c>
       <c r="B15">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C15">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D15">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E15">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F15">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G15">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N15">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O15">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U15">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V15">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
@@ -7195,67 +7195,67 @@
         <v>2038</v>
       </c>
       <c r="B16">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C16">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D16">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E16">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F16">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H16">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N16">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O16">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U16">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V16">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
@@ -7263,67 +7263,67 @@
         <v>2039</v>
       </c>
       <c r="B17">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C17">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D17">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E17">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F17">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G17">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N17">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O17">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U17">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V17">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.25">
@@ -7331,67 +7331,67 @@
         <v>2040</v>
       </c>
       <c r="B18">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C18">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D18">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E18">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F18">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G18">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H18">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N18">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O18">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U18">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V18">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.25">
@@ -7399,67 +7399,67 @@
         <v>2041</v>
       </c>
       <c r="B19">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C19">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D19">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E19">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F19">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G19">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H19">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N19">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O19">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U19">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V19">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.25">
@@ -7467,67 +7467,67 @@
         <v>2042</v>
       </c>
       <c r="B20">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C20">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D20">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E20">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F20">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G20">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H20">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N20">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O20">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U20">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V20">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.25">
@@ -7535,67 +7535,67 @@
         <v>2043</v>
       </c>
       <c r="B21">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C21">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D21">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E21">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F21">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G21">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H21">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N21">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O21">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U21">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V21">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.25">
@@ -7603,67 +7603,67 @@
         <v>2044</v>
       </c>
       <c r="B22">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C22">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D22">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E22">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F22">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H22">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N22">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O22">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U22">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V22">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.25">
@@ -7671,67 +7671,67 @@
         <v>2045</v>
       </c>
       <c r="B23">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C23">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D23">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E23">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F23">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G23">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H23">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N23">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O23">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U23">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V23">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
@@ -7739,67 +7739,67 @@
         <v>2046</v>
       </c>
       <c r="B24">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C24">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D24">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E24">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F24">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H24">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N24">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O24">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U24">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V24">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.25">
@@ -7807,67 +7807,67 @@
         <v>2047</v>
       </c>
       <c r="B25">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C25">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D25">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E25">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F25">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G25">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H25">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N25">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O25">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U25">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V25">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.25">
@@ -7875,67 +7875,67 @@
         <v>2048</v>
       </c>
       <c r="B26">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C26">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D26">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E26">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F26">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G26">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H26">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N26">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O26">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U26">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V26">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.25">
@@ -7943,67 +7943,67 @@
         <v>2049</v>
       </c>
       <c r="B27">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C27">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D27">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E27">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F27">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G27">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H27">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N27">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O27">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U27">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V27">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.25">
@@ -8011,67 +8011,67 @@
         <v>2050</v>
       </c>
       <c r="B28">
-        <v>700000</v>
+        <v>83.72</v>
       </c>
       <c r="C28">
-        <v>150</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D28">
-        <v>3500</v>
+        <v>2540000</v>
       </c>
       <c r="E28">
-        <v>800</v>
+        <v>2484</v>
       </c>
       <c r="F28">
-        <v>9500</v>
+        <v>1</v>
       </c>
       <c r="G28">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="H28">
-        <v>18000</v>
+        <v>1</v>
       </c>
       <c r="I28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="J28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="K28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="L28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="M28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="N28">
-        <v>35000</v>
+        <v>1800</v>
       </c>
       <c r="O28">
-        <v>35000</v>
+        <v>6800</v>
       </c>
       <c r="P28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="Q28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="R28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="S28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="T28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="U28">
-        <v>35000</v>
+        <v>1</v>
       </c>
       <c r="V28">
-        <v>35000</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds energy demand and scenario constraints
Implements a factory energy demand calculation and distribution rule for more accurate energy consumption modeling.
Introduces scenario constraints for NZIA (Net-Zero Industry Act) and CRMA (Critical Raw Materials Act) compliance, allowing for flexible configuration via parameters.
Adds option to configure constraints as strict or flexible.
The holding cost for stockpiled materials was increased.
Fixes a bug related to price reduction calculation for single technologies.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-extension/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="688" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF99B2D8-6013-44D2-BC0C-7C6E7DC34F3E}"/>
+  <xr:revisionPtr revIDLastSave="693" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AD85F33-426E-44BB-A093-4FD93EDE6565}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" firstSheet="7" activeTab="13" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="38280" yWindow="-1710" windowWidth="38640" windowHeight="21120" firstSheet="7" activeTab="12" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -707,7 +707,7 @@
     </xf>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -743,10 +743,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -1690,13 +1686,13 @@
       <c r="C9" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9">
         <v>0.94859999999999989</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9">
         <v>0.94859999999999989</v>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1710,13 +1706,13 @@
       <c r="C10" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10">
         <v>6.9563999999999995</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10">
         <v>6.9563999999999995</v>
       </c>
-      <c r="F10" s="17">
+      <c r="F10" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1730,13 +1726,13 @@
       <c r="C11" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11">
         <v>1.17E-3</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11">
         <v>1.17E-3</v>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1750,13 +1746,13 @@
       <c r="C12" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12">
         <v>8.1</v>
       </c>
-      <c r="E12" s="16">
+      <c r="E12">
         <v>8.1</v>
       </c>
-      <c r="F12" s="17">
+      <c r="F12" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1770,13 +1766,13 @@
       <c r="C13" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="D13" s="16">
+      <c r="D13">
         <v>114.72499999999999</v>
       </c>
-      <c r="E13" s="16">
+      <c r="E13">
         <v>114.72499999999999</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="9" t="s">
         <v>148</v>
       </c>
     </row>
@@ -1790,13 +1786,13 @@
       <c r="C14" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14">
         <v>5.5</v>
       </c>
-      <c r="E14" s="16">
+      <c r="E14">
         <v>5.5</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="9" t="s">
         <v>149</v>
       </c>
     </row>
@@ -1810,13 +1806,13 @@
       <c r="C15" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15">
         <v>5.47E-3</v>
       </c>
-      <c r="E15" s="16">
+      <c r="E15">
         <v>5.47E-3</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1830,13 +1826,13 @@
       <c r="C16" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16">
         <v>4.7689999999999996E-2</v>
       </c>
-      <c r="E16" s="16">
+      <c r="E16">
         <v>4.7689999999999996E-2</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1850,13 +1846,13 @@
       <c r="C17" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17">
         <v>7.2699999999999996E-3</v>
       </c>
-      <c r="E17" s="16">
+      <c r="E17">
         <v>7.2699999999999996E-3</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1870,13 +1866,13 @@
       <c r="C18" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="D18" s="16">
+      <c r="D18">
         <v>2.7909999999999999</v>
       </c>
-      <c r="E18" s="16">
+      <c r="E18">
         <v>2.7909999999999999</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="9" t="s">
         <v>148</v>
       </c>
     </row>
@@ -1890,13 +1886,13 @@
       <c r="C19" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="D19" s="16">
+      <c r="D19">
         <v>2.2925</v>
       </c>
-      <c r="E19" s="16">
+      <c r="E19">
         <v>2.2925</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="9" t="s">
         <v>148</v>
       </c>
     </row>
@@ -1910,13 +1906,13 @@
       <c r="C20" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="D20" s="16">
+      <c r="D20">
         <v>18.945</v>
       </c>
-      <c r="E20" s="16">
+      <c r="E20">
         <v>18.945</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1930,13 +1926,13 @@
       <c r="C21" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="D21" s="16">
+      <c r="D21">
         <v>0.78549999999999998</v>
       </c>
-      <c r="E21" s="16">
+      <c r="E21">
         <v>0.78549999999999998</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="F21" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1950,13 +1946,13 @@
       <c r="C22" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22">
         <v>0.1045</v>
       </c>
-      <c r="E22" s="16">
+      <c r="E22">
         <v>0.1045</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1970,13 +1966,13 @@
       <c r="C23" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23">
         <v>0.39200000000000002</v>
       </c>
-      <c r="E23" s="16">
+      <c r="E23">
         <v>0.39200000000000002</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F23" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1990,13 +1986,13 @@
       <c r="C24" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D24">
         <v>0.50024999999999997</v>
       </c>
-      <c r="E24" s="16">
+      <c r="E24">
         <v>0.50024999999999997</v>
       </c>
-      <c r="F24" s="17" t="s">
+      <c r="F24" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2010,13 +2006,13 @@
       <c r="C25" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="D25" s="16">
+      <c r="D25">
         <v>0.97139999999999993</v>
       </c>
-      <c r="E25" s="16">
+      <c r="E25">
         <v>0.97139999999999993</v>
       </c>
-      <c r="F25" s="17">
+      <c r="F25" s="9">
         <v>0</v>
       </c>
     </row>
@@ -2030,13 +2026,13 @@
       <c r="C26" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="D26" s="16">
+      <c r="D26">
         <v>7.1236000000000006</v>
       </c>
-      <c r="E26" s="16">
+      <c r="E26">
         <v>7.1236000000000006</v>
       </c>
-      <c r="F26" s="17">
+      <c r="F26" s="9">
         <v>0</v>
       </c>
     </row>
@@ -2050,13 +2046,13 @@
       <c r="C27" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="D27" s="16">
+      <c r="D27">
         <v>3.4500000000000004E-3</v>
       </c>
-      <c r="E27" s="16">
+      <c r="E27">
         <v>3.4500000000000004E-3</v>
       </c>
-      <c r="F27" s="17">
+      <c r="F27" s="9">
         <v>0</v>
       </c>
     </row>
@@ -2070,13 +2066,13 @@
       <c r="C28" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="D28" s="16">
+      <c r="D28">
         <v>11.6</v>
       </c>
-      <c r="E28" s="16">
+      <c r="E28">
         <v>11.6</v>
       </c>
-      <c r="F28" s="17">
+      <c r="F28" s="9">
         <v>0</v>
       </c>
     </row>
@@ -2090,13 +2086,13 @@
       <c r="C29" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="D29" s="16">
+      <c r="D29">
         <v>116.77</v>
       </c>
-      <c r="E29" s="16">
+      <c r="E29">
         <v>116.77</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="F29" s="9" t="s">
         <v>148</v>
       </c>
     </row>
@@ -2110,13 +2106,13 @@
       <c r="C30" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30">
         <v>5.5</v>
       </c>
-      <c r="E30" s="16">
+      <c r="E30">
         <v>5.5</v>
       </c>
-      <c r="F30" s="17" t="s">
+      <c r="F30" s="9" t="s">
         <v>149</v>
       </c>
     </row>
@@ -2130,13 +2126,13 @@
       <c r="C31" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="D31" s="16">
+      <c r="D31">
         <v>1.1259999999999999E-2</v>
       </c>
-      <c r="E31" s="16">
+      <c r="E31">
         <v>1.1259999999999999E-2</v>
       </c>
-      <c r="F31" s="17" t="s">
+      <c r="F31" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2150,13 +2146,13 @@
       <c r="C32" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="D32" s="16">
+      <c r="D32">
         <v>0.11219</v>
       </c>
-      <c r="E32" s="16">
+      <c r="E32">
         <v>0.11219</v>
       </c>
-      <c r="F32" s="17" t="s">
+      <c r="F32" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2170,13 +2166,13 @@
       <c r="C33" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="D33" s="16">
+      <c r="D33">
         <v>2.0460000000000002E-2</v>
       </c>
-      <c r="E33" s="16">
+      <c r="E33">
         <v>2.0460000000000002E-2</v>
       </c>
-      <c r="F33" s="17" t="s">
+      <c r="F33" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2190,13 +2186,13 @@
       <c r="C34" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="D34" s="16">
+      <c r="D34">
         <v>4.04</v>
       </c>
-      <c r="E34" s="16">
+      <c r="E34">
         <v>4.04</v>
       </c>
-      <c r="F34" s="17" t="s">
+      <c r="F34" s="9" t="s">
         <v>148</v>
       </c>
     </row>
@@ -2210,13 +2206,13 @@
       <c r="C35" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="D35" s="16">
+      <c r="D35">
         <v>3.2574999999999998</v>
       </c>
-      <c r="E35" s="16">
+      <c r="E35">
         <v>3.2574999999999998</v>
       </c>
-      <c r="F35" s="17" t="s">
+      <c r="F35" s="9" t="s">
         <v>148</v>
       </c>
     </row>
@@ -2230,13 +2226,13 @@
       <c r="C36" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="D36" s="16">
+      <c r="D36">
         <v>19.89</v>
       </c>
-      <c r="E36" s="16">
+      <c r="E36">
         <v>19.89</v>
       </c>
-      <c r="F36" s="17" t="s">
+      <c r="F36" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2250,13 +2246,13 @@
       <c r="C37" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="D37" s="16">
+      <c r="D37">
         <v>0.79039999999999999</v>
       </c>
-      <c r="E37" s="16">
+      <c r="E37">
         <v>0.79039999999999999</v>
       </c>
-      <c r="F37" s="17" t="s">
+      <c r="F37" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2270,13 +2266,13 @@
       <c r="C38" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="D38" s="16">
+      <c r="D38">
         <v>0.10940000000000001</v>
       </c>
-      <c r="E38" s="16">
+      <c r="E38">
         <v>0.10940000000000001</v>
       </c>
-      <c r="F38" s="17" t="s">
+      <c r="F38" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2290,13 +2286,13 @@
       <c r="C39" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="D39" s="16">
+      <c r="D39">
         <v>0.32230000000000003</v>
       </c>
-      <c r="E39" s="16">
+      <c r="E39">
         <v>0.32230000000000003</v>
       </c>
-      <c r="F39" s="17" t="s">
+      <c r="F39" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2310,13 +2306,13 @@
       <c r="C40" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="D40" s="16">
+      <c r="D40">
         <v>0.5272</v>
       </c>
-      <c r="E40" s="16">
+      <c r="E40">
         <v>0.5272</v>
       </c>
-      <c r="F40" s="17" t="s">
+      <c r="F40" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -6285,28 +6281,28 @@
         <v>2484</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N2">
         <v>3135</v>
@@ -6315,25 +6311,25 @@
         <v>12905</v>
       </c>
       <c r="P2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V2">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
@@ -6353,28 +6349,28 @@
         <v>2484</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N3">
         <v>3135</v>
@@ -6383,25 +6379,25 @@
         <v>12905</v>
       </c>
       <c r="P3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V3">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
@@ -6421,28 +6417,28 @@
         <v>2484</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N4">
         <v>3135</v>
@@ -6451,25 +6447,25 @@
         <v>12905</v>
       </c>
       <c r="P4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V4">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
@@ -6489,28 +6485,28 @@
         <v>2484</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N5">
         <v>3135</v>
@@ -6519,25 +6515,25 @@
         <v>12905</v>
       </c>
       <c r="P5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V5">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
@@ -6557,28 +6553,28 @@
         <v>2484</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N6">
         <v>3135</v>
@@ -6587,25 +6583,25 @@
         <v>12905</v>
       </c>
       <c r="P6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V6">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
@@ -6625,28 +6621,28 @@
         <v>2484</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N7">
         <v>3135</v>
@@ -6655,25 +6651,25 @@
         <v>12905</v>
       </c>
       <c r="P7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V7">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
@@ -6693,28 +6689,28 @@
         <v>2484</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N8">
         <v>3135</v>
@@ -6723,25 +6719,25 @@
         <v>12905</v>
       </c>
       <c r="P8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V8">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
@@ -6761,28 +6757,28 @@
         <v>2484</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N9">
         <v>3135</v>
@@ -6791,25 +6787,25 @@
         <v>12905</v>
       </c>
       <c r="P9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V9">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.25">
@@ -6829,28 +6825,28 @@
         <v>2484</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N10">
         <v>3135</v>
@@ -6859,25 +6855,25 @@
         <v>12905</v>
       </c>
       <c r="P10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V10">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
@@ -6897,28 +6893,28 @@
         <v>2484</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N11">
         <v>3135</v>
@@ -6927,25 +6923,25 @@
         <v>12905</v>
       </c>
       <c r="P11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V11">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.25">
@@ -6965,28 +6961,28 @@
         <v>2484</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N12">
         <v>3135</v>
@@ -6995,25 +6991,25 @@
         <v>12905</v>
       </c>
       <c r="P12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V12">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.25">
@@ -7033,28 +7029,28 @@
         <v>2484</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N13">
         <v>3135</v>
@@ -7063,25 +7059,25 @@
         <v>12905</v>
       </c>
       <c r="P13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V13">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.25">
@@ -7101,28 +7097,28 @@
         <v>2484</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N14">
         <v>3135</v>
@@ -7131,25 +7127,25 @@
         <v>12905</v>
       </c>
       <c r="P14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V14">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
@@ -7169,28 +7165,28 @@
         <v>2484</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N15">
         <v>3135</v>
@@ -7199,25 +7195,25 @@
         <v>12905</v>
       </c>
       <c r="P15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V15">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
@@ -7237,28 +7233,28 @@
         <v>2484</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N16">
         <v>3135</v>
@@ -7267,25 +7263,25 @@
         <v>12905</v>
       </c>
       <c r="P16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V16">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
@@ -7305,28 +7301,28 @@
         <v>2484</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N17">
         <v>3135</v>
@@ -7335,25 +7331,25 @@
         <v>12905</v>
       </c>
       <c r="P17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V17">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.25">
@@ -7373,28 +7369,28 @@
         <v>2484</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N18">
         <v>3135</v>
@@ -7403,25 +7399,25 @@
         <v>12905</v>
       </c>
       <c r="P18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V18">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.25">
@@ -7441,28 +7437,28 @@
         <v>2484</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N19">
         <v>3135</v>
@@ -7471,25 +7467,25 @@
         <v>12905</v>
       </c>
       <c r="P19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V19">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.25">
@@ -7509,28 +7505,28 @@
         <v>2484</v>
       </c>
       <c r="F20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N20">
         <v>3135</v>
@@ -7539,25 +7535,25 @@
         <v>12905</v>
       </c>
       <c r="P20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V20">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.25">
@@ -7577,28 +7573,28 @@
         <v>2484</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N21">
         <v>3135</v>
@@ -7607,25 +7603,25 @@
         <v>12905</v>
       </c>
       <c r="P21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V21">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.25">
@@ -7645,28 +7641,28 @@
         <v>2484</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N22">
         <v>3135</v>
@@ -7675,25 +7671,25 @@
         <v>12905</v>
       </c>
       <c r="P22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V22">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.25">
@@ -7713,28 +7709,28 @@
         <v>2484</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N23">
         <v>3135</v>
@@ -7743,25 +7739,25 @@
         <v>12905</v>
       </c>
       <c r="P23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V23">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
@@ -7781,28 +7777,28 @@
         <v>2484</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N24">
         <v>3135</v>
@@ -7811,25 +7807,25 @@
         <v>12905</v>
       </c>
       <c r="P24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V24">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.25">
@@ -7849,28 +7845,28 @@
         <v>2484</v>
       </c>
       <c r="F25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N25">
         <v>3135</v>
@@ -7879,25 +7875,25 @@
         <v>12905</v>
       </c>
       <c r="P25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V25">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.25">
@@ -7917,28 +7913,28 @@
         <v>2484</v>
       </c>
       <c r="F26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N26">
         <v>3135</v>
@@ -7947,25 +7943,25 @@
         <v>12905</v>
       </c>
       <c r="P26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V26">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.25">
@@ -7985,28 +7981,28 @@
         <v>2484</v>
       </c>
       <c r="F27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N27">
         <v>3135</v>
@@ -8015,25 +8011,25 @@
         <v>12905</v>
       </c>
       <c r="P27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V27">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.25">
@@ -8053,28 +8049,28 @@
         <v>2484</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="G28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="H28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="J28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="K28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="L28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="M28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="N28">
         <v>3135</v>
@@ -8083,25 +8079,25 @@
         <v>12905</v>
       </c>
       <c r="P28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="Q28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="R28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="S28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="T28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="U28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
       <c r="V28">
-        <v>1</v>
+        <v>9999999</v>
       </c>
     </row>
   </sheetData>
@@ -12267,13 +12263,13 @@
       <c r="D6" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6">
         <v>73600</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6">
         <v>20976.000000000007</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6">
         <v>3680.0000000000009</v>
       </c>
     </row>
@@ -12290,13 +12286,13 @@
       <c r="D7" t="s">
         <v>90</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7">
         <v>82800</v>
       </c>
-      <c r="F7" s="16">
+      <c r="F7">
         <v>7866</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7">
         <v>4140</v>
       </c>
     </row>
@@ -12313,13 +12309,13 @@
       <c r="D8" t="s">
         <v>92</v>
       </c>
-      <c r="E8" s="16">
+      <c r="E8">
         <v>276000</v>
       </c>
-      <c r="F8" s="16">
+      <c r="F8">
         <v>26220</v>
       </c>
-      <c r="G8" s="16">
+      <c r="G8">
         <v>13800</v>
       </c>
     </row>
@@ -12336,13 +12332,13 @@
       <c r="D9" t="s">
         <v>102</v>
       </c>
-      <c r="E9" s="16">
-        <v>1</v>
-      </c>
-      <c r="F9" s="16">
-        <v>1</v>
-      </c>
-      <c r="G9" s="16">
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
         <v>1</v>
       </c>
     </row>
@@ -12359,13 +12355,13 @@
       <c r="D10" t="s">
         <v>89</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10">
         <v>165600</v>
       </c>
-      <c r="F10" s="16">
+      <c r="F10">
         <v>47196</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10">
         <v>8280</v>
       </c>
     </row>
@@ -12382,13 +12378,13 @@
       <c r="D11" t="s">
         <v>90</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11">
         <v>202400</v>
       </c>
-      <c r="F11" s="16">
+      <c r="F11">
         <v>19228</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11">
         <v>10120</v>
       </c>
     </row>
@@ -12405,13 +12401,13 @@
       <c r="D12" t="s">
         <v>92</v>
       </c>
-      <c r="E12" s="16">
+      <c r="E12">
         <v>202400</v>
       </c>
-      <c r="F12" s="16">
+      <c r="F12">
         <v>19228</v>
       </c>
-      <c r="G12" s="16">
+      <c r="G12">
         <v>10120</v>
       </c>
     </row>
@@ -12428,13 +12424,13 @@
       <c r="D13" t="s">
         <v>102</v>
       </c>
-      <c r="E13" s="16">
-        <v>1</v>
-      </c>
-      <c r="F13" s="16">
-        <v>1</v>
-      </c>
-      <c r="G13" s="16">
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
         <v>1</v>
       </c>
     </row>
@@ -12451,13 +12447,13 @@
       <c r="D14" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="16">
+      <c r="E14">
         <v>92000</v>
       </c>
-      <c r="F14" s="16">
+      <c r="F14">
         <v>13524</v>
       </c>
-      <c r="G14" s="16">
+      <c r="G14">
         <v>4600</v>
       </c>
     </row>
@@ -12474,13 +12470,13 @@
       <c r="D15" t="s">
         <v>102</v>
       </c>
-      <c r="E15" s="16">
-        <v>1</v>
-      </c>
-      <c r="F15" s="16">
-        <v>1</v>
-      </c>
-      <c r="G15" s="16">
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
         <v>1</v>
       </c>
     </row>
@@ -25583,26 +25579,6 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -25610,6 +25586,26 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new cost to represent bulk materials
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="762" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F15EF054-2427-4D2D-BE91-3CB9DFE66F3B}"/>
+  <xr:revisionPtr revIDLastSave="778" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09613109-F906-46D9-B1AE-A17BDBE63962}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="7" activeTab="9" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" firstSheet="12" activeTab="17" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="153">
   <si>
     <t>Value</t>
   </si>
@@ -514,6 +514,9 @@
   <si>
     <t>Batteries_CellBatt</t>
   </si>
+  <si>
+    <t>material_downstream_manufacturing</t>
+  </si>
 </sst>
 </file>
 
@@ -580,6 +583,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -12133,10 +12137,10 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CE844EE-882F-4833-8B87-00A8BB665263}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>96</v>
       </c>
@@ -12158,8 +12162,11 @@
       <c r="G1" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -12181,8 +12188,11 @@
       <c r="G2" s="12">
         <v>3220</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2024</v>
       </c>
@@ -12204,8 +12214,11 @@
       <c r="G3" s="12">
         <v>4600</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2024</v>
       </c>
@@ -12227,8 +12240,11 @@
       <c r="G4" s="12">
         <v>8280</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2024</v>
       </c>
@@ -12250,8 +12266,11 @@
       <c r="G5" s="12">
         <v>2300</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2024</v>
       </c>
@@ -12264,17 +12283,20 @@
       <c r="D6" t="s">
         <v>89</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="12">
         <v>73600</v>
       </c>
-      <c r="F6">
-        <v>20976.000000000007</v>
-      </c>
-      <c r="G6">
+      <c r="F6" s="12">
+        <v>40142</v>
+      </c>
+      <c r="G6" s="12">
         <v>3680.0000000000009</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" s="12">
+        <v>74006</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2024</v>
       </c>
@@ -12287,17 +12309,20 @@
       <c r="D7" t="s">
         <v>90</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="12">
         <v>82800</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="12">
         <v>7866</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="12">
         <v>4140</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" s="12">
+        <v>264948.33858154103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -12310,17 +12335,20 @@
       <c r="D8" t="s">
         <v>92</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="12">
         <v>276000</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="12">
         <v>26220</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="12">
         <v>13800</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8" s="12">
+        <v>493032.21042160509</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2024</v>
       </c>
@@ -12333,17 +12361,18 @@
       <c r="D9" t="s">
         <v>100</v>
       </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E9" s="12">
+        <v>1</v>
+      </c>
+      <c r="F9" s="12">
+        <v>1</v>
+      </c>
+      <c r="G9" s="12">
+        <v>1</v>
+      </c>
+      <c r="H9" s="12"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2024</v>
       </c>
@@ -12356,17 +12385,20 @@
       <c r="D10" t="s">
         <v>89</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="12">
         <v>165600</v>
       </c>
-      <c r="F10">
-        <v>47196</v>
-      </c>
-      <c r="G10">
+      <c r="F10" s="12">
+        <v>120522</v>
+      </c>
+      <c r="G10" s="12">
         <v>8280</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H10" s="12">
+        <v>229760</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2024</v>
       </c>
@@ -12379,17 +12411,20 @@
       <c r="D11" t="s">
         <v>90</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="12">
         <v>202400</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="12">
         <v>19228</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="12">
         <v>10120</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H11" s="12">
+        <v>231566.55902280001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2024</v>
       </c>
@@ -12402,17 +12437,20 @@
       <c r="D12" t="s">
         <v>92</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="12">
         <v>202400</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="12">
         <v>19228</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="12">
         <v>10120</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H12" s="12">
+        <v>901215.14350847807</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2024</v>
       </c>
@@ -12435,7 +12473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2024</v>
       </c>
@@ -12458,7 +12496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2024</v>
       </c>
@@ -25586,26 +25624,6 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -25613,6 +25631,26 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Individualized the stages name to distinguish between on and offshore stages
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="778" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09613109-F906-46D9-B1AE-A17BDBE63962}"/>
+  <xr:revisionPtr revIDLastSave="806" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FC4A7EF-48AA-4ADE-81C0-85A7670B0A6F}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" firstSheet="12" activeTab="17" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" activeTab="9" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -36,7 +36,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">gas_block!$B$1:$B$109</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="165">
   <si>
     <t>Value</t>
   </si>
@@ -517,6 +517,42 @@
   <si>
     <t>material_downstream_manufacturing</t>
   </si>
+  <si>
+    <t>blade_bulk_on</t>
+  </si>
+  <si>
+    <t>blade_bulk_off</t>
+  </si>
+  <si>
+    <t>tower_bulk_on</t>
+  </si>
+  <si>
+    <t>tower_bulk_off</t>
+  </si>
+  <si>
+    <t>BladeOn</t>
+  </si>
+  <si>
+    <t>TowerOn</t>
+  </si>
+  <si>
+    <t>NacelleOn</t>
+  </si>
+  <si>
+    <t>AssemblyOn</t>
+  </si>
+  <si>
+    <t>BladeOff</t>
+  </si>
+  <si>
+    <t>TowerOff</t>
+  </si>
+  <si>
+    <t>NacelleOff</t>
+  </si>
+  <si>
+    <t>AssemblyOff</t>
+  </si>
 </sst>
 </file>
 
@@ -774,6 +810,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1267,7 +1307,7 @@
         <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>89</v>
+        <v>157</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1293,7 +1333,7 @@
         <v>76</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>158</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1319,7 +1359,7 @@
         <v>76</v>
       </c>
       <c r="C8" t="s">
-        <v>92</v>
+        <v>159</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1345,7 +1385,7 @@
         <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1371,7 +1411,7 @@
         <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>161</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1397,7 +1437,7 @@
         <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>162</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1420,7 +1460,7 @@
         <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>92</v>
+        <v>163</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1443,7 +1483,7 @@
         <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>100</v>
+        <v>164</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1515,7 +1555,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FA1A697-84AA-4F97-BE70-81695B57512E}">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="12" customWidth="1"/>
@@ -1689,13 +1729,13 @@
         <v>89</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="D9">
-        <v>0.94859999999999989</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>0.94859999999999989</v>
+        <v>1</v>
       </c>
       <c r="F9" s="9">
         <v>0</v>
@@ -1706,16 +1746,16 @@
         <v>76</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="D10">
-        <v>6.9563999999999995</v>
+        <v>1</v>
       </c>
       <c r="E10">
-        <v>6.9563999999999995</v>
+        <v>1</v>
       </c>
       <c r="F10" s="9">
         <v>0</v>
@@ -1726,19 +1766,19 @@
         <v>76</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D11">
-        <v>1.17E-3</v>
+        <v>5.5</v>
       </c>
       <c r="E11">
-        <v>1.17E-3</v>
-      </c>
-      <c r="F11" s="9">
-        <v>0</v>
+        <v>5.5</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1746,19 +1786,19 @@
         <v>76</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="D12">
-        <v>8.1</v>
+        <v>5.47E-3</v>
       </c>
       <c r="E12">
-        <v>8.1</v>
-      </c>
-      <c r="F12" s="9">
-        <v>0</v>
+        <v>5.47E-3</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1766,19 +1806,19 @@
         <v>76</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>91</v>
+        <v>138</v>
       </c>
       <c r="D13">
-        <v>114.72499999999999</v>
+        <v>4.7689999999999996E-2</v>
       </c>
       <c r="E13">
-        <v>114.72499999999999</v>
+        <v>4.7689999999999996E-2</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>145</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1786,19 +1826,19 @@
         <v>76</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D14">
-        <v>5.5</v>
+        <v>7.2699999999999996E-3</v>
       </c>
       <c r="E14">
-        <v>5.5</v>
+        <v>7.2699999999999996E-3</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>146</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1809,16 +1849,16 @@
         <v>92</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="D15">
-        <v>5.47E-3</v>
+        <v>2.7909999999999999</v>
       </c>
       <c r="E15">
-        <v>5.47E-3</v>
+        <v>2.7909999999999999</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>85</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1829,16 +1869,16 @@
         <v>92</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="D16">
-        <v>4.7689999999999996E-2</v>
+        <v>2.2925</v>
       </c>
       <c r="E16">
-        <v>4.7689999999999996E-2</v>
+        <v>2.2925</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>85</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1849,13 +1889,13 @@
         <v>92</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D17">
-        <v>7.2699999999999996E-3</v>
+        <v>18.945</v>
       </c>
       <c r="E17">
-        <v>7.2699999999999996E-3</v>
+        <v>18.945</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>85</v>
@@ -1869,16 +1909,16 @@
         <v>92</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="D18">
-        <v>2.7909999999999999</v>
+        <v>0.78549999999999998</v>
       </c>
       <c r="E18">
-        <v>2.7909999999999999</v>
+        <v>0.78549999999999998</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>145</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1889,16 +1929,16 @@
         <v>92</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="D19">
-        <v>2.2925</v>
+        <v>0.1045</v>
       </c>
       <c r="E19">
-        <v>2.2925</v>
+        <v>0.1045</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>145</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1909,13 +1949,13 @@
         <v>92</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D20">
-        <v>18.945</v>
+        <v>0.39200000000000002</v>
       </c>
       <c r="E20">
-        <v>18.945</v>
+        <v>0.39200000000000002</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>85</v>
@@ -1929,13 +1969,13 @@
         <v>92</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D21">
-        <v>0.78549999999999998</v>
+        <v>0.50024999999999997</v>
       </c>
       <c r="E21">
-        <v>0.78549999999999998</v>
+        <v>0.50024999999999997</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>85</v>
@@ -1943,62 +1983,62 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="D22">
-        <v>0.1045</v>
+        <v>1</v>
       </c>
       <c r="E22">
-        <v>0.1045</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>85</v>
+        <v>1</v>
+      </c>
+      <c r="F22" s="9">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="D23">
-        <v>0.39200000000000002</v>
+        <v>1</v>
       </c>
       <c r="E23">
-        <v>0.39200000000000002</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>85</v>
+        <v>1</v>
+      </c>
+      <c r="F23" s="9">
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D24">
-        <v>0.50024999999999997</v>
+        <v>5.5</v>
       </c>
       <c r="E24">
-        <v>0.50024999999999997</v>
+        <v>5.5</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>85</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2006,19 +2046,19 @@
         <v>77</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D25">
-        <v>0.97139999999999993</v>
+        <v>1.1259999999999999E-2</v>
       </c>
       <c r="E25">
-        <v>0.97139999999999993</v>
-      </c>
-      <c r="F25" s="9">
-        <v>0</v>
+        <v>1.1259999999999999E-2</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -2026,19 +2066,19 @@
         <v>77</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D26">
-        <v>7.1236000000000006</v>
+        <v>0.11219</v>
       </c>
       <c r="E26">
-        <v>7.1236000000000006</v>
-      </c>
-      <c r="F26" s="9">
-        <v>0</v>
+        <v>0.11219</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2046,19 +2086,19 @@
         <v>77</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D27">
-        <v>3.4500000000000004E-3</v>
+        <v>2.0460000000000002E-2</v>
       </c>
       <c r="E27">
-        <v>3.4500000000000004E-3</v>
-      </c>
-      <c r="F27" s="9">
-        <v>0</v>
+        <v>2.0460000000000002E-2</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2066,19 +2106,19 @@
         <v>77</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D28">
-        <v>11.6</v>
+        <v>4.04</v>
       </c>
       <c r="E28">
-        <v>11.6</v>
-      </c>
-      <c r="F28" s="9">
-        <v>0</v>
+        <v>4.04</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -2086,16 +2126,16 @@
         <v>77</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>91</v>
+        <v>130</v>
       </c>
       <c r="D29">
-        <v>116.77</v>
+        <v>3.2574999999999998</v>
       </c>
       <c r="E29">
-        <v>116.77</v>
+        <v>3.2574999999999998</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>145</v>
@@ -2106,19 +2146,19 @@
         <v>77</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D30">
-        <v>5.5</v>
+        <v>19.89</v>
       </c>
       <c r="E30">
-        <v>5.5</v>
+        <v>19.89</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>146</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2129,13 +2169,13 @@
         <v>92</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D31">
-        <v>1.1259999999999999E-2</v>
+        <v>0.79039999999999999</v>
       </c>
       <c r="E31">
-        <v>1.1259999999999999E-2</v>
+        <v>0.79039999999999999</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>85</v>
@@ -2149,13 +2189,13 @@
         <v>92</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D32">
-        <v>0.11219</v>
+        <v>0.10940000000000001</v>
       </c>
       <c r="E32">
-        <v>0.11219</v>
+        <v>0.10940000000000001</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>85</v>
@@ -2169,13 +2209,13 @@
         <v>92</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D33">
-        <v>2.0460000000000002E-2</v>
+        <v>0.32230000000000003</v>
       </c>
       <c r="E33">
-        <v>2.0460000000000002E-2</v>
+        <v>0.32230000000000003</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>85</v>
@@ -2189,175 +2229,55 @@
         <v>92</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="D34">
-        <v>4.04</v>
+        <v>0.5272</v>
       </c>
       <c r="E34">
-        <v>4.04</v>
+        <v>0.5272</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>145</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>130</v>
+      <c r="A35" t="s">
+        <v>93</v>
+      </c>
+      <c r="B35" t="s">
+        <v>150</v>
+      </c>
+      <c r="C35" t="s">
+        <v>94</v>
       </c>
       <c r="D35">
-        <v>3.2574999999999998</v>
+        <v>50</v>
       </c>
       <c r="E35">
-        <v>3.2574999999999998</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>145</v>
+        <v>50</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="C36" s="12" t="s">
-        <v>140</v>
+      <c r="A36" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36" t="s">
+        <v>150</v>
+      </c>
+      <c r="C36" t="s">
+        <v>95</v>
       </c>
       <c r="D36">
-        <v>19.89</v>
+        <v>50</v>
       </c>
       <c r="E36">
-        <v>19.89</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="D37">
-        <v>0.79039999999999999</v>
-      </c>
-      <c r="E37">
-        <v>0.79039999999999999</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="C38" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="D38">
-        <v>0.10940000000000001</v>
-      </c>
-      <c r="E38">
-        <v>0.10940000000000001</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="C39" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="D39">
-        <v>0.32230000000000003</v>
-      </c>
-      <c r="E39">
-        <v>0.32230000000000003</v>
-      </c>
-      <c r="F39" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="C40" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="D40">
-        <v>0.5272</v>
-      </c>
-      <c r="E40">
-        <v>0.5272</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>93</v>
-      </c>
-      <c r="B41" t="s">
-        <v>150</v>
-      </c>
-      <c r="C41" t="s">
-        <v>94</v>
-      </c>
-      <c r="D41">
         <v>50</v>
       </c>
-      <c r="E41">
-        <v>50</v>
-      </c>
-      <c r="F41">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>93</v>
-      </c>
-      <c r="B42" t="s">
-        <v>150</v>
-      </c>
-      <c r="C42" t="s">
-        <v>95</v>
-      </c>
-      <c r="D42">
-        <v>50</v>
-      </c>
-      <c r="E42">
-        <v>50</v>
-      </c>
-      <c r="F42">
+      <c r="F36">
         <v>0</v>
       </c>
     </row>
@@ -25624,6 +25544,26 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -25631,26 +25571,6 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Got rid of ghost caps and refined the crma scenario constraints
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1096" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F95914E4-E465-4F60-BC82-3474F0D31125}"/>
+  <xr:revisionPtr revIDLastSave="1098" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{280D284B-9121-4E13-AEAE-5874AF8D5C6E}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" firstSheet="12" activeTab="18" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="9" activeTab="17" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -36,7 +36,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">gas_block!$B$1:$B$109</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -866,11 +866,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{1C1ADB5D-62B2-4A88-A962-14B0B3D457AA}"/>
@@ -1305,7 +1305,7 @@
       <c r="E2" s="12">
         <v>150</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="20">
         <v>24000</v>
       </c>
       <c r="G2">
@@ -1328,7 +1328,7 @@
       <c r="E3" s="12">
         <v>125</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="20">
         <v>2000</v>
       </c>
       <c r="G3">
@@ -1351,7 +1351,7 @@
       <c r="E4" s="12">
         <v>76</v>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="20">
         <v>7000</v>
       </c>
       <c r="G4">
@@ -1400,7 +1400,7 @@
       <c r="E6" s="12">
         <v>60</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="20">
         <v>18000</v>
       </c>
       <c r="G6">
@@ -1426,7 +1426,7 @@
       <c r="E7" s="12">
         <v>55</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="20">
         <v>14000</v>
       </c>
       <c r="G7">
@@ -1452,7 +1452,7 @@
       <c r="E8" s="12">
         <v>35</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="20">
         <v>13000</v>
       </c>
       <c r="G8">
@@ -1504,7 +1504,7 @@
       <c r="E10" s="12">
         <v>60</v>
       </c>
-      <c r="F10" s="21">
+      <c r="F10" s="20">
         <v>5000</v>
       </c>
       <c r="G10">
@@ -1530,7 +1530,7 @@
       <c r="E11" s="12">
         <v>55</v>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="20">
         <v>9000</v>
       </c>
       <c r="G11">
@@ -1553,7 +1553,7 @@
       <c r="E12" s="12">
         <v>35</v>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="20">
         <v>7000</v>
       </c>
       <c r="G12">
@@ -1844,7 +1844,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="9">
-        <v>0</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2184,7 +2184,7 @@
         <v>1</v>
       </c>
       <c r="F27" s="9">
-        <v>0</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -4946,10 +4946,10 @@
       <c r="L2" s="12">
         <v>450000</v>
       </c>
-      <c r="M2" s="22">
+      <c r="M2" s="21">
         <v>1200</v>
       </c>
-      <c r="N2" s="22">
+      <c r="N2" s="21">
         <v>5000</v>
       </c>
       <c r="O2" s="12">
@@ -5026,10 +5026,10 @@
       <c r="L3" s="12">
         <v>450000</v>
       </c>
-      <c r="M3" s="22">
+      <c r="M3" s="21">
         <v>1200</v>
       </c>
-      <c r="N3" s="22">
+      <c r="N3" s="21">
         <v>5000</v>
       </c>
       <c r="O3" s="12">
@@ -5106,10 +5106,10 @@
       <c r="L4" s="12">
         <v>450000</v>
       </c>
-      <c r="M4" s="22">
+      <c r="M4" s="21">
         <v>1200</v>
       </c>
-      <c r="N4" s="22">
+      <c r="N4" s="21">
         <v>5000</v>
       </c>
       <c r="O4" s="12">
@@ -5186,10 +5186,10 @@
       <c r="L5" s="12">
         <v>450000</v>
       </c>
-      <c r="M5" s="22">
+      <c r="M5" s="21">
         <v>1200</v>
       </c>
-      <c r="N5" s="22">
+      <c r="N5" s="21">
         <v>5000</v>
       </c>
       <c r="O5" s="12">
@@ -5266,10 +5266,10 @@
       <c r="L6" s="12">
         <v>450000</v>
       </c>
-      <c r="M6" s="22">
+      <c r="M6" s="21">
         <v>1200</v>
       </c>
-      <c r="N6" s="22">
+      <c r="N6" s="21">
         <v>5000</v>
       </c>
       <c r="O6" s="12">
@@ -5346,10 +5346,10 @@
       <c r="L7" s="12">
         <v>450000</v>
       </c>
-      <c r="M7" s="22">
+      <c r="M7" s="21">
         <v>1200</v>
       </c>
-      <c r="N7" s="22">
+      <c r="N7" s="21">
         <v>5000</v>
       </c>
       <c r="O7" s="12">
@@ -5426,10 +5426,10 @@
       <c r="L8" s="12">
         <v>450000</v>
       </c>
-      <c r="M8" s="22">
+      <c r="M8" s="21">
         <v>1200</v>
       </c>
-      <c r="N8" s="22">
+      <c r="N8" s="21">
         <v>5000</v>
       </c>
       <c r="O8" s="12">
@@ -5506,10 +5506,10 @@
       <c r="L9" s="12">
         <v>450000</v>
       </c>
-      <c r="M9" s="22">
+      <c r="M9" s="21">
         <v>1200</v>
       </c>
-      <c r="N9" s="22">
+      <c r="N9" s="21">
         <v>5000</v>
       </c>
       <c r="O9" s="12">
@@ -5586,10 +5586,10 @@
       <c r="L10" s="12">
         <v>450000</v>
       </c>
-      <c r="M10" s="22">
+      <c r="M10" s="21">
         <v>1200</v>
       </c>
-      <c r="N10" s="22">
+      <c r="N10" s="21">
         <v>5000</v>
       </c>
       <c r="O10" s="12">
@@ -5666,10 +5666,10 @@
       <c r="L11" s="12">
         <v>450000</v>
       </c>
-      <c r="M11" s="22">
+      <c r="M11" s="21">
         <v>1200</v>
       </c>
-      <c r="N11" s="22">
+      <c r="N11" s="21">
         <v>5000</v>
       </c>
       <c r="O11" s="12">
@@ -5746,10 +5746,10 @@
       <c r="L12" s="12">
         <v>450000</v>
       </c>
-      <c r="M12" s="22">
+      <c r="M12" s="21">
         <v>1200</v>
       </c>
-      <c r="N12" s="22">
+      <c r="N12" s="21">
         <v>5000</v>
       </c>
       <c r="O12" s="12">
@@ -5826,10 +5826,10 @@
       <c r="L13" s="12">
         <v>450000</v>
       </c>
-      <c r="M13" s="22">
+      <c r="M13" s="21">
         <v>1200</v>
       </c>
-      <c r="N13" s="22">
+      <c r="N13" s="21">
         <v>5000</v>
       </c>
       <c r="O13" s="12">
@@ -5906,10 +5906,10 @@
       <c r="L14" s="12">
         <v>450000</v>
       </c>
-      <c r="M14" s="22">
+      <c r="M14" s="21">
         <v>1200</v>
       </c>
-      <c r="N14" s="22">
+      <c r="N14" s="21">
         <v>5000</v>
       </c>
       <c r="O14" s="12">
@@ -5986,10 +5986,10 @@
       <c r="L15" s="12">
         <v>450000</v>
       </c>
-      <c r="M15" s="22">
+      <c r="M15" s="21">
         <v>1200</v>
       </c>
-      <c r="N15" s="22">
+      <c r="N15" s="21">
         <v>5000</v>
       </c>
       <c r="O15" s="12">
@@ -6066,10 +6066,10 @@
       <c r="L16" s="12">
         <v>450000</v>
       </c>
-      <c r="M16" s="22">
+      <c r="M16" s="21">
         <v>1200</v>
       </c>
-      <c r="N16" s="22">
+      <c r="N16" s="21">
         <v>5000</v>
       </c>
       <c r="O16" s="12">
@@ -6146,10 +6146,10 @@
       <c r="L17" s="12">
         <v>450000</v>
       </c>
-      <c r="M17" s="22">
+      <c r="M17" s="21">
         <v>1200</v>
       </c>
-      <c r="N17" s="22">
+      <c r="N17" s="21">
         <v>5000</v>
       </c>
       <c r="O17" s="12">
@@ -6226,10 +6226,10 @@
       <c r="L18" s="12">
         <v>450000</v>
       </c>
-      <c r="M18" s="22">
+      <c r="M18" s="21">
         <v>1200</v>
       </c>
-      <c r="N18" s="22">
+      <c r="N18" s="21">
         <v>5000</v>
       </c>
       <c r="O18" s="12">
@@ -6306,10 +6306,10 @@
       <c r="L19" s="12">
         <v>450000</v>
       </c>
-      <c r="M19" s="22">
+      <c r="M19" s="21">
         <v>1200</v>
       </c>
-      <c r="N19" s="22">
+      <c r="N19" s="21">
         <v>5000</v>
       </c>
       <c r="O19" s="12">
@@ -6386,10 +6386,10 @@
       <c r="L20" s="12">
         <v>450000</v>
       </c>
-      <c r="M20" s="22">
+      <c r="M20" s="21">
         <v>1200</v>
       </c>
-      <c r="N20" s="22">
+      <c r="N20" s="21">
         <v>5000</v>
       </c>
       <c r="O20" s="12">
@@ -6466,10 +6466,10 @@
       <c r="L21" s="12">
         <v>450000</v>
       </c>
-      <c r="M21" s="22">
+      <c r="M21" s="21">
         <v>1200</v>
       </c>
-      <c r="N21" s="22">
+      <c r="N21" s="21">
         <v>5000</v>
       </c>
       <c r="O21" s="12">
@@ -6546,10 +6546,10 @@
       <c r="L22" s="12">
         <v>450000</v>
       </c>
-      <c r="M22" s="22">
+      <c r="M22" s="21">
         <v>1200</v>
       </c>
-      <c r="N22" s="22">
+      <c r="N22" s="21">
         <v>5000</v>
       </c>
       <c r="O22" s="12">
@@ -6626,10 +6626,10 @@
       <c r="L23" s="12">
         <v>450000</v>
       </c>
-      <c r="M23" s="22">
+      <c r="M23" s="21">
         <v>1200</v>
       </c>
-      <c r="N23" s="22">
+      <c r="N23" s="21">
         <v>5000</v>
       </c>
       <c r="O23" s="12">
@@ -6706,10 +6706,10 @@
       <c r="L24" s="12">
         <v>450000</v>
       </c>
-      <c r="M24" s="22">
+      <c r="M24" s="21">
         <v>1200</v>
       </c>
-      <c r="N24" s="22">
+      <c r="N24" s="21">
         <v>5000</v>
       </c>
       <c r="O24" s="12">
@@ -6786,10 +6786,10 @@
       <c r="L25" s="12">
         <v>450000</v>
       </c>
-      <c r="M25" s="22">
+      <c r="M25" s="21">
         <v>1200</v>
       </c>
-      <c r="N25" s="22">
+      <c r="N25" s="21">
         <v>5000</v>
       </c>
       <c r="O25" s="12">
@@ -6866,10 +6866,10 @@
       <c r="L26" s="12">
         <v>450000</v>
       </c>
-      <c r="M26" s="22">
+      <c r="M26" s="21">
         <v>1200</v>
       </c>
-      <c r="N26" s="22">
+      <c r="N26" s="21">
         <v>5000</v>
       </c>
       <c r="O26" s="12">
@@ -6946,10 +6946,10 @@
       <c r="L27" s="12">
         <v>450000</v>
       </c>
-      <c r="M27" s="22">
+      <c r="M27" s="21">
         <v>1200</v>
       </c>
-      <c r="N27" s="22">
+      <c r="N27" s="21">
         <v>5000</v>
       </c>
       <c r="O27" s="12">
@@ -7026,10 +7026,10 @@
       <c r="L28" s="12">
         <v>450000</v>
       </c>
-      <c r="M28" s="22">
+      <c r="M28" s="21">
         <v>1200</v>
       </c>
-      <c r="N28" s="22">
+      <c r="N28" s="21">
         <v>5000</v>
       </c>
       <c r="O28" s="12">
@@ -7196,10 +7196,10 @@
       <c r="L2" s="12">
         <v>450000</v>
       </c>
-      <c r="M2" s="22">
+      <c r="M2" s="21">
         <v>1200</v>
       </c>
-      <c r="N2" s="22">
+      <c r="N2" s="21">
         <v>5000</v>
       </c>
       <c r="O2" s="12">
@@ -7276,10 +7276,10 @@
       <c r="L3" s="12">
         <v>450000</v>
       </c>
-      <c r="M3" s="22">
+      <c r="M3" s="21">
         <v>1200</v>
       </c>
-      <c r="N3" s="22">
+      <c r="N3" s="21">
         <v>5000</v>
       </c>
       <c r="O3" s="12">
@@ -7356,10 +7356,10 @@
       <c r="L4" s="12">
         <v>450000</v>
       </c>
-      <c r="M4" s="22">
+      <c r="M4" s="21">
         <v>1200</v>
       </c>
-      <c r="N4" s="22">
+      <c r="N4" s="21">
         <v>5000</v>
       </c>
       <c r="O4" s="12">
@@ -7436,10 +7436,10 @@
       <c r="L5" s="12">
         <v>450000</v>
       </c>
-      <c r="M5" s="22">
+      <c r="M5" s="21">
         <v>1200</v>
       </c>
-      <c r="N5" s="22">
+      <c r="N5" s="21">
         <v>5000</v>
       </c>
       <c r="O5" s="12">
@@ -7516,10 +7516,10 @@
       <c r="L6" s="12">
         <v>450000</v>
       </c>
-      <c r="M6" s="22">
+      <c r="M6" s="21">
         <v>1200</v>
       </c>
-      <c r="N6" s="22">
+      <c r="N6" s="21">
         <v>5000</v>
       </c>
       <c r="O6" s="12">
@@ -7596,10 +7596,10 @@
       <c r="L7" s="12">
         <v>450000</v>
       </c>
-      <c r="M7" s="22">
+      <c r="M7" s="21">
         <v>1200</v>
       </c>
-      <c r="N7" s="22">
+      <c r="N7" s="21">
         <v>5000</v>
       </c>
       <c r="O7" s="12">
@@ -7676,10 +7676,10 @@
       <c r="L8" s="12">
         <v>450000</v>
       </c>
-      <c r="M8" s="22">
+      <c r="M8" s="21">
         <v>1200</v>
       </c>
-      <c r="N8" s="22">
+      <c r="N8" s="21">
         <v>5000</v>
       </c>
       <c r="O8" s="12">
@@ -7756,10 +7756,10 @@
       <c r="L9" s="12">
         <v>450000</v>
       </c>
-      <c r="M9" s="22">
+      <c r="M9" s="21">
         <v>1200</v>
       </c>
-      <c r="N9" s="22">
+      <c r="N9" s="21">
         <v>5000</v>
       </c>
       <c r="O9" s="12">
@@ -7836,10 +7836,10 @@
       <c r="L10" s="12">
         <v>450000</v>
       </c>
-      <c r="M10" s="22">
+      <c r="M10" s="21">
         <v>1200</v>
       </c>
-      <c r="N10" s="22">
+      <c r="N10" s="21">
         <v>5000</v>
       </c>
       <c r="O10" s="12">
@@ -7916,10 +7916,10 @@
       <c r="L11" s="12">
         <v>450000</v>
       </c>
-      <c r="M11" s="22">
+      <c r="M11" s="21">
         <v>1200</v>
       </c>
-      <c r="N11" s="22">
+      <c r="N11" s="21">
         <v>5000</v>
       </c>
       <c r="O11" s="12">
@@ -7996,10 +7996,10 @@
       <c r="L12" s="12">
         <v>450000</v>
       </c>
-      <c r="M12" s="22">
+      <c r="M12" s="21">
         <v>1200</v>
       </c>
-      <c r="N12" s="22">
+      <c r="N12" s="21">
         <v>5000</v>
       </c>
       <c r="O12" s="12">
@@ -8076,10 +8076,10 @@
       <c r="L13" s="12">
         <v>450000</v>
       </c>
-      <c r="M13" s="22">
+      <c r="M13" s="21">
         <v>1200</v>
       </c>
-      <c r="N13" s="22">
+      <c r="N13" s="21">
         <v>5000</v>
       </c>
       <c r="O13" s="12">
@@ -8156,10 +8156,10 @@
       <c r="L14" s="12">
         <v>450000</v>
       </c>
-      <c r="M14" s="22">
+      <c r="M14" s="21">
         <v>1200</v>
       </c>
-      <c r="N14" s="22">
+      <c r="N14" s="21">
         <v>5000</v>
       </c>
       <c r="O14" s="12">
@@ -8236,10 +8236,10 @@
       <c r="L15" s="12">
         <v>450000</v>
       </c>
-      <c r="M15" s="22">
+      <c r="M15" s="21">
         <v>1200</v>
       </c>
-      <c r="N15" s="22">
+      <c r="N15" s="21">
         <v>5000</v>
       </c>
       <c r="O15" s="12">
@@ -8316,10 +8316,10 @@
       <c r="L16" s="12">
         <v>450000</v>
       </c>
-      <c r="M16" s="22">
+      <c r="M16" s="21">
         <v>1200</v>
       </c>
-      <c r="N16" s="22">
+      <c r="N16" s="21">
         <v>5000</v>
       </c>
       <c r="O16" s="12">
@@ -8396,10 +8396,10 @@
       <c r="L17" s="12">
         <v>450000</v>
       </c>
-      <c r="M17" s="22">
+      <c r="M17" s="21">
         <v>1200</v>
       </c>
-      <c r="N17" s="22">
+      <c r="N17" s="21">
         <v>5000</v>
       </c>
       <c r="O17" s="12">
@@ -8476,10 +8476,10 @@
       <c r="L18" s="12">
         <v>450000</v>
       </c>
-      <c r="M18" s="22">
+      <c r="M18" s="21">
         <v>1200</v>
       </c>
-      <c r="N18" s="22">
+      <c r="N18" s="21">
         <v>5000</v>
       </c>
       <c r="O18" s="12">
@@ -8556,10 +8556,10 @@
       <c r="L19" s="12">
         <v>450000</v>
       </c>
-      <c r="M19" s="22">
+      <c r="M19" s="21">
         <v>1200</v>
       </c>
-      <c r="N19" s="22">
+      <c r="N19" s="21">
         <v>5000</v>
       </c>
       <c r="O19" s="12">
@@ -8636,10 +8636,10 @@
       <c r="L20" s="12">
         <v>450000</v>
       </c>
-      <c r="M20" s="22">
+      <c r="M20" s="21">
         <v>1200</v>
       </c>
-      <c r="N20" s="22">
+      <c r="N20" s="21">
         <v>5000</v>
       </c>
       <c r="O20" s="12">
@@ -8716,10 +8716,10 @@
       <c r="L21" s="12">
         <v>450000</v>
       </c>
-      <c r="M21" s="22">
+      <c r="M21" s="21">
         <v>1200</v>
       </c>
-      <c r="N21" s="22">
+      <c r="N21" s="21">
         <v>5000</v>
       </c>
       <c r="O21" s="12">
@@ -8796,10 +8796,10 @@
       <c r="L22" s="12">
         <v>450000</v>
       </c>
-      <c r="M22" s="22">
+      <c r="M22" s="21">
         <v>1200</v>
       </c>
-      <c r="N22" s="22">
+      <c r="N22" s="21">
         <v>5000</v>
       </c>
       <c r="O22" s="12">
@@ -8876,10 +8876,10 @@
       <c r="L23" s="12">
         <v>450000</v>
       </c>
-      <c r="M23" s="22">
+      <c r="M23" s="21">
         <v>1200</v>
       </c>
-      <c r="N23" s="22">
+      <c r="N23" s="21">
         <v>5000</v>
       </c>
       <c r="O23" s="12">
@@ -8956,10 +8956,10 @@
       <c r="L24" s="12">
         <v>450000</v>
       </c>
-      <c r="M24" s="22">
+      <c r="M24" s="21">
         <v>1200</v>
       </c>
-      <c r="N24" s="22">
+      <c r="N24" s="21">
         <v>5000</v>
       </c>
       <c r="O24" s="12">
@@ -9036,10 +9036,10 @@
       <c r="L25" s="12">
         <v>450000</v>
       </c>
-      <c r="M25" s="22">
+      <c r="M25" s="21">
         <v>1200</v>
       </c>
-      <c r="N25" s="22">
+      <c r="N25" s="21">
         <v>5000</v>
       </c>
       <c r="O25" s="12">
@@ -9116,10 +9116,10 @@
       <c r="L26" s="12">
         <v>450000</v>
       </c>
-      <c r="M26" s="22">
+      <c r="M26" s="21">
         <v>1200</v>
       </c>
-      <c r="N26" s="22">
+      <c r="N26" s="21">
         <v>5000</v>
       </c>
       <c r="O26" s="12">
@@ -9196,10 +9196,10 @@
       <c r="L27" s="12">
         <v>450000</v>
       </c>
-      <c r="M27" s="22">
+      <c r="M27" s="21">
         <v>1200</v>
       </c>
-      <c r="N27" s="22">
+      <c r="N27" s="21">
         <v>5000</v>
       </c>
       <c r="O27" s="12">
@@ -9276,10 +9276,10 @@
       <c r="L28" s="12">
         <v>450000</v>
       </c>
-      <c r="M28" s="22">
+      <c r="M28" s="21">
         <v>1200</v>
       </c>
-      <c r="N28" s="22">
+      <c r="N28" s="21">
         <v>5000</v>
       </c>
       <c r="O28" s="12">
@@ -26142,7 +26142,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="20">
+      <c r="A2" s="22">
         <v>2024</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -26156,7 +26156,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="20"/>
+      <c r="A3" s="22"/>
       <c r="B3" s="11" t="s">
         <v>70</v>
       </c>
@@ -26169,7 +26169,7 @@
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="20"/>
+      <c r="A4" s="22"/>
       <c r="B4" s="11" t="s">
         <v>71</v>
       </c>
@@ -26181,7 +26181,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="20"/>
+      <c r="A5" s="22"/>
       <c r="B5" s="11" t="s">
         <v>68</v>
       </c>
@@ -26193,7 +26193,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="20">
+      <c r="A6" s="22">
         <v>2025</v>
       </c>
       <c r="B6" s="11" t="s">
@@ -26207,7 +26207,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="20"/>
+      <c r="A7" s="22"/>
       <c r="B7" s="11" t="s">
         <v>70</v>
       </c>
@@ -26219,7 +26219,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="20"/>
+      <c r="A8" s="22"/>
       <c r="B8" s="11" t="s">
         <v>71</v>
       </c>
@@ -26231,7 +26231,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="20"/>
+      <c r="A9" s="22"/>
       <c r="B9" s="11" t="s">
         <v>68</v>
       </c>
@@ -26244,7 +26244,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="20">
+      <c r="A10" s="22">
         <v>2026</v>
       </c>
       <c r="B10" s="11" t="s">
@@ -26258,7 +26258,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="20"/>
+      <c r="A11" s="22"/>
       <c r="B11" s="11" t="s">
         <v>70</v>
       </c>
@@ -26270,7 +26270,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="20"/>
+      <c r="A12" s="22"/>
       <c r="B12" s="11" t="s">
         <v>71</v>
       </c>
@@ -26282,7 +26282,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="20"/>
+      <c r="A13" s="22"/>
       <c r="B13" s="11" t="s">
         <v>68</v>
       </c>
@@ -26295,7 +26295,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="20">
+      <c r="A14" s="22">
         <v>2027</v>
       </c>
       <c r="B14" s="11" t="s">
@@ -26309,7 +26309,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="20"/>
+      <c r="A15" s="22"/>
       <c r="B15" s="11" t="s">
         <v>70</v>
       </c>
@@ -26321,7 +26321,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="20"/>
+      <c r="A16" s="22"/>
       <c r="B16" s="11" t="s">
         <v>71</v>
       </c>
@@ -26333,7 +26333,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="20"/>
+      <c r="A17" s="22"/>
       <c r="B17" s="11" t="s">
         <v>68</v>
       </c>
@@ -26346,7 +26346,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="20">
+      <c r="A18" s="22">
         <v>2028</v>
       </c>
       <c r="B18" s="11" t="s">
@@ -26360,7 +26360,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="20"/>
+      <c r="A19" s="22"/>
       <c r="B19" s="11" t="s">
         <v>70</v>
       </c>
@@ -26372,7 +26372,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="20"/>
+      <c r="A20" s="22"/>
       <c r="B20" s="11" t="s">
         <v>71</v>
       </c>
@@ -26384,7 +26384,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="20"/>
+      <c r="A21" s="22"/>
       <c r="B21" s="11" t="s">
         <v>68</v>
       </c>
@@ -26397,7 +26397,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="20">
+      <c r="A22" s="22">
         <v>2029</v>
       </c>
       <c r="B22" s="11" t="s">
@@ -26411,7 +26411,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="20"/>
+      <c r="A23" s="22"/>
       <c r="B23" s="11" t="s">
         <v>70</v>
       </c>
@@ -26423,7 +26423,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="20"/>
+      <c r="A24" s="22"/>
       <c r="B24" s="11" t="s">
         <v>71</v>
       </c>
@@ -26435,7 +26435,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="20"/>
+      <c r="A25" s="22"/>
       <c r="B25" s="11" t="s">
         <v>68</v>
       </c>
@@ -26448,7 +26448,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="20">
+      <c r="A26" s="22">
         <v>2030</v>
       </c>
       <c r="B26" s="11" t="s">
@@ -26462,7 +26462,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="20"/>
+      <c r="A27" s="22"/>
       <c r="B27" s="11" t="s">
         <v>70</v>
       </c>
@@ -26474,7 +26474,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="20"/>
+      <c r="A28" s="22"/>
       <c r="B28" s="11" t="s">
         <v>71</v>
       </c>
@@ -26486,7 +26486,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="20"/>
+      <c r="A29" s="22"/>
       <c r="B29" s="11" t="s">
         <v>68</v>
       </c>
@@ -26499,7 +26499,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="20">
+      <c r="A30" s="22">
         <v>2031</v>
       </c>
       <c r="B30" s="11" t="s">
@@ -26513,7 +26513,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="20"/>
+      <c r="A31" s="22"/>
       <c r="B31" s="11" t="s">
         <v>70</v>
       </c>
@@ -26525,7 +26525,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="20"/>
+      <c r="A32" s="22"/>
       <c r="B32" s="11" t="s">
         <v>71</v>
       </c>
@@ -26537,7 +26537,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="20"/>
+      <c r="A33" s="22"/>
       <c r="B33" s="11" t="s">
         <v>68</v>
       </c>
@@ -26550,7 +26550,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="20">
+      <c r="A34" s="22">
         <v>2032</v>
       </c>
       <c r="B34" s="11" t="s">
@@ -26564,7 +26564,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="20"/>
+      <c r="A35" s="22"/>
       <c r="B35" s="11" t="s">
         <v>70</v>
       </c>
@@ -26576,7 +26576,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="20"/>
+      <c r="A36" s="22"/>
       <c r="B36" s="11" t="s">
         <v>71</v>
       </c>
@@ -26588,7 +26588,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="20"/>
+      <c r="A37" s="22"/>
       <c r="B37" s="11" t="s">
         <v>68</v>
       </c>
@@ -26601,7 +26601,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="20">
+      <c r="A38" s="22">
         <v>2033</v>
       </c>
       <c r="B38" s="11" t="s">
@@ -26615,7 +26615,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="20"/>
+      <c r="A39" s="22"/>
       <c r="B39" s="11" t="s">
         <v>70</v>
       </c>
@@ -26627,7 +26627,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="20"/>
+      <c r="A40" s="22"/>
       <c r="B40" s="11" t="s">
         <v>71</v>
       </c>
@@ -26639,7 +26639,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="20"/>
+      <c r="A41" s="22"/>
       <c r="B41" s="11" t="s">
         <v>68</v>
       </c>
@@ -26652,7 +26652,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="20">
+      <c r="A42" s="22">
         <v>2034</v>
       </c>
       <c r="B42" s="11" t="s">
@@ -26666,7 +26666,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="20"/>
+      <c r="A43" s="22"/>
       <c r="B43" s="11" t="s">
         <v>70</v>
       </c>
@@ -26678,7 +26678,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="20"/>
+      <c r="A44" s="22"/>
       <c r="B44" s="11" t="s">
         <v>71</v>
       </c>
@@ -26690,7 +26690,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="20"/>
+      <c r="A45" s="22"/>
       <c r="B45" s="11" t="s">
         <v>68</v>
       </c>
@@ -26703,7 +26703,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="20">
+      <c r="A46" s="22">
         <v>2035</v>
       </c>
       <c r="B46" s="11" t="s">
@@ -26717,7 +26717,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="20"/>
+      <c r="A47" s="22"/>
       <c r="B47" s="11" t="s">
         <v>70</v>
       </c>
@@ -26729,7 +26729,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="20"/>
+      <c r="A48" s="22"/>
       <c r="B48" s="11" t="s">
         <v>71</v>
       </c>
@@ -26741,7 +26741,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="20"/>
+      <c r="A49" s="22"/>
       <c r="B49" s="11" t="s">
         <v>68</v>
       </c>
@@ -26754,7 +26754,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="20">
+      <c r="A50" s="22">
         <v>2036</v>
       </c>
       <c r="B50" s="11" t="s">
@@ -26768,7 +26768,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="20"/>
+      <c r="A51" s="22"/>
       <c r="B51" s="11" t="s">
         <v>70</v>
       </c>
@@ -26780,7 +26780,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="20"/>
+      <c r="A52" s="22"/>
       <c r="B52" s="11" t="s">
         <v>71</v>
       </c>
@@ -26792,7 +26792,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="20"/>
+      <c r="A53" s="22"/>
       <c r="B53" s="11" t="s">
         <v>68</v>
       </c>
@@ -26805,7 +26805,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="20">
+      <c r="A54" s="22">
         <v>2037</v>
       </c>
       <c r="B54" s="11" t="s">
@@ -26819,7 +26819,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="20"/>
+      <c r="A55" s="22"/>
       <c r="B55" s="11" t="s">
         <v>70</v>
       </c>
@@ -26831,7 +26831,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="20"/>
+      <c r="A56" s="22"/>
       <c r="B56" s="11" t="s">
         <v>71</v>
       </c>
@@ -26843,7 +26843,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="20"/>
+      <c r="A57" s="22"/>
       <c r="B57" s="11" t="s">
         <v>68</v>
       </c>
@@ -26856,7 +26856,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="20">
+      <c r="A58" s="22">
         <v>2038</v>
       </c>
       <c r="B58" s="11" t="s">
@@ -26870,7 +26870,7 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="20"/>
+      <c r="A59" s="22"/>
       <c r="B59" s="11" t="s">
         <v>70</v>
       </c>
@@ -26882,7 +26882,7 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="20"/>
+      <c r="A60" s="22"/>
       <c r="B60" s="11" t="s">
         <v>71</v>
       </c>
@@ -26894,7 +26894,7 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="20"/>
+      <c r="A61" s="22"/>
       <c r="B61" s="11" t="s">
         <v>68</v>
       </c>
@@ -26907,7 +26907,7 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="20">
+      <c r="A62" s="22">
         <v>2039</v>
       </c>
       <c r="B62" s="11" t="s">
@@ -26921,7 +26921,7 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="20"/>
+      <c r="A63" s="22"/>
       <c r="B63" s="11" t="s">
         <v>70</v>
       </c>
@@ -26933,7 +26933,7 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="20"/>
+      <c r="A64" s="22"/>
       <c r="B64" s="11" t="s">
         <v>71</v>
       </c>
@@ -26945,7 +26945,7 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="20"/>
+      <c r="A65" s="22"/>
       <c r="B65" s="11" t="s">
         <v>68</v>
       </c>
@@ -26958,7 +26958,7 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="20">
+      <c r="A66" s="22">
         <v>2040</v>
       </c>
       <c r="B66" s="11" t="s">
@@ -26972,7 +26972,7 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="20"/>
+      <c r="A67" s="22"/>
       <c r="B67" s="11" t="s">
         <v>70</v>
       </c>
@@ -26984,7 +26984,7 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="20"/>
+      <c r="A68" s="22"/>
       <c r="B68" s="11" t="s">
         <v>71</v>
       </c>
@@ -26996,7 +26996,7 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="20"/>
+      <c r="A69" s="22"/>
       <c r="B69" s="11" t="s">
         <v>68</v>
       </c>
@@ -27009,7 +27009,7 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="20">
+      <c r="A70" s="22">
         <v>2041</v>
       </c>
       <c r="B70" s="11" t="s">
@@ -27023,7 +27023,7 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="20"/>
+      <c r="A71" s="22"/>
       <c r="B71" s="11" t="s">
         <v>70</v>
       </c>
@@ -27035,7 +27035,7 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="20"/>
+      <c r="A72" s="22"/>
       <c r="B72" s="11" t="s">
         <v>71</v>
       </c>
@@ -27047,7 +27047,7 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="20"/>
+      <c r="A73" s="22"/>
       <c r="B73" s="11" t="s">
         <v>68</v>
       </c>
@@ -27060,7 +27060,7 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="20">
+      <c r="A74" s="22">
         <v>2042</v>
       </c>
       <c r="B74" s="11" t="s">
@@ -27074,7 +27074,7 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="20"/>
+      <c r="A75" s="22"/>
       <c r="B75" s="11" t="s">
         <v>70</v>
       </c>
@@ -27086,7 +27086,7 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="20"/>
+      <c r="A76" s="22"/>
       <c r="B76" s="11" t="s">
         <v>71</v>
       </c>
@@ -27098,7 +27098,7 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="20"/>
+      <c r="A77" s="22"/>
       <c r="B77" s="11" t="s">
         <v>68</v>
       </c>
@@ -27111,7 +27111,7 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="20">
+      <c r="A78" s="22">
         <v>2043</v>
       </c>
       <c r="B78" s="11" t="s">
@@ -27125,7 +27125,7 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="20"/>
+      <c r="A79" s="22"/>
       <c r="B79" s="11" t="s">
         <v>70</v>
       </c>
@@ -27137,7 +27137,7 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="20"/>
+      <c r="A80" s="22"/>
       <c r="B80" s="11" t="s">
         <v>71</v>
       </c>
@@ -27149,7 +27149,7 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="20"/>
+      <c r="A81" s="22"/>
       <c r="B81" s="11" t="s">
         <v>68</v>
       </c>
@@ -27162,7 +27162,7 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="20">
+      <c r="A82" s="22">
         <v>2044</v>
       </c>
       <c r="B82" s="11" t="s">
@@ -27176,7 +27176,7 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="20"/>
+      <c r="A83" s="22"/>
       <c r="B83" s="11" t="s">
         <v>70</v>
       </c>
@@ -27188,7 +27188,7 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="20"/>
+      <c r="A84" s="22"/>
       <c r="B84" s="11" t="s">
         <v>71</v>
       </c>
@@ -27200,7 +27200,7 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="20"/>
+      <c r="A85" s="22"/>
       <c r="B85" s="11" t="s">
         <v>68</v>
       </c>
@@ -27213,7 +27213,7 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="20">
+      <c r="A86" s="22">
         <v>2045</v>
       </c>
       <c r="B86" s="11" t="s">
@@ -27227,7 +27227,7 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="20"/>
+      <c r="A87" s="22"/>
       <c r="B87" s="11" t="s">
         <v>70</v>
       </c>
@@ -27239,7 +27239,7 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="20"/>
+      <c r="A88" s="22"/>
       <c r="B88" s="11" t="s">
         <v>71</v>
       </c>
@@ -27251,7 +27251,7 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="20"/>
+      <c r="A89" s="22"/>
       <c r="B89" s="11" t="s">
         <v>68</v>
       </c>
@@ -27264,7 +27264,7 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="20">
+      <c r="A90" s="22">
         <v>2046</v>
       </c>
       <c r="B90" s="11" t="s">
@@ -27278,7 +27278,7 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="20"/>
+      <c r="A91" s="22"/>
       <c r="B91" s="11" t="s">
         <v>70</v>
       </c>
@@ -27290,7 +27290,7 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="20"/>
+      <c r="A92" s="22"/>
       <c r="B92" s="11" t="s">
         <v>71</v>
       </c>
@@ -27302,7 +27302,7 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="20"/>
+      <c r="A93" s="22"/>
       <c r="B93" s="11" t="s">
         <v>68</v>
       </c>
@@ -27315,7 +27315,7 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="20">
+      <c r="A94" s="22">
         <v>2047</v>
       </c>
       <c r="B94" s="11" t="s">
@@ -27329,7 +27329,7 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="20"/>
+      <c r="A95" s="22"/>
       <c r="B95" s="11" t="s">
         <v>70</v>
       </c>
@@ -27341,7 +27341,7 @@
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="20"/>
+      <c r="A96" s="22"/>
       <c r="B96" s="11" t="s">
         <v>71</v>
       </c>
@@ -27353,7 +27353,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="20"/>
+      <c r="A97" s="22"/>
       <c r="B97" s="11" t="s">
         <v>68</v>
       </c>
@@ -27366,7 +27366,7 @@
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="20">
+      <c r="A98" s="22">
         <v>2048</v>
       </c>
       <c r="B98" s="11" t="s">
@@ -27380,7 +27380,7 @@
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" s="20"/>
+      <c r="A99" s="22"/>
       <c r="B99" s="11" t="s">
         <v>70</v>
       </c>
@@ -27392,7 +27392,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="20"/>
+      <c r="A100" s="22"/>
       <c r="B100" s="11" t="s">
         <v>71</v>
       </c>
@@ -27404,7 +27404,7 @@
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" s="20"/>
+      <c r="A101" s="22"/>
       <c r="B101" s="11" t="s">
         <v>68</v>
       </c>
@@ -27417,7 +27417,7 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" s="20">
+      <c r="A102" s="22">
         <v>2049</v>
       </c>
       <c r="B102" s="11" t="s">
@@ -27431,7 +27431,7 @@
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A103" s="20"/>
+      <c r="A103" s="22"/>
       <c r="B103" s="11" t="s">
         <v>70</v>
       </c>
@@ -27443,7 +27443,7 @@
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="20"/>
+      <c r="A104" s="22"/>
       <c r="B104" s="11" t="s">
         <v>71</v>
       </c>
@@ -27455,7 +27455,7 @@
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="20"/>
+      <c r="A105" s="22"/>
       <c r="B105" s="11" t="s">
         <v>68</v>
       </c>
@@ -27468,7 +27468,7 @@
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" s="20">
+      <c r="A106" s="22">
         <v>2050</v>
       </c>
       <c r="B106" s="11" t="s">
@@ -27482,7 +27482,7 @@
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" s="20"/>
+      <c r="A107" s="22"/>
       <c r="B107" s="11" t="s">
         <v>70</v>
       </c>
@@ -27494,7 +27494,7 @@
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" s="20"/>
+      <c r="A108" s="22"/>
       <c r="B108" s="11" t="s">
         <v>71</v>
       </c>
@@ -27506,7 +27506,7 @@
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" s="20"/>
+      <c r="A109" s="22"/>
       <c r="B109" s="11" t="s">
         <v>68</v>
       </c>

</xml_diff>

<commit_message>
Added presolve debug output
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1155" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{898C7E9C-83DA-4DD8-8EF3-751FB916CEA0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="9" activeTab="10" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="5" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -37,7 +37,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">gas_block!$B$1:$B$109</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -920,11 +919,11 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="11">
@@ -2719,7 +2718,7 @@
       <c r="A2" s="14">
         <v>2024</v>
       </c>
-      <c r="B2" s="23">
+      <c r="B2" s="22">
         <v>2024431</v>
       </c>
       <c r="C2" s="15">
@@ -2728,7 +2727,7 @@
       <c r="D2" s="15">
         <v>58100000</v>
       </c>
-      <c r="E2" s="23">
+      <c r="E2" s="22">
         <v>860748</v>
       </c>
       <c r="F2" s="15">
@@ -2743,7 +2742,7 @@
       <c r="I2">
         <v>999999999</v>
       </c>
-      <c r="J2" s="23">
+      <c r="J2" s="22">
         <v>1235</v>
       </c>
       <c r="K2">
@@ -2752,19 +2751,19 @@
       <c r="L2">
         <v>0</v>
       </c>
-      <c r="M2" s="23">
+      <c r="M2" s="22">
         <v>485</v>
       </c>
-      <c r="N2" s="23">
+      <c r="N2" s="22">
         <v>280</v>
       </c>
-      <c r="O2" s="23">
+      <c r="O2" s="22">
         <v>15000</v>
       </c>
       <c r="P2">
         <v>0</v>
       </c>
-      <c r="Q2" s="23">
+      <c r="Q2" s="22">
         <v>47673</v>
       </c>
       <c r="R2">
@@ -2799,7 +2798,7 @@
       <c r="A3" s="14">
         <v>2025</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="22">
         <v>2024431</v>
       </c>
       <c r="C3" s="15">
@@ -2808,7 +2807,7 @@
       <c r="D3" s="15">
         <v>58100000</v>
       </c>
-      <c r="E3" s="23">
+      <c r="E3" s="22">
         <v>860748</v>
       </c>
       <c r="F3" s="15">
@@ -2823,7 +2822,7 @@
       <c r="I3">
         <v>999999999</v>
       </c>
-      <c r="J3" s="23">
+      <c r="J3" s="22">
         <v>1235</v>
       </c>
       <c r="K3">
@@ -2832,19 +2831,19 @@
       <c r="L3">
         <v>0</v>
       </c>
-      <c r="M3" s="23">
+      <c r="M3" s="22">
         <v>485</v>
       </c>
-      <c r="N3" s="23">
+      <c r="N3" s="22">
         <v>280</v>
       </c>
-      <c r="O3" s="23">
+      <c r="O3" s="22">
         <v>15000</v>
       </c>
       <c r="P3">
         <v>0</v>
       </c>
-      <c r="Q3" s="23">
+      <c r="Q3" s="22">
         <v>47673</v>
       </c>
       <c r="R3">
@@ -2879,7 +2878,7 @@
       <c r="A4" s="14">
         <v>2026</v>
       </c>
-      <c r="B4" s="23">
+      <c r="B4" s="22">
         <v>2024431</v>
       </c>
       <c r="C4" s="15">
@@ -2888,7 +2887,7 @@
       <c r="D4" s="15">
         <v>58100000</v>
       </c>
-      <c r="E4" s="23">
+      <c r="E4" s="22">
         <v>860748</v>
       </c>
       <c r="F4" s="15">
@@ -2903,7 +2902,7 @@
       <c r="I4">
         <v>999999999</v>
       </c>
-      <c r="J4" s="23">
+      <c r="J4" s="22">
         <v>1235</v>
       </c>
       <c r="K4">
@@ -2912,19 +2911,19 @@
       <c r="L4">
         <v>0</v>
       </c>
-      <c r="M4" s="23">
+      <c r="M4" s="22">
         <v>485</v>
       </c>
-      <c r="N4" s="23">
+      <c r="N4" s="22">
         <v>280</v>
       </c>
-      <c r="O4" s="23">
+      <c r="O4" s="22">
         <v>15000</v>
       </c>
       <c r="P4">
         <v>0</v>
       </c>
-      <c r="Q4" s="23">
+      <c r="Q4" s="22">
         <v>47673</v>
       </c>
       <c r="R4">
@@ -2959,7 +2958,7 @@
       <c r="A5" s="14">
         <v>2027</v>
       </c>
-      <c r="B5" s="23">
+      <c r="B5" s="22">
         <v>2024431</v>
       </c>
       <c r="C5" s="15">
@@ -2968,7 +2967,7 @@
       <c r="D5" s="15">
         <v>58100000</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="22">
         <v>860748</v>
       </c>
       <c r="F5" s="15">
@@ -2983,7 +2982,7 @@
       <c r="I5">
         <v>999999999</v>
       </c>
-      <c r="J5" s="23">
+      <c r="J5" s="22">
         <v>1235</v>
       </c>
       <c r="K5">
@@ -2992,19 +2991,19 @@
       <c r="L5">
         <v>0</v>
       </c>
-      <c r="M5" s="23">
+      <c r="M5" s="22">
         <v>485</v>
       </c>
-      <c r="N5" s="23">
+      <c r="N5" s="22">
         <v>280</v>
       </c>
-      <c r="O5" s="23">
+      <c r="O5" s="22">
         <v>15000</v>
       </c>
       <c r="P5">
         <v>0</v>
       </c>
-      <c r="Q5" s="23">
+      <c r="Q5" s="22">
         <v>47673</v>
       </c>
       <c r="R5">
@@ -3039,7 +3038,7 @@
       <c r="A6" s="14">
         <v>2028</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="22">
         <v>2024431</v>
       </c>
       <c r="C6" s="15">
@@ -3048,7 +3047,7 @@
       <c r="D6" s="15">
         <v>58100000</v>
       </c>
-      <c r="E6" s="23">
+      <c r="E6" s="22">
         <v>860748</v>
       </c>
       <c r="F6" s="15">
@@ -3063,7 +3062,7 @@
       <c r="I6">
         <v>999999999</v>
       </c>
-      <c r="J6" s="23">
+      <c r="J6" s="22">
         <v>1235</v>
       </c>
       <c r="K6">
@@ -3072,19 +3071,19 @@
       <c r="L6">
         <v>0</v>
       </c>
-      <c r="M6" s="23">
+      <c r="M6" s="22">
         <v>485</v>
       </c>
-      <c r="N6" s="23">
+      <c r="N6" s="22">
         <v>280</v>
       </c>
-      <c r="O6" s="23">
+      <c r="O6" s="22">
         <v>15000</v>
       </c>
       <c r="P6">
         <v>0</v>
       </c>
-      <c r="Q6" s="23">
+      <c r="Q6" s="22">
         <v>47673</v>
       </c>
       <c r="R6">
@@ -3119,7 +3118,7 @@
       <c r="A7" s="14">
         <v>2029</v>
       </c>
-      <c r="B7" s="23">
+      <c r="B7" s="22">
         <v>2024431</v>
       </c>
       <c r="C7" s="15">
@@ -3128,7 +3127,7 @@
       <c r="D7" s="15">
         <v>58100000</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="22">
         <v>860748</v>
       </c>
       <c r="F7" s="15">
@@ -3143,7 +3142,7 @@
       <c r="I7">
         <v>999999999</v>
       </c>
-      <c r="J7" s="23">
+      <c r="J7" s="22">
         <v>1235</v>
       </c>
       <c r="K7">
@@ -3152,19 +3151,19 @@
       <c r="L7">
         <v>0</v>
       </c>
-      <c r="M7" s="23">
+      <c r="M7" s="22">
         <v>485</v>
       </c>
-      <c r="N7" s="23">
+      <c r="N7" s="22">
         <v>280</v>
       </c>
-      <c r="O7" s="23">
+      <c r="O7" s="22">
         <v>15000</v>
       </c>
       <c r="P7">
         <v>0</v>
       </c>
-      <c r="Q7" s="23">
+      <c r="Q7" s="22">
         <v>47673</v>
       </c>
       <c r="R7">
@@ -3199,7 +3198,7 @@
       <c r="A8" s="14">
         <v>2030</v>
       </c>
-      <c r="B8" s="23">
+      <c r="B8" s="22">
         <v>2024431</v>
       </c>
       <c r="C8" s="15">
@@ -3208,7 +3207,7 @@
       <c r="D8" s="15">
         <v>58100000</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="22">
         <v>860748</v>
       </c>
       <c r="F8" s="15">
@@ -3223,7 +3222,7 @@
       <c r="I8">
         <v>999999999</v>
       </c>
-      <c r="J8" s="23">
+      <c r="J8" s="22">
         <v>1235</v>
       </c>
       <c r="K8">
@@ -3232,19 +3231,19 @@
       <c r="L8">
         <v>0</v>
       </c>
-      <c r="M8" s="23">
+      <c r="M8" s="22">
         <v>485</v>
       </c>
-      <c r="N8" s="23">
+      <c r="N8" s="22">
         <v>280</v>
       </c>
-      <c r="O8" s="23">
+      <c r="O8" s="22">
         <v>15000</v>
       </c>
       <c r="P8">
         <v>0</v>
       </c>
-      <c r="Q8" s="23">
+      <c r="Q8" s="22">
         <v>47673</v>
       </c>
       <c r="R8">
@@ -3279,7 +3278,7 @@
       <c r="A9" s="14">
         <v>2031</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="22">
         <v>2024431</v>
       </c>
       <c r="C9" s="15">
@@ -3288,7 +3287,7 @@
       <c r="D9" s="15">
         <v>58100000</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9" s="22">
         <v>860748</v>
       </c>
       <c r="F9" s="15">
@@ -3303,7 +3302,7 @@
       <c r="I9">
         <v>999999999</v>
       </c>
-      <c r="J9" s="23">
+      <c r="J9" s="22">
         <v>1235</v>
       </c>
       <c r="K9">
@@ -3312,19 +3311,19 @@
       <c r="L9">
         <v>0</v>
       </c>
-      <c r="M9" s="23">
+      <c r="M9" s="22">
         <v>485</v>
       </c>
-      <c r="N9" s="23">
+      <c r="N9" s="22">
         <v>280</v>
       </c>
-      <c r="O9" s="23">
+      <c r="O9" s="22">
         <v>15000</v>
       </c>
       <c r="P9">
         <v>0</v>
       </c>
-      <c r="Q9" s="23">
+      <c r="Q9" s="22">
         <v>47673</v>
       </c>
       <c r="R9">
@@ -3359,7 +3358,7 @@
       <c r="A10" s="14">
         <v>2032</v>
       </c>
-      <c r="B10" s="23">
+      <c r="B10" s="22">
         <v>2024431</v>
       </c>
       <c r="C10" s="15">
@@ -3368,7 +3367,7 @@
       <c r="D10" s="15">
         <v>58100000</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="22">
         <v>860748</v>
       </c>
       <c r="F10" s="15">
@@ -3383,7 +3382,7 @@
       <c r="I10">
         <v>999999999</v>
       </c>
-      <c r="J10" s="23">
+      <c r="J10" s="22">
         <v>1235</v>
       </c>
       <c r="K10">
@@ -3392,19 +3391,19 @@
       <c r="L10">
         <v>0</v>
       </c>
-      <c r="M10" s="23">
+      <c r="M10" s="22">
         <v>485</v>
       </c>
-      <c r="N10" s="23">
+      <c r="N10" s="22">
         <v>280</v>
       </c>
-      <c r="O10" s="23">
+      <c r="O10" s="22">
         <v>15000</v>
       </c>
       <c r="P10">
         <v>0</v>
       </c>
-      <c r="Q10" s="23">
+      <c r="Q10" s="22">
         <v>47673</v>
       </c>
       <c r="R10">
@@ -3439,7 +3438,7 @@
       <c r="A11" s="14">
         <v>2033</v>
       </c>
-      <c r="B11" s="23">
+      <c r="B11" s="22">
         <v>2024431</v>
       </c>
       <c r="C11" s="15">
@@ -3448,7 +3447,7 @@
       <c r="D11" s="15">
         <v>58100000</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11" s="22">
         <v>860748</v>
       </c>
       <c r="F11" s="15">
@@ -3463,7 +3462,7 @@
       <c r="I11">
         <v>999999999</v>
       </c>
-      <c r="J11" s="23">
+      <c r="J11" s="22">
         <v>1235</v>
       </c>
       <c r="K11">
@@ -3472,19 +3471,19 @@
       <c r="L11">
         <v>0</v>
       </c>
-      <c r="M11" s="23">
+      <c r="M11" s="22">
         <v>485</v>
       </c>
-      <c r="N11" s="23">
+      <c r="N11" s="22">
         <v>280</v>
       </c>
-      <c r="O11" s="23">
+      <c r="O11" s="22">
         <v>15000</v>
       </c>
       <c r="P11">
         <v>0</v>
       </c>
-      <c r="Q11" s="23">
+      <c r="Q11" s="22">
         <v>47673</v>
       </c>
       <c r="R11">
@@ -3519,7 +3518,7 @@
       <c r="A12" s="14">
         <v>2034</v>
       </c>
-      <c r="B12" s="23">
+      <c r="B12" s="22">
         <v>2024431</v>
       </c>
       <c r="C12" s="15">
@@ -3528,7 +3527,7 @@
       <c r="D12" s="15">
         <v>58100000</v>
       </c>
-      <c r="E12" s="23">
+      <c r="E12" s="22">
         <v>860748</v>
       </c>
       <c r="F12" s="15">
@@ -3543,7 +3542,7 @@
       <c r="I12">
         <v>999999999</v>
       </c>
-      <c r="J12" s="23">
+      <c r="J12" s="22">
         <v>1235</v>
       </c>
       <c r="K12">
@@ -3552,19 +3551,19 @@
       <c r="L12">
         <v>0</v>
       </c>
-      <c r="M12" s="23">
+      <c r="M12" s="22">
         <v>485</v>
       </c>
-      <c r="N12" s="23">
+      <c r="N12" s="22">
         <v>280</v>
       </c>
-      <c r="O12" s="23">
+      <c r="O12" s="22">
         <v>15000</v>
       </c>
       <c r="P12">
         <v>0</v>
       </c>
-      <c r="Q12" s="23">
+      <c r="Q12" s="22">
         <v>47673</v>
       </c>
       <c r="R12">
@@ -3599,7 +3598,7 @@
       <c r="A13" s="14">
         <v>2035</v>
       </c>
-      <c r="B13" s="23">
+      <c r="B13" s="22">
         <v>2024431</v>
       </c>
       <c r="C13" s="15">
@@ -3608,7 +3607,7 @@
       <c r="D13" s="15">
         <v>58100000</v>
       </c>
-      <c r="E13" s="23">
+      <c r="E13" s="22">
         <v>860748</v>
       </c>
       <c r="F13" s="15">
@@ -3623,7 +3622,7 @@
       <c r="I13">
         <v>999999999</v>
       </c>
-      <c r="J13" s="23">
+      <c r="J13" s="22">
         <v>1235</v>
       </c>
       <c r="K13">
@@ -3632,19 +3631,19 @@
       <c r="L13">
         <v>0</v>
       </c>
-      <c r="M13" s="23">
+      <c r="M13" s="22">
         <v>485</v>
       </c>
-      <c r="N13" s="23">
+      <c r="N13" s="22">
         <v>280</v>
       </c>
-      <c r="O13" s="23">
+      <c r="O13" s="22">
         <v>15000</v>
       </c>
       <c r="P13">
         <v>0</v>
       </c>
-      <c r="Q13" s="23">
+      <c r="Q13" s="22">
         <v>47673</v>
       </c>
       <c r="R13">
@@ -3679,7 +3678,7 @@
       <c r="A14" s="14">
         <v>2036</v>
       </c>
-      <c r="B14" s="23">
+      <c r="B14" s="22">
         <v>2024431</v>
       </c>
       <c r="C14" s="15">
@@ -3688,7 +3687,7 @@
       <c r="D14" s="15">
         <v>58100000</v>
       </c>
-      <c r="E14" s="23">
+      <c r="E14" s="22">
         <v>860748</v>
       </c>
       <c r="F14" s="15">
@@ -3703,7 +3702,7 @@
       <c r="I14">
         <v>999999999</v>
       </c>
-      <c r="J14" s="23">
+      <c r="J14" s="22">
         <v>1235</v>
       </c>
       <c r="K14">
@@ -3712,19 +3711,19 @@
       <c r="L14">
         <v>0</v>
       </c>
-      <c r="M14" s="23">
+      <c r="M14" s="22">
         <v>485</v>
       </c>
-      <c r="N14" s="23">
+      <c r="N14" s="22">
         <v>280</v>
       </c>
-      <c r="O14" s="23">
+      <c r="O14" s="22">
         <v>15000</v>
       </c>
       <c r="P14">
         <v>0</v>
       </c>
-      <c r="Q14" s="23">
+      <c r="Q14" s="22">
         <v>47673</v>
       </c>
       <c r="R14">
@@ -3759,7 +3758,7 @@
       <c r="A15" s="14">
         <v>2037</v>
       </c>
-      <c r="B15" s="23">
+      <c r="B15" s="22">
         <v>2024431</v>
       </c>
       <c r="C15" s="15">
@@ -3768,7 +3767,7 @@
       <c r="D15" s="15">
         <v>58100000</v>
       </c>
-      <c r="E15" s="23">
+      <c r="E15" s="22">
         <v>860748</v>
       </c>
       <c r="F15" s="15">
@@ -3783,7 +3782,7 @@
       <c r="I15">
         <v>999999999</v>
       </c>
-      <c r="J15" s="23">
+      <c r="J15" s="22">
         <v>1235</v>
       </c>
       <c r="K15">
@@ -3792,19 +3791,19 @@
       <c r="L15">
         <v>0</v>
       </c>
-      <c r="M15" s="23">
+      <c r="M15" s="22">
         <v>485</v>
       </c>
-      <c r="N15" s="23">
+      <c r="N15" s="22">
         <v>280</v>
       </c>
-      <c r="O15" s="23">
+      <c r="O15" s="22">
         <v>15000</v>
       </c>
       <c r="P15">
         <v>0</v>
       </c>
-      <c r="Q15" s="23">
+      <c r="Q15" s="22">
         <v>47673</v>
       </c>
       <c r="R15">
@@ -3839,7 +3838,7 @@
       <c r="A16" s="14">
         <v>2038</v>
       </c>
-      <c r="B16" s="23">
+      <c r="B16" s="22">
         <v>2024431</v>
       </c>
       <c r="C16" s="15">
@@ -3848,7 +3847,7 @@
       <c r="D16" s="15">
         <v>58100000</v>
       </c>
-      <c r="E16" s="23">
+      <c r="E16" s="22">
         <v>860748</v>
       </c>
       <c r="F16" s="15">
@@ -3863,7 +3862,7 @@
       <c r="I16">
         <v>999999999</v>
       </c>
-      <c r="J16" s="23">
+      <c r="J16" s="22">
         <v>1235</v>
       </c>
       <c r="K16">
@@ -3872,19 +3871,19 @@
       <c r="L16">
         <v>0</v>
       </c>
-      <c r="M16" s="23">
+      <c r="M16" s="22">
         <v>485</v>
       </c>
-      <c r="N16" s="23">
+      <c r="N16" s="22">
         <v>280</v>
       </c>
-      <c r="O16" s="23">
+      <c r="O16" s="22">
         <v>15000</v>
       </c>
       <c r="P16">
         <v>0</v>
       </c>
-      <c r="Q16" s="23">
+      <c r="Q16" s="22">
         <v>47673</v>
       </c>
       <c r="R16">
@@ -3919,7 +3918,7 @@
       <c r="A17" s="14">
         <v>2039</v>
       </c>
-      <c r="B17" s="23">
+      <c r="B17" s="22">
         <v>2024431</v>
       </c>
       <c r="C17" s="15">
@@ -3928,7 +3927,7 @@
       <c r="D17" s="15">
         <v>58100000</v>
       </c>
-      <c r="E17" s="23">
+      <c r="E17" s="22">
         <v>860748</v>
       </c>
       <c r="F17" s="15">
@@ -3943,7 +3942,7 @@
       <c r="I17">
         <v>999999999</v>
       </c>
-      <c r="J17" s="23">
+      <c r="J17" s="22">
         <v>1235</v>
       </c>
       <c r="K17">
@@ -3952,19 +3951,19 @@
       <c r="L17">
         <v>0</v>
       </c>
-      <c r="M17" s="23">
+      <c r="M17" s="22">
         <v>485</v>
       </c>
-      <c r="N17" s="23">
+      <c r="N17" s="22">
         <v>280</v>
       </c>
-      <c r="O17" s="23">
+      <c r="O17" s="22">
         <v>15000</v>
       </c>
       <c r="P17">
         <v>0</v>
       </c>
-      <c r="Q17" s="23">
+      <c r="Q17" s="22">
         <v>47673</v>
       </c>
       <c r="R17">
@@ -3999,7 +3998,7 @@
       <c r="A18" s="14">
         <v>2040</v>
       </c>
-      <c r="B18" s="23">
+      <c r="B18" s="22">
         <v>2024431</v>
       </c>
       <c r="C18" s="15">
@@ -4008,7 +4007,7 @@
       <c r="D18" s="15">
         <v>58100000</v>
       </c>
-      <c r="E18" s="23">
+      <c r="E18" s="22">
         <v>860748</v>
       </c>
       <c r="F18" s="15">
@@ -4023,7 +4022,7 @@
       <c r="I18">
         <v>999999999</v>
       </c>
-      <c r="J18" s="23">
+      <c r="J18" s="22">
         <v>1235</v>
       </c>
       <c r="K18">
@@ -4032,19 +4031,19 @@
       <c r="L18">
         <v>0</v>
       </c>
-      <c r="M18" s="23">
+      <c r="M18" s="22">
         <v>485</v>
       </c>
-      <c r="N18" s="23">
+      <c r="N18" s="22">
         <v>280</v>
       </c>
-      <c r="O18" s="23">
+      <c r="O18" s="22">
         <v>15000</v>
       </c>
       <c r="P18">
         <v>0</v>
       </c>
-      <c r="Q18" s="23">
+      <c r="Q18" s="22">
         <v>47673</v>
       </c>
       <c r="R18">
@@ -4079,7 +4078,7 @@
       <c r="A19" s="14">
         <v>2041</v>
       </c>
-      <c r="B19" s="23">
+      <c r="B19" s="22">
         <v>2024431</v>
       </c>
       <c r="C19" s="15">
@@ -4088,7 +4087,7 @@
       <c r="D19" s="15">
         <v>58100000</v>
       </c>
-      <c r="E19" s="23">
+      <c r="E19" s="22">
         <v>860748</v>
       </c>
       <c r="F19" s="15">
@@ -4103,7 +4102,7 @@
       <c r="I19">
         <v>999999999</v>
       </c>
-      <c r="J19" s="23">
+      <c r="J19" s="22">
         <v>1235</v>
       </c>
       <c r="K19">
@@ -4112,19 +4111,19 @@
       <c r="L19">
         <v>0</v>
       </c>
-      <c r="M19" s="23">
+      <c r="M19" s="22">
         <v>485</v>
       </c>
-      <c r="N19" s="23">
+      <c r="N19" s="22">
         <v>280</v>
       </c>
-      <c r="O19" s="23">
+      <c r="O19" s="22">
         <v>15000</v>
       </c>
       <c r="P19">
         <v>0</v>
       </c>
-      <c r="Q19" s="23">
+      <c r="Q19" s="22">
         <v>47673</v>
       </c>
       <c r="R19">
@@ -4159,7 +4158,7 @@
       <c r="A20" s="14">
         <v>2042</v>
       </c>
-      <c r="B20" s="23">
+      <c r="B20" s="22">
         <v>2024431</v>
       </c>
       <c r="C20" s="15">
@@ -4168,7 +4167,7 @@
       <c r="D20" s="15">
         <v>58100000</v>
       </c>
-      <c r="E20" s="23">
+      <c r="E20" s="22">
         <v>860748</v>
       </c>
       <c r="F20" s="15">
@@ -4183,7 +4182,7 @@
       <c r="I20">
         <v>999999999</v>
       </c>
-      <c r="J20" s="23">
+      <c r="J20" s="22">
         <v>1235</v>
       </c>
       <c r="K20">
@@ -4192,19 +4191,19 @@
       <c r="L20">
         <v>0</v>
       </c>
-      <c r="M20" s="23">
+      <c r="M20" s="22">
         <v>485</v>
       </c>
-      <c r="N20" s="23">
+      <c r="N20" s="22">
         <v>280</v>
       </c>
-      <c r="O20" s="23">
+      <c r="O20" s="22">
         <v>15000</v>
       </c>
       <c r="P20">
         <v>0</v>
       </c>
-      <c r="Q20" s="23">
+      <c r="Q20" s="22">
         <v>47673</v>
       </c>
       <c r="R20">
@@ -4239,7 +4238,7 @@
       <c r="A21" s="14">
         <v>2043</v>
       </c>
-      <c r="B21" s="23">
+      <c r="B21" s="22">
         <v>2024431</v>
       </c>
       <c r="C21" s="15">
@@ -4248,7 +4247,7 @@
       <c r="D21" s="15">
         <v>58100000</v>
       </c>
-      <c r="E21" s="23">
+      <c r="E21" s="22">
         <v>860748</v>
       </c>
       <c r="F21" s="15">
@@ -4263,7 +4262,7 @@
       <c r="I21">
         <v>999999999</v>
       </c>
-      <c r="J21" s="23">
+      <c r="J21" s="22">
         <v>1235</v>
       </c>
       <c r="K21">
@@ -4272,19 +4271,19 @@
       <c r="L21">
         <v>0</v>
       </c>
-      <c r="M21" s="23">
+      <c r="M21" s="22">
         <v>485</v>
       </c>
-      <c r="N21" s="23">
+      <c r="N21" s="22">
         <v>280</v>
       </c>
-      <c r="O21" s="23">
+      <c r="O21" s="22">
         <v>15000</v>
       </c>
       <c r="P21">
         <v>0</v>
       </c>
-      <c r="Q21" s="23">
+      <c r="Q21" s="22">
         <v>47673</v>
       </c>
       <c r="R21">
@@ -4319,7 +4318,7 @@
       <c r="A22" s="14">
         <v>2044</v>
       </c>
-      <c r="B22" s="23">
+      <c r="B22" s="22">
         <v>2024431</v>
       </c>
       <c r="C22" s="15">
@@ -4328,7 +4327,7 @@
       <c r="D22" s="15">
         <v>58100000</v>
       </c>
-      <c r="E22" s="23">
+      <c r="E22" s="22">
         <v>860748</v>
       </c>
       <c r="F22" s="15">
@@ -4343,7 +4342,7 @@
       <c r="I22">
         <v>999999999</v>
       </c>
-      <c r="J22" s="23">
+      <c r="J22" s="22">
         <v>1235</v>
       </c>
       <c r="K22">
@@ -4352,19 +4351,19 @@
       <c r="L22">
         <v>0</v>
       </c>
-      <c r="M22" s="23">
+      <c r="M22" s="22">
         <v>485</v>
       </c>
-      <c r="N22" s="23">
+      <c r="N22" s="22">
         <v>280</v>
       </c>
-      <c r="O22" s="23">
+      <c r="O22" s="22">
         <v>15000</v>
       </c>
       <c r="P22">
         <v>0</v>
       </c>
-      <c r="Q22" s="23">
+      <c r="Q22" s="22">
         <v>47673</v>
       </c>
       <c r="R22">
@@ -4399,7 +4398,7 @@
       <c r="A23" s="14">
         <v>2045</v>
       </c>
-      <c r="B23" s="23">
+      <c r="B23" s="22">
         <v>2024431</v>
       </c>
       <c r="C23" s="15">
@@ -4408,7 +4407,7 @@
       <c r="D23" s="15">
         <v>58100000</v>
       </c>
-      <c r="E23" s="23">
+      <c r="E23" s="22">
         <v>860748</v>
       </c>
       <c r="F23" s="15">
@@ -4423,7 +4422,7 @@
       <c r="I23">
         <v>999999999</v>
       </c>
-      <c r="J23" s="23">
+      <c r="J23" s="22">
         <v>1235</v>
       </c>
       <c r="K23">
@@ -4432,19 +4431,19 @@
       <c r="L23">
         <v>0</v>
       </c>
-      <c r="M23" s="23">
+      <c r="M23" s="22">
         <v>485</v>
       </c>
-      <c r="N23" s="23">
+      <c r="N23" s="22">
         <v>280</v>
       </c>
-      <c r="O23" s="23">
+      <c r="O23" s="22">
         <v>15000</v>
       </c>
       <c r="P23">
         <v>0</v>
       </c>
-      <c r="Q23" s="23">
+      <c r="Q23" s="22">
         <v>47673</v>
       </c>
       <c r="R23">
@@ -4479,7 +4478,7 @@
       <c r="A24" s="14">
         <v>2046</v>
       </c>
-      <c r="B24" s="23">
+      <c r="B24" s="22">
         <v>2024431</v>
       </c>
       <c r="C24" s="15">
@@ -4488,7 +4487,7 @@
       <c r="D24" s="15">
         <v>58100000</v>
       </c>
-      <c r="E24" s="23">
+      <c r="E24" s="22">
         <v>860748</v>
       </c>
       <c r="F24" s="15">
@@ -4503,7 +4502,7 @@
       <c r="I24">
         <v>999999999</v>
       </c>
-      <c r="J24" s="23">
+      <c r="J24" s="22">
         <v>1235</v>
       </c>
       <c r="K24">
@@ -4512,19 +4511,19 @@
       <c r="L24">
         <v>0</v>
       </c>
-      <c r="M24" s="23">
+      <c r="M24" s="22">
         <v>485</v>
       </c>
-      <c r="N24" s="23">
+      <c r="N24" s="22">
         <v>280</v>
       </c>
-      <c r="O24" s="23">
+      <c r="O24" s="22">
         <v>15000</v>
       </c>
       <c r="P24">
         <v>0</v>
       </c>
-      <c r="Q24" s="23">
+      <c r="Q24" s="22">
         <v>47673</v>
       </c>
       <c r="R24">
@@ -4559,7 +4558,7 @@
       <c r="A25" s="14">
         <v>2047</v>
       </c>
-      <c r="B25" s="23">
+      <c r="B25" s="22">
         <v>2024431</v>
       </c>
       <c r="C25" s="15">
@@ -4568,7 +4567,7 @@
       <c r="D25" s="15">
         <v>58100000</v>
       </c>
-      <c r="E25" s="23">
+      <c r="E25" s="22">
         <v>860748</v>
       </c>
       <c r="F25" s="15">
@@ -4583,7 +4582,7 @@
       <c r="I25">
         <v>999999999</v>
       </c>
-      <c r="J25" s="23">
+      <c r="J25" s="22">
         <v>1235</v>
       </c>
       <c r="K25">
@@ -4592,19 +4591,19 @@
       <c r="L25">
         <v>0</v>
       </c>
-      <c r="M25" s="23">
+      <c r="M25" s="22">
         <v>485</v>
       </c>
-      <c r="N25" s="23">
+      <c r="N25" s="22">
         <v>280</v>
       </c>
-      <c r="O25" s="23">
+      <c r="O25" s="22">
         <v>15000</v>
       </c>
       <c r="P25">
         <v>0</v>
       </c>
-      <c r="Q25" s="23">
+      <c r="Q25" s="22">
         <v>47673</v>
       </c>
       <c r="R25">
@@ -4639,7 +4638,7 @@
       <c r="A26" s="14">
         <v>2048</v>
       </c>
-      <c r="B26" s="23">
+      <c r="B26" s="22">
         <v>2024431</v>
       </c>
       <c r="C26" s="15">
@@ -4648,7 +4647,7 @@
       <c r="D26" s="15">
         <v>58100000</v>
       </c>
-      <c r="E26" s="23">
+      <c r="E26" s="22">
         <v>860748</v>
       </c>
       <c r="F26" s="15">
@@ -4663,7 +4662,7 @@
       <c r="I26">
         <v>999999999</v>
       </c>
-      <c r="J26" s="23">
+      <c r="J26" s="22">
         <v>1235</v>
       </c>
       <c r="K26">
@@ -4672,19 +4671,19 @@
       <c r="L26">
         <v>0</v>
       </c>
-      <c r="M26" s="23">
+      <c r="M26" s="22">
         <v>485</v>
       </c>
-      <c r="N26" s="23">
+      <c r="N26" s="22">
         <v>280</v>
       </c>
-      <c r="O26" s="23">
+      <c r="O26" s="22">
         <v>15000</v>
       </c>
       <c r="P26">
         <v>0</v>
       </c>
-      <c r="Q26" s="23">
+      <c r="Q26" s="22">
         <v>47673</v>
       </c>
       <c r="R26">
@@ -4719,7 +4718,7 @@
       <c r="A27" s="14">
         <v>2049</v>
       </c>
-      <c r="B27" s="23">
+      <c r="B27" s="22">
         <v>2024431</v>
       </c>
       <c r="C27" s="15">
@@ -4728,7 +4727,7 @@
       <c r="D27" s="15">
         <v>58100000</v>
       </c>
-      <c r="E27" s="23">
+      <c r="E27" s="22">
         <v>860748</v>
       </c>
       <c r="F27" s="15">
@@ -4743,7 +4742,7 @@
       <c r="I27">
         <v>999999999</v>
       </c>
-      <c r="J27" s="23">
+      <c r="J27" s="22">
         <v>1235</v>
       </c>
       <c r="K27">
@@ -4752,19 +4751,19 @@
       <c r="L27">
         <v>0</v>
       </c>
-      <c r="M27" s="23">
+      <c r="M27" s="22">
         <v>485</v>
       </c>
-      <c r="N27" s="23">
+      <c r="N27" s="22">
         <v>280</v>
       </c>
-      <c r="O27" s="23">
+      <c r="O27" s="22">
         <v>15000</v>
       </c>
       <c r="P27">
         <v>0</v>
       </c>
-      <c r="Q27" s="23">
+      <c r="Q27" s="22">
         <v>47673</v>
       </c>
       <c r="R27">
@@ -4799,7 +4798,7 @@
       <c r="A28" s="14">
         <v>2050</v>
       </c>
-      <c r="B28" s="23">
+      <c r="B28" s="22">
         <v>2024431</v>
       </c>
       <c r="C28" s="15">
@@ -4808,7 +4807,7 @@
       <c r="D28" s="15">
         <v>58100000</v>
       </c>
-      <c r="E28" s="23">
+      <c r="E28" s="22">
         <v>860748</v>
       </c>
       <c r="F28" s="15">
@@ -4823,7 +4822,7 @@
       <c r="I28">
         <v>999999999</v>
       </c>
-      <c r="J28" s="23">
+      <c r="J28" s="22">
         <v>1235</v>
       </c>
       <c r="K28">
@@ -4832,19 +4831,19 @@
       <c r="L28">
         <v>0</v>
       </c>
-      <c r="M28" s="23">
+      <c r="M28" s="22">
         <v>485</v>
       </c>
-      <c r="N28" s="23">
+      <c r="N28" s="22">
         <v>280</v>
       </c>
-      <c r="O28" s="23">
+      <c r="O28" s="22">
         <v>15000</v>
       </c>
       <c r="P28">
         <v>0</v>
       </c>
-      <c r="Q28" s="23">
+      <c r="Q28" s="22">
         <v>47673</v>
       </c>
       <c r="R28">
@@ -26198,7 +26197,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="22">
+      <c r="A2" s="23">
         <v>2024</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -26212,7 +26211,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="22"/>
+      <c r="A3" s="23"/>
       <c r="B3" s="11" t="s">
         <v>70</v>
       </c>
@@ -26225,7 +26224,7 @@
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="22"/>
+      <c r="A4" s="23"/>
       <c r="B4" s="11" t="s">
         <v>71</v>
       </c>
@@ -26237,7 +26236,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="22"/>
+      <c r="A5" s="23"/>
       <c r="B5" s="11" t="s">
         <v>68</v>
       </c>
@@ -26249,7 +26248,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="22">
+      <c r="A6" s="23">
         <v>2025</v>
       </c>
       <c r="B6" s="11" t="s">
@@ -26263,7 +26262,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="22"/>
+      <c r="A7" s="23"/>
       <c r="B7" s="11" t="s">
         <v>70</v>
       </c>
@@ -26275,7 +26274,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="22"/>
+      <c r="A8" s="23"/>
       <c r="B8" s="11" t="s">
         <v>71</v>
       </c>
@@ -26287,7 +26286,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="22"/>
+      <c r="A9" s="23"/>
       <c r="B9" s="11" t="s">
         <v>68</v>
       </c>
@@ -26300,7 +26299,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="22">
+      <c r="A10" s="23">
         <v>2026</v>
       </c>
       <c r="B10" s="11" t="s">
@@ -26314,7 +26313,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="22"/>
+      <c r="A11" s="23"/>
       <c r="B11" s="11" t="s">
         <v>70</v>
       </c>
@@ -26326,7 +26325,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="22"/>
+      <c r="A12" s="23"/>
       <c r="B12" s="11" t="s">
         <v>71</v>
       </c>
@@ -26338,7 +26337,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="22"/>
+      <c r="A13" s="23"/>
       <c r="B13" s="11" t="s">
         <v>68</v>
       </c>
@@ -26351,7 +26350,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="22">
+      <c r="A14" s="23">
         <v>2027</v>
       </c>
       <c r="B14" s="11" t="s">
@@ -26365,7 +26364,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="22"/>
+      <c r="A15" s="23"/>
       <c r="B15" s="11" t="s">
         <v>70</v>
       </c>
@@ -26377,7 +26376,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="22"/>
+      <c r="A16" s="23"/>
       <c r="B16" s="11" t="s">
         <v>71</v>
       </c>
@@ -26389,7 +26388,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="22"/>
+      <c r="A17" s="23"/>
       <c r="B17" s="11" t="s">
         <v>68</v>
       </c>
@@ -26402,7 +26401,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="22">
+      <c r="A18" s="23">
         <v>2028</v>
       </c>
       <c r="B18" s="11" t="s">
@@ -26416,7 +26415,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="22"/>
+      <c r="A19" s="23"/>
       <c r="B19" s="11" t="s">
         <v>70</v>
       </c>
@@ -26428,7 +26427,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="22"/>
+      <c r="A20" s="23"/>
       <c r="B20" s="11" t="s">
         <v>71</v>
       </c>
@@ -26440,7 +26439,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="22"/>
+      <c r="A21" s="23"/>
       <c r="B21" s="11" t="s">
         <v>68</v>
       </c>
@@ -26453,7 +26452,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="22">
+      <c r="A22" s="23">
         <v>2029</v>
       </c>
       <c r="B22" s="11" t="s">
@@ -26467,7 +26466,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="22"/>
+      <c r="A23" s="23"/>
       <c r="B23" s="11" t="s">
         <v>70</v>
       </c>
@@ -26479,7 +26478,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="22"/>
+      <c r="A24" s="23"/>
       <c r="B24" s="11" t="s">
         <v>71</v>
       </c>
@@ -26491,7 +26490,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="22"/>
+      <c r="A25" s="23"/>
       <c r="B25" s="11" t="s">
         <v>68</v>
       </c>
@@ -26504,7 +26503,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="22">
+      <c r="A26" s="23">
         <v>2030</v>
       </c>
       <c r="B26" s="11" t="s">
@@ -26518,7 +26517,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="22"/>
+      <c r="A27" s="23"/>
       <c r="B27" s="11" t="s">
         <v>70</v>
       </c>
@@ -26530,7 +26529,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="22"/>
+      <c r="A28" s="23"/>
       <c r="B28" s="11" t="s">
         <v>71</v>
       </c>
@@ -26542,7 +26541,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="22"/>
+      <c r="A29" s="23"/>
       <c r="B29" s="11" t="s">
         <v>68</v>
       </c>
@@ -26555,7 +26554,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="22">
+      <c r="A30" s="23">
         <v>2031</v>
       </c>
       <c r="B30" s="11" t="s">
@@ -26569,7 +26568,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="22"/>
+      <c r="A31" s="23"/>
       <c r="B31" s="11" t="s">
         <v>70</v>
       </c>
@@ -26581,7 +26580,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="22"/>
+      <c r="A32" s="23"/>
       <c r="B32" s="11" t="s">
         <v>71</v>
       </c>
@@ -26593,7 +26592,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="22"/>
+      <c r="A33" s="23"/>
       <c r="B33" s="11" t="s">
         <v>68</v>
       </c>
@@ -26606,7 +26605,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="22">
+      <c r="A34" s="23">
         <v>2032</v>
       </c>
       <c r="B34" s="11" t="s">
@@ -26620,7 +26619,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="22"/>
+      <c r="A35" s="23"/>
       <c r="B35" s="11" t="s">
         <v>70</v>
       </c>
@@ -26632,7 +26631,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="22"/>
+      <c r="A36" s="23"/>
       <c r="B36" s="11" t="s">
         <v>71</v>
       </c>
@@ -26644,7 +26643,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="22"/>
+      <c r="A37" s="23"/>
       <c r="B37" s="11" t="s">
         <v>68</v>
       </c>
@@ -26657,7 +26656,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="22">
+      <c r="A38" s="23">
         <v>2033</v>
       </c>
       <c r="B38" s="11" t="s">
@@ -26671,7 +26670,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="22"/>
+      <c r="A39" s="23"/>
       <c r="B39" s="11" t="s">
         <v>70</v>
       </c>
@@ -26683,7 +26682,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="22"/>
+      <c r="A40" s="23"/>
       <c r="B40" s="11" t="s">
         <v>71</v>
       </c>
@@ -26695,7 +26694,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="22"/>
+      <c r="A41" s="23"/>
       <c r="B41" s="11" t="s">
         <v>68</v>
       </c>
@@ -26708,7 +26707,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="22">
+      <c r="A42" s="23">
         <v>2034</v>
       </c>
       <c r="B42" s="11" t="s">
@@ -26722,7 +26721,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="22"/>
+      <c r="A43" s="23"/>
       <c r="B43" s="11" t="s">
         <v>70</v>
       </c>
@@ -26734,7 +26733,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="22"/>
+      <c r="A44" s="23"/>
       <c r="B44" s="11" t="s">
         <v>71</v>
       </c>
@@ -26746,7 +26745,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="22"/>
+      <c r="A45" s="23"/>
       <c r="B45" s="11" t="s">
         <v>68</v>
       </c>
@@ -26759,7 +26758,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="22">
+      <c r="A46" s="23">
         <v>2035</v>
       </c>
       <c r="B46" s="11" t="s">
@@ -26773,7 +26772,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="22"/>
+      <c r="A47" s="23"/>
       <c r="B47" s="11" t="s">
         <v>70</v>
       </c>
@@ -26785,7 +26784,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="22"/>
+      <c r="A48" s="23"/>
       <c r="B48" s="11" t="s">
         <v>71</v>
       </c>
@@ -26797,7 +26796,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="22"/>
+      <c r="A49" s="23"/>
       <c r="B49" s="11" t="s">
         <v>68</v>
       </c>
@@ -26810,7 +26809,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="22">
+      <c r="A50" s="23">
         <v>2036</v>
       </c>
       <c r="B50" s="11" t="s">
@@ -26824,7 +26823,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="22"/>
+      <c r="A51" s="23"/>
       <c r="B51" s="11" t="s">
         <v>70</v>
       </c>
@@ -26836,7 +26835,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="22"/>
+      <c r="A52" s="23"/>
       <c r="B52" s="11" t="s">
         <v>71</v>
       </c>
@@ -26848,7 +26847,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="22"/>
+      <c r="A53" s="23"/>
       <c r="B53" s="11" t="s">
         <v>68</v>
       </c>
@@ -26861,7 +26860,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="22">
+      <c r="A54" s="23">
         <v>2037</v>
       </c>
       <c r="B54" s="11" t="s">
@@ -26875,7 +26874,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="22"/>
+      <c r="A55" s="23"/>
       <c r="B55" s="11" t="s">
         <v>70</v>
       </c>
@@ -26887,7 +26886,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="22"/>
+      <c r="A56" s="23"/>
       <c r="B56" s="11" t="s">
         <v>71</v>
       </c>
@@ -26899,7 +26898,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="22"/>
+      <c r="A57" s="23"/>
       <c r="B57" s="11" t="s">
         <v>68</v>
       </c>
@@ -26912,7 +26911,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="22">
+      <c r="A58" s="23">
         <v>2038</v>
       </c>
       <c r="B58" s="11" t="s">
@@ -26926,7 +26925,7 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="22"/>
+      <c r="A59" s="23"/>
       <c r="B59" s="11" t="s">
         <v>70</v>
       </c>
@@ -26938,7 +26937,7 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="22"/>
+      <c r="A60" s="23"/>
       <c r="B60" s="11" t="s">
         <v>71</v>
       </c>
@@ -26950,7 +26949,7 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="22"/>
+      <c r="A61" s="23"/>
       <c r="B61" s="11" t="s">
         <v>68</v>
       </c>
@@ -26963,7 +26962,7 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="22">
+      <c r="A62" s="23">
         <v>2039</v>
       </c>
       <c r="B62" s="11" t="s">
@@ -26977,7 +26976,7 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="22"/>
+      <c r="A63" s="23"/>
       <c r="B63" s="11" t="s">
         <v>70</v>
       </c>
@@ -26989,7 +26988,7 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="22"/>
+      <c r="A64" s="23"/>
       <c r="B64" s="11" t="s">
         <v>71</v>
       </c>
@@ -27001,7 +27000,7 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="22"/>
+      <c r="A65" s="23"/>
       <c r="B65" s="11" t="s">
         <v>68</v>
       </c>
@@ -27014,7 +27013,7 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="22">
+      <c r="A66" s="23">
         <v>2040</v>
       </c>
       <c r="B66" s="11" t="s">
@@ -27028,7 +27027,7 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="22"/>
+      <c r="A67" s="23"/>
       <c r="B67" s="11" t="s">
         <v>70</v>
       </c>
@@ -27040,7 +27039,7 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="22"/>
+      <c r="A68" s="23"/>
       <c r="B68" s="11" t="s">
         <v>71</v>
       </c>
@@ -27052,7 +27051,7 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="22"/>
+      <c r="A69" s="23"/>
       <c r="B69" s="11" t="s">
         <v>68</v>
       </c>
@@ -27065,7 +27064,7 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="22">
+      <c r="A70" s="23">
         <v>2041</v>
       </c>
       <c r="B70" s="11" t="s">
@@ -27079,7 +27078,7 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="22"/>
+      <c r="A71" s="23"/>
       <c r="B71" s="11" t="s">
         <v>70</v>
       </c>
@@ -27091,7 +27090,7 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="22"/>
+      <c r="A72" s="23"/>
       <c r="B72" s="11" t="s">
         <v>71</v>
       </c>
@@ -27103,7 +27102,7 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="22"/>
+      <c r="A73" s="23"/>
       <c r="B73" s="11" t="s">
         <v>68</v>
       </c>
@@ -27116,7 +27115,7 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="22">
+      <c r="A74" s="23">
         <v>2042</v>
       </c>
       <c r="B74" s="11" t="s">
@@ -27130,7 +27129,7 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="22"/>
+      <c r="A75" s="23"/>
       <c r="B75" s="11" t="s">
         <v>70</v>
       </c>
@@ -27142,7 +27141,7 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="22"/>
+      <c r="A76" s="23"/>
       <c r="B76" s="11" t="s">
         <v>71</v>
       </c>
@@ -27154,7 +27153,7 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="22"/>
+      <c r="A77" s="23"/>
       <c r="B77" s="11" t="s">
         <v>68</v>
       </c>
@@ -27167,7 +27166,7 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="22">
+      <c r="A78" s="23">
         <v>2043</v>
       </c>
       <c r="B78" s="11" t="s">
@@ -27181,7 +27180,7 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="22"/>
+      <c r="A79" s="23"/>
       <c r="B79" s="11" t="s">
         <v>70</v>
       </c>
@@ -27193,7 +27192,7 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="22"/>
+      <c r="A80" s="23"/>
       <c r="B80" s="11" t="s">
         <v>71</v>
       </c>
@@ -27205,7 +27204,7 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="22"/>
+      <c r="A81" s="23"/>
       <c r="B81" s="11" t="s">
         <v>68</v>
       </c>
@@ -27218,7 +27217,7 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="22">
+      <c r="A82" s="23">
         <v>2044</v>
       </c>
       <c r="B82" s="11" t="s">
@@ -27232,7 +27231,7 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="22"/>
+      <c r="A83" s="23"/>
       <c r="B83" s="11" t="s">
         <v>70</v>
       </c>
@@ -27244,7 +27243,7 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="22"/>
+      <c r="A84" s="23"/>
       <c r="B84" s="11" t="s">
         <v>71</v>
       </c>
@@ -27256,7 +27255,7 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="22"/>
+      <c r="A85" s="23"/>
       <c r="B85" s="11" t="s">
         <v>68</v>
       </c>
@@ -27269,7 +27268,7 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="22">
+      <c r="A86" s="23">
         <v>2045</v>
       </c>
       <c r="B86" s="11" t="s">
@@ -27283,7 +27282,7 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="22"/>
+      <c r="A87" s="23"/>
       <c r="B87" s="11" t="s">
         <v>70</v>
       </c>
@@ -27295,7 +27294,7 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="22"/>
+      <c r="A88" s="23"/>
       <c r="B88" s="11" t="s">
         <v>71</v>
       </c>
@@ -27307,7 +27306,7 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="22"/>
+      <c r="A89" s="23"/>
       <c r="B89" s="11" t="s">
         <v>68</v>
       </c>
@@ -27320,7 +27319,7 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="22">
+      <c r="A90" s="23">
         <v>2046</v>
       </c>
       <c r="B90" s="11" t="s">
@@ -27334,7 +27333,7 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="22"/>
+      <c r="A91" s="23"/>
       <c r="B91" s="11" t="s">
         <v>70</v>
       </c>
@@ -27346,7 +27345,7 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="22"/>
+      <c r="A92" s="23"/>
       <c r="B92" s="11" t="s">
         <v>71</v>
       </c>
@@ -27358,7 +27357,7 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="22"/>
+      <c r="A93" s="23"/>
       <c r="B93" s="11" t="s">
         <v>68</v>
       </c>
@@ -27371,7 +27370,7 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="22">
+      <c r="A94" s="23">
         <v>2047</v>
       </c>
       <c r="B94" s="11" t="s">
@@ -27385,7 +27384,7 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="22"/>
+      <c r="A95" s="23"/>
       <c r="B95" s="11" t="s">
         <v>70</v>
       </c>
@@ -27397,7 +27396,7 @@
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="22"/>
+      <c r="A96" s="23"/>
       <c r="B96" s="11" t="s">
         <v>71</v>
       </c>
@@ -27409,7 +27408,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="22"/>
+      <c r="A97" s="23"/>
       <c r="B97" s="11" t="s">
         <v>68</v>
       </c>
@@ -27422,7 +27421,7 @@
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="22">
+      <c r="A98" s="23">
         <v>2048</v>
       </c>
       <c r="B98" s="11" t="s">
@@ -27436,7 +27435,7 @@
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" s="22"/>
+      <c r="A99" s="23"/>
       <c r="B99" s="11" t="s">
         <v>70</v>
       </c>
@@ -27448,7 +27447,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="22"/>
+      <c r="A100" s="23"/>
       <c r="B100" s="11" t="s">
         <v>71</v>
       </c>
@@ -27460,7 +27459,7 @@
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" s="22"/>
+      <c r="A101" s="23"/>
       <c r="B101" s="11" t="s">
         <v>68</v>
       </c>
@@ -27473,7 +27472,7 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" s="22">
+      <c r="A102" s="23">
         <v>2049</v>
       </c>
       <c r="B102" s="11" t="s">
@@ -27487,7 +27486,7 @@
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A103" s="22"/>
+      <c r="A103" s="23"/>
       <c r="B103" s="11" t="s">
         <v>70</v>
       </c>
@@ -27499,7 +27498,7 @@
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="22"/>
+      <c r="A104" s="23"/>
       <c r="B104" s="11" t="s">
         <v>71</v>
       </c>
@@ -27511,7 +27510,7 @@
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="22"/>
+      <c r="A105" s="23"/>
       <c r="B105" s="11" t="s">
         <v>68</v>
       </c>
@@ -27524,7 +27523,7 @@
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" s="22">
+      <c r="A106" s="23">
         <v>2050</v>
       </c>
       <c r="B106" s="11" t="s">
@@ -27538,7 +27537,7 @@
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" s="22"/>
+      <c r="A107" s="23"/>
       <c r="B107" s="11" t="s">
         <v>70</v>
       </c>
@@ -27550,7 +27549,7 @@
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" s="22"/>
+      <c r="A108" s="23"/>
       <c r="B108" s="11" t="s">
         <v>71</v>
       </c>
@@ -27562,7 +27561,7 @@
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" s="22"/>
+      <c r="A109" s="23"/>
       <c r="B109" s="11" t="s">
         <v>68</v>
       </c>
@@ -27577,26 +27576,6 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -27604,6 +27583,26 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Applied EOS onto bulk prices
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1155" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{898C7E9C-83DA-4DD8-8EF3-751FB916CEA0}"/>
+  <xr:revisionPtr revIDLastSave="1170" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E7549D9-7045-45AC-8066-5808153A4E87}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="5" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -1699,6 +1699,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="25.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2593,10 +2594,10 @@
         <v>146</v>
       </c>
       <c r="D45">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E45">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F45">
         <v>0</v>
@@ -2613,10 +2614,10 @@
         <v>141</v>
       </c>
       <c r="D46">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E46">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F46">
         <v>0</v>
@@ -24384,10 +24385,10 @@
         <v>5</v>
       </c>
       <c r="P2" s="6">
-        <v>70.922028124999997</v>
+        <v>68.997492539999996</v>
       </c>
       <c r="Q2" s="6">
-        <v>70.922028124999997</v>
+        <v>68.997492539999996</v>
       </c>
       <c r="R2" s="13">
         <v>0.85</v>
@@ -24467,10 +24468,10 @@
         <v>5</v>
       </c>
       <c r="P3" s="6">
-        <v>171.04915999999997</v>
+        <v>6.4290486009999999</v>
       </c>
       <c r="Q3" s="6">
-        <v>171.04915999999997</v>
+        <v>6.4290486009999999</v>
       </c>
       <c r="R3" s="13">
         <v>0.95</v>
@@ -24550,10 +24551,10 @@
         <v>5</v>
       </c>
       <c r="P4" s="6">
-        <v>162.10234999999997</v>
+        <v>8.0020722230000008</v>
       </c>
       <c r="Q4" s="6">
-        <v>162.10234999999997</v>
+        <v>8.0020722230000008</v>
       </c>
       <c r="R4" s="13">
         <v>0.95</v>
@@ -24633,10 +24634,10 @@
         <v>5</v>
       </c>
       <c r="P5" s="6">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="6">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="R5" s="13">
         <v>0.7</v>
@@ -27576,6 +27577,26 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -27583,26 +27604,6 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Material Block Pricing
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/urbs-materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1170" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E7549D9-7045-45AC-8066-5808153A4E87}"/>
+  <xr:revisionPtr revIDLastSave="1187" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12E46AA0-D504-45D6-96B5-A3EC0E86EF18}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="11" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -24,14 +24,15 @@
     <sheet name="gas_block" sheetId="13" r:id="rId9"/>
     <sheet name="Tech_Stage_Specs" sheetId="14" r:id="rId10"/>
     <sheet name="Material_Intensity" sheetId="15" r:id="rId11"/>
-    <sheet name="mining_limit" sheetId="20" r:id="rId12"/>
-    <sheet name="mining_cost" sheetId="21" r:id="rId13"/>
-    <sheet name="import_cost_mining" sheetId="22" r:id="rId14"/>
-    <sheet name="energy_transition_factor" sheetId="23" r:id="rId15"/>
-    <sheet name="ore_metal_factor" sheetId="24" r:id="rId16"/>
-    <sheet name="Component_Map" sheetId="18" r:id="rId17"/>
-    <sheet name="Cost_Data" sheetId="16" r:id="rId18"/>
-    <sheet name="Import_Cost_Stage" sheetId="19" r:id="rId19"/>
+    <sheet name="material_blocks" sheetId="25" r:id="rId12"/>
+    <sheet name="mining_limit" sheetId="20" r:id="rId13"/>
+    <sheet name="mining_cost" sheetId="21" r:id="rId14"/>
+    <sheet name="import_cost_mining" sheetId="22" r:id="rId15"/>
+    <sheet name="energy_transition_factor" sheetId="23" r:id="rId16"/>
+    <sheet name="ore_metal_factor" sheetId="24" r:id="rId17"/>
+    <sheet name="Component_Map" sheetId="18" r:id="rId18"/>
+    <sheet name="Cost_Data" sheetId="16" r:id="rId19"/>
+    <sheet name="Import_Cost_Stage" sheetId="19" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">gas_block!$B$1:$B$109</definedName>
@@ -57,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="194">
   <si>
     <t>Value</t>
   </si>
@@ -612,6 +613,33 @@
   </si>
   <si>
     <t>silicon</t>
+  </si>
+  <si>
+    <t>material</t>
+  </si>
+  <si>
+    <t>base_2024</t>
+  </si>
+  <si>
+    <t>lds_2030</t>
+  </si>
+  <si>
+    <t>lds_2050</t>
+  </si>
+  <si>
+    <t>hds_2030</t>
+  </si>
+  <si>
+    <t>hds_2050</t>
+  </si>
+  <si>
+    <t>price_t1</t>
+  </si>
+  <si>
+    <t>price_t2</t>
+  </si>
+  <si>
+    <t>price_t3</t>
   </si>
 </sst>
 </file>
@@ -2631,6 +2659,773 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C48FFD33-43EA-4828-A0BA-4DF40CC0ECAB}">
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F1" t="s">
+        <v>190</v>
+      </c>
+      <c r="G1" t="s">
+        <v>191</v>
+      </c>
+      <c r="H1" t="s">
+        <v>192</v>
+      </c>
+      <c r="I1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B2">
+        <v>100</v>
+      </c>
+      <c r="C2">
+        <v>150</v>
+      </c>
+      <c r="D2">
+        <v>200</v>
+      </c>
+      <c r="E2">
+        <v>200</v>
+      </c>
+      <c r="F2">
+        <v>300</v>
+      </c>
+      <c r="G2">
+        <v>50</v>
+      </c>
+      <c r="H2">
+        <v>100</v>
+      </c>
+      <c r="I2">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3">
+        <v>100</v>
+      </c>
+      <c r="C3">
+        <v>150</v>
+      </c>
+      <c r="D3">
+        <v>200</v>
+      </c>
+      <c r="E3">
+        <v>200</v>
+      </c>
+      <c r="F3">
+        <v>300</v>
+      </c>
+      <c r="G3">
+        <v>50</v>
+      </c>
+      <c r="H3">
+        <v>100</v>
+      </c>
+      <c r="I3">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B4">
+        <v>100</v>
+      </c>
+      <c r="C4">
+        <v>150</v>
+      </c>
+      <c r="D4">
+        <v>200</v>
+      </c>
+      <c r="E4">
+        <v>200</v>
+      </c>
+      <c r="F4">
+        <v>300</v>
+      </c>
+      <c r="G4">
+        <v>50</v>
+      </c>
+      <c r="H4">
+        <v>100</v>
+      </c>
+      <c r="I4">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B5">
+        <v>100</v>
+      </c>
+      <c r="C5">
+        <v>150</v>
+      </c>
+      <c r="D5">
+        <v>200</v>
+      </c>
+      <c r="E5">
+        <v>200</v>
+      </c>
+      <c r="F5">
+        <v>300</v>
+      </c>
+      <c r="G5">
+        <v>50</v>
+      </c>
+      <c r="H5">
+        <v>100</v>
+      </c>
+      <c r="I5">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B6">
+        <v>100</v>
+      </c>
+      <c r="C6">
+        <v>150</v>
+      </c>
+      <c r="D6">
+        <v>200</v>
+      </c>
+      <c r="E6">
+        <v>200</v>
+      </c>
+      <c r="F6">
+        <v>300</v>
+      </c>
+      <c r="G6">
+        <v>50</v>
+      </c>
+      <c r="H6">
+        <v>100</v>
+      </c>
+      <c r="I6">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7">
+        <v>100</v>
+      </c>
+      <c r="C7">
+        <v>150</v>
+      </c>
+      <c r="D7">
+        <v>200</v>
+      </c>
+      <c r="E7">
+        <v>200</v>
+      </c>
+      <c r="F7">
+        <v>300</v>
+      </c>
+      <c r="G7">
+        <v>50</v>
+      </c>
+      <c r="H7">
+        <v>100</v>
+      </c>
+      <c r="I7">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B8">
+        <v>100</v>
+      </c>
+      <c r="C8">
+        <v>150</v>
+      </c>
+      <c r="D8">
+        <v>200</v>
+      </c>
+      <c r="E8">
+        <v>200</v>
+      </c>
+      <c r="F8">
+        <v>300</v>
+      </c>
+      <c r="G8">
+        <v>50</v>
+      </c>
+      <c r="H8">
+        <v>100</v>
+      </c>
+      <c r="I8">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>143</v>
+      </c>
+      <c r="B9">
+        <v>100</v>
+      </c>
+      <c r="C9">
+        <v>150</v>
+      </c>
+      <c r="D9">
+        <v>200</v>
+      </c>
+      <c r="E9">
+        <v>200</v>
+      </c>
+      <c r="F9">
+        <v>300</v>
+      </c>
+      <c r="G9">
+        <v>50</v>
+      </c>
+      <c r="H9">
+        <v>100</v>
+      </c>
+      <c r="I9">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>144</v>
+      </c>
+      <c r="B10">
+        <v>100</v>
+      </c>
+      <c r="C10">
+        <v>150</v>
+      </c>
+      <c r="D10">
+        <v>200</v>
+      </c>
+      <c r="E10">
+        <v>200</v>
+      </c>
+      <c r="F10">
+        <v>300</v>
+      </c>
+      <c r="G10">
+        <v>50</v>
+      </c>
+      <c r="H10">
+        <v>100</v>
+      </c>
+      <c r="I10">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>145</v>
+      </c>
+      <c r="B11">
+        <v>100</v>
+      </c>
+      <c r="C11">
+        <v>150</v>
+      </c>
+      <c r="D11">
+        <v>200</v>
+      </c>
+      <c r="E11">
+        <v>200</v>
+      </c>
+      <c r="F11">
+        <v>300</v>
+      </c>
+      <c r="G11">
+        <v>50</v>
+      </c>
+      <c r="H11">
+        <v>100</v>
+      </c>
+      <c r="I11">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>146</v>
+      </c>
+      <c r="B12">
+        <v>100</v>
+      </c>
+      <c r="C12">
+        <v>150</v>
+      </c>
+      <c r="D12">
+        <v>200</v>
+      </c>
+      <c r="E12">
+        <v>200</v>
+      </c>
+      <c r="F12">
+        <v>300</v>
+      </c>
+      <c r="G12">
+        <v>50</v>
+      </c>
+      <c r="H12">
+        <v>100</v>
+      </c>
+      <c r="I12">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>147</v>
+      </c>
+      <c r="B13">
+        <v>100</v>
+      </c>
+      <c r="C13">
+        <v>150</v>
+      </c>
+      <c r="D13">
+        <v>200</v>
+      </c>
+      <c r="E13">
+        <v>200</v>
+      </c>
+      <c r="F13">
+        <v>300</v>
+      </c>
+      <c r="G13">
+        <v>50</v>
+      </c>
+      <c r="H13">
+        <v>100</v>
+      </c>
+      <c r="I13">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>148</v>
+      </c>
+      <c r="B14">
+        <v>100</v>
+      </c>
+      <c r="C14">
+        <v>150</v>
+      </c>
+      <c r="D14">
+        <v>200</v>
+      </c>
+      <c r="E14">
+        <v>200</v>
+      </c>
+      <c r="F14">
+        <v>300</v>
+      </c>
+      <c r="G14">
+        <v>50</v>
+      </c>
+      <c r="H14">
+        <v>100</v>
+      </c>
+      <c r="I14">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>149</v>
+      </c>
+      <c r="B15">
+        <v>100</v>
+      </c>
+      <c r="C15">
+        <v>150</v>
+      </c>
+      <c r="D15">
+        <v>200</v>
+      </c>
+      <c r="E15">
+        <v>200</v>
+      </c>
+      <c r="F15">
+        <v>300</v>
+      </c>
+      <c r="G15">
+        <v>50</v>
+      </c>
+      <c r="H15">
+        <v>100</v>
+      </c>
+      <c r="I15">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>150</v>
+      </c>
+      <c r="B16">
+        <v>100</v>
+      </c>
+      <c r="C16">
+        <v>150</v>
+      </c>
+      <c r="D16">
+        <v>200</v>
+      </c>
+      <c r="E16">
+        <v>200</v>
+      </c>
+      <c r="F16">
+        <v>300</v>
+      </c>
+      <c r="G16">
+        <v>50</v>
+      </c>
+      <c r="H16">
+        <v>100</v>
+      </c>
+      <c r="I16">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>151</v>
+      </c>
+      <c r="B17">
+        <v>100</v>
+      </c>
+      <c r="C17">
+        <v>150</v>
+      </c>
+      <c r="D17">
+        <v>200</v>
+      </c>
+      <c r="E17">
+        <v>200</v>
+      </c>
+      <c r="F17">
+        <v>300</v>
+      </c>
+      <c r="G17">
+        <v>50</v>
+      </c>
+      <c r="H17">
+        <v>100</v>
+      </c>
+      <c r="I17">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>152</v>
+      </c>
+      <c r="B18">
+        <v>100</v>
+      </c>
+      <c r="C18">
+        <v>150</v>
+      </c>
+      <c r="D18">
+        <v>200</v>
+      </c>
+      <c r="E18">
+        <v>200</v>
+      </c>
+      <c r="F18">
+        <v>300</v>
+      </c>
+      <c r="G18">
+        <v>50</v>
+      </c>
+      <c r="H18">
+        <v>100</v>
+      </c>
+      <c r="I18">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>153</v>
+      </c>
+      <c r="B19">
+        <v>100</v>
+      </c>
+      <c r="C19">
+        <v>150</v>
+      </c>
+      <c r="D19">
+        <v>200</v>
+      </c>
+      <c r="E19">
+        <v>200</v>
+      </c>
+      <c r="F19">
+        <v>300</v>
+      </c>
+      <c r="G19">
+        <v>50</v>
+      </c>
+      <c r="H19">
+        <v>100</v>
+      </c>
+      <c r="I19">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>154</v>
+      </c>
+      <c r="B20">
+        <v>100</v>
+      </c>
+      <c r="C20">
+        <v>150</v>
+      </c>
+      <c r="D20">
+        <v>200</v>
+      </c>
+      <c r="E20">
+        <v>200</v>
+      </c>
+      <c r="F20">
+        <v>300</v>
+      </c>
+      <c r="G20">
+        <v>50</v>
+      </c>
+      <c r="H20">
+        <v>100</v>
+      </c>
+      <c r="I20">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>155</v>
+      </c>
+      <c r="B21">
+        <v>100</v>
+      </c>
+      <c r="C21">
+        <v>150</v>
+      </c>
+      <c r="D21">
+        <v>200</v>
+      </c>
+      <c r="E21">
+        <v>200</v>
+      </c>
+      <c r="F21">
+        <v>300</v>
+      </c>
+      <c r="G21">
+        <v>50</v>
+      </c>
+      <c r="H21">
+        <v>100</v>
+      </c>
+      <c r="I21">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>156</v>
+      </c>
+      <c r="B22">
+        <v>100</v>
+      </c>
+      <c r="C22">
+        <v>150</v>
+      </c>
+      <c r="D22">
+        <v>200</v>
+      </c>
+      <c r="E22">
+        <v>200</v>
+      </c>
+      <c r="F22">
+        <v>300</v>
+      </c>
+      <c r="G22">
+        <v>50</v>
+      </c>
+      <c r="H22">
+        <v>100</v>
+      </c>
+      <c r="I22">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>121</v>
+      </c>
+      <c r="B23">
+        <v>999999</v>
+      </c>
+      <c r="C23">
+        <v>999999</v>
+      </c>
+      <c r="D23">
+        <v>999999</v>
+      </c>
+      <c r="E23">
+        <v>999999</v>
+      </c>
+      <c r="F23">
+        <v>999999</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24">
+        <v>999999</v>
+      </c>
+      <c r="C24">
+        <v>999999</v>
+      </c>
+      <c r="D24">
+        <v>999999</v>
+      </c>
+      <c r="E24">
+        <v>999999</v>
+      </c>
+      <c r="F24">
+        <v>999999</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>123</v>
+      </c>
+      <c r="B25">
+        <v>999999</v>
+      </c>
+      <c r="C25">
+        <v>999999</v>
+      </c>
+      <c r="D25">
+        <v>999999</v>
+      </c>
+      <c r="E25">
+        <v>999999</v>
+      </c>
+      <c r="F25">
+        <v>999999</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
+      </c>
+      <c r="I25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>122</v>
+      </c>
+      <c r="B26">
+        <v>999999</v>
+      </c>
+      <c r="C26">
+        <v>999999</v>
+      </c>
+      <c r="D26">
+        <v>999999</v>
+      </c>
+      <c r="E26">
+        <v>999999</v>
+      </c>
+      <c r="F26">
+        <v>999999</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA468E9E-004D-4F86-817A-29F43A769A51}">
   <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4880,7 +5675,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3497A18D-E10F-4371-B6A4-3051915122F0}">
   <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7130,7 +7925,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0643026C-02E1-4FD1-A973-B34B54E790E8}">
   <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9380,7 +10175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28476978-BEE9-428F-A843-1F40BF462E1E}">
   <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11630,7 +12425,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3AB9FD-44ED-4E59-8956-C20ADB98B718}">
   <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13880,7 +14675,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{996B2112-D2EE-4E9F-B294-4222E881A3C9}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14077,7 +14872,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CE844EE-882F-4833-8B87-00A8BB665263}">
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14475,1339 +15270,6 @@
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B74DFEF-01D9-4B2D-A936-BF616F091054}">
-  <dimension ref="A1:O34"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E1" t="s">
-        <v>107</v>
-      </c>
-      <c r="F1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G1" t="s">
-        <v>133</v>
-      </c>
-      <c r="H1" t="s">
-        <v>134</v>
-      </c>
-      <c r="I1" t="s">
-        <v>135</v>
-      </c>
-      <c r="J1" t="s">
-        <v>136</v>
-      </c>
-      <c r="K1" t="s">
-        <v>137</v>
-      </c>
-      <c r="L1" t="s">
-        <v>138</v>
-      </c>
-      <c r="M1" t="s">
-        <v>139</v>
-      </c>
-      <c r="N1" t="s">
-        <v>118</v>
-      </c>
-      <c r="O1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>2024</v>
-      </c>
-      <c r="B2">
-        <v>38640</v>
-      </c>
-      <c r="C2">
-        <v>55200</v>
-      </c>
-      <c r="D2">
-        <v>82800</v>
-      </c>
-      <c r="E2">
-        <v>149960</v>
-      </c>
-      <c r="F2">
-        <v>9999999</v>
-      </c>
-      <c r="G2">
-        <v>9999999</v>
-      </c>
-      <c r="H2">
-        <v>382762.9</v>
-      </c>
-      <c r="I2">
-        <v>679793.6</v>
-      </c>
-      <c r="J2">
-        <v>9999999</v>
-      </c>
-      <c r="K2">
-        <v>9999999</v>
-      </c>
-      <c r="L2">
-        <v>479917.1</v>
-      </c>
-      <c r="M2">
-        <v>787018</v>
-      </c>
-      <c r="N2">
-        <v>9999999</v>
-      </c>
-      <c r="O2">
-        <v>280439.83</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2025</v>
-      </c>
-      <c r="B3">
-        <v>38060.400000000001</v>
-      </c>
-      <c r="C3">
-        <v>54372</v>
-      </c>
-      <c r="D3">
-        <v>81558</v>
-      </c>
-      <c r="E3">
-        <v>148580</v>
-      </c>
-      <c r="F3">
-        <v>9999999</v>
-      </c>
-      <c r="G3">
-        <v>9999999</v>
-      </c>
-      <c r="H3">
-        <v>382762.9</v>
-      </c>
-      <c r="I3">
-        <v>679793.6</v>
-      </c>
-      <c r="J3">
-        <v>9999999</v>
-      </c>
-      <c r="K3">
-        <v>9999999</v>
-      </c>
-      <c r="L3">
-        <v>479917.1</v>
-      </c>
-      <c r="M3">
-        <v>787018</v>
-      </c>
-      <c r="N3">
-        <v>9999999</v>
-      </c>
-      <c r="O3">
-        <v>274754.90999999997</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2026</v>
-      </c>
-      <c r="B4">
-        <v>37489.493999999999</v>
-      </c>
-      <c r="C4">
-        <v>53556.42</v>
-      </c>
-      <c r="D4">
-        <v>80334.63</v>
-      </c>
-      <c r="E4">
-        <v>147200</v>
-      </c>
-      <c r="F4">
-        <v>9999999</v>
-      </c>
-      <c r="G4">
-        <v>9999999</v>
-      </c>
-      <c r="H4">
-        <v>382762.9</v>
-      </c>
-      <c r="I4">
-        <v>679793.6</v>
-      </c>
-      <c r="J4">
-        <v>9999999</v>
-      </c>
-      <c r="K4">
-        <v>9999999</v>
-      </c>
-      <c r="L4">
-        <v>479917.1</v>
-      </c>
-      <c r="M4">
-        <v>787018</v>
-      </c>
-      <c r="N4">
-        <v>9999999</v>
-      </c>
-      <c r="O4">
-        <v>269179.44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>2027</v>
-      </c>
-      <c r="B5">
-        <v>36927.151590000001</v>
-      </c>
-      <c r="C5">
-        <v>52753.073700000001</v>
-      </c>
-      <c r="D5">
-        <v>79129.610549999998</v>
-      </c>
-      <c r="E5">
-        <v>145820</v>
-      </c>
-      <c r="F5">
-        <v>9999999</v>
-      </c>
-      <c r="G5">
-        <v>9999999</v>
-      </c>
-      <c r="H5">
-        <v>382762.9</v>
-      </c>
-      <c r="I5">
-        <v>679793.6</v>
-      </c>
-      <c r="J5">
-        <v>9999999</v>
-      </c>
-      <c r="K5">
-        <v>9999999</v>
-      </c>
-      <c r="L5">
-        <v>479917.1</v>
-      </c>
-      <c r="M5">
-        <v>787018</v>
-      </c>
-      <c r="N5">
-        <v>9999999</v>
-      </c>
-      <c r="O5">
-        <v>263711.78000000003</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>2028</v>
-      </c>
-      <c r="B6">
-        <v>36373.244316149998</v>
-      </c>
-      <c r="C6">
-        <v>51961.777594500003</v>
-      </c>
-      <c r="D6">
-        <v>77942.666391749997</v>
-      </c>
-      <c r="E6">
-        <v>144440</v>
-      </c>
-      <c r="F6">
-        <v>9999999</v>
-      </c>
-      <c r="G6">
-        <v>9999999</v>
-      </c>
-      <c r="H6">
-        <v>382762.9</v>
-      </c>
-      <c r="I6">
-        <v>679793.6</v>
-      </c>
-      <c r="J6">
-        <v>9999999</v>
-      </c>
-      <c r="K6">
-        <v>9999999</v>
-      </c>
-      <c r="L6">
-        <v>479917.1</v>
-      </c>
-      <c r="M6">
-        <v>787018</v>
-      </c>
-      <c r="N6">
-        <v>9999999</v>
-      </c>
-      <c r="O6">
-        <v>258350.32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2029</v>
-      </c>
-      <c r="B7">
-        <v>35827.645651407751</v>
-      </c>
-      <c r="C7">
-        <v>51182.350930582499</v>
-      </c>
-      <c r="D7">
-        <v>76773.526395873749</v>
-      </c>
-      <c r="E7">
-        <v>143060</v>
-      </c>
-      <c r="F7">
-        <v>9999999</v>
-      </c>
-      <c r="G7">
-        <v>9999999</v>
-      </c>
-      <c r="H7">
-        <v>382762.9</v>
-      </c>
-      <c r="I7">
-        <v>679793.6</v>
-      </c>
-      <c r="J7">
-        <v>9999999</v>
-      </c>
-      <c r="K7">
-        <v>9999999</v>
-      </c>
-      <c r="L7">
-        <v>479917.1</v>
-      </c>
-      <c r="M7">
-        <v>787018</v>
-      </c>
-      <c r="N7">
-        <v>9999999</v>
-      </c>
-      <c r="O7">
-        <v>253093.46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>2030</v>
-      </c>
-      <c r="B8">
-        <v>35290.230966636635</v>
-      </c>
-      <c r="C8">
-        <v>50414.615666623758</v>
-      </c>
-      <c r="D8">
-        <v>75621.923499935641</v>
-      </c>
-      <c r="E8">
-        <v>141680</v>
-      </c>
-      <c r="F8">
-        <v>9999999</v>
-      </c>
-      <c r="G8">
-        <v>9999999</v>
-      </c>
-      <c r="H8">
-        <v>382762.9</v>
-      </c>
-      <c r="I8">
-        <v>679793.6</v>
-      </c>
-      <c r="J8">
-        <v>9999999</v>
-      </c>
-      <c r="K8">
-        <v>9999999</v>
-      </c>
-      <c r="L8">
-        <v>479917.1</v>
-      </c>
-      <c r="M8">
-        <v>787018</v>
-      </c>
-      <c r="N8">
-        <v>9999999</v>
-      </c>
-      <c r="O8">
-        <v>247939.65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>2031</v>
-      </c>
-      <c r="B9">
-        <v>34760.877502137082</v>
-      </c>
-      <c r="C9">
-        <v>49658.396431624402</v>
-      </c>
-      <c r="D9">
-        <v>74487.594647436606</v>
-      </c>
-      <c r="E9">
-        <v>140300</v>
-      </c>
-      <c r="F9">
-        <v>9999999</v>
-      </c>
-      <c r="G9">
-        <v>9999999</v>
-      </c>
-      <c r="H9">
-        <v>382762.9</v>
-      </c>
-      <c r="I9">
-        <v>679793.6</v>
-      </c>
-      <c r="J9">
-        <v>9999999</v>
-      </c>
-      <c r="K9">
-        <v>9999999</v>
-      </c>
-      <c r="L9">
-        <v>479917.1</v>
-      </c>
-      <c r="M9">
-        <v>787018</v>
-      </c>
-      <c r="N9">
-        <v>9999999</v>
-      </c>
-      <c r="O9">
-        <v>242887.37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>2032</v>
-      </c>
-      <c r="B10">
-        <v>34239.464339605023</v>
-      </c>
-      <c r="C10">
-        <v>48913.520485150038</v>
-      </c>
-      <c r="D10">
-        <v>73370.280727725054</v>
-      </c>
-      <c r="E10">
-        <v>138920</v>
-      </c>
-      <c r="F10">
-        <v>9999999</v>
-      </c>
-      <c r="G10">
-        <v>9999999</v>
-      </c>
-      <c r="H10">
-        <v>382762.9</v>
-      </c>
-      <c r="I10">
-        <v>679793.6</v>
-      </c>
-      <c r="J10">
-        <v>9999999</v>
-      </c>
-      <c r="K10">
-        <v>9999999</v>
-      </c>
-      <c r="L10">
-        <v>479917.1</v>
-      </c>
-      <c r="M10">
-        <v>787018</v>
-      </c>
-      <c r="N10">
-        <v>9999999</v>
-      </c>
-      <c r="O10">
-        <v>237935.1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>2033</v>
-      </c>
-      <c r="B11">
-        <v>33725.872374510946</v>
-      </c>
-      <c r="C11">
-        <v>48179.817677872787</v>
-      </c>
-      <c r="D11">
-        <v>72269.726516809184</v>
-      </c>
-      <c r="E11">
-        <v>137540</v>
-      </c>
-      <c r="F11">
-        <v>9999999</v>
-      </c>
-      <c r="G11">
-        <v>9999999</v>
-      </c>
-      <c r="H11">
-        <v>382762.9</v>
-      </c>
-      <c r="I11">
-        <v>679793.6</v>
-      </c>
-      <c r="J11">
-        <v>9999999</v>
-      </c>
-      <c r="K11">
-        <v>9999999</v>
-      </c>
-      <c r="L11">
-        <v>479917.1</v>
-      </c>
-      <c r="M11">
-        <v>787018</v>
-      </c>
-      <c r="N11">
-        <v>9999999</v>
-      </c>
-      <c r="O11">
-        <v>233081.4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>2034</v>
-      </c>
-      <c r="B12">
-        <v>33219.984288893284</v>
-      </c>
-      <c r="C12">
-        <v>47457.120412704695</v>
-      </c>
-      <c r="D12">
-        <v>71185.68061905705</v>
-      </c>
-      <c r="E12">
-        <v>136160</v>
-      </c>
-      <c r="F12">
-        <v>9999999</v>
-      </c>
-      <c r="G12">
-        <v>9999999</v>
-      </c>
-      <c r="H12">
-        <v>382762.9</v>
-      </c>
-      <c r="I12">
-        <v>679793.6</v>
-      </c>
-      <c r="J12">
-        <v>9999999</v>
-      </c>
-      <c r="K12">
-        <v>9999999</v>
-      </c>
-      <c r="L12">
-        <v>479917.1</v>
-      </c>
-      <c r="M12">
-        <v>787018</v>
-      </c>
-      <c r="N12">
-        <v>9999999</v>
-      </c>
-      <c r="O12">
-        <v>228324.82</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>2035</v>
-      </c>
-      <c r="B13">
-        <v>32721.684524559885</v>
-      </c>
-      <c r="C13">
-        <v>46745.263606514127</v>
-      </c>
-      <c r="D13">
-        <v>70117.895409771198</v>
-      </c>
-      <c r="E13">
-        <v>134780</v>
-      </c>
-      <c r="F13">
-        <v>9999999</v>
-      </c>
-      <c r="G13">
-        <v>9999999</v>
-      </c>
-      <c r="H13">
-        <v>382762.9</v>
-      </c>
-      <c r="I13">
-        <v>679793.6</v>
-      </c>
-      <c r="J13">
-        <v>9999999</v>
-      </c>
-      <c r="K13">
-        <v>9999999</v>
-      </c>
-      <c r="L13">
-        <v>479917.1</v>
-      </c>
-      <c r="M13">
-        <v>787018</v>
-      </c>
-      <c r="N13">
-        <v>9999999</v>
-      </c>
-      <c r="O13">
-        <v>223663.91</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>2036</v>
-      </c>
-      <c r="B14">
-        <v>32230.859256691485</v>
-      </c>
-      <c r="C14">
-        <v>46044.084652416415</v>
-      </c>
-      <c r="D14">
-        <v>69066.126978624627</v>
-      </c>
-      <c r="E14">
-        <v>133400</v>
-      </c>
-      <c r="F14">
-        <v>9999999</v>
-      </c>
-      <c r="G14">
-        <v>9999999</v>
-      </c>
-      <c r="H14">
-        <v>382762.9</v>
-      </c>
-      <c r="I14">
-        <v>679793.6</v>
-      </c>
-      <c r="J14">
-        <v>9999999</v>
-      </c>
-      <c r="K14">
-        <v>9999999</v>
-      </c>
-      <c r="L14">
-        <v>479917.1</v>
-      </c>
-      <c r="M14">
-        <v>787018</v>
-      </c>
-      <c r="N14">
-        <v>9999999</v>
-      </c>
-      <c r="O14">
-        <v>219097.32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>2037</v>
-      </c>
-      <c r="B15">
-        <v>31747.396367841113</v>
-      </c>
-      <c r="C15">
-        <v>45353.423382630172</v>
-      </c>
-      <c r="D15">
-        <v>68030.135073945261</v>
-      </c>
-      <c r="E15">
-        <v>132020</v>
-      </c>
-      <c r="F15">
-        <v>9999999</v>
-      </c>
-      <c r="G15">
-        <v>9999999</v>
-      </c>
-      <c r="H15">
-        <v>382762.9</v>
-      </c>
-      <c r="I15">
-        <v>679793.6</v>
-      </c>
-      <c r="J15">
-        <v>9999999</v>
-      </c>
-      <c r="K15">
-        <v>9999999</v>
-      </c>
-      <c r="L15">
-        <v>479917.1</v>
-      </c>
-      <c r="M15">
-        <v>787018</v>
-      </c>
-      <c r="N15">
-        <v>9999999</v>
-      </c>
-      <c r="O15">
-        <v>214623.65</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>2038</v>
-      </c>
-      <c r="B16">
-        <v>31271.185422323495</v>
-      </c>
-      <c r="C16">
-        <v>44673.122031890722</v>
-      </c>
-      <c r="D16">
-        <v>67009.683047836079</v>
-      </c>
-      <c r="E16">
-        <v>130640</v>
-      </c>
-      <c r="F16">
-        <v>9999999</v>
-      </c>
-      <c r="G16">
-        <v>9999999</v>
-      </c>
-      <c r="H16">
-        <v>382762.9</v>
-      </c>
-      <c r="I16">
-        <v>679793.6</v>
-      </c>
-      <c r="J16">
-        <v>9999999</v>
-      </c>
-      <c r="K16">
-        <v>9999999</v>
-      </c>
-      <c r="L16">
-        <v>479917.1</v>
-      </c>
-      <c r="M16">
-        <v>787018</v>
-      </c>
-      <c r="N16">
-        <v>9999999</v>
-      </c>
-      <c r="O16">
-        <v>210241.6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>2039</v>
-      </c>
-      <c r="B17">
-        <v>30802.117640988643</v>
-      </c>
-      <c r="C17">
-        <v>44003.025201412362</v>
-      </c>
-      <c r="D17">
-        <v>66004.537802118532</v>
-      </c>
-      <c r="E17">
-        <v>129260</v>
-      </c>
-      <c r="F17">
-        <v>9999999</v>
-      </c>
-      <c r="G17">
-        <v>9999999</v>
-      </c>
-      <c r="H17">
-        <v>382762.9</v>
-      </c>
-      <c r="I17">
-        <v>679793.6</v>
-      </c>
-      <c r="J17">
-        <v>9999999</v>
-      </c>
-      <c r="K17">
-        <v>9999999</v>
-      </c>
-      <c r="L17">
-        <v>479917.1</v>
-      </c>
-      <c r="M17">
-        <v>787018</v>
-      </c>
-      <c r="N17">
-        <v>9999999</v>
-      </c>
-      <c r="O17">
-        <v>205949.84</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>2040</v>
-      </c>
-      <c r="B18">
-        <v>30340.085876373814</v>
-      </c>
-      <c r="C18">
-        <v>43342.979823391179</v>
-      </c>
-      <c r="D18">
-        <v>65014.46973508675</v>
-      </c>
-      <c r="E18">
-        <v>127880</v>
-      </c>
-      <c r="F18">
-        <v>9999999</v>
-      </c>
-      <c r="G18">
-        <v>9999999</v>
-      </c>
-      <c r="H18">
-        <v>382762.9</v>
-      </c>
-      <c r="I18">
-        <v>679793.6</v>
-      </c>
-      <c r="J18">
-        <v>9999999</v>
-      </c>
-      <c r="K18">
-        <v>9999999</v>
-      </c>
-      <c r="L18">
-        <v>479917.1</v>
-      </c>
-      <c r="M18">
-        <v>787018</v>
-      </c>
-      <c r="N18">
-        <v>9999999</v>
-      </c>
-      <c r="O18">
-        <v>201747.12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>2041</v>
-      </c>
-      <c r="B19">
-        <v>29884.984588228206</v>
-      </c>
-      <c r="C19">
-        <v>42692.835126040307</v>
-      </c>
-      <c r="D19">
-        <v>64039.252689060449</v>
-      </c>
-      <c r="E19">
-        <v>126500</v>
-      </c>
-      <c r="F19">
-        <v>9999999</v>
-      </c>
-      <c r="G19">
-        <v>9999999</v>
-      </c>
-      <c r="H19">
-        <v>382762.9</v>
-      </c>
-      <c r="I19">
-        <v>679793.6</v>
-      </c>
-      <c r="J19">
-        <v>9999999</v>
-      </c>
-      <c r="K19">
-        <v>9999999</v>
-      </c>
-      <c r="L19">
-        <v>479917.1</v>
-      </c>
-      <c r="M19">
-        <v>787018</v>
-      </c>
-      <c r="N19">
-        <v>9999999</v>
-      </c>
-      <c r="O19">
-        <v>197632.19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>2042</v>
-      </c>
-      <c r="B20">
-        <v>29436.709819404783</v>
-      </c>
-      <c r="C20">
-        <v>42052.442599149705</v>
-      </c>
-      <c r="D20">
-        <v>63078.663898724539</v>
-      </c>
-      <c r="E20">
-        <v>125120</v>
-      </c>
-      <c r="F20">
-        <v>9999999</v>
-      </c>
-      <c r="G20">
-        <v>9999999</v>
-      </c>
-      <c r="H20">
-        <v>382762.9</v>
-      </c>
-      <c r="I20">
-        <v>679793.6</v>
-      </c>
-      <c r="J20">
-        <v>9999999</v>
-      </c>
-      <c r="K20">
-        <v>9999999</v>
-      </c>
-      <c r="L20">
-        <v>479917.1</v>
-      </c>
-      <c r="M20">
-        <v>787018</v>
-      </c>
-      <c r="N20">
-        <v>9999999</v>
-      </c>
-      <c r="O20">
-        <v>193603.83</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>2043</v>
-      </c>
-      <c r="B21">
-        <v>28995.159172113712</v>
-      </c>
-      <c r="C21">
-        <v>41421.655960162461</v>
-      </c>
-      <c r="D21">
-        <v>62132.48394024367</v>
-      </c>
-      <c r="E21">
-        <v>123740</v>
-      </c>
-      <c r="F21">
-        <v>9999999</v>
-      </c>
-      <c r="G21">
-        <v>9999999</v>
-      </c>
-      <c r="H21">
-        <v>382762.9</v>
-      </c>
-      <c r="I21">
-        <v>679793.6</v>
-      </c>
-      <c r="J21">
-        <v>9999999</v>
-      </c>
-      <c r="K21">
-        <v>9999999</v>
-      </c>
-      <c r="L21">
-        <v>479917.1</v>
-      </c>
-      <c r="M21">
-        <v>787018</v>
-      </c>
-      <c r="N21">
-        <v>9999999</v>
-      </c>
-      <c r="O21">
-        <v>189660.87</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>2044</v>
-      </c>
-      <c r="B22">
-        <v>28560.231784532007</v>
-      </c>
-      <c r="C22">
-        <v>40800.331120760027</v>
-      </c>
-      <c r="D22">
-        <v>61200.496681140015</v>
-      </c>
-      <c r="E22">
-        <v>122360</v>
-      </c>
-      <c r="F22">
-        <v>9999999</v>
-      </c>
-      <c r="G22">
-        <v>9999999</v>
-      </c>
-      <c r="H22">
-        <v>382762.9</v>
-      </c>
-      <c r="I22">
-        <v>679793.6</v>
-      </c>
-      <c r="J22">
-        <v>9999999</v>
-      </c>
-      <c r="K22">
-        <v>9999999</v>
-      </c>
-      <c r="L22">
-        <v>479917.1</v>
-      </c>
-      <c r="M22">
-        <v>787018</v>
-      </c>
-      <c r="N22">
-        <v>9999999</v>
-      </c>
-      <c r="O22">
-        <v>185802.14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>2045</v>
-      </c>
-      <c r="B23">
-        <v>28131.828307764026</v>
-      </c>
-      <c r="C23">
-        <v>40188.326153948627</v>
-      </c>
-      <c r="D23">
-        <v>60282.489230922911</v>
-      </c>
-      <c r="E23">
-        <v>120980</v>
-      </c>
-      <c r="F23">
-        <v>9999999</v>
-      </c>
-      <c r="G23">
-        <v>9999999</v>
-      </c>
-      <c r="H23">
-        <v>382762.9</v>
-      </c>
-      <c r="I23">
-        <v>679793.6</v>
-      </c>
-      <c r="J23">
-        <v>9999999</v>
-      </c>
-      <c r="K23">
-        <v>9999999</v>
-      </c>
-      <c r="L23">
-        <v>479917.1</v>
-      </c>
-      <c r="M23">
-        <v>787018</v>
-      </c>
-      <c r="N23">
-        <v>9999999</v>
-      </c>
-      <c r="O23">
-        <v>182026.51</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>2046</v>
-      </c>
-      <c r="B24">
-        <v>27709.850883147566</v>
-      </c>
-      <c r="C24">
-        <v>39585.501261639394</v>
-      </c>
-      <c r="D24">
-        <v>59378.251892459069</v>
-      </c>
-      <c r="E24">
-        <v>119600</v>
-      </c>
-      <c r="F24">
-        <v>9999999</v>
-      </c>
-      <c r="G24">
-        <v>9999999</v>
-      </c>
-      <c r="H24">
-        <v>382762.9</v>
-      </c>
-      <c r="I24">
-        <v>679793.6</v>
-      </c>
-      <c r="J24">
-        <v>9999999</v>
-      </c>
-      <c r="K24">
-        <v>9999999</v>
-      </c>
-      <c r="L24">
-        <v>479917.1</v>
-      </c>
-      <c r="M24">
-        <v>787018</v>
-      </c>
-      <c r="N24">
-        <v>9999999</v>
-      </c>
-      <c r="O24">
-        <v>178332.87</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>2047</v>
-      </c>
-      <c r="B25">
-        <v>27294.203119900354</v>
-      </c>
-      <c r="C25">
-        <v>38991.718742714802</v>
-      </c>
-      <c r="D25">
-        <v>58487.578114072181</v>
-      </c>
-      <c r="E25">
-        <v>118220</v>
-      </c>
-      <c r="F25">
-        <v>9999999</v>
-      </c>
-      <c r="G25">
-        <v>9999999</v>
-      </c>
-      <c r="H25">
-        <v>382762.9</v>
-      </c>
-      <c r="I25">
-        <v>679793.6</v>
-      </c>
-      <c r="J25">
-        <v>9999999</v>
-      </c>
-      <c r="K25">
-        <v>9999999</v>
-      </c>
-      <c r="L25">
-        <v>479917.1</v>
-      </c>
-      <c r="M25">
-        <v>787018</v>
-      </c>
-      <c r="N25">
-        <v>9999999</v>
-      </c>
-      <c r="O25">
-        <v>174720.11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>2048</v>
-      </c>
-      <c r="B26">
-        <v>26884.790073101849</v>
-      </c>
-      <c r="C26">
-        <v>38406.842961574082</v>
-      </c>
-      <c r="D26">
-        <v>57610.264442361098</v>
-      </c>
-      <c r="E26">
-        <v>116840</v>
-      </c>
-      <c r="F26">
-        <v>9999999</v>
-      </c>
-      <c r="G26">
-        <v>9999999</v>
-      </c>
-      <c r="H26">
-        <v>382762.9</v>
-      </c>
-      <c r="I26">
-        <v>679793.6</v>
-      </c>
-      <c r="J26">
-        <v>9999999</v>
-      </c>
-      <c r="K26">
-        <v>9999999</v>
-      </c>
-      <c r="L26">
-        <v>479917.1</v>
-      </c>
-      <c r="M26">
-        <v>787018</v>
-      </c>
-      <c r="N26">
-        <v>9999999</v>
-      </c>
-      <c r="O26">
-        <v>171187.17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>2049</v>
-      </c>
-      <c r="B27">
-        <v>26481.518222005321</v>
-      </c>
-      <c r="C27">
-        <v>37830.74031715047</v>
-      </c>
-      <c r="D27">
-        <v>56746.110475725684</v>
-      </c>
-      <c r="E27">
-        <v>115460</v>
-      </c>
-      <c r="F27">
-        <v>9999999</v>
-      </c>
-      <c r="G27">
-        <v>9999999</v>
-      </c>
-      <c r="H27">
-        <v>382762.9</v>
-      </c>
-      <c r="I27">
-        <v>679793.6</v>
-      </c>
-      <c r="J27">
-        <v>9999999</v>
-      </c>
-      <c r="K27">
-        <v>9999999</v>
-      </c>
-      <c r="L27">
-        <v>479917.1</v>
-      </c>
-      <c r="M27">
-        <v>787018</v>
-      </c>
-      <c r="N27">
-        <v>9999999</v>
-      </c>
-      <c r="O27">
-        <v>167732.98000000001</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>2050</v>
-      </c>
-      <c r="B28">
-        <v>26084.295448675242</v>
-      </c>
-      <c r="C28">
-        <v>37263.279212393216</v>
-      </c>
-      <c r="D28">
-        <v>55894.918818589795</v>
-      </c>
-      <c r="E28">
-        <v>114080</v>
-      </c>
-      <c r="F28">
-        <v>9999999</v>
-      </c>
-      <c r="G28">
-        <v>9999999</v>
-      </c>
-      <c r="H28">
-        <v>382762.9</v>
-      </c>
-      <c r="I28">
-        <v>679793.6</v>
-      </c>
-      <c r="J28">
-        <v>9999999</v>
-      </c>
-      <c r="K28">
-        <v>9999999</v>
-      </c>
-      <c r="L28">
-        <v>479917.1</v>
-      </c>
-      <c r="M28">
-        <v>787018</v>
-      </c>
-      <c r="N28">
-        <v>9999999</v>
-      </c>
-      <c r="O28">
-        <v>164356.51999999999</v>
-      </c>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B33" s="17"/>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="G34" s="16"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -17655,6 +17117,1339 @@
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B74DFEF-01D9-4B2D-A936-BF616F091054}">
+  <dimension ref="A1:O34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F1" t="s">
+        <v>132</v>
+      </c>
+      <c r="G1" t="s">
+        <v>133</v>
+      </c>
+      <c r="H1" t="s">
+        <v>134</v>
+      </c>
+      <c r="I1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J1" t="s">
+        <v>136</v>
+      </c>
+      <c r="K1" t="s">
+        <v>137</v>
+      </c>
+      <c r="L1" t="s">
+        <v>138</v>
+      </c>
+      <c r="M1" t="s">
+        <v>139</v>
+      </c>
+      <c r="N1" t="s">
+        <v>118</v>
+      </c>
+      <c r="O1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2024</v>
+      </c>
+      <c r="B2">
+        <v>38640</v>
+      </c>
+      <c r="C2">
+        <v>55200</v>
+      </c>
+      <c r="D2">
+        <v>82800</v>
+      </c>
+      <c r="E2">
+        <v>149960</v>
+      </c>
+      <c r="F2">
+        <v>9999999</v>
+      </c>
+      <c r="G2">
+        <v>9999999</v>
+      </c>
+      <c r="H2">
+        <v>382762.9</v>
+      </c>
+      <c r="I2">
+        <v>679793.6</v>
+      </c>
+      <c r="J2">
+        <v>9999999</v>
+      </c>
+      <c r="K2">
+        <v>9999999</v>
+      </c>
+      <c r="L2">
+        <v>479917.1</v>
+      </c>
+      <c r="M2">
+        <v>787018</v>
+      </c>
+      <c r="N2">
+        <v>9999999</v>
+      </c>
+      <c r="O2">
+        <v>280439.83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2025</v>
+      </c>
+      <c r="B3">
+        <v>38060.400000000001</v>
+      </c>
+      <c r="C3">
+        <v>54372</v>
+      </c>
+      <c r="D3">
+        <v>81558</v>
+      </c>
+      <c r="E3">
+        <v>148580</v>
+      </c>
+      <c r="F3">
+        <v>9999999</v>
+      </c>
+      <c r="G3">
+        <v>9999999</v>
+      </c>
+      <c r="H3">
+        <v>382762.9</v>
+      </c>
+      <c r="I3">
+        <v>679793.6</v>
+      </c>
+      <c r="J3">
+        <v>9999999</v>
+      </c>
+      <c r="K3">
+        <v>9999999</v>
+      </c>
+      <c r="L3">
+        <v>479917.1</v>
+      </c>
+      <c r="M3">
+        <v>787018</v>
+      </c>
+      <c r="N3">
+        <v>9999999</v>
+      </c>
+      <c r="O3">
+        <v>274754.90999999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2026</v>
+      </c>
+      <c r="B4">
+        <v>37489.493999999999</v>
+      </c>
+      <c r="C4">
+        <v>53556.42</v>
+      </c>
+      <c r="D4">
+        <v>80334.63</v>
+      </c>
+      <c r="E4">
+        <v>147200</v>
+      </c>
+      <c r="F4">
+        <v>9999999</v>
+      </c>
+      <c r="G4">
+        <v>9999999</v>
+      </c>
+      <c r="H4">
+        <v>382762.9</v>
+      </c>
+      <c r="I4">
+        <v>679793.6</v>
+      </c>
+      <c r="J4">
+        <v>9999999</v>
+      </c>
+      <c r="K4">
+        <v>9999999</v>
+      </c>
+      <c r="L4">
+        <v>479917.1</v>
+      </c>
+      <c r="M4">
+        <v>787018</v>
+      </c>
+      <c r="N4">
+        <v>9999999</v>
+      </c>
+      <c r="O4">
+        <v>269179.44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2027</v>
+      </c>
+      <c r="B5">
+        <v>36927.151590000001</v>
+      </c>
+      <c r="C5">
+        <v>52753.073700000001</v>
+      </c>
+      <c r="D5">
+        <v>79129.610549999998</v>
+      </c>
+      <c r="E5">
+        <v>145820</v>
+      </c>
+      <c r="F5">
+        <v>9999999</v>
+      </c>
+      <c r="G5">
+        <v>9999999</v>
+      </c>
+      <c r="H5">
+        <v>382762.9</v>
+      </c>
+      <c r="I5">
+        <v>679793.6</v>
+      </c>
+      <c r="J5">
+        <v>9999999</v>
+      </c>
+      <c r="K5">
+        <v>9999999</v>
+      </c>
+      <c r="L5">
+        <v>479917.1</v>
+      </c>
+      <c r="M5">
+        <v>787018</v>
+      </c>
+      <c r="N5">
+        <v>9999999</v>
+      </c>
+      <c r="O5">
+        <v>263711.78000000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2028</v>
+      </c>
+      <c r="B6">
+        <v>36373.244316149998</v>
+      </c>
+      <c r="C6">
+        <v>51961.777594500003</v>
+      </c>
+      <c r="D6">
+        <v>77942.666391749997</v>
+      </c>
+      <c r="E6">
+        <v>144440</v>
+      </c>
+      <c r="F6">
+        <v>9999999</v>
+      </c>
+      <c r="G6">
+        <v>9999999</v>
+      </c>
+      <c r="H6">
+        <v>382762.9</v>
+      </c>
+      <c r="I6">
+        <v>679793.6</v>
+      </c>
+      <c r="J6">
+        <v>9999999</v>
+      </c>
+      <c r="K6">
+        <v>9999999</v>
+      </c>
+      <c r="L6">
+        <v>479917.1</v>
+      </c>
+      <c r="M6">
+        <v>787018</v>
+      </c>
+      <c r="N6">
+        <v>9999999</v>
+      </c>
+      <c r="O6">
+        <v>258350.32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2029</v>
+      </c>
+      <c r="B7">
+        <v>35827.645651407751</v>
+      </c>
+      <c r="C7">
+        <v>51182.350930582499</v>
+      </c>
+      <c r="D7">
+        <v>76773.526395873749</v>
+      </c>
+      <c r="E7">
+        <v>143060</v>
+      </c>
+      <c r="F7">
+        <v>9999999</v>
+      </c>
+      <c r="G7">
+        <v>9999999</v>
+      </c>
+      <c r="H7">
+        <v>382762.9</v>
+      </c>
+      <c r="I7">
+        <v>679793.6</v>
+      </c>
+      <c r="J7">
+        <v>9999999</v>
+      </c>
+      <c r="K7">
+        <v>9999999</v>
+      </c>
+      <c r="L7">
+        <v>479917.1</v>
+      </c>
+      <c r="M7">
+        <v>787018</v>
+      </c>
+      <c r="N7">
+        <v>9999999</v>
+      </c>
+      <c r="O7">
+        <v>253093.46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2030</v>
+      </c>
+      <c r="B8">
+        <v>35290.230966636635</v>
+      </c>
+      <c r="C8">
+        <v>50414.615666623758</v>
+      </c>
+      <c r="D8">
+        <v>75621.923499935641</v>
+      </c>
+      <c r="E8">
+        <v>141680</v>
+      </c>
+      <c r="F8">
+        <v>9999999</v>
+      </c>
+      <c r="G8">
+        <v>9999999</v>
+      </c>
+      <c r="H8">
+        <v>382762.9</v>
+      </c>
+      <c r="I8">
+        <v>679793.6</v>
+      </c>
+      <c r="J8">
+        <v>9999999</v>
+      </c>
+      <c r="K8">
+        <v>9999999</v>
+      </c>
+      <c r="L8">
+        <v>479917.1</v>
+      </c>
+      <c r="M8">
+        <v>787018</v>
+      </c>
+      <c r="N8">
+        <v>9999999</v>
+      </c>
+      <c r="O8">
+        <v>247939.65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2031</v>
+      </c>
+      <c r="B9">
+        <v>34760.877502137082</v>
+      </c>
+      <c r="C9">
+        <v>49658.396431624402</v>
+      </c>
+      <c r="D9">
+        <v>74487.594647436606</v>
+      </c>
+      <c r="E9">
+        <v>140300</v>
+      </c>
+      <c r="F9">
+        <v>9999999</v>
+      </c>
+      <c r="G9">
+        <v>9999999</v>
+      </c>
+      <c r="H9">
+        <v>382762.9</v>
+      </c>
+      <c r="I9">
+        <v>679793.6</v>
+      </c>
+      <c r="J9">
+        <v>9999999</v>
+      </c>
+      <c r="K9">
+        <v>9999999</v>
+      </c>
+      <c r="L9">
+        <v>479917.1</v>
+      </c>
+      <c r="M9">
+        <v>787018</v>
+      </c>
+      <c r="N9">
+        <v>9999999</v>
+      </c>
+      <c r="O9">
+        <v>242887.37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2032</v>
+      </c>
+      <c r="B10">
+        <v>34239.464339605023</v>
+      </c>
+      <c r="C10">
+        <v>48913.520485150038</v>
+      </c>
+      <c r="D10">
+        <v>73370.280727725054</v>
+      </c>
+      <c r="E10">
+        <v>138920</v>
+      </c>
+      <c r="F10">
+        <v>9999999</v>
+      </c>
+      <c r="G10">
+        <v>9999999</v>
+      </c>
+      <c r="H10">
+        <v>382762.9</v>
+      </c>
+      <c r="I10">
+        <v>679793.6</v>
+      </c>
+      <c r="J10">
+        <v>9999999</v>
+      </c>
+      <c r="K10">
+        <v>9999999</v>
+      </c>
+      <c r="L10">
+        <v>479917.1</v>
+      </c>
+      <c r="M10">
+        <v>787018</v>
+      </c>
+      <c r="N10">
+        <v>9999999</v>
+      </c>
+      <c r="O10">
+        <v>237935.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2033</v>
+      </c>
+      <c r="B11">
+        <v>33725.872374510946</v>
+      </c>
+      <c r="C11">
+        <v>48179.817677872787</v>
+      </c>
+      <c r="D11">
+        <v>72269.726516809184</v>
+      </c>
+      <c r="E11">
+        <v>137540</v>
+      </c>
+      <c r="F11">
+        <v>9999999</v>
+      </c>
+      <c r="G11">
+        <v>9999999</v>
+      </c>
+      <c r="H11">
+        <v>382762.9</v>
+      </c>
+      <c r="I11">
+        <v>679793.6</v>
+      </c>
+      <c r="J11">
+        <v>9999999</v>
+      </c>
+      <c r="K11">
+        <v>9999999</v>
+      </c>
+      <c r="L11">
+        <v>479917.1</v>
+      </c>
+      <c r="M11">
+        <v>787018</v>
+      </c>
+      <c r="N11">
+        <v>9999999</v>
+      </c>
+      <c r="O11">
+        <v>233081.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2034</v>
+      </c>
+      <c r="B12">
+        <v>33219.984288893284</v>
+      </c>
+      <c r="C12">
+        <v>47457.120412704695</v>
+      </c>
+      <c r="D12">
+        <v>71185.68061905705</v>
+      </c>
+      <c r="E12">
+        <v>136160</v>
+      </c>
+      <c r="F12">
+        <v>9999999</v>
+      </c>
+      <c r="G12">
+        <v>9999999</v>
+      </c>
+      <c r="H12">
+        <v>382762.9</v>
+      </c>
+      <c r="I12">
+        <v>679793.6</v>
+      </c>
+      <c r="J12">
+        <v>9999999</v>
+      </c>
+      <c r="K12">
+        <v>9999999</v>
+      </c>
+      <c r="L12">
+        <v>479917.1</v>
+      </c>
+      <c r="M12">
+        <v>787018</v>
+      </c>
+      <c r="N12">
+        <v>9999999</v>
+      </c>
+      <c r="O12">
+        <v>228324.82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2035</v>
+      </c>
+      <c r="B13">
+        <v>32721.684524559885</v>
+      </c>
+      <c r="C13">
+        <v>46745.263606514127</v>
+      </c>
+      <c r="D13">
+        <v>70117.895409771198</v>
+      </c>
+      <c r="E13">
+        <v>134780</v>
+      </c>
+      <c r="F13">
+        <v>9999999</v>
+      </c>
+      <c r="G13">
+        <v>9999999</v>
+      </c>
+      <c r="H13">
+        <v>382762.9</v>
+      </c>
+      <c r="I13">
+        <v>679793.6</v>
+      </c>
+      <c r="J13">
+        <v>9999999</v>
+      </c>
+      <c r="K13">
+        <v>9999999</v>
+      </c>
+      <c r="L13">
+        <v>479917.1</v>
+      </c>
+      <c r="M13">
+        <v>787018</v>
+      </c>
+      <c r="N13">
+        <v>9999999</v>
+      </c>
+      <c r="O13">
+        <v>223663.91</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2036</v>
+      </c>
+      <c r="B14">
+        <v>32230.859256691485</v>
+      </c>
+      <c r="C14">
+        <v>46044.084652416415</v>
+      </c>
+      <c r="D14">
+        <v>69066.126978624627</v>
+      </c>
+      <c r="E14">
+        <v>133400</v>
+      </c>
+      <c r="F14">
+        <v>9999999</v>
+      </c>
+      <c r="G14">
+        <v>9999999</v>
+      </c>
+      <c r="H14">
+        <v>382762.9</v>
+      </c>
+      <c r="I14">
+        <v>679793.6</v>
+      </c>
+      <c r="J14">
+        <v>9999999</v>
+      </c>
+      <c r="K14">
+        <v>9999999</v>
+      </c>
+      <c r="L14">
+        <v>479917.1</v>
+      </c>
+      <c r="M14">
+        <v>787018</v>
+      </c>
+      <c r="N14">
+        <v>9999999</v>
+      </c>
+      <c r="O14">
+        <v>219097.32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2037</v>
+      </c>
+      <c r="B15">
+        <v>31747.396367841113</v>
+      </c>
+      <c r="C15">
+        <v>45353.423382630172</v>
+      </c>
+      <c r="D15">
+        <v>68030.135073945261</v>
+      </c>
+      <c r="E15">
+        <v>132020</v>
+      </c>
+      <c r="F15">
+        <v>9999999</v>
+      </c>
+      <c r="G15">
+        <v>9999999</v>
+      </c>
+      <c r="H15">
+        <v>382762.9</v>
+      </c>
+      <c r="I15">
+        <v>679793.6</v>
+      </c>
+      <c r="J15">
+        <v>9999999</v>
+      </c>
+      <c r="K15">
+        <v>9999999</v>
+      </c>
+      <c r="L15">
+        <v>479917.1</v>
+      </c>
+      <c r="M15">
+        <v>787018</v>
+      </c>
+      <c r="N15">
+        <v>9999999</v>
+      </c>
+      <c r="O15">
+        <v>214623.65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2038</v>
+      </c>
+      <c r="B16">
+        <v>31271.185422323495</v>
+      </c>
+      <c r="C16">
+        <v>44673.122031890722</v>
+      </c>
+      <c r="D16">
+        <v>67009.683047836079</v>
+      </c>
+      <c r="E16">
+        <v>130640</v>
+      </c>
+      <c r="F16">
+        <v>9999999</v>
+      </c>
+      <c r="G16">
+        <v>9999999</v>
+      </c>
+      <c r="H16">
+        <v>382762.9</v>
+      </c>
+      <c r="I16">
+        <v>679793.6</v>
+      </c>
+      <c r="J16">
+        <v>9999999</v>
+      </c>
+      <c r="K16">
+        <v>9999999</v>
+      </c>
+      <c r="L16">
+        <v>479917.1</v>
+      </c>
+      <c r="M16">
+        <v>787018</v>
+      </c>
+      <c r="N16">
+        <v>9999999</v>
+      </c>
+      <c r="O16">
+        <v>210241.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>2039</v>
+      </c>
+      <c r="B17">
+        <v>30802.117640988643</v>
+      </c>
+      <c r="C17">
+        <v>44003.025201412362</v>
+      </c>
+      <c r="D17">
+        <v>66004.537802118532</v>
+      </c>
+      <c r="E17">
+        <v>129260</v>
+      </c>
+      <c r="F17">
+        <v>9999999</v>
+      </c>
+      <c r="G17">
+        <v>9999999</v>
+      </c>
+      <c r="H17">
+        <v>382762.9</v>
+      </c>
+      <c r="I17">
+        <v>679793.6</v>
+      </c>
+      <c r="J17">
+        <v>9999999</v>
+      </c>
+      <c r="K17">
+        <v>9999999</v>
+      </c>
+      <c r="L17">
+        <v>479917.1</v>
+      </c>
+      <c r="M17">
+        <v>787018</v>
+      </c>
+      <c r="N17">
+        <v>9999999</v>
+      </c>
+      <c r="O17">
+        <v>205949.84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>2040</v>
+      </c>
+      <c r="B18">
+        <v>30340.085876373814</v>
+      </c>
+      <c r="C18">
+        <v>43342.979823391179</v>
+      </c>
+      <c r="D18">
+        <v>65014.46973508675</v>
+      </c>
+      <c r="E18">
+        <v>127880</v>
+      </c>
+      <c r="F18">
+        <v>9999999</v>
+      </c>
+      <c r="G18">
+        <v>9999999</v>
+      </c>
+      <c r="H18">
+        <v>382762.9</v>
+      </c>
+      <c r="I18">
+        <v>679793.6</v>
+      </c>
+      <c r="J18">
+        <v>9999999</v>
+      </c>
+      <c r="K18">
+        <v>9999999</v>
+      </c>
+      <c r="L18">
+        <v>479917.1</v>
+      </c>
+      <c r="M18">
+        <v>787018</v>
+      </c>
+      <c r="N18">
+        <v>9999999</v>
+      </c>
+      <c r="O18">
+        <v>201747.12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2041</v>
+      </c>
+      <c r="B19">
+        <v>29884.984588228206</v>
+      </c>
+      <c r="C19">
+        <v>42692.835126040307</v>
+      </c>
+      <c r="D19">
+        <v>64039.252689060449</v>
+      </c>
+      <c r="E19">
+        <v>126500</v>
+      </c>
+      <c r="F19">
+        <v>9999999</v>
+      </c>
+      <c r="G19">
+        <v>9999999</v>
+      </c>
+      <c r="H19">
+        <v>382762.9</v>
+      </c>
+      <c r="I19">
+        <v>679793.6</v>
+      </c>
+      <c r="J19">
+        <v>9999999</v>
+      </c>
+      <c r="K19">
+        <v>9999999</v>
+      </c>
+      <c r="L19">
+        <v>479917.1</v>
+      </c>
+      <c r="M19">
+        <v>787018</v>
+      </c>
+      <c r="N19">
+        <v>9999999</v>
+      </c>
+      <c r="O19">
+        <v>197632.19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>2042</v>
+      </c>
+      <c r="B20">
+        <v>29436.709819404783</v>
+      </c>
+      <c r="C20">
+        <v>42052.442599149705</v>
+      </c>
+      <c r="D20">
+        <v>63078.663898724539</v>
+      </c>
+      <c r="E20">
+        <v>125120</v>
+      </c>
+      <c r="F20">
+        <v>9999999</v>
+      </c>
+      <c r="G20">
+        <v>9999999</v>
+      </c>
+      <c r="H20">
+        <v>382762.9</v>
+      </c>
+      <c r="I20">
+        <v>679793.6</v>
+      </c>
+      <c r="J20">
+        <v>9999999</v>
+      </c>
+      <c r="K20">
+        <v>9999999</v>
+      </c>
+      <c r="L20">
+        <v>479917.1</v>
+      </c>
+      <c r="M20">
+        <v>787018</v>
+      </c>
+      <c r="N20">
+        <v>9999999</v>
+      </c>
+      <c r="O20">
+        <v>193603.83</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>2043</v>
+      </c>
+      <c r="B21">
+        <v>28995.159172113712</v>
+      </c>
+      <c r="C21">
+        <v>41421.655960162461</v>
+      </c>
+      <c r="D21">
+        <v>62132.48394024367</v>
+      </c>
+      <c r="E21">
+        <v>123740</v>
+      </c>
+      <c r="F21">
+        <v>9999999</v>
+      </c>
+      <c r="G21">
+        <v>9999999</v>
+      </c>
+      <c r="H21">
+        <v>382762.9</v>
+      </c>
+      <c r="I21">
+        <v>679793.6</v>
+      </c>
+      <c r="J21">
+        <v>9999999</v>
+      </c>
+      <c r="K21">
+        <v>9999999</v>
+      </c>
+      <c r="L21">
+        <v>479917.1</v>
+      </c>
+      <c r="M21">
+        <v>787018</v>
+      </c>
+      <c r="N21">
+        <v>9999999</v>
+      </c>
+      <c r="O21">
+        <v>189660.87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>2044</v>
+      </c>
+      <c r="B22">
+        <v>28560.231784532007</v>
+      </c>
+      <c r="C22">
+        <v>40800.331120760027</v>
+      </c>
+      <c r="D22">
+        <v>61200.496681140015</v>
+      </c>
+      <c r="E22">
+        <v>122360</v>
+      </c>
+      <c r="F22">
+        <v>9999999</v>
+      </c>
+      <c r="G22">
+        <v>9999999</v>
+      </c>
+      <c r="H22">
+        <v>382762.9</v>
+      </c>
+      <c r="I22">
+        <v>679793.6</v>
+      </c>
+      <c r="J22">
+        <v>9999999</v>
+      </c>
+      <c r="K22">
+        <v>9999999</v>
+      </c>
+      <c r="L22">
+        <v>479917.1</v>
+      </c>
+      <c r="M22">
+        <v>787018</v>
+      </c>
+      <c r="N22">
+        <v>9999999</v>
+      </c>
+      <c r="O22">
+        <v>185802.14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>2045</v>
+      </c>
+      <c r="B23">
+        <v>28131.828307764026</v>
+      </c>
+      <c r="C23">
+        <v>40188.326153948627</v>
+      </c>
+      <c r="D23">
+        <v>60282.489230922911</v>
+      </c>
+      <c r="E23">
+        <v>120980</v>
+      </c>
+      <c r="F23">
+        <v>9999999</v>
+      </c>
+      <c r="G23">
+        <v>9999999</v>
+      </c>
+      <c r="H23">
+        <v>382762.9</v>
+      </c>
+      <c r="I23">
+        <v>679793.6</v>
+      </c>
+      <c r="J23">
+        <v>9999999</v>
+      </c>
+      <c r="K23">
+        <v>9999999</v>
+      </c>
+      <c r="L23">
+        <v>479917.1</v>
+      </c>
+      <c r="M23">
+        <v>787018</v>
+      </c>
+      <c r="N23">
+        <v>9999999</v>
+      </c>
+      <c r="O23">
+        <v>182026.51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>2046</v>
+      </c>
+      <c r="B24">
+        <v>27709.850883147566</v>
+      </c>
+      <c r="C24">
+        <v>39585.501261639394</v>
+      </c>
+      <c r="D24">
+        <v>59378.251892459069</v>
+      </c>
+      <c r="E24">
+        <v>119600</v>
+      </c>
+      <c r="F24">
+        <v>9999999</v>
+      </c>
+      <c r="G24">
+        <v>9999999</v>
+      </c>
+      <c r="H24">
+        <v>382762.9</v>
+      </c>
+      <c r="I24">
+        <v>679793.6</v>
+      </c>
+      <c r="J24">
+        <v>9999999</v>
+      </c>
+      <c r="K24">
+        <v>9999999</v>
+      </c>
+      <c r="L24">
+        <v>479917.1</v>
+      </c>
+      <c r="M24">
+        <v>787018</v>
+      </c>
+      <c r="N24">
+        <v>9999999</v>
+      </c>
+      <c r="O24">
+        <v>178332.87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2047</v>
+      </c>
+      <c r="B25">
+        <v>27294.203119900354</v>
+      </c>
+      <c r="C25">
+        <v>38991.718742714802</v>
+      </c>
+      <c r="D25">
+        <v>58487.578114072181</v>
+      </c>
+      <c r="E25">
+        <v>118220</v>
+      </c>
+      <c r="F25">
+        <v>9999999</v>
+      </c>
+      <c r="G25">
+        <v>9999999</v>
+      </c>
+      <c r="H25">
+        <v>382762.9</v>
+      </c>
+      <c r="I25">
+        <v>679793.6</v>
+      </c>
+      <c r="J25">
+        <v>9999999</v>
+      </c>
+      <c r="K25">
+        <v>9999999</v>
+      </c>
+      <c r="L25">
+        <v>479917.1</v>
+      </c>
+      <c r="M25">
+        <v>787018</v>
+      </c>
+      <c r="N25">
+        <v>9999999</v>
+      </c>
+      <c r="O25">
+        <v>174720.11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>2048</v>
+      </c>
+      <c r="B26">
+        <v>26884.790073101849</v>
+      </c>
+      <c r="C26">
+        <v>38406.842961574082</v>
+      </c>
+      <c r="D26">
+        <v>57610.264442361098</v>
+      </c>
+      <c r="E26">
+        <v>116840</v>
+      </c>
+      <c r="F26">
+        <v>9999999</v>
+      </c>
+      <c r="G26">
+        <v>9999999</v>
+      </c>
+      <c r="H26">
+        <v>382762.9</v>
+      </c>
+      <c r="I26">
+        <v>679793.6</v>
+      </c>
+      <c r="J26">
+        <v>9999999</v>
+      </c>
+      <c r="K26">
+        <v>9999999</v>
+      </c>
+      <c r="L26">
+        <v>479917.1</v>
+      </c>
+      <c r="M26">
+        <v>787018</v>
+      </c>
+      <c r="N26">
+        <v>9999999</v>
+      </c>
+      <c r="O26">
+        <v>171187.17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>2049</v>
+      </c>
+      <c r="B27">
+        <v>26481.518222005321</v>
+      </c>
+      <c r="C27">
+        <v>37830.74031715047</v>
+      </c>
+      <c r="D27">
+        <v>56746.110475725684</v>
+      </c>
+      <c r="E27">
+        <v>115460</v>
+      </c>
+      <c r="F27">
+        <v>9999999</v>
+      </c>
+      <c r="G27">
+        <v>9999999</v>
+      </c>
+      <c r="H27">
+        <v>382762.9</v>
+      </c>
+      <c r="I27">
+        <v>679793.6</v>
+      </c>
+      <c r="J27">
+        <v>9999999</v>
+      </c>
+      <c r="K27">
+        <v>9999999</v>
+      </c>
+      <c r="L27">
+        <v>479917.1</v>
+      </c>
+      <c r="M27">
+        <v>787018</v>
+      </c>
+      <c r="N27">
+        <v>9999999</v>
+      </c>
+      <c r="O27">
+        <v>167732.98000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>2050</v>
+      </c>
+      <c r="B28">
+        <v>26084.295448675242</v>
+      </c>
+      <c r="C28">
+        <v>37263.279212393216</v>
+      </c>
+      <c r="D28">
+        <v>55894.918818589795</v>
+      </c>
+      <c r="E28">
+        <v>114080</v>
+      </c>
+      <c r="F28">
+        <v>9999999</v>
+      </c>
+      <c r="G28">
+        <v>9999999</v>
+      </c>
+      <c r="H28">
+        <v>382762.9</v>
+      </c>
+      <c r="I28">
+        <v>679793.6</v>
+      </c>
+      <c r="J28">
+        <v>9999999</v>
+      </c>
+      <c r="K28">
+        <v>9999999</v>
+      </c>
+      <c r="L28">
+        <v>479917.1</v>
+      </c>
+      <c r="M28">
+        <v>787018</v>
+      </c>
+      <c r="N28">
+        <v>9999999</v>
+      </c>
+      <c r="O28">
+        <v>164356.51999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B33" s="17"/>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="G34" s="16"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Added Excel Long Fomrat for standard Data and cleaned repo
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1372" documentId="13_ncr:1_{A1CEE875-B6E7-4616-ADB8-CAA4FD821F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DDDAFC0-16ED-4EDE-85EF-DEE291449E41}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="15" activeTab="19" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-28920" yWindow="5115" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -1020,10 +1020,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -2785,6 +2781,26 @@
   </sheetData>
   <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -2792,26 +2808,6 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>